<commit_message>
US03: documentação (requisitos, use case, BPMN, prompt), estado e backlog
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E9QzPgdcfwB8xR8d5sAuMb
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -174,31 +174,29 @@
 • Páginas privadas redirecionam para o login.</t>
   </si>
   <si>
+    <t xml:space="preserve">Código, testes e documentação no GitHub (PR #4 e #5 aceites, com o ícone para mostrar a palavra-passe).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perfis de aluno e administrador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como administrador, quero ter uma conta própria, separada das contas dos alunos e numa área escondida, para gerir a aplicação sem que os alunos vejam ou consigam usar essas funções.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Os administradores têm contas próprias (nome de utilizador, sem email), separadas dos alunos.
+• O primeiro administrador é criado no terminal (flask --app app create-admin).
+• A gestão tem início de sessão próprio, com mensagem genérica.
+• A área de gestão está escondida: sem ligações nas páginas dos alunos e com endereço configurável.
+• Um administrador cria e remove outros administradores (não a si próprio).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Em curso</t>
   </si>
   <si>
-    <t xml:space="preserve">Feita; em revisão no GitHub (PR #4 e PR #5, ícone para mostrar a palavra-passe).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perfis de aluno e administrador</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como administrador, quero ter um perfil próprio, distinto do perfil de aluno, para gerir o catálogo e os períodos sem dar essas permissões aos alunos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Quem se regista fica com o perfil Aluno.
-• Um administrador é criado por comando (flask --app app promote-admin &lt;email&gt;), sobre uma conta já confirmada.
-• As páginas de administração só abrem para administradores; um aluno recebe «sem permissão».
-• A barra do topo mostra as opções conforme o perfil.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Por fazer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 07/10: story nova. O RF04 não tinha story e a importação do catálogo (US04) precisa de um administrador.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: story nova (o RF04 não tinha story). Revista pelo PO: administradores independentes e área escondida (3 → 5 SP). Feita; em revisão no GitHub (PR #7).</t>
   </si>
   <si>
     <t xml:space="preserve">—</t>
@@ -222,6 +220,9 @@
   </si>
   <si>
     <t xml:space="preserve">Sprint 2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por fazer</t>
   </si>
   <si>
     <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2.</t>
@@ -967,16 +968,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1000,7 +1005,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1008,11 +1013,11 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1044,7 +1049,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1056,11 +1061,11 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1085,7 +1090,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="22">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1228,20 +1233,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFEDEDED"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDDEBF7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFE2EFDA"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1398,22 +1389,26 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
@@ -1448,7 +1443,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>8</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>24</c:v>
@@ -1488,22 +1483,26 @@
           <c:invertIfNegative val="0"/>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
@@ -1538,7 +1537,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>3</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1555,17 +1554,17 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="92672184"/>
-        <c:axId val="51052424"/>
+        <c:axId val="1302559"/>
+        <c:axId val="55718072"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="92672184"/>
+        <c:axId val="1302559"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1590,7 +1589,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="51052424"/>
+        <c:crossAx val="55718072"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1598,7 +1597,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="51052424"/>
+        <c:axId val="55718072"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1638,7 +1637,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1663,7 +1662,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="92672184"/>
+        <c:crossAx val="1302559"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1730,9 +1729,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2094480</xdr:colOff>
+      <xdr:colOff>2094120</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>91440</xdr:rowOff>
+      <xdr:rowOff>91080</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1740,8 +1739,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="775440" y="4000680"/>
-        <a:ext cx="5759640" cy="2519640"/>
+        <a:off x="775440" y="3992040"/>
+        <a:ext cx="5759280" cy="2518920"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1937,1164 +1936,1164 @@
   <dimension ref="A1:M36"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="24"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="9" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="1" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="10"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="3" t="s">
+      <c r="H4" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="3" t="s">
+      <c r="I4" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="J4" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="3" t="s">
+      <c r="K4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="L4" s="3" t="s">
+      <c r="L4" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="M4" s="3" t="s">
+      <c r="M4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="F5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="G5" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="I5" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="J5" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="K5" s="7"/>
-      <c r="L5" s="7" t="s">
+      <c r="K5" s="8"/>
+      <c r="L5" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="M5" s="4" t="s">
+      <c r="M5" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4" t="n">
+      <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="C6" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E6" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="F6" s="5" t="s">
+      <c r="F6" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="G6" s="6" t="n">
+      <c r="G6" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="H6" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="6" t="s">
+      <c r="I6" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="J6" s="6" t="s">
+      <c r="J6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="K6" s="8"/>
+      <c r="L6" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="K6" s="7"/>
-      <c r="L6" s="7" t="s">
+      <c r="M6" s="5" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="M6" s="4" t="s">
+      <c r="C7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="K7" s="8"/>
+      <c r="L7" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="G8" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I8" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="J8" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K8" s="8"/>
+      <c r="L8" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="M8" s="5" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="G9" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="J9" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K9" s="8"/>
+      <c r="L9" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="M9" s="5" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="G10" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H10" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I10" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="J10" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K10" s="8"/>
+      <c r="L10" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="M10" s="5" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I11" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="J11" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K11" s="8"/>
+      <c r="L11" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="M11" s="5" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="G12" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I12" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="J12" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K12" s="8"/>
+      <c r="L12" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="M12" s="5" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H13" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I13" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="J13" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K13" s="8"/>
+      <c r="L13" s="8"/>
+      <c r="M13" s="5" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="G14" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H14" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I14" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="J14" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K14" s="8"/>
+      <c r="L14" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="M14" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G15" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I15" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="J15" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K15" s="8"/>
+      <c r="L15" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="M15" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="G16" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I16" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="J16" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K16" s="8"/>
+      <c r="L16" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="M16" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G17" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="J17" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K17" s="8"/>
+      <c r="L17" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="M17" s="5" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="G18" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I18" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="J18" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K18" s="8"/>
+      <c r="L18" s="8"/>
+      <c r="M18" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="G19" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I19" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="J19" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K19" s="8"/>
+      <c r="L19" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="M19" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="G20" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H20" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="I20" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="J20" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K20" s="8"/>
+      <c r="L20" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="M20" s="5" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="G21" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="I21" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="J21" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K21" s="8"/>
+      <c r="L21" s="8"/>
+      <c r="M21" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="G22" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="J22" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K22" s="8"/>
+      <c r="L22" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="M22" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="G23" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H23" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="J23" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K23" s="8"/>
+      <c r="L23" s="8"/>
+      <c r="M23" s="5" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="G24" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>97</v>
+      </c>
+      <c r="J24" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K24" s="8"/>
+      <c r="L24" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="M24" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="5" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H25" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="I25" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="J25" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K25" s="8"/>
+      <c r="L25" s="8" t="s">
+        <v>127</v>
+      </c>
+      <c r="M25" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="G26" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H26" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="J26" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K26" s="8"/>
+      <c r="L26" s="8" t="s">
+        <v>133</v>
+      </c>
+      <c r="M26" s="5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="J27" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K27" s="8"/>
+      <c r="L27" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="M27" s="5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="n">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
+      <c r="B28" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="E28" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="F28" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="G28" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G7" s="6" t="n">
+      <c r="H28" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="J28" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K28" s="8"/>
+      <c r="L28" s="8"/>
+      <c r="M28" s="5" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="G29" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="H7" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="J7" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K7" s="7"/>
-      <c r="L7" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="M7" s="4" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="G8" s="6" t="n">
+      <c r="H29" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="J29" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K29" s="8"/>
+      <c r="L29" s="8"/>
+      <c r="M29" s="5" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="E30" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="G30" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H8" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" s="6" t="s">
+      <c r="H30" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="J30" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="J8" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K8" s="7"/>
-      <c r="L8" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="M8" s="4" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="4" t="n">
+      <c r="K30" s="8"/>
+      <c r="L30" s="8"/>
+      <c r="M30" s="5" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="G31" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="H31" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="J31" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K31" s="8"/>
+      <c r="L31" s="8"/>
+      <c r="M31" s="5" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="E32" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="F32" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="G32" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H32" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="I32" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="J32" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="K32" s="8"/>
+      <c r="L32" s="8"/>
+      <c r="M32" s="5" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F34" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="G34" s="9" t="n">
+        <f aca="false">SUM(G5:G32)</f>
+        <v>109</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F35" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="G35" s="9" t="n">
+        <f aca="false">SUMIF(J5:J32,"Feito",G5:G32)</f>
         <v>5</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="G9" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="J9" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K9" s="7"/>
-      <c r="L9" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="M9" s="4" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C10" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I10" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="J10" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K10" s="7"/>
-      <c r="L10" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="M10" s="4" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="G11" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I11" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="J11" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K11" s="7"/>
-      <c r="L11" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="M11" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="G12" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I12" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="J12" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K12" s="7"/>
-      <c r="L12" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="M12" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="G13" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I13" s="6" t="s">
-        <v>42</v>
-      </c>
-      <c r="J13" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7"/>
-      <c r="M13" s="4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="G14" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I14" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="J14" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K14" s="7"/>
-      <c r="L14" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="M14" s="4" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="n">
-        <v>11</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="G15" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="J15" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="M15" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="4" t="n">
-        <v>12</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="D16" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="F16" s="5" t="s">
-        <v>82</v>
-      </c>
-      <c r="G16" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="J16" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K16" s="7"/>
-      <c r="L16" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="M16" s="4" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="n">
-        <v>13</v>
-      </c>
-      <c r="B17" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="G17" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="H17" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I17" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="J17" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K17" s="7"/>
-      <c r="L17" s="7" t="s">
-        <v>72</v>
-      </c>
-      <c r="M17" s="4" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="4" t="n">
-        <v>14</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="C18" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>92</v>
-      </c>
-      <c r="F18" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="G18" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="H18" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I18" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="J18" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K18" s="7"/>
-      <c r="L18" s="7"/>
-      <c r="M18" s="4" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="C19" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D19" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="G19" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="H19" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="I19" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="J19" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K19" s="7"/>
-      <c r="L19" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="M19" s="4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="B20" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D20" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="E20" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="G20" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H20" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="I20" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="J20" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K20" s="7"/>
-      <c r="L20" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="M20" s="4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="B21" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="C21" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="E21" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="F21" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="G21" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H21" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="I21" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="J21" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K21" s="7"/>
-      <c r="L21" s="7"/>
-      <c r="M21" s="4" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="F22" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="G22" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H22" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="I22" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="J22" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K22" s="7"/>
-      <c r="L22" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="M22" s="4" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="4" t="n">
-        <v>19</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="C23" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="F23" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="G23" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H23" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="I23" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="J23" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K23" s="7"/>
-      <c r="L23" s="7"/>
-      <c r="M23" s="4" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="B24" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="C24" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="E24" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="G24" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="H24" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="I24" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="J24" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K24" s="7"/>
-      <c r="L24" s="7" t="s">
-        <v>98</v>
-      </c>
-      <c r="M24" s="4" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="n">
-        <v>21</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="F25" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="G25" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="H25" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="I25" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J25" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K25" s="7"/>
-      <c r="L25" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="M25" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="n">
-        <v>22</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="C26" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="D26" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="E26" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="F26" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="G26" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H26" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="I26" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J26" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K26" s="7"/>
-      <c r="L26" s="7" t="s">
-        <v>133</v>
-      </c>
-      <c r="M26" s="4" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D27" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="E27" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="F27" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="G27" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H27" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="I27" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J27" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K27" s="7"/>
-      <c r="L27" s="7" t="s">
-        <v>139</v>
-      </c>
-      <c r="M27" s="4" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="B28" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="C28" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>141</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="G28" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H28" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="I28" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J28" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K28" s="7"/>
-      <c r="L28" s="7"/>
-      <c r="M28" s="4" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>143</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="F29" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="G29" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H29" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="I29" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J29" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K29" s="7"/>
-      <c r="L29" s="7"/>
-      <c r="M29" s="4" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="4" t="n">
-        <v>26</v>
-      </c>
-      <c r="B30" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="D30" s="5" t="s">
-        <v>147</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="F30" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="G30" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="H30" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="I30" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J30" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K30" s="7"/>
-      <c r="L30" s="7"/>
-      <c r="M30" s="4" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="4" t="n">
-        <v>27</v>
-      </c>
-      <c r="B31" s="4" t="s">
-        <v>150</v>
-      </c>
-      <c r="C31" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="F31" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="G31" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="H31" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="I31" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J31" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K31" s="7"/>
-      <c r="L31" s="7"/>
-      <c r="M31" s="4" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="B32" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="E32" s="5" t="s">
-        <v>156</v>
-      </c>
-      <c r="F32" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="G32" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="H32" s="4" t="s">
-        <v>158</v>
-      </c>
-      <c r="I32" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="J32" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="K32" s="7"/>
-      <c r="L32" s="7"/>
-      <c r="M32" s="4" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F34" s="8" t="s">
-        <v>159</v>
-      </c>
-      <c r="G34" s="8" t="n">
-        <f aca="false">SUM(G5:G32)</f>
-        <v>107</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F35" s="8" t="s">
-        <v>160</v>
-      </c>
-      <c r="G35" s="8" t="n">
-        <f aca="false">SUMIF(J5:J32,"Feito",G5:G32)</f>
-        <v>3</v>
-      </c>
     </row>
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F36" s="9" t="s">
+      <c r="F36" s="10" t="s">
         <v>161</v>
       </c>
     </row>
@@ -3123,19 +3122,19 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5:I32">
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Sprint 1"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>"Sprint 2"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"Sprint 3"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="22">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
       <formula>"Sprint 4"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="23">
+    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
       <formula>"Backlog"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3177,275 +3176,275 @@
   <dimension ref="A1:H36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="10"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="11" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="12" t="s">
         <v>164</v>
       </c>
-      <c r="C3" s="6" t="n">
+      <c r="C3" s="7" t="n">
         <v>23</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="D5" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="E5" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G5" s="4" t="s">
         <v>170</v>
       </c>
-      <c r="H5" s="3" t="s">
+      <c r="H5" s="4" t="s">
         <v>171</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="14" t="s">
         <v>172</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$32,$A6,'Product Backlog'!$G$5:$G$32)</f>
-        <v>8</v>
-      </c>
-      <c r="E6" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$32,'Product Backlog'!$I$5:$I$32,$A6,'Product Backlog'!$J$5:$J$32,"Feito")</f>
-        <v>3</v>
-      </c>
-      <c r="F6" s="14" t="n">
+        <v>5</v>
+      </c>
+      <c r="F6" s="15" t="n">
         <f aca="false">IF(D6=0,0,E6/D6)</f>
-        <v>0.375</v>
-      </c>
-      <c r="G6" s="15" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G6" s="16" t="n">
         <f aca="false">$C$3-D6</f>
-        <v>15</v>
-      </c>
-      <c r="H6" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="H6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$32,$A6)</f>
         <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="B7" s="13" t="s">
+      <c r="A7" s="17" t="s">
+        <v>41</v>
+      </c>
+      <c r="B7" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="C7" s="13" t="s">
+      <c r="C7" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$32,$A7,'Product Backlog'!$G$5:$G$32)</f>
         <v>24</v>
       </c>
-      <c r="E7" s="4" t="n">
+      <c r="E7" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$32,'Product Backlog'!$I$5:$I$32,$A7,'Product Backlog'!$J$5:$J$32,"Feito")</f>
         <v>0</v>
       </c>
-      <c r="F7" s="14" t="n">
+      <c r="F7" s="15" t="n">
         <f aca="false">IF(D7=0,0,E7/D7)</f>
         <v>0</v>
       </c>
-      <c r="G7" s="15" t="n">
+      <c r="G7" s="16" t="n">
         <f aca="false">$C$3-D7</f>
         <v>-1</v>
       </c>
-      <c r="H7" s="4" t="n">
+      <c r="H7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$32,$A7)</f>
         <v>6</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="14" t="s">
         <v>176</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="C8" s="14" t="s">
         <v>177</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$32,$A8,'Product Backlog'!$G$5:$G$32)</f>
         <v>23</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$32,'Product Backlog'!$I$5:$I$32,$A8,'Product Backlog'!$J$5:$J$32,"Feito")</f>
         <v>0</v>
       </c>
-      <c r="F8" s="14" t="n">
+      <c r="F8" s="15" t="n">
         <f aca="false">IF(D8=0,0,E8/D8)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="15" t="n">
+      <c r="G8" s="16" t="n">
         <f aca="false">$C$3-D8</f>
         <v>0</v>
       </c>
-      <c r="H8" s="4" t="n">
+      <c r="H8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$32,$A8)</f>
         <v>5</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="18" t="s">
+      <c r="A9" s="19" t="s">
         <v>97</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="14" t="s">
         <v>178</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="14" t="s">
         <v>179</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$32,$A9,'Product Backlog'!$G$5:$G$32)</f>
         <v>19</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$32,'Product Backlog'!$I$5:$I$32,$A9,'Product Backlog'!$J$5:$J$32,"Feito")</f>
         <v>0</v>
       </c>
-      <c r="F9" s="14" t="n">
+      <c r="F9" s="15" t="n">
         <f aca="false">IF(D9=0,0,E9/D9)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="15" t="n">
+      <c r="G9" s="16" t="n">
         <f aca="false">$C$3-D9</f>
         <v>4</v>
       </c>
-      <c r="H9" s="4" t="n">
+      <c r="H9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$32,$A9)</f>
         <v>6</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="4" t="s">
+      <c r="A10" s="5" t="s">
         <v>126</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="14" t="s">
         <v>181</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$32,$A10,'Product Backlog'!$G$5:$G$32)</f>
         <v>33</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$32,'Product Backlog'!$I$5:$I$32,$A10,'Product Backlog'!$J$5:$J$32,"Feito")</f>
         <v>0</v>
       </c>
-      <c r="F10" s="14" t="n">
+      <c r="F10" s="15" t="n">
         <f aca="false">IF(D10=0,0,E10/D10)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="H10" s="4" t="n">
+      <c r="G10" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="H10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$32,$A10)</f>
         <v>8</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="20" t="s">
         <v>182</v>
       </c>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="20" t="n">
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="21" t="n">
         <f aca="false">SUM(D6:D10)</f>
-        <v>107</v>
-      </c>
-      <c r="E11" s="20" t="n">
+        <v>109</v>
+      </c>
+      <c r="E11" s="21" t="n">
         <f aca="false">SUM(E6:E10)</f>
-        <v>3</v>
-      </c>
-      <c r="F11" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F11" s="22" t="n">
         <f aca="false">IF(D11=0,0,E11/D11)</f>
-        <v>0.0280373831775701</v>
-      </c>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20" t="n">
+        <v>0.0458715596330275</v>
+      </c>
+      <c r="G11" s="21"/>
+      <c r="H11" s="21" t="n">
         <f aca="false">SUM(H6:H10)</f>
         <v>28</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="22" t="s">
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="23" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="23" t="s">
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="24" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="23" t="s">
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="24" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="23" t="s">
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="24" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="23" t="s">
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="24" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="23" t="s">
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="24" t="s">
         <v>188</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="23" t="s">
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="24" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="23" t="s">
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="24" t="s">
         <v>190</v>
       </c>
     </row>
@@ -3470,126 +3469,126 @@
   <dimension ref="A1:E9"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="42"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="42"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>191</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+    <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>171</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="D4" s="4" t="s">
         <v>194</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="E4" s="4" t="s">
         <v>195</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="24" t="s">
+    <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="25" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>196</v>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$32,A5)</f>
         <v>15</v>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$H$5:$H$32,A5,'Product Backlog'!$G$5:$G$32)</f>
-        <v>60</v>
-      </c>
-      <c r="E5" s="14" t="n">
+        <v>62</v>
+      </c>
+      <c r="E5" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D5/SUM($D$5:$D$8))</f>
-        <v>0.560747663551402</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
+        <v>0.568807339449541</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="13" t="s">
         <v>105</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>197</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$32,A6)</f>
         <v>7</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$H$5:$H$32,A6,'Product Backlog'!$G$5:$G$32)</f>
         <v>22</v>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="E6" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D6/SUM($D$5:$D$8))</f>
-        <v>0.205607476635514</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
+        <v>0.201834862385321</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="17" t="s">
         <v>138</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$32,A7)</f>
         <v>5</v>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$H$5:$H$32,A7,'Product Backlog'!$G$5:$G$32)</f>
         <v>22</v>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="E7" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D7/SUM($D$5:$D$8))</f>
-        <v>0.205607476635514</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="25" t="s">
+        <v>0.201834862385321</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="26" t="s">
         <v>158</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="C8" s="4" t="n">
+      <c r="C8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$32,A8)</f>
         <v>1</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$H$5:$H$32,A8,'Product Backlog'!$G$5:$G$32)</f>
         <v>3</v>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="E8" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D8/SUM($D$5:$D$8))</f>
-        <v>0.0280373831775701</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="s">
+        <v>0.0275229357798165</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="C9" s="26" t="n">
+      <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>
         <v>28</v>
       </c>
-      <c r="D9" s="26" t="n">
+      <c r="D9" s="27" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fechar o Sprint 1: US02 e US03 concluídas
Estado das stories no README, em docs/US02 e docs/US03 e no Product
Backlog (Sprint 1: 10 de 10 SP).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E9QzPgdcfwB8xR8d5sAuMb
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="199">
   <si>
     <t xml:space="preserve">Product Backlog — Recomendador de UCs Opcionais</t>
   </si>
@@ -193,10 +193,7 @@
 • Um administrador cria e remove outros administradores (não a si próprio).</t>
   </si>
   <si>
-    <t xml:space="preserve">Em curso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 07/10: story nova (o RF04 não tinha story). Revista pelo PO: administradores independentes e área escondida (3 → 5 SP). Feita; em revisão no GitHub (PR #7).</t>
+    <t xml:space="preserve">Replaneamento de 07/10: story nova (o RF04 não tinha story). Revista pelos PO: administradores independentes e área escondida (3 → 5 SP). Código, testes e documentação no GitHub (PR #7 aceite).</t>
   </si>
   <si>
     <t xml:space="preserve">—</t>
@@ -1090,7 +1087,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="22">
+  <dxfs count="21">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1182,14 +1179,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1537,7 +1526,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>5</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="1">
                   <c:v>0</c:v>
@@ -1554,11 +1543,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="1302559"/>
-        <c:axId val="55718072"/>
+        <c:axId val="19613223"/>
+        <c:axId val="79555399"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1302559"/>
+        <c:axId val="19613223"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1589,7 +1578,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55718072"/>
+        <c:crossAx val="79555399"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1597,7 +1586,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="55718072"/>
+        <c:axId val="79555399"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1662,7 +1651,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1302559"/>
+        <c:crossAx val="19613223"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1729,9 +1718,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2094120</xdr:colOff>
+      <xdr:colOff>2093760</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>91080</xdr:rowOff>
+      <xdr:rowOff>90720</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1740,7 +1729,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5759280" cy="2518920"/>
+        <a:ext cx="5758920" cy="2518560"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2107,14 +2096,14 @@
         <v>21</v>
       </c>
       <c r="J7" s="7" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="K7" s="8"/>
       <c r="L7" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="M7" s="5" t="s">
         <v>34</v>
-      </c>
-      <c r="M7" s="5" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2122,19 +2111,19 @@
         <v>4</v>
       </c>
       <c r="B8" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>40</v>
       </c>
       <c r="G8" s="7" t="n">
         <v>5</v>
@@ -2143,14 +2132,14 @@
         <v>20</v>
       </c>
       <c r="I8" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="J8" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="J8" s="7" t="s">
-        <v>42</v>
       </c>
       <c r="K8" s="8"/>
       <c r="L8" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M8" s="5" t="s">
         <v>29</v>
@@ -2161,19 +2150,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="D9" s="6" t="s">
+      <c r="E9" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="6" t="s">
         <v>46</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>47</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>3</v>
@@ -2182,17 +2171,17 @@
         <v>20</v>
       </c>
       <c r="I9" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="J9" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="J9" s="7" t="s">
-        <v>42</v>
       </c>
       <c r="K9" s="8"/>
       <c r="L9" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2200,19 +2189,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="E10" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>51</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="G10" s="7" t="n">
         <v>3</v>
@@ -2221,17 +2210,17 @@
         <v>20</v>
       </c>
       <c r="I10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="J10" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="J10" s="7" t="s">
-        <v>42</v>
       </c>
       <c r="K10" s="8"/>
       <c r="L10" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="M10" s="5" t="s">
         <v>43</v>
-      </c>
-      <c r="M10" s="5" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2239,19 +2228,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D11" s="6" t="s">
+      <c r="E11" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>55</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>56</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>5</v>
@@ -2260,17 +2249,17 @@
         <v>20</v>
       </c>
       <c r="I11" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="J11" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="J11" s="7" t="s">
-        <v>42</v>
       </c>
       <c r="K11" s="8"/>
       <c r="L11" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2278,19 +2267,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="C12" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D12" s="6" t="s">
+      <c r="E12" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="F12" s="6" t="s">
         <v>59</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>60</v>
       </c>
       <c r="G12" s="7" t="n">
         <v>3</v>
@@ -2299,17 +2288,17 @@
         <v>20</v>
       </c>
       <c r="I12" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="J12" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="J12" s="7" t="s">
-        <v>42</v>
       </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2317,19 +2306,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="E13" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="F13" s="6" t="s">
         <v>64</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>65</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>5</v>
@@ -2338,15 +2327,15 @@
         <v>20</v>
       </c>
       <c r="I13" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="J13" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="J13" s="7" t="s">
-        <v>42</v>
       </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8"/>
       <c r="M13" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2354,19 +2343,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="E14" s="6" t="s">
         <v>68</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>70</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>5</v>
@@ -2375,17 +2364,17 @@
         <v>20</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="M14" s="5" t="s">
         <v>72</v>
-      </c>
-      <c r="M14" s="5" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2393,19 +2382,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="E15" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="6" t="s">
         <v>77</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>78</v>
       </c>
       <c r="G15" s="7" t="n">
         <v>3</v>
@@ -2414,17 +2403,17 @@
         <v>20</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2432,19 +2421,19 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="D16" s="6" t="s">
+      <c r="E16" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>81</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>82</v>
       </c>
       <c r="G16" s="7" t="n">
         <v>8</v>
@@ -2453,17 +2442,17 @@
         <v>20</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2471,19 +2460,19 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="D17" s="6" t="s">
+      <c r="E17" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="F17" s="6" t="s">
         <v>86</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>87</v>
       </c>
       <c r="G17" s="7" t="n">
         <v>2</v>
@@ -2492,17 +2481,17 @@
         <v>20</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K17" s="8"/>
       <c r="L17" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2510,19 +2499,19 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="E18" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="F18" s="6" t="s">
         <v>92</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>93</v>
       </c>
       <c r="G18" s="7" t="n">
         <v>5</v>
@@ -2531,15 +2520,15 @@
         <v>20</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8"/>
       <c r="M18" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2547,19 +2536,19 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D19" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="E19" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="F19" s="6" t="s">
         <v>95</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>96</v>
       </c>
       <c r="G19" s="7" t="n">
         <v>5</v>
@@ -2568,17 +2557,17 @@
         <v>20</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="M19" s="5" t="s">
         <v>98</v>
-      </c>
-      <c r="M19" s="5" t="s">
-        <v>99</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2586,38 +2575,38 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="E20" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="F20" s="6" t="s">
         <v>103</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>104</v>
       </c>
       <c r="G20" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2625,36 +2614,36 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D21" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="C21" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="D21" s="6" t="s">
+      <c r="E21" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="F21" s="6" t="s">
         <v>109</v>
-      </c>
-      <c r="F21" s="6" t="s">
-        <v>110</v>
       </c>
       <c r="G21" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8"/>
       <c r="M21" s="5" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2662,38 +2651,38 @@
         <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="D22" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="C22" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="D22" s="6" t="s">
+      <c r="E22" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="F22" s="6" t="s">
         <v>113</v>
-      </c>
-      <c r="F22" s="6" t="s">
-        <v>114</v>
       </c>
       <c r="G22" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2701,36 +2690,36 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D23" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="D23" s="6" t="s">
+      <c r="E23" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="F23" s="6" t="s">
         <v>117</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>118</v>
       </c>
       <c r="G23" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8"/>
       <c r="M23" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2738,38 +2727,38 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D24" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="E24" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="F24" s="6" t="s">
         <v>121</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>122</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2777,38 +2766,38 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D25" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="E25" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="F25" s="6" t="s">
         <v>124</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>125</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2816,38 +2805,38 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="D26" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="E26" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="F26" s="6" t="s">
         <v>131</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>132</v>
       </c>
       <c r="G26" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
+        <v>132</v>
+      </c>
+      <c r="M26" s="5" t="s">
         <v>133</v>
-      </c>
-      <c r="M26" s="5" t="s">
-        <v>134</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2855,38 +2844,38 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D27" s="6" t="s">
         <v>134</v>
       </c>
-      <c r="C27" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D27" s="6" t="s">
+      <c r="E27" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="F27" s="6" t="s">
         <v>136</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>137</v>
       </c>
       <c r="G27" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2894,36 +2883,36 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D28" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="E28" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="F28" s="6" t="s">
         <v>141</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>142</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8"/>
       <c r="M28" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2931,36 +2920,36 @@
         <v>25</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D29" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="E29" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="F29" s="6" t="s">
         <v>144</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>145</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8"/>
       <c r="M29" s="5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2968,36 +2957,36 @@
         <v>26</v>
       </c>
       <c r="B30" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D30" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="C30" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="D30" s="6" t="s">
+      <c r="E30" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="F30" s="6" t="s">
         <v>148</v>
-      </c>
-      <c r="F30" s="6" t="s">
-        <v>149</v>
       </c>
       <c r="G30" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8"/>
       <c r="M30" s="5" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3005,36 +2994,36 @@
         <v>27</v>
       </c>
       <c r="B31" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="D31" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="C31" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D31" s="6" t="s">
+      <c r="E31" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="F31" s="6" t="s">
         <v>152</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>153</v>
       </c>
       <c r="G31" s="7" t="n">
         <v>8</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
       <c r="M31" s="5" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3042,41 +3031,41 @@
         <v>28</v>
       </c>
       <c r="B32" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="D32" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="C32" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="D32" s="6" t="s">
+      <c r="E32" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="F32" s="6" t="s">
         <v>156</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>157</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
       <c r="M32" s="5" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F34" s="9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="G34" s="9" t="n">
         <f aca="false">SUM(G5:G32)</f>
@@ -3085,56 +3074,56 @@
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F35" s="9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="G35" s="9" t="n">
         <f aca="false">SUMIF(J5:J32,"Feito",G5:G32)</f>
-        <v>5</v>
+        <v>10</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F36" s="10" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:M32"/>
   <conditionalFormatting sqref="J5:J32">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>"Feito"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Em curso"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:H32">
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>"Must"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Should"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Could"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>"Won't"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5:I32">
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Sprint 1"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Sprint 2"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Sprint 3"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"Sprint 4"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
+    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
       <formula>"Backlog"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3188,17 +3177,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>23</v>
@@ -3209,25 +3198,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>164</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>165</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>166</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>167</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>168</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>169</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="H5" s="4" t="s">
         <v>170</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3235,10 +3224,10 @@
         <v>21</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>171</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>172</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>173</v>
       </c>
       <c r="D6" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$32,$A6,'Product Backlog'!$G$5:$G$32)</f>
@@ -3246,11 +3235,11 @@
       </c>
       <c r="E6" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$32,'Product Backlog'!$I$5:$I$32,$A6,'Product Backlog'!$J$5:$J$32,"Feito")</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F6" s="15" t="n">
         <f aca="false">IF(D6=0,0,E6/D6)</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G6" s="16" t="n">
         <f aca="false">$C$3-D6</f>
@@ -3263,13 +3252,13 @@
     </row>
     <row r="7" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" s="14" t="s">
+        <v>173</v>
+      </c>
+      <c r="C7" s="14" t="s">
         <v>174</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>175</v>
       </c>
       <c r="D7" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$32,$A7,'Product Backlog'!$G$5:$G$32)</f>
@@ -3294,13 +3283,13 @@
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>175</v>
+      </c>
+      <c r="C8" s="14" t="s">
         <v>176</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>177</v>
       </c>
       <c r="D8" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$32,$A8,'Product Backlog'!$G$5:$G$32)</f>
@@ -3325,13 +3314,13 @@
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B9" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="C9" s="14" t="s">
         <v>178</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>179</v>
       </c>
       <c r="D9" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$32,$A9,'Product Backlog'!$G$5:$G$32)</f>
@@ -3356,13 +3345,13 @@
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B10" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="C10" s="14" t="s">
         <v>180</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>181</v>
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$32,$A10,'Product Backlog'!$G$5:$G$32)</f>
@@ -3377,7 +3366,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="H10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$32,$A10)</f>
@@ -3386,7 +3375,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
@@ -3396,11 +3385,11 @@
       </c>
       <c r="E11" s="21" t="n">
         <f aca="false">SUM(E6:E10)</f>
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F11" s="22" t="n">
         <f aca="false">IF(D11=0,0,E11/D11)</f>
-        <v>0.0458715596330275</v>
+        <v>0.0917431192660551</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21" t="n">
@@ -3410,42 +3399,42 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
   </sheetData>
@@ -3478,24 +3467,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
+        <v>191</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>192</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>193</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>171</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>194</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3503,7 +3492,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$32,A5)</f>
@@ -3520,10 +3509,10 @@
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$32,A6)</f>
@@ -3540,10 +3529,10 @@
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$32,A7)</f>
@@ -3560,10 +3549,10 @@
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$32,A8)</f>
@@ -3580,7 +3569,7 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>

</xml_diff>

<commit_message>
Nova visão do produto: orientação de curso, várias instituições e LLM
Decisão dos Product Owners de 13/10/2026, com sugestões do docente
(LLM e design patterns):
- docs/geral/00-visao-do-produto.md: públicos, percurso como sequência
  de decisões, âmbito do MVP e metas
- docs/geral/03-arquitetura-e-padroes.md: padrões existentes e previstos
  (Strategy, Adapter, Factory, Decorator, Chain of Responsibility, State)
- Requisitos 1.3: RF03, RF05 e RF07 alterados; RF34 a RF39, RNF12,
  RN09 e RN10 novos; rastreabilidade e pontos em aberto 10 a 12
- Backlog: US29 a US31 novas, US04 a US06 revistas, novo plano de sprints
- dados/catalogo-cursos-mvp.csv: 30 licenciaturas de 12 instituições (DGES)
- PROJETO.md, índice da documentação, regras de código, checklist do PR
  e registo de uso de IA

Sem alterações de código; 136 testes a passar.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01K3W6WeaKcJNZGLwpdCFawJ
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Product Backlog'!$4:$4</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$32</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$35</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -82,12 +82,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="230">
   <si>
     <t xml:space="preserve">Product Backlog — Recomendador de UCs Opcionais</t>
   </si>
   <si>
-    <t xml:space="preserve">Ordenado por sprint e prioridade. Células a amarelo são para a equipa atualizar (Sprint, Estado, Responsável, SP, Notas). Replaneado a 07/10/2026 (ver folha «Plano de sprints»).</t>
+    <t xml:space="preserve">Ordenado pela ordem de trabalho (sprint e prioridade). Células a amarelo são para a equipa atualizar (Sprint, Estado, Responsável, SP, Notas). Replaneado a 13/10/2026 com a nova visão do produto (ver folha «Plano de sprints» e docs/geral/00-visao-do-produto.md). A partir de 13/10 os IDs não mudam.</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -205,15 +205,16 @@
     <t xml:space="preserve">E2</t>
   </si>
   <si>
-    <t xml:space="preserve">Importar catálogo de cursos e UCs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como administrador, quero importar as UCs a partir de um ficheiro CSV, para não ter de as introduzir uma a uma.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• O CSV é validado (colunas obrigatórias, tipos, códigos duplicados).
+    <t xml:space="preserve">Importar catálogo de instituições e cursos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como administrador, quero importar instituições e cursos a partir de um ficheiro CSV, para que o catálogo tenha várias instituições sem introduzir os dados um a um.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Aceita o formato de dados/catalogo-cursos-mvp.csv (códigos DGES, curso, instituição, área, vagas, nota do último colocado, descrição, saídas, fontes).
+• O CSV é validado (colunas obrigatórias, tipos, códigos duplicados).
 • Linhas inválidas são reportadas sem bloquear as válidas.
-• Reimportar atualiza UCs existentes pelo código.</t>
+• Reimportar atualiza cursos existentes pelo par código de instituição + código de curso.</t>
   </si>
   <si>
     <t xml:space="preserve">Sprint 2</t>
@@ -222,21 +223,82 @@
     <t xml:space="preserve">Por fazer</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa a importar instituições e cursos (nova visão). As UCs de cada curso entram com a US06.</t>
   </si>
   <si>
     <t xml:space="preserve">US05</t>
   </si>
   <si>
-    <t xml:space="preserve">Consultar catálogo de opcionais</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como aluno, quero consultar as opcionais disponíveis para o meu curso, com descrição e médias de interesse, carga e dificuldade, para conhecer as alternativas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Lista filtrada pelo curso do aluno.
-• As médias só aparecem com ≥ 5 avaliações; caso contrário mostra "dados insuficientes".
-• Pesquisa por nome.</t>
+    <t xml:space="preserve">Consultar e comparar cursos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como pessoa indecisa, quero consultar e comparar cursos de várias instituições, para perceber as diferenças antes de decidir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Filtros por área, instituição e localidade.
+• Ficha de cada curso com descrição, saídas profissionais, vagas, nota do último colocado e ligação à fonte.
+• Comparação de até 3 cursos lado a lado.
+• Funciona sem sessão iniciada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Questionário de orientação</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como pessoa indecisa, quero responder a um questionário curto sobre os meus interesses e preferências, para receber sugestões de curso que façam sentido para mim.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Perguntas sobre interesses, tipo de trabalho preferido, saídas que imagina, localidade e regime.
+• As perguntas e opções ficam num ficheiro editável pelo Product Owner (como app/texts.py).
+• As respostas ficam guardadas na conta e o questionário pode ser refeito (as respostas anteriores mantêm-se no histórico).
+• Responder demora menos de 2 minutos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 13/10: story nova (nova visão do produto, sugestão do docente).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sugestão de cursos com LLM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como pessoa indecisa, quero receber 2 a 3 cursos sugeridos a partir das minhas respostas, cada um com uma explicação, para saber por onde começar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Os cursos sugeridos existem no catálogo; os que não existem são descartados (RN09).
+• Cada sugestão tem uma explicação curta em português de Portugal.
+• Ao LLM só seguem as respostas e o catálogo, nunca email ou nome (RNF12).
+• O fornecedor é configurável (anthropic, ollama, falso) sem mudar o resto do código (padrões Adapter e Factory, docs/geral/03).
+• Os testes usam o LLM falso e correm sem rede.
+• Se o LLM falhar ou demorar mais de 15 s, o utilizador recebe uma mensagem clara e pode tentar de novo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Escolher curso e linha do tempo do percurso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como utilizador, quero escolher um dos cursos sugeridos (ou outro do catálogo) e ver as decisões que fui tomando, para acompanhar o meu percurso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• A escolha nunca é automática: o utilizador confirma (RN10).
+• Depois de escolher, o curso e a instituição ficam no perfil (RF03).
+• Cada decisão fica registada com data, opções sugeridas e opção escolhida (RF35).
+• Linha do tempo com as decisões, da mais recente para a mais antiga.
+• O utilizador pode mudar de curso, o que cria uma nova decisão.</t>
   </si>
   <si>
     <t xml:space="preserve">US06</t>
@@ -248,12 +310,19 @@
     <t xml:space="preserve">Registar percurso</t>
   </si>
   <si>
-    <t xml:space="preserve">Como aluno, quero indicar cursos ou UCs que já concluí e em que ano letivo, para que o sistema conheça o meu percurso.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Seleção a partir do catálogo.
+    <t xml:space="preserve">Como aluno, quero indicar as UCs do meu curso que já concluí e em que ano letivo, para que o sistema conheça o meu percurso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• O administrador importa as UCs de cada curso por CSV (código, nome, ano, semestre, ECTS, tipo, descrição).
+• O aluno seleciona UCs do catálogo do seu curso.
 • Não permite duplicados no mesmo ano letivo.
 • O aluno pode remover um registo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4; inclui a importação das UCs; 3 → 5 SP.</t>
   </si>
   <si>
     <t xml:space="preserve">US07</t>
@@ -271,18 +340,7 @@
 • Só é possível avaliar dentro de um período aberto (até à US16, o período está sempre aberto).</t>
   </si>
   <si>
-    <t xml:space="preserve">US08</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Avaliação rápida de obrigatórias</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como aluno, quero avaliar rapidamente o interesse das obrigatórias que fiz numa só página, para que o sistema me conheça mesmo antes de eu ter feito opcionais.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Vista em grelha com todas as obrigatórias do percurso.
-• Gravação de todas de uma vez.
-• Avaliar 10 UCs demora menos de 2 minutos.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4.</t>
   </si>
   <si>
     <t xml:space="preserve">US09</t>
@@ -303,6 +361,53 @@
 • Teste automático que verifica RN04.</t>
   </si>
   <si>
+    <t xml:space="preserve">Replaneamento de 13/10: Sprint 2 → Sprint 4, com a US07 para as avaliações serem anónimas desde o início.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recomendações de popularidade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como aluno com poucas avaliações, quero ver as opcionais mais bem avaliadas pelos colegas, para ter sugestões mesmo sem historial.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Aparece quando o aluno não cumpre RN05.
+• A interface indica que são "populares" e não personalizadas.
+• Nunca inclui UCs que o aluno já concluiu (RN03).
+• Implementada como estratégia intercambiável (padrão Strategy, docs/geral/03).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 2 para Sprint 3. Replaneamento de 13/10: Sprint 3 → Sprint 4; segue o padrão Strategy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avaliação rápida de obrigatórias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como aluno, quero avaliar rapidamente o interesse das obrigatórias que fiz numa só página, para que o sistema me conheça mesmo antes de eu ter feito opcionais.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Vista em grelha com todas as obrigatórias do percurso.
+• Gravação de todas de uma vez.
+• Avaliar 10 UCs demora menos de 2 minutos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Should</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backlog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release.</t>
+  </si>
+  <si>
     <t xml:space="preserve">US10</t>
   </si>
   <si>
@@ -319,29 +424,10 @@
 • O motor recomenda UCs do perfil "plantado" na maioria dos casos.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sprint 3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 2 para Sprint 3.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 2 para Sprint 3. Replaneamento de 13/10: Sprint 3 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release.</t>
   </si>
   <si>
     <t xml:space="preserve">US20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recomendações de popularidade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como aluno com poucas avaliações, quero ver as opcionais mais bem avaliadas pelos colegas, para ter sugestões mesmo sem historial.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Aparece quando o aluno não cumpre RN05.
-• A interface indica que são "populares" e não personalizadas.</t>
   </si>
   <si>
     <t xml:space="preserve">US12</t>
@@ -395,6 +481,9 @@
 • A explicação não revela identidades.</t>
   </si>
   <si>
+    <t xml:space="preserve">Replaneamento de 13/10: Sprint 3 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Avaliação offline do motor</t>
   </si>
   <si>
@@ -406,10 +495,7 @@
 • Resultados guardados e comparáveis entre estratégias.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sprint 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 3 para Sprint 4.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 3 para Sprint 4. Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release.</t>
   </si>
   <si>
     <t xml:space="preserve">US21</t>
@@ -431,7 +517,7 @@
 • Fora do período, o formulário de avaliação fica bloqueado com mensagem explicativa.</t>
   </si>
   <si>
-    <t xml:space="preserve">Should</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 3 para Sprint 4. Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro).</t>
   </si>
   <si>
     <t xml:space="preserve">US24</t>
@@ -449,6 +535,9 @@
     <t xml:space="preserve">• Exportação em JSON/CSV.
 • Apagar remove conta, percurso e avaliações.
 • A ação pede confirmação.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro).</t>
   </si>
   <si>
     <t xml:space="preserve">US18</t>
@@ -504,9 +593,6 @@
 • "Indiferente" mantém a ordenação original.</t>
   </si>
   <si>
-    <t xml:space="preserve">Backlog</t>
-  </si>
-  <si>
     <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 3 para Backlog.</t>
   </si>
   <si>
@@ -617,7 +703,7 @@
     <t xml:space="preserve">Story points concluídos (Estado = Feito)</t>
   </si>
   <si>
-    <t xml:space="preserve">Nota: a US22 (fatorização de matrizes, SVD) não estava nesta folha. Fica fora do plano da release, como a US23.</t>
+    <t xml:space="preserve">Nota: a fatorização de matrizes (SVD, antiga US22) fica fora do plano da release. Épico E11 (novo): Orientação de curso.</t>
   </si>
   <si>
     <t xml:space="preserve">Plano de sprints — Recomendador de UCs Opcionais</t>
@@ -656,28 +742,28 @@
     <t xml:space="preserve">US01, US02, US03</t>
   </si>
   <si>
-    <t xml:space="preserve">O catálogo existe e o aluno regista o percurso e avalia UCs, de forma anónima.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US04, US05, US06, US07, US08, US09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O sistema dá recomendações personalizadas e explicadas.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US10, US11, US12, US13, US14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O motor é avaliado, os alunos controlam os seus dados e o produto está pronto para demonstração.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US15, US16, US17, US18, US19, US20</t>
+    <t xml:space="preserve">Uma pessoa indecisa descobre e compara cursos de várias instituições e responde ao questionário de orientação.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US04, US05, US29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O OptaBem sugere cursos com explicação e o utilizador escolhe, ficando a decisão registada no percurso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US30, US31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quem já é aluno regista o percurso, avalia opcionais de forma anónima e recebe sugestões por popularidade.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US06, US07, US09, US11</t>
   </si>
   <si>
     <t xml:space="preserve">Fora do plano desta release; entra se houver folga.</t>
   </si>
   <si>
-    <t xml:space="preserve">US21, US22, US23, US24, US25, US26, US27, US28</t>
+    <t xml:space="preserve">US08, US10, US12–US28</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -705,6 +791,30 @@
   </si>
   <si>
     <t xml:space="preserve">• As stories foram renumeradas pela nova ordem (US01 a US28). A coluna «ID anterior» da folha «Product Backlog» mostra o número antigo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 13/10/2026 (decisão dos Product Owners, com sugestões do docente)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Nova visão do produto: o utilizador pode ainda não ter curso; o OptaBem orienta a escolha do curso e depois a das opcionais (docs/geral/00-visao-do-produto.md).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Catálogo com várias instituições: MVP com 12 instituições e 30 licenciaturas (dados/catalogo-cursos-mvp.csv, fonte DGES).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Stories novas: US29 (questionário), US30 (sugestão de cursos com LLM) e US31 (escolher curso e linha do tempo). Épico novo E11.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US04 e US05 passam a tratar instituições e cursos; US06 inclui a importação das UCs e passa para o Sprint 4.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US08, US10 e US12 a US20 passam para o Backlog; as que eram Must passam a Should nesta release.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• A partir de 13/10 os IDs ficam fixos (stories novas recebem o número seguinte). A ordem de trabalho é a deste plano.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Atenção: o plano soma 13, 13 e 18 SP; a velocidade real do Sprint 1 foi 10 SP (ponto 10 da secção 5 dos requisitos).</t>
   </si>
   <si>
     <t xml:space="preserve">Resumo por prioridade (MoSCoW)</t>
@@ -1435,13 +1545,13 @@
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>24</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>23</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>19</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1543,11 +1653,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="19613223"/>
-        <c:axId val="79555399"/>
+        <c:axId val="42986021"/>
+        <c:axId val="37217584"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="19613223"/>
+        <c:axId val="42986021"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1578,7 +1688,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79555399"/>
+        <c:crossAx val="37217584"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1586,7 +1696,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="79555399"/>
+        <c:axId val="37217584"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1651,7 +1761,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19613223"/>
+        <c:crossAx val="42986021"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1718,9 +1828,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2093760</xdr:colOff>
+      <xdr:colOff>2093040</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>90720</xdr:rowOff>
+      <xdr:rowOff>90000</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1729,7 +1839,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5758920" cy="2518560"/>
+        <a:ext cx="5758200" cy="2517840"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1922,7 +2032,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:M36"/>
+  <dimension ref="A1:M39"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
@@ -2165,7 +2275,7 @@
         <v>46</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>20</v>
@@ -2178,7 +2288,7 @@
       </c>
       <c r="K9" s="8"/>
       <c r="L9" s="8" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="M9" s="5" t="s">
         <v>35</v>
@@ -2189,19 +2299,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G10" s="7" t="n">
         <v>3</v>
@@ -2217,10 +2327,10 @@
       </c>
       <c r="K10" s="8"/>
       <c r="L10" s="8" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="M10" s="5" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2228,38 +2338,38 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>20</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="J11" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K11" s="8"/>
       <c r="L11" s="8" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>47</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2267,38 +2377,38 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H12" s="5" t="s">
         <v>20</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>40</v>
+        <v>58</v>
       </c>
       <c r="J12" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>52</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2306,19 +2416,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>5</v>
@@ -2327,15 +2437,17 @@
         <v>20</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>40</v>
+        <v>68</v>
       </c>
       <c r="J13" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K13" s="8"/>
-      <c r="L13" s="8"/>
+      <c r="L13" s="8" t="s">
+        <v>69</v>
+      </c>
       <c r="M13" s="5" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2343,19 +2455,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>5</v>
@@ -2364,17 +2476,17 @@
         <v>20</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J14" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2382,38 +2494,38 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H15" s="5" t="s">
         <v>20</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J15" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2421,38 +2533,38 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="G16" s="7" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H16" s="5" t="s">
         <v>20</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="J16" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8" t="s">
-        <v>71</v>
+        <v>86</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2460,38 +2572,38 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>70</v>
+        <v>92</v>
       </c>
       <c r="J17" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K17" s="8"/>
       <c r="L17" s="8" t="s">
-        <v>71</v>
+        <v>93</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>87</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2499,36 +2611,38 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="G18" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>70</v>
+        <v>92</v>
       </c>
       <c r="J18" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K18" s="8"/>
-      <c r="L18" s="8"/>
+      <c r="L18" s="8" t="s">
+        <v>99</v>
+      </c>
       <c r="M18" s="5" t="s">
-        <v>82</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2536,38 +2650,38 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>87</v>
+        <v>101</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>20</v>
+        <v>91</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="J19" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2575,38 +2689,38 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="J20" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2614,36 +2728,38 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>61</v>
+        <v>112</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="J21" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K21" s="8"/>
-      <c r="L21" s="8"/>
+      <c r="L21" s="8" t="s">
+        <v>116</v>
+      </c>
       <c r="M21" s="5" t="s">
-        <v>65</v>
+        <v>105</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2654,35 +2770,35 @@
         <v>110</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>48</v>
+        <v>95</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="J22" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
-        <v>97</v>
+        <v>120</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>56</v>
+        <v>121</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2690,36 +2806,38 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="G23" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="J23" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K23" s="8"/>
-      <c r="L23" s="8"/>
+      <c r="L23" s="8" t="s">
+        <v>127</v>
+      </c>
       <c r="M23" s="5" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2727,38 +2845,38 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>72</v>
+        <v>129</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="J24" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2766,38 +2884,38 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>98</v>
+        <v>134</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>83</v>
+        <v>64</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>122</v>
+        <v>135</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>123</v>
+        <v>136</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>124</v>
+        <v>137</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>125</v>
+        <v>92</v>
       </c>
       <c r="J25" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2805,38 +2923,38 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>129</v>
+        <v>139</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>131</v>
+        <v>141</v>
       </c>
       <c r="G26" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>125</v>
+        <v>92</v>
       </c>
       <c r="J26" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2844,38 +2962,38 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>133</v>
+        <v>100</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>83</v>
+        <v>106</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>137</v>
+        <v>91</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>125</v>
+        <v>92</v>
       </c>
       <c r="J27" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
-        <v>138</v>
+        <v>127</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2883,36 +3001,38 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>89</v>
+        <v>106</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="G28" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>137</v>
+        <v>91</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>125</v>
+        <v>92</v>
       </c>
       <c r="J28" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K28" s="8"/>
-      <c r="L28" s="8"/>
+      <c r="L28" s="8" t="s">
+        <v>149</v>
+      </c>
       <c r="M28" s="5" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2920,36 +3040,38 @@
         <v>25</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>118</v>
+        <v>150</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>100</v>
+        <v>151</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>143</v>
+        <v>153</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>144</v>
+        <v>154</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>137</v>
+        <v>91</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>125</v>
+        <v>92</v>
       </c>
       <c r="J29" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K29" s="8"/>
-      <c r="L29" s="8"/>
+      <c r="L29" s="8" t="s">
+        <v>155</v>
+      </c>
       <c r="M29" s="5" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2957,36 +3079,38 @@
         <v>26</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>128</v>
+        <v>106</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>125</v>
+        <v>92</v>
       </c>
       <c r="J30" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K30" s="8"/>
-      <c r="L30" s="8"/>
+      <c r="L30" s="8" t="s">
+        <v>161</v>
+      </c>
       <c r="M30" s="5" t="s">
-        <v>149</v>
+        <v>129</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2994,28 +3118,28 @@
         <v>27</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>149</v>
+        <v>128</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>83</v>
+        <v>112</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="G31" s="7" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>125</v>
+        <v>92</v>
       </c>
       <c r="J31" s="7" t="s">
         <v>41</v>
@@ -3023,7 +3147,7 @@
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
       <c r="M31" s="5" t="s">
-        <v>110</v>
+        <v>138</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3031,28 +3155,28 @@
         <v>28</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>156</v>
+        <v>167</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>125</v>
+        <v>92</v>
       </c>
       <c r="J32" s="7" t="s">
         <v>41</v>
@@ -3060,35 +3184,147 @@
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
       <c r="M32" s="5" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F34" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="G34" s="9" t="n">
-        <f aca="false">SUM(G5:G32)</f>
-        <v>109</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F35" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="G35" s="9" t="n">
-        <f aca="false">SUMIF(J5:J32,"Feito",G5:G32)</f>
+        <v>168</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="F33" s="6" t="s">
+        <v>171</v>
+      </c>
+      <c r="G33" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H33" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="J33" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="K33" s="8"/>
+      <c r="L33" s="8"/>
+      <c r="M33" s="5" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>173</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>175</v>
+      </c>
+      <c r="G34" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="I34" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="J34" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="K34" s="8"/>
+      <c r="L34" s="8"/>
+      <c r="M34" s="5" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>177</v>
+      </c>
+      <c r="E35" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="F35" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="G35" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H35" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="J35" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="K35" s="8"/>
+      <c r="L35" s="8"/>
+      <c r="M35" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F37" s="9" t="s">
+        <v>181</v>
+      </c>
+      <c r="G37" s="9" t="n">
+        <f aca="false">SUM(G5:G35)</f>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F38" s="9" t="s">
+        <v>182</v>
+      </c>
+      <c r="G38" s="9" t="n">
+        <f aca="false">SUMIF(J5:J35,"Feito",G5:G35)</f>
         <v>10</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F36" s="10" t="s">
-        <v>160</v>
+    <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F39" s="10" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:M32"/>
-  <conditionalFormatting sqref="J5:J32">
+  <autoFilter ref="A4:M35"/>
+  <conditionalFormatting sqref="J5:J35">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>"Feito"</formula>
     </cfRule>
@@ -3096,7 +3332,7 @@
       <formula>"Em curso"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H32">
+  <conditionalFormatting sqref="H5:H35">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>"Must"</formula>
     </cfRule>
@@ -3110,7 +3346,7 @@
       <formula>"Won't"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I32">
+  <conditionalFormatting sqref="I5:I35">
     <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Sprint 1"</formula>
     </cfRule>
@@ -3128,19 +3364,19 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G32" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G35" type="list">
       <formula1>"1,2,3,5,8,13,21"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H32" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H35" type="list">
       <formula1>"Must,Should,Could,Won't"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I32" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I35" type="list">
       <formula1>"Sprint 1,Sprint 2,Sprint 3,Sprint 4,Backlog"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J32" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J35" type="list">
       <formula1>"Por fazer,Em curso,Feito"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3162,7 +3398,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -3177,17 +3413,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>161</v>
+        <v>184</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>162</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>163</v>
+        <v>186</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>23</v>
@@ -3198,25 +3434,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>164</v>
+        <v>187</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>165</v>
+        <v>188</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>166</v>
+        <v>189</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>167</v>
+        <v>190</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>168</v>
+        <v>191</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>169</v>
+        <v>192</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>170</v>
+        <v>193</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3224,17 +3460,17 @@
         <v>21</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>171</v>
+        <v>194</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>172</v>
+        <v>195</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$32,$A6,'Product Backlog'!$G$5:$G$32)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$35,$A6,'Product Backlog'!$G$5:$G$35)</f>
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$32,'Product Backlog'!$I$5:$I$32,$A6,'Product Backlog'!$J$5:$J$32,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$35,'Product Backlog'!$I$5:$I$35,$A6,'Product Backlog'!$J$5:$J$35,"Feito")</f>
         <v>10</v>
       </c>
       <c r="F6" s="15" t="n">
@@ -3246,7 +3482,7 @@
         <v>13</v>
       </c>
       <c r="H6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$32,$A6)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$35,$A6)</f>
         <v>3</v>
       </c>
     </row>
@@ -3255,17 +3491,17 @@
         <v>40</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>173</v>
+        <v>196</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>174</v>
+        <v>197</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$32,$A7,'Product Backlog'!$G$5:$G$32)</f>
-        <v>24</v>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$35,$A7,'Product Backlog'!$G$5:$G$35)</f>
+        <v>13</v>
       </c>
       <c r="E7" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$32,'Product Backlog'!$I$5:$I$32,$A7,'Product Backlog'!$J$5:$J$32,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$35,'Product Backlog'!$I$5:$I$35,$A7,'Product Backlog'!$J$5:$J$35,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F7" s="15" t="n">
@@ -3274,29 +3510,29 @@
       </c>
       <c r="G7" s="16" t="n">
         <f aca="false">$C$3-D7</f>
-        <v>-1</v>
+        <v>10</v>
       </c>
       <c r="H7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$32,$A7)</f>
-        <v>6</v>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$35,$A7)</f>
+        <v>3</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>175</v>
+        <v>198</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>176</v>
+        <v>199</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$32,$A8,'Product Backlog'!$G$5:$G$32)</f>
-        <v>23</v>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$35,$A8,'Product Backlog'!$G$5:$G$35)</f>
+        <v>13</v>
       </c>
       <c r="E8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$32,'Product Backlog'!$I$5:$I$32,$A8,'Product Backlog'!$J$5:$J$32,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$35,'Product Backlog'!$I$5:$I$35,$A8,'Product Backlog'!$J$5:$J$35,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F8" s="15" t="n">
@@ -3305,29 +3541,29 @@
       </c>
       <c r="G8" s="16" t="n">
         <f aca="false">$C$3-D8</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$32,$A8)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$35,$A8)</f>
+        <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>96</v>
+        <v>68</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>177</v>
+        <v>200</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>178</v>
+        <v>201</v>
       </c>
       <c r="D9" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$32,$A9,'Product Backlog'!$G$5:$G$32)</f>
-        <v>19</v>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$35,$A9,'Product Backlog'!$G$5:$G$35)</f>
+        <v>18</v>
       </c>
       <c r="E9" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$32,'Product Backlog'!$I$5:$I$32,$A9,'Product Backlog'!$J$5:$J$32,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$35,'Product Backlog'!$I$5:$I$35,$A9,'Product Backlog'!$J$5:$J$35,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F9" s="15" t="n">
@@ -3336,29 +3572,29 @@
       </c>
       <c r="G9" s="16" t="n">
         <f aca="false">$C$3-D9</f>
+        <v>5</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$35,$A9)</f>
         <v>4</v>
-      </c>
-      <c r="H9" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$32,$A9)</f>
-        <v>6</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>125</v>
+        <v>92</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>179</v>
+        <v>202</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>180</v>
+        <v>203</v>
       </c>
       <c r="D10" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$32,$A10,'Product Backlog'!$G$5:$G$32)</f>
-        <v>33</v>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$35,$A10,'Product Backlog'!$G$5:$G$35)</f>
+        <v>75</v>
       </c>
       <c r="E10" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$32,'Product Backlog'!$I$5:$I$32,$A10,'Product Backlog'!$J$5:$J$32,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$35,'Product Backlog'!$I$5:$I$35,$A10,'Product Backlog'!$J$5:$J$35,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F10" s="15" t="n">
@@ -3369,19 +3605,19 @@
         <v>34</v>
       </c>
       <c r="H10" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$32,$A10)</f>
-        <v>8</v>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$35,$A10)</f>
+        <v>19</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
       <c r="D11" s="21" t="n">
         <f aca="false">SUM(D6:D10)</f>
-        <v>109</v>
+        <v>129</v>
       </c>
       <c r="E11" s="21" t="n">
         <f aca="false">SUM(E6:E10)</f>
@@ -3389,52 +3625,92 @@
       </c>
       <c r="F11" s="22" t="n">
         <f aca="false">IF(D11=0,0,E11/D11)</f>
-        <v>0.0917431192660551</v>
+        <v>0.0775193798449612</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21" t="n">
         <f aca="false">SUM(H6:H10)</f>
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>182</v>
+        <v>205</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>183</v>
+        <v>206</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>184</v>
+        <v>207</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>185</v>
+        <v>208</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>186</v>
+        <v>209</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>187</v>
+        <v>210</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>188</v>
+        <v>211</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>189</v>
+        <v>212</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="23" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="24" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="24" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="24" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="24" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="24" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="24" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="24" t="s">
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -3467,24 +3743,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>190</v>
+        <v>221</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>191</v>
+        <v>222</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>192</v>
+        <v>223</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>170</v>
+        <v>193</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>193</v>
+        <v>224</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>194</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3492,92 +3768,92 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>195</v>
+        <v>226</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$32,A5)</f>
-        <v>15</v>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$35,A5)</f>
+        <v>12</v>
       </c>
       <c r="D5" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$32,A5,'Product Backlog'!$G$5:$G$32)</f>
-        <v>62</v>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$35,A5,'Product Backlog'!$G$5:$G$35)</f>
+        <v>54</v>
       </c>
       <c r="E5" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D5/SUM($D$5:$D$8))</f>
-        <v>0.568807339449541</v>
+        <v>0.418604651162791</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>196</v>
+        <v>227</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$32,A6)</f>
-        <v>7</v>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$35,A6)</f>
+        <v>13</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$32,A6,'Product Backlog'!$G$5:$G$32)</f>
-        <v>22</v>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$35,A6,'Product Backlog'!$G$5:$G$35)</f>
+        <v>50</v>
       </c>
       <c r="E6" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D6/SUM($D$5:$D$8))</f>
-        <v>0.201834862385321</v>
+        <v>0.387596899224806</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>197</v>
+        <v>228</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$32,A7)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$35,A7)</f>
         <v>5</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$32,A7,'Product Backlog'!$G$5:$G$32)</f>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$35,A7,'Product Backlog'!$G$5:$G$35)</f>
         <v>22</v>
       </c>
       <c r="E7" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D7/SUM($D$5:$D$8))</f>
-        <v>0.201834862385321</v>
+        <v>0.170542635658915</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>157</v>
+        <v>180</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>198</v>
+        <v>229</v>
       </c>
       <c r="C8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$32,A8)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$35,A8)</f>
         <v>1</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$32,A8,'Product Backlog'!$G$5:$G$32)</f>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$35,A8,'Product Backlog'!$G$5:$G$35)</f>
         <v>3</v>
       </c>
       <c r="E8" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D8/SUM($D$5:$D$8))</f>
-        <v>0.0275229357798165</v>
+        <v>0.0232558139534884</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>181</v>
+        <v>204</v>
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D9" s="27" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>109</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Backlog: US03 revista, US05 em curso e US32 (assistente LLM) por avaliar
- Excel: notas da US03 (início de sessão único) e da US05 (pesquisa
  antecipada; faltam filtros, ficha e comparação); story nova US32 no
  Backlog, por avaliar; fórmulas alargadas à linha nova; notas da
  revisão de 14/10 na folha «Plano de sprints».
- Requisitos: ponto em aberto 13 (assistente LLM conversacional).
- PROJETO.md: estado das stories atualizado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E9QzPgdcfwB8xR8d5sAuMb
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="243">
   <si>
     <t xml:space="preserve">Product Backlog — Recomendador de UCs Opcionais</t>
   </si>
@@ -193,7 +193,7 @@
 • Um administrador cria e remove outros administradores (não a si próprio).</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: story nova (o RF04 não tinha story). Revista pelos PO: administradores independentes e área escondida (3 → 5 SP). Código, testes e documentação no GitHub (PR #7 aceite).</t>
+    <t xml:space="preserve">Replaneamento de 07/10: story nova (o RF04 não tinha story). Revista pelos PO: administradores independentes e área escondida (3 → 5 SP). Código, testes e documentação no GitHub (PR #7 aceite). Revisão de 14/10 (PO): um só início de sessão para alunos e administradores, com os padrões Strategy, Chain of Responsibility e Factory (app/auth/perfis.py, PR #14).</t>
   </si>
   <si>
     <t xml:space="preserve">—</t>
@@ -241,7 +241,10 @@
 • Funciona sem sessão iniciada.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11.</t>
+    <t xml:space="preserve">Em curso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11. 14/10: trabalho antecipado no PR #14 — pesquisa de cursos reais na página de apresentação (app/catalogo/, dados da DGES lidos do CSV). Falta: filtros por área/instituição/localidade, ficha completa do curso e comparação de até 3 cursos.</t>
   </si>
   <si>
     <t xml:space="preserve">US29</t>
@@ -697,6 +700,30 @@
     <t xml:space="preserve">Won't</t>
   </si>
   <si>
+    <t xml:space="preserve">US32</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assistente LLM que conversa com o utilizador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como pessoa indecisa, quero conversar com um assistente que me faça perguntas e me ajude a perceber que cursos e opcionais fazem sentido para mim, para decidir com mais confiança.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• A AVALIAR pelos Product Owners antes de ser estimada (ver docs/geral/01, ponto em aberto 13).
+• O assistente só fala de cursos e opcionais do catálogo (RN09) e explica cada sugestão.
+• Não recebe email, nome nem identificadores do utilizador (RNF12).
+• Funciona com o LLMFalso nos testes (sem rede).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por avaliar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14/10: pedido do PO para verificar a inserção de um agente LLM que interaja com o utilizador. Pode estender a US29/US30 (questionário + sugestão) para uma conversa; decidir âmbito, custo e privacidade antes de estimar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nova</t>
+  </si>
+  <si>
     <t xml:space="preserve">Total de story points</t>
   </si>
   <si>
@@ -763,7 +790,7 @@
     <t xml:space="preserve">Fora do plano desta release; entra se houver folga.</t>
   </si>
   <si>
-    <t xml:space="preserve">US08, US10, US12–US28</t>
+    <t xml:space="preserve">US08, US10, US12–US28, US32</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -815,6 +842,21 @@
   </si>
   <si>
     <t xml:space="preserve">• Atenção: o plano soma 13, 13 e 18 SP; a velocidade real do Sprint 1 foi 10 SP (ponto 10 da secção 5 dos requisitos).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisão de 14/10/2026 (decisões dos Product Owners)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US03 revista: um só início de sessão para alunos e administradores (design patterns Strategy, Chain of Responsibility e Factory).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US05 começada antes do Sprint 2: pesquisa de cursos reais na página de apresentação. Os SP contam no Sprint 2, quando a story estiver completa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Story nova US32 (assistente LLM que conversa com o utilizador), no Backlog e por avaliar: decidir âmbito, custo e privacidade antes de estimar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Redesenho visual do site (sem story própria): fica registado no PR #14 e no registo de uso de IA.</t>
   </si>
   <si>
     <t xml:space="preserve">Resumo por prioridade (MoSCoW)</t>
@@ -1197,7 +1239,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="22">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1289,6 +1331,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1653,11 +1703,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="42986021"/>
-        <c:axId val="37217584"/>
+        <c:axId val="90681899"/>
+        <c:axId val="55780184"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="42986021"/>
+        <c:axId val="90681899"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1688,7 +1738,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37217584"/>
+        <c:crossAx val="55780184"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1696,7 +1746,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="37217584"/>
+        <c:axId val="55780184"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1761,7 +1811,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42986021"/>
+        <c:crossAx val="90681899"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1828,9 +1878,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2093040</xdr:colOff>
+      <xdr:colOff>2092680</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>90000</xdr:rowOff>
+      <xdr:rowOff>89640</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1839,7 +1889,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5758200" cy="2517840"/>
+        <a:ext cx="5757840" cy="2517480"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2284,11 +2334,11 @@
         <v>40</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K9" s="8"/>
       <c r="L9" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M9" s="5" t="s">
         <v>35</v>
@@ -2299,19 +2349,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G10" s="7" t="n">
         <v>3</v>
@@ -2327,7 +2377,7 @@
       </c>
       <c r="K10" s="8"/>
       <c r="L10" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M10" s="5" t="s">
         <v>34</v>
@@ -2338,19 +2388,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>8</v>
@@ -2359,14 +2409,14 @@
         <v>20</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J11" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K11" s="8"/>
       <c r="L11" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M11" s="5" t="s">
         <v>34</v>
@@ -2377,19 +2427,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G12" s="7" t="n">
         <v>5</v>
@@ -2398,14 +2448,14 @@
         <v>20</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J12" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M12" s="5" t="s">
         <v>34</v>
@@ -2416,19 +2466,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>5</v>
@@ -2437,14 +2487,14 @@
         <v>20</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J13" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="M13" s="5" t="s">
         <v>43</v>
@@ -2455,19 +2505,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>5</v>
@@ -2476,17 +2526,17 @@
         <v>20</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J14" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2494,19 +2544,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="G15" s="7" t="n">
         <v>5</v>
@@ -2515,17 +2565,17 @@
         <v>20</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J15" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2533,19 +2583,19 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G16" s="7" t="n">
         <v>3</v>
@@ -2554,17 +2604,17 @@
         <v>20</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="J16" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2572,38 +2622,38 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="G17" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J17" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K17" s="8"/>
       <c r="L17" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2611,38 +2661,38 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G18" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J18" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2650,38 +2700,38 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G19" s="7" t="n">
         <v>8</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J19" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2689,38 +2739,38 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="G20" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J20" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2728,38 +2778,38 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G21" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J21" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="M21" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2767,38 +2817,38 @@
         <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G22" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J22" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2806,38 +2856,38 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G23" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J23" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="M23" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2845,38 +2895,38 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J24" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2884,38 +2934,38 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J25" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2923,38 +2973,38 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G26" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J26" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2962,38 +3012,38 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G27" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J27" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3001,38 +3051,38 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J28" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3040,38 +3090,38 @@
         <v>25</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J29" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="M29" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3079,38 +3129,38 @@
         <v>26</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G30" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J30" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3118,28 +3168,28 @@
         <v>27</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="G31" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J31" s="7" t="s">
         <v>41</v>
@@ -3147,7 +3197,7 @@
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
       <c r="M31" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3155,28 +3205,28 @@
         <v>28</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J32" s="7" t="s">
         <v>41</v>
@@ -3184,7 +3234,7 @@
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
       <c r="M32" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3192,28 +3242,28 @@
         <v>29</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="G33" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I33" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J33" s="7" t="s">
         <v>41</v>
@@ -3221,7 +3271,7 @@
       <c r="K33" s="8"/>
       <c r="L33" s="8"/>
       <c r="M33" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3229,28 +3279,28 @@
         <v>30</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="G34" s="7" t="n">
         <v>8</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J34" s="7" t="s">
         <v>41</v>
@@ -3258,7 +3308,7 @@
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
       <c r="M34" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3266,28 +3316,28 @@
         <v>31</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G35" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="I35" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="J35" s="7" t="s">
         <v>41</v>
@@ -3295,13 +3345,49 @@
       <c r="K35" s="8"/>
       <c r="L35" s="8"/>
       <c r="M35" s="5" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+        <v>177</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="C36" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>183</v>
+      </c>
+      <c r="E36" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="F36" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="G36" s="7"/>
+      <c r="H36" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="I36" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="J36" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="K36" s="8"/>
+      <c r="L36" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="M36" s="5" t="s">
+        <v>188</v>
+      </c>
+    </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F37" s="9" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="G37" s="9" t="n">
         <f aca="false">SUM(G5:G35)</f>
@@ -3310,7 +3396,7 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F38" s="9" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="G38" s="9" t="n">
         <f aca="false">SUMIF(J5:J35,"Feito",G5:G35)</f>
@@ -3319,47 +3405,47 @@
     </row>
     <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F39" s="10" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:M35"/>
   <conditionalFormatting sqref="J5:J35">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Feito"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>"Em curso"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:H35">
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Must"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Should"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>"Could"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Won't"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5:I35">
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Sprint 1"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>"Sprint 2"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"Sprint 3"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
       <formula>"Sprint 4"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
       <formula>"Backlog"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3398,7 +3484,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:H51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -3413,17 +3499,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>23</v>
@@ -3434,25 +3520,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3460,17 +3546,17 @@
         <v>21</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$35,$A6,'Product Backlog'!$G$5:$G$35)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A6,'Product Backlog'!$G$5:$G$36)</f>
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$35,'Product Backlog'!$I$5:$I$35,$A6,'Product Backlog'!$J$5:$J$35,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A6,'Product Backlog'!$J$5:$J$36,"Feito")</f>
         <v>10</v>
       </c>
       <c r="F6" s="15" t="n">
@@ -3482,7 +3568,7 @@
         <v>13</v>
       </c>
       <c r="H6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$35,$A6)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A6)</f>
         <v>3</v>
       </c>
     </row>
@@ -3491,17 +3577,17 @@
         <v>40</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$35,$A7,'Product Backlog'!$G$5:$G$35)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A7,'Product Backlog'!$G$5:$G$36)</f>
         <v>13</v>
       </c>
       <c r="E7" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$35,'Product Backlog'!$I$5:$I$35,$A7,'Product Backlog'!$J$5:$J$35,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A7,'Product Backlog'!$J$5:$J$36,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F7" s="15" t="n">
@@ -3513,26 +3599,26 @@
         <v>10</v>
       </c>
       <c r="H7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$35,$A7)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A7)</f>
         <v>3</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$35,$A8,'Product Backlog'!$G$5:$G$35)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$G$5:$G$36)</f>
         <v>13</v>
       </c>
       <c r="E8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$35,'Product Backlog'!$I$5:$I$35,$A8,'Product Backlog'!$J$5:$J$35,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$J$5:$J$36,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F8" s="15" t="n">
@@ -3544,26 +3630,26 @@
         <v>10</v>
       </c>
       <c r="H8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$35,$A8)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A8)</f>
         <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="D9" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$35,$A9,'Product Backlog'!$G$5:$G$35)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A9,'Product Backlog'!$G$5:$G$36)</f>
         <v>18</v>
       </c>
       <c r="E9" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$35,'Product Backlog'!$I$5:$I$35,$A9,'Product Backlog'!$J$5:$J$35,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A9,'Product Backlog'!$J$5:$J$36,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F9" s="15" t="n">
@@ -3575,26 +3661,26 @@
         <v>5</v>
       </c>
       <c r="H9" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$35,$A9)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A9)</f>
         <v>4</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
       <c r="D10" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$35,$A10,'Product Backlog'!$G$5:$G$35)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A10,'Product Backlog'!$G$5:$G$36)</f>
         <v>75</v>
       </c>
       <c r="E10" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$35,'Product Backlog'!$I$5:$I$35,$A10,'Product Backlog'!$J$5:$J$35,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A10,'Product Backlog'!$J$5:$J$36,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F10" s="15" t="n">
@@ -3605,13 +3691,13 @@
         <v>34</v>
       </c>
       <c r="H10" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$35,$A10)</f>
-        <v>19</v>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A10)</f>
+        <v>20</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
@@ -3630,87 +3716,112 @@
       <c r="G11" s="21"/>
       <c r="H11" s="21" t="n">
         <f aca="false">SUM(H6:H10)</f>
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="24" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="24" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="24" t="s">
-        <v>220</v>
+        <v>228</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="23" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="24" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="24" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="24" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="24" t="s">
+        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -3743,24 +3854,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>221</v>
+        <v>234</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>222</v>
+        <v>235</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>223</v>
+        <v>236</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>224</v>
+        <v>237</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>225</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3768,14 +3879,14 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>226</v>
+        <v>239</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$35,A5)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A5)</f>
         <v>12</v>
       </c>
       <c r="D5" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$35,A5,'Product Backlog'!$G$5:$G$35)</f>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$36,A5,'Product Backlog'!$G$5:$G$36)</f>
         <v>54</v>
       </c>
       <c r="E5" s="15" t="n">
@@ -3785,17 +3896,17 @@
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>227</v>
+        <v>240</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$35,A6)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A6)</f>
         <v>13</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$35,A6,'Product Backlog'!$G$5:$G$35)</f>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$36,A6,'Product Backlog'!$G$5:$G$36)</f>
         <v>50</v>
       </c>
       <c r="E6" s="15" t="n">
@@ -3805,17 +3916,17 @@
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>228</v>
+        <v>241</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$35,A7)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A7)</f>
+        <v>6</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$35,A7,'Product Backlog'!$G$5:$G$35)</f>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$36,A7,'Product Backlog'!$G$5:$G$36)</f>
         <v>22</v>
       </c>
       <c r="E7" s="15" t="n">
@@ -3825,17 +3936,17 @@
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>229</v>
+        <v>242</v>
       </c>
       <c r="C8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$35,A8)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A8)</f>
         <v>1</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$35,A8,'Product Backlog'!$G$5:$G$35)</f>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$36,A8,'Product Backlog'!$G$5:$G$36)</f>
         <v>3</v>
       </c>
       <c r="E8" s="15" t="n">
@@ -3845,11 +3956,11 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D9" s="27" t="n">
         <f aca="false">SUM(D5:D8)</f>

</xml_diff>

<commit_message>
Replaneamento de 14/10: LLM conduz a orientação, plano a 10 SP
- US29 reescrita (conversa de orientação com o LLM, 5 SP) e US32 fundida nela
- US30 reescrita (sugestão de 2 a 3 cursos no fim da conversa, 3 SP), passa para o Sprint 2
- Plano à velocidade real: Sprints 2-4 com 8, 10 e 10 SP; US04, US09 e US11 no backlog
- Excel: velocidade 10 SP; totais, validações e formatação passam a incluir a última linha
- Requisitos 1.4 (RF36-RF38, RNF12, pontos 14 e 15), visão 1.1, PROJETO.md

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jxs1JgMiGoE8QQAeMbxyRn
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Product Backlog'!$4:$4</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$35</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$36</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -82,12 +82,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="252">
   <si>
     <t xml:space="preserve">Product Backlog — Recomendador de UCs Opcionais</t>
   </si>
   <si>
-    <t xml:space="preserve">Ordenado pela ordem de trabalho (sprint e prioridade). Células a amarelo são para a equipa atualizar (Sprint, Estado, Responsável, SP, Notas). Replaneado a 13/10/2026 com a nova visão do produto (ver folha «Plano de sprints» e docs/geral/00-visao-do-produto.md). A partir de 13/10 os IDs não mudam.</t>
+    <t xml:space="preserve">Ordenado pela ordem de trabalho (sprint e prioridade). Células a amarelo são para a equipa atualizar (Sprint, Estado, Responsável, SP, Notas). Replaneado a 14/10/2026 com a velocidade real (10 SP por sprint) e a decisão de o LLM conduzir a orientação (ver folha «Plano de sprints»). A partir de 13/10 os IDs não mudam.</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -199,22 +199,24 @@
     <t xml:space="preserve">—</t>
   </si>
   <si>
-    <t xml:space="preserve">US04</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Importar catálogo de instituições e cursos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como administrador, quero importar instituições e cursos a partir de um ficheiro CSV, para que o catálogo tenha várias instituições sem introduzir os dados um a um.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Aceita o formato de dados/catalogo-cursos-mvp.csv (códigos DGES, curso, instituição, área, vagas, nota do último colocado, descrição, saídas, fontes).
-• O CSV é validado (colunas obrigatórias, tipos, códigos duplicados).
-• Linhas inválidas são reportadas sem bloquear as válidas.
-• Reimportar atualiza cursos existentes pelo par código de instituição + código de curso.</t>
+    <t xml:space="preserve">US29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conversa de orientação com o LLM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como pessoa indecisa, quero conversar com um assistente que me vai fazendo perguntas sobre os meus interesses, para perceber o que procuro num curso sem preencher um questionário fixo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• As perguntas não são fixas: o LLM faz uma de cada vez, a partir das respostas anteriores, no máximo 6.
+• A página avisa para não escrever dados pessoais; emails e números longos são apagados antes de enviar, e o LLM nunca recebe email, nome ou identificadores da conta (RNF12).
+• Disponível com sessão iniciada (o limite diário do fornecedor é partilhado por todos os utilizadores).
+• Se o LLM falhar, atingir o limite ou demorar mais de 15 s, aparece uma mensagem clara e a pessoa pode tentar de novo sem perder a conversa.
+• A pessoa pode recomeçar a conversa.
+• Os testes usam o LLM falso e correm sem rede.</t>
   </si>
   <si>
     <t xml:space="preserve">Sprint 2</t>
@@ -223,69 +225,26 @@
     <t xml:space="preserve">Por fazer</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa a importar instituições e cursos (nova visão). As UCs de cada curso entram com a US06.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US05</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Consultar e comparar cursos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como pessoa indecisa, quero consultar e comparar cursos de várias instituições, para perceber as diferenças antes de decidir.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Filtros por área, instituição e localidade.
-• Ficha de cada curso com descrição, saídas profissionais, vagas, nota do último colocado e ligação à fonte.
-• Comparação de até 3 cursos lado a lado.
-• Funciona sem sessão iniciada.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Em curso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11. 14/10: trabalho antecipado no PR #14 — pesquisa de cursos reais na página de apresentação (app/catalogo/, dados da DGES lidos do CSV). Falta: filtros por área/instituição/localidade, ficha completa do curso e comparação de até 3 cursos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Questionário de orientação</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como pessoa indecisa, quero responder a um questionário curto sobre os meus interesses e preferências, para receber sugestões de curso que façam sentido para mim.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Perguntas sobre interesses, tipo de trabalho preferido, saídas que imagina, localidade e regime.
-• As perguntas e opções ficam num ficheiro editável pelo Product Owner (como app/texts.py).
-• As respostas ficam guardadas na conta e o questionário pode ser refeito (as respostas anteriores mantêm-se no histórico).
-• Responder demora menos de 2 minutos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 13/10: story nova (nova visão do produto, sugestão do docente).</t>
+    <t xml:space="preserve">Replaneamento de 13/10: story nova (questionário de perguntas fixas). 14/10: reescrita por decisão do PO — as perguntas deixam de ser fixas e o LLM conduz a conversa; absorve a US32. 3 → 5 SP (página de conversa, estado entre pedidos, erros do fornecedor). Base técnica feita no spike (PR #17: app/llm, app/orientacao). Antes de começar: decisão do PO sobre idade e plano do Gemini (docs/geral/05-spike-llm.md, secção 5). Atenção: a conversa não cabe no cookie de sessão (4 KB); tem de ficar no servidor.</t>
   </si>
   <si>
     <t xml:space="preserve">US30</t>
   </si>
   <si>
-    <t xml:space="preserve">Sugestão de cursos com LLM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como pessoa indecisa, quero receber 2 a 3 cursos sugeridos a partir das minhas respostas, cada um com uma explicação, para saber por onde começar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Os cursos sugeridos existem no catálogo; os que não existem são descartados (RN09).
-• Cada sugestão tem uma explicação curta em português de Portugal.
-• Ao LLM só seguem as respostas e o catálogo, nunca email ou nome (RNF12).
-• O fornecedor é configurável (anthropic, ollama, falso) sem mudar o resto do código (padrões Adapter e Factory, docs/geral/03).
-• Os testes usam o LLM falso e correm sem rede.
-• Se o LLM falhar ou demorar mais de 15 s, o utilizador recebe uma mensagem clara e pode tentar de novo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint 3</t>
+    <t xml:space="preserve">Sugestão de 2 a 3 cursos no fim da conversa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como pessoa indecisa, quero que a conversa termine com 2 a 3 cursos do catálogo, cada um com a explicação de porque combina comigo, para saber por onde começar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• A sugestão aparece quando o LLM tem informação suficiente ou ao fim de 6 respostas; a pessoa pode pedi-la antes («Ver sugestões»).
+• Só aparecem cursos do catálogo; os outros são descartados (RN09). Se sobrarem menos de 2, a página diz isso e propõe continuar a conversa ou ver o catálogo.
+• Cada curso mostra os dados do catálogo (instituição, localidade, vagas, nota do último colocado, ligação à DGES) e a explicação do LLM.
+• Nenhum curso é atribuído automaticamente: a escolha é feita na US31 (RN10).
+• Os testes usam o LLM falso, incluindo respostas com cursos inventados.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 13/10: story nova (sugestão a partir do questionário). 14/10: passa a ser o fim da conversa da US29 e passa do Sprint 3 para o Sprint 2 (decisão do PO). 8 → 3 SP: o fornecedor configurável, a validação contra o catálogo e os testes sem rede foram feitos no spike (PR #17).</t>
   </si>
   <si>
     <t xml:space="preserve">US31</t>
@@ -304,6 +263,39 @@
 • O utilizador pode mudar de curso, o que cria uma nova decisão.</t>
   </si>
   <si>
+    <t xml:space="preserve">Sprint 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 13/10: story nova (nova visão do produto, sugestão do docente). 14/10: mantém-se no Sprint 3; a escolha parte das sugestões da US30.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consultar e comparar cursos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como pessoa indecisa, quero consultar e comparar cursos de várias instituições, para perceber as diferenças antes de decidir.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Filtros por área, instituição e localidade.
+• Ficha de cada curso com descrição, saídas profissionais, vagas, nota do último colocado e ligação à fonte.
+• Comparação de até 3 cursos lado a lado.
+• Funciona sem sessão iniciada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Em curso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11. 14/10: trabalho antecipado no PR #14 — pesquisa de cursos reais na página de apresentação (app/catalogo/, dados da DGES lidos do CSV). Falta: filtros por área/instituição/localidade, ficha completa do curso e comparação de até 3 cursos. 14/10: Sprint 2 → Sprint 3, para o LLM entrar no Sprint 2 com a velocidade real (10 SP).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US04</t>
+  </si>
+  <si>
     <t xml:space="preserve">US06</t>
   </si>
   <si>
@@ -325,7 +317,7 @@
     <t xml:space="preserve">Sprint 4</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4; inclui a importação das UCs; 3 → 5 SP.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4; inclui a importação das UCs; 3 → 5 SP. 14/10: mantém-se no Sprint 4.</t>
   </si>
   <si>
     <t xml:space="preserve">US07</t>
@@ -340,10 +332,32 @@
     <t xml:space="preserve">• Só aparecem cursos ou UCs do meu percurso (RN01).
 • Os três campos são obrigatórios.
 • Posso editar ou apagar a avaliação.
-• Só é possível avaliar dentro de um período aberto (até à US16, o período está sempre aberto).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4.</t>
+• Só é possível avaliar dentro de um período aberto (até à US16, o período está sempre aberto).
+• As avaliações ficam ligadas a um pseudo_id desde o início, e não ao email (ponto 2 dos requisitos); as regras de visualização e exportação ficam na US09.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4. 14/10: fica no Sprint 4 sem a US09 (velocidade de 10 SP); por isso guarda já com pseudo_id.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Importar catálogo de instituições e cursos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como administrador, quero importar instituições e cursos a partir de um ficheiro CSV, para que o catálogo tenha várias instituições sem introduzir os dados um a um.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Aceita o formato de dados/catalogo-cursos-mvp.csv (códigos DGES, curso, instituição, área, vagas, nota do último colocado, descrição, saídas, fontes).
+• O CSV é validado (colunas obrigatórias, tipos, códigos duplicados).
+• Linhas inválidas são reportadas sem bloquear as válidas.
+• Reimportar atualiza cursos existentes pelo par código de instituição + código de curso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Should</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backlog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa a importar instituições e cursos (nova visão). As UCs de cada curso entram com a US06. 14/10: Sprint 2 → Backlog, Must → Should: a aplicação já lê o catálogo do CSV (app/catalogo) e o LLM trabalha sobre ele; importar para a base de dados não muda nada para o utilizador nesta release.</t>
   </si>
   <si>
     <t xml:space="preserve">US09</t>
@@ -364,7 +378,7 @@
 • Teste automático que verifica RN04.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: Sprint 2 → Sprint 4, com a US07 para as avaliações serem anónimas desde o início.</t>
+    <t xml:space="preserve">Replaneamento de 13/10: Sprint 2 → Sprint 4, com a US07 para as avaliações serem anónimas desde o início. 14/10: Sprint 4 → Backlog, Must → Should (velocidade de 10 SP). A US07 guarda já com pseudo_id; sem agregados (US11) a RN04 ainda não se aplica.</t>
   </si>
   <si>
     <t xml:space="preserve">US11</t>
@@ -385,7 +399,7 @@
 • Implementada como estratégia intercambiável (padrão Strategy, docs/geral/03).</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 2 para Sprint 3. Replaneamento de 13/10: Sprint 3 → Sprint 4; segue o padrão Strategy.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 2 para Sprint 3. Replaneamento de 13/10: Sprint 3 → Sprint 4; segue o padrão Strategy. 14/10: Sprint 4 → Backlog, Must → Should (velocidade de 10 SP). Primeira candidata se houver um Sprint 5 ou folga.</t>
   </si>
   <si>
     <t xml:space="preserve">US08</t>
@@ -400,12 +414,6 @@
     <t xml:space="preserve">• Vista em grelha com todas as obrigatórias do percurso.
 • Gravação de todas de uma vez.
 • Avaliar 10 UCs demora menos de 2 minutos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Should</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Backlog</t>
   </si>
   <si>
     <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release.</t>
@@ -709,16 +717,13 @@
     <t xml:space="preserve">Como pessoa indecisa, quero conversar com um assistente que me faça perguntas e me ajude a perceber que cursos e opcionais fazem sentido para mim, para decidir com mais confiança.</t>
   </si>
   <si>
-    <t xml:space="preserve">• A AVALIAR pelos Product Owners antes de ser estimada (ver docs/geral/01, ponto em aberto 13).
-• O assistente só fala de cursos e opcionais do catálogo (RN09) e explica cada sugestão.
-• Não recebe email, nome nem identificadores do utilizador (RNF12).
-• Funciona com o LLMFalso nos testes (sem rede).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Por avaliar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14/10: pedido do PO para verificar a inserção de um agente LLM que interaja com o utilizador. Pode estender a US29/US30 (questionário + sugestão) para uma conversa; decidir âmbito, custo e privacidade antes de estimar.</t>
+    <t xml:space="preserve">• Fundida na US29 a 14/10/2026 (decisão do PO na issue #15): a conversa com o assistente passa a ser a própria orientação. A sugestão de cursos é a US30.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fundida</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14/10: pedido do PO para verificar a inserção de um agente LLM. No mesmo dia, o PO decidiu que o LLM conduz a conversa: a story foi fundida na US29. O ID fica, para a rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">nova</t>
@@ -739,7 +744,7 @@
     <t xml:space="preserve">Calculado a partir da folha «Product Backlog»: mudar o Sprint ou o Estado de uma story lá atualiza esta tabela.</t>
   </si>
   <si>
-    <t xml:space="preserve">Velocidade estimada por sprint (SP)</t>
+    <t xml:space="preserve">Velocidade por sprint (SP) — real do Sprint 1</t>
   </si>
   <si>
     <t xml:space="preserve">Sprint Goal</t>
@@ -769,28 +774,28 @@
     <t xml:space="preserve">US01, US02, US03</t>
   </si>
   <si>
-    <t xml:space="preserve">Uma pessoa indecisa descobre e compara cursos de várias instituições e responde ao questionário de orientação.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US04, US05, US29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O OptaBem sugere cursos com explicação e o utilizador escolhe, ficando a decisão registada no percurso.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US30, US31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quem já é aluno regista o percurso, avalia opcionais de forma anónima e recebe sugestões por popularidade.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US06, US07, US09, US11</t>
+    <t xml:space="preserve">Uma pessoa indecisa conversa com o assistente (LLM), que lhe faz perguntas e lhe sugere 2 a 3 cursos do catálogo com explicação.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US29, US30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O utilizador escolhe um curso sugerido (fica registado no percurso) e consulta e compara cursos de várias instituições.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US31, US05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quem já é aluno regista as UCs que concluiu e avalia as opcionais que fez, com as avaliações pseudonimizadas desde o início.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US06, US07</t>
   </si>
   <si>
     <t xml:space="preserve">Fora do plano desta release; entra se houver folga.</t>
   </si>
   <si>
-    <t xml:space="preserve">US08, US10, US12–US28, US32</t>
+    <t xml:space="preserve">US04, US09, US11, US08, US10, US12–US28 (US32 fundida na US29)</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -857,6 +862,27 @@
   </si>
   <si>
     <t xml:space="preserve">• Redesenho visual do site (sem story própria): fica registado no PR #14 e no registo de uso de IA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 14/10/2026 (decisão do PO na issue #15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• As perguntas deixam de ser fixas: o LLM conduz a conversa. US29 reescrita (conversa, 5 SP) e US32 fundida nela; US30 passa a ser o fim da conversa (3 SP).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Spike técnico feito antes do Sprint 2 (PR #17): Gemini e Groq atrás de ClienteLLM, testes sem rede, conclusões em docs/geral/05-spike-llm.md. Não tem SP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• O LLM passa para o Sprint 2. Velocidade ajustada à real (de 23 para 10 SP): Sprint 2 com 8 SP (2 de folga pela tecnologia nova), Sprints 3 e 4 com 10 SP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US05 passa para o Sprint 3. US04, US09 e US11 passam para o Backlog (Must → Should). A US07 guarda as avaliações com pseudo_id desde o início.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Consequência: nesta release não há recomendação de opcionais (US11). Se houver um Sprint 5, entram primeiro a US09 e a US11 (8 SP).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Por decidir antes do Sprint 2: idade mínima e plano do Gemini (os termos excluem menores de 18 e o plano gratuito com utilizadores no EEE).</t>
   </si>
   <si>
     <t xml:space="preserve">Resumo por prioridade (MoSCoW)</t>
@@ -1595,13 +1621,13 @@
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>13</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>18</c:v>
+                  <c:v>10</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1703,11 +1729,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="90681899"/>
-        <c:axId val="55780184"/>
+        <c:axId val="13824179"/>
+        <c:axId val="52095193"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="90681899"/>
+        <c:axId val="13824179"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1738,7 +1764,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55780184"/>
+        <c:crossAx val="52095193"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1746,7 +1772,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="55780184"/>
+        <c:axId val="52095193"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1811,7 +1837,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="90681899"/>
+        <c:crossAx val="13824179"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1878,9 +1904,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2092680</xdr:colOff>
+      <xdr:colOff>2092320</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>89640</xdr:rowOff>
+      <xdr:rowOff>89280</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1889,7 +1915,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5757840" cy="2517480"/>
+        <a:ext cx="5757480" cy="2517120"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2266,7 +2292,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="139.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="n">
         <v>4</v>
       </c>
@@ -2302,10 +2328,10 @@
         <v>42</v>
       </c>
       <c r="M8" s="5" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="139.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="n">
         <v>5</v>
       </c>
@@ -2325,7 +2351,7 @@
         <v>46</v>
       </c>
       <c r="G9" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H9" s="5" t="s">
         <v>20</v>
@@ -2334,14 +2360,14 @@
         <v>40</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="K9" s="8"/>
       <c r="L9" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2349,35 +2375,35 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D10" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="E10" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="D10" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="E10" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>53</v>
-      </c>
       <c r="G10" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>20</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="J10" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K10" s="8"/>
       <c r="L10" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M10" s="5" t="s">
         <v>34</v>
@@ -2388,10 +2414,10 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>55</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>50</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>56</v>
@@ -2403,23 +2429,23 @@
         <v>58</v>
       </c>
       <c r="G11" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>20</v>
       </c>
       <c r="I11" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="J11" s="7" t="s">
         <v>59</v>
-      </c>
-      <c r="J11" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="K11" s="8"/>
       <c r="L11" s="8" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>34</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2427,19 +2453,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G12" s="7" t="n">
         <v>5</v>
@@ -2448,17 +2474,17 @@
         <v>20</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="J12" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="M12" s="5" t="s">
         <v>54</v>
-      </c>
-      <c r="M12" s="5" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2466,19 +2492,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>5</v>
@@ -2487,17 +2513,17 @@
         <v>20</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="J13" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2505,38 +2531,38 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>65</v>
+        <v>55</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="J14" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>64</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2544,38 +2570,38 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="G15" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="J15" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2583,38 +2609,38 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="G16" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="J16" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2622,38 +2648,38 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="G17" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J17" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K17" s="8"/>
       <c r="L17" s="8" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2661,38 +2687,38 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G18" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J18" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2700,38 +2726,38 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G19" s="7" t="n">
         <v>8</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J19" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2739,38 +2765,38 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G20" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J20" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2778,38 +2804,38 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G21" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J21" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="M21" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2817,38 +2843,38 @@
         <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="G22" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J22" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2856,38 +2882,38 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G23" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J23" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="M23" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2895,38 +2921,38 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J24" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2934,38 +2960,38 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J25" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2973,38 +2999,38 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="G26" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J26" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3012,38 +3038,38 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="G27" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J27" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3051,38 +3077,38 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J28" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3090,38 +3116,38 @@
         <v>25</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J29" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="M29" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3129,38 +3155,38 @@
         <v>26</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G30" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J30" s="7" t="s">
         <v>41</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3168,28 +3194,28 @@
         <v>27</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="G31" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J31" s="7" t="s">
         <v>41</v>
@@ -3197,7 +3223,7 @@
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
       <c r="M31" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3205,28 +3231,28 @@
         <v>28</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J32" s="7" t="s">
         <v>41</v>
@@ -3234,7 +3260,7 @@
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
       <c r="M32" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3242,28 +3268,28 @@
         <v>29</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="G33" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I33" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J33" s="7" t="s">
         <v>41</v>
@@ -3271,7 +3297,7 @@
       <c r="K33" s="8"/>
       <c r="L33" s="8"/>
       <c r="M33" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3279,28 +3305,28 @@
         <v>30</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="G34" s="7" t="n">
         <v>8</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J34" s="7" t="s">
         <v>41</v>
@@ -3308,7 +3334,7 @@
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
       <c r="M34" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3316,28 +3342,28 @@
         <v>31</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="G35" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="I35" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J35" s="7" t="s">
         <v>41</v>
@@ -3345,72 +3371,70 @@
       <c r="K35" s="8"/>
       <c r="L35" s="8"/>
       <c r="M35" s="5" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="n">
         <v>32</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="G36" s="7"/>
-      <c r="H36" s="5" t="s">
-        <v>161</v>
-      </c>
+      <c r="H36" s="5"/>
       <c r="I36" s="7" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="J36" s="7" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K36" s="8"/>
       <c r="L36" s="8" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="M36" s="5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F37" s="9" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="G37" s="9" t="n">
-        <f aca="false">SUM(G5:G35)</f>
-        <v>129</v>
+        <f aca="false">SUM(G5:G36)</f>
+        <v>126</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F38" s="9" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="G38" s="9" t="n">
-        <f aca="false">SUMIF(J5:J35,"Feito",G5:G35)</f>
+        <f aca="false">SUMIF(J5:J36,"Feito",G5:G36)</f>
         <v>10</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F39" s="10" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:M35"/>
-  <conditionalFormatting sqref="J5:J35">
+  <autoFilter ref="A4:M36"/>
+  <conditionalFormatting sqref="J5:J36">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Feito"</formula>
     </cfRule>
@@ -3418,7 +3442,7 @@
       <formula>"Em curso"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H35">
+  <conditionalFormatting sqref="H5:H36">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Must"</formula>
     </cfRule>
@@ -3432,7 +3456,7 @@
       <formula>"Won't"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I35">
+  <conditionalFormatting sqref="I5:I36">
     <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Sprint 1"</formula>
     </cfRule>
@@ -3450,20 +3474,20 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G35" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G36" type="list">
       <formula1>"1,2,3,5,8,13,21"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H35" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H36" type="list">
       <formula1>"Must,Should,Could,Won't"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I35" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I36" type="list">
       <formula1>"Sprint 1,Sprint 2,Sprint 3,Sprint 4,Backlog"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J35" type="list">
-      <formula1>"Por fazer,Em curso,Feito"</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J36" type="list">
+      <formula1>"Por fazer,Em curso,Feito,Fundida"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -3484,7 +3508,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H51"/>
+  <dimension ref="A1:H59"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -3499,20 +3523,20 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C3" s="7" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3520,25 +3544,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3546,10 +3570,10 @@
         <v>21</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D6" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A6,'Product Backlog'!$G$5:$G$36)</f>
@@ -3565,7 +3589,7 @@
       </c>
       <c r="G6" s="16" t="n">
         <f aca="false">$C$3-D6</f>
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="H6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A6)</f>
@@ -3577,14 +3601,14 @@
         <v>40</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D7" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A7,'Product Backlog'!$G$5:$G$36)</f>
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="E7" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A7,'Product Backlog'!$J$5:$J$36,"Feito")</f>
@@ -3596,26 +3620,26 @@
       </c>
       <c r="G7" s="16" t="n">
         <f aca="false">$C$3-D7</f>
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A7)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D8" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$G$5:$G$36)</f>
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="E8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$J$5:$J$36,"Feito")</f>
@@ -3627,7 +3651,7 @@
       </c>
       <c r="G8" s="16" t="n">
         <f aca="false">$C$3-D8</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="H8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A8)</f>
@@ -3636,17 +3660,17 @@
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D9" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A9,'Product Backlog'!$G$5:$G$36)</f>
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="E9" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A9,'Product Backlog'!$J$5:$J$36,"Feito")</f>
@@ -3658,26 +3682,26 @@
       </c>
       <c r="G9" s="16" t="n">
         <f aca="false">$C$3-D9</f>
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A9)</f>
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A10,'Product Backlog'!$G$5:$G$36)</f>
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="E10" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A10,'Product Backlog'!$J$5:$J$36,"Feito")</f>
@@ -3692,18 +3716,18 @@
       </c>
       <c r="H10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A10)</f>
-        <v>20</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
       <c r="D11" s="21" t="n">
         <f aca="false">SUM(D6:D10)</f>
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="E11" s="21" t="n">
         <f aca="false">SUM(E6:E10)</f>
@@ -3711,7 +3735,7 @@
       </c>
       <c r="F11" s="22" t="n">
         <f aca="false">IF(D11=0,0,E11/D11)</f>
-        <v>0.0775193798449612</v>
+        <v>0.0793650793650794</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21" t="n">
@@ -3721,107 +3745,142 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="24" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="24" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="24" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="23" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="24" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="24" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="24" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="24" t="s">
-        <v>233</v>
+        <v>235</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="23" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="24" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="24" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="24" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="24" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="24" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="24" t="s">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -3854,24 +3913,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>234</v>
+        <v>243</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>235</v>
+        <v>244</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>236</v>
+        <v>245</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>237</v>
+        <v>246</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>238</v>
+        <v>247</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3879,51 +3938,51 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="C5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A5)</f>
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D5" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$H$5:$H$36,A5,'Product Backlog'!$G$5:$G$36)</f>
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="E5" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D5/SUM($D$5:$D$8))</f>
-        <v>0.418604651162791</v>
+        <v>0.301587301587302</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>92</v>
+        <v>77</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>240</v>
+        <v>249</v>
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A6)</f>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D6" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$H$5:$H$36,A6,'Product Backlog'!$G$5:$G$36)</f>
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="E6" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D6/SUM($D$5:$D$8))</f>
-        <v>0.387596899224806</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>241</v>
+        <v>250</v>
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A7)</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D7" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$H$5:$H$36,A7,'Product Backlog'!$G$5:$G$36)</f>
@@ -3931,15 +3990,15 @@
       </c>
       <c r="E7" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D7/SUM($D$5:$D$8))</f>
-        <v>0.170542635658915</v>
+        <v>0.174603174603175</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>242</v>
+        <v>251</v>
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A8)</f>
@@ -3951,20 +4010,20 @@
       </c>
       <c r="E8" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D8/SUM($D$5:$D$8))</f>
-        <v>0.0232558139534884</v>
+        <v>0.0238095238095238</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D9" s="27" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
US29: conversa de orientação com o LLM
- Página /orientacao/ (só com sessão): o LLM faz as perguntas, uma de cada vez, no máximo 6
- Conversa guardada no servidor (tabela conversas_orientacao), sem emails nem números (RNF12)
- Erros claros, «Tentar de novo» sem perder a conversa, recomeçar
- Botão «Começar a conversa» na linha do tempo; conversa terminada avança o percurso
- LLM_TIMEOUT passa a 15 s (RNF12)
- 21 testes novos (231 no total); docs/US29 com use case, BPMN e diagramas

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jxs1JgMiGoE8QQAeMbxyRn
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -222,10 +222,10 @@
     <t xml:space="preserve">Sprint 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Por fazer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 13/10: story nova (questionário de perguntas fixas). 14/10: reescrita por decisão do PO — as perguntas deixam de ser fixas e o LLM conduz a conversa; absorve a US32. 3 → 5 SP (página de conversa, estado entre pedidos, erros do fornecedor). Base técnica feita no spike (PR #17: app/llm, app/orientacao). Antes de começar: decisão do PO sobre idade e plano do Gemini (docs/geral/05-spike-llm.md, secção 5). Atenção: a conversa não cabe no cookie de sessão (4 KB); tem de ficar no servidor.</t>
+    <t xml:space="preserve">Em curso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 13/10: story nova (questionário de perguntas fixas). 14/10: reescrita por decisão do PO — as perguntas deixam de ser fixas e o LLM conduz a conversa; absorve a US32. 3 → 5 SP (página de conversa, estado entre pedidos, erros do fornecedor). Base técnica feita no spike (PR #17: app/llm, app/orientacao). Antes de começar: decisão do PO sobre idade e plano do Gemini (docs/geral/05-spike-llm.md, secção 5). Atenção: a conversa não cabe no cookie de sessão (4 KB); tem de ficar no servidor. 14/10: feita antes do Sprint 2 por decisão do PO (PR #19), à espera de revisão; docs/US29/.</t>
   </si>
   <si>
     <t xml:space="preserve">US30</t>
@@ -244,6 +244,9 @@
 • Os testes usam o LLM falso, incluindo respostas com cursos inventados.</t>
   </si>
   <si>
+    <t xml:space="preserve">Por fazer</t>
+  </si>
+  <si>
     <t xml:space="preserve">Replaneamento de 13/10: story nova (sugestão a partir do questionário). 14/10: passa a ser o fim da conversa da US29 e passa do Sprint 3 para o Sprint 2 (decisão do PO). 8 → 3 SP: o fornecedor configurável, a validação contra o catálogo e os testes sem rede foram feitos no spike (PR #17).</t>
   </si>
   <si>
@@ -285,9 +288,6 @@
 • Ficha de cada curso com descrição, saídas profissionais, vagas, nota do último colocado e ligação à fonte.
 • Comparação de até 3 cursos lado a lado.
 • Funciona sem sessão iniciada.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Em curso</t>
   </si>
   <si>
     <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11. 14/10: trabalho antecipado no PR #14 — pesquisa de cursos reais na página de apresentação (app/catalogo/, dados da DGES lidos do CSV). Falta: filtros por área/instituição/localidade, ficha completa do curso e comparação de até 3 cursos. 14/10: Sprint 2 → Sprint 3, para o LLM entrar no Sprint 2 com a velocidade real (10 SP).</t>
@@ -1729,11 +1729,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="13824179"/>
-        <c:axId val="52095193"/>
+        <c:axId val="94559607"/>
+        <c:axId val="25671691"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="13824179"/>
+        <c:axId val="94559607"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1764,7 +1764,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="52095193"/>
+        <c:crossAx val="25671691"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1772,7 +1772,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="52095193"/>
+        <c:axId val="25671691"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1837,7 +1837,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13824179"/>
+        <c:crossAx val="94559607"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1904,9 +1904,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2092320</xdr:colOff>
+      <xdr:colOff>2091960</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>89280</xdr:rowOff>
+      <xdr:rowOff>88920</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1915,7 +1915,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5757480" cy="2517120"/>
+        <a:ext cx="5757120" cy="2516760"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2360,11 +2360,11 @@
         <v>40</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K9" s="8"/>
       <c r="L9" s="8" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M9" s="5" t="s">
         <v>34</v>
@@ -2375,19 +2375,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>36</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G10" s="7" t="n">
         <v>5</v>
@@ -2396,14 +2396,14 @@
         <v>20</v>
       </c>
       <c r="I10" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K10" s="8"/>
       <c r="L10" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="M10" s="5" t="s">
         <v>34</v>
@@ -2414,19 +2414,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>5</v>
@@ -2435,10 +2435,10 @@
         <v>20</v>
       </c>
       <c r="I11" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>59</v>
+        <v>41</v>
       </c>
       <c r="K11" s="8"/>
       <c r="L11" s="8" t="s">
@@ -2477,14 +2477,14 @@
         <v>67</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8" t="s">
         <v>68</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2516,7 +2516,7 @@
         <v>67</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8" t="s">
@@ -2534,7 +2534,7 @@
         <v>61</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>74</v>
@@ -2555,7 +2555,7 @@
         <v>78</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8" t="s">
@@ -2594,7 +2594,7 @@
         <v>78</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8" t="s">
@@ -2633,7 +2633,7 @@
         <v>78</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8" t="s">
@@ -2672,7 +2672,7 @@
         <v>78</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K17" s="8"/>
       <c r="L17" s="8" t="s">
@@ -2711,7 +2711,7 @@
         <v>78</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8" t="s">
@@ -2750,7 +2750,7 @@
         <v>78</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
@@ -2789,7 +2789,7 @@
         <v>78</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
@@ -2828,7 +2828,7 @@
         <v>78</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8" t="s">
@@ -2867,7 +2867,7 @@
         <v>78</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
@@ -2906,7 +2906,7 @@
         <v>78</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8" t="s">
@@ -2945,7 +2945,7 @@
         <v>78</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
@@ -2984,7 +2984,7 @@
         <v>78</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
@@ -3023,7 +3023,7 @@
         <v>78</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
@@ -3062,7 +3062,7 @@
         <v>78</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
@@ -3101,7 +3101,7 @@
         <v>78</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8" t="s">
@@ -3140,7 +3140,7 @@
         <v>78</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8" t="s">
@@ -3179,7 +3179,7 @@
         <v>78</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8" t="s">
@@ -3218,7 +3218,7 @@
         <v>78</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
@@ -3255,7 +3255,7 @@
         <v>78</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
@@ -3292,7 +3292,7 @@
         <v>78</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K33" s="8"/>
       <c r="L33" s="8"/>
@@ -3329,7 +3329,7 @@
         <v>78</v>
       </c>
       <c r="J34" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
@@ -3366,7 +3366,7 @@
         <v>78</v>
       </c>
       <c r="J35" s="7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="K35" s="8"/>
       <c r="L35" s="8"/>
@@ -3629,7 +3629,7 @@
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B8" s="14" t="s">
         <v>208</v>
@@ -3848,37 +3848,37 @@
         <v>235</v>
       </c>
     </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="23" t="s">
         <v>236</v>
       </c>
     </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="24" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="24" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="24" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="24" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="24" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="24" t="s">
         <v>242</v>
       </c>

</xml_diff>

<commit_message>
Revisão de 20/10: corrigir histórico dos requisitos e estado da US05
- Histórico dos requisitos por ordem (1.3 antes de 1.4); frase sobre o
  Excel e o Word atualizada
- US05 volta a «Por fazer» (Excel e PROJETO.md): não fica trabalho em
  curso num sprint que ainda não começou; a pesquisa de 14/10 e a página
  /cursos/ contam como parte já entregue
- Registo de uso de IA

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015vDh8NssB4QRgbuJ248CJh
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -244,9 +244,6 @@
 • Os testes usam o LLM falso, incluindo respostas com cursos inventados.</t>
   </si>
   <si>
-    <t xml:space="preserve">Por fazer</t>
-  </si>
-  <si>
     <t xml:space="preserve">Replaneamento de 13/10: story nova (sugestão a partir do questionário). 14/10: passa a ser o fim da conversa da US29 e passa do Sprint 3 para o Sprint 2 (decisão do PO). 8 → 3 SP: o fornecedor configurável, a validação contra o catálogo e os testes sem rede foram feitos no spike (PR #17).</t>
   </si>
   <si>
@@ -269,6 +266,9 @@
     <t xml:space="preserve">Sprint 3</t>
   </si>
   <si>
+    <t xml:space="preserve">Por fazer</t>
+  </si>
+  <si>
     <t xml:space="preserve">Replaneamento de 13/10: story nova (nova visão do produto, sugestão do docente). 14/10: mantém-se no Sprint 3; a escolha parte das sugestões da US30.</t>
   </si>
   <si>
@@ -290,7 +290,7 @@
 • Funciona sem sessão iniciada.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11. 14/10: trabalho antecipado no PR #14 — pesquisa de cursos reais na página de apresentação (app/catalogo/, dados da DGES lidos do CSV). Falta: filtros por área/instituição/localidade, ficha completa do curso e comparação de até 3 cursos. 14/10: Sprint 2 → Sprint 3, para o LLM entrar no Sprint 2 com a velocidade real (10 SP).</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11. 14/10: trabalho antecipado no PR #14 — pesquisa de cursos reais na página de apresentação (app/catalogo/, dados da DGES lidos do CSV). Falta: filtros por área/instituição/localidade, ficha completa do curso e comparação de até 3 cursos. 14/10: Sprint 2 → Sprint 3, para o LLM entrar no Sprint 2 com a velocidade real (10 SP). 20/10: estado volta a «Por fazer» (não fica trabalho em curso num sprint que ainda não começou); a pesquisa de 14/10 e a página /cursos/ (US30) contam como parte já entregue.</t>
   </si>
   <si>
     <t xml:space="preserve">US04</t>
@@ -1148,111 +1148,111 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1729,11 +1729,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="94559607"/>
-        <c:axId val="25671691"/>
+        <c:axId val="40819930"/>
+        <c:axId val="97489759"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="94559607"/>
+        <c:axId val="40819930"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1764,7 +1764,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="25671691"/>
+        <c:crossAx val="97489759"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1772,7 +1772,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="25671691"/>
+        <c:axId val="97489759"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1837,7 +1837,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94559607"/>
+        <c:crossAx val="40819930"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1904,9 +1904,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2091960</xdr:colOff>
+      <xdr:colOff>2091600</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>88920</xdr:rowOff>
+      <xdr:rowOff>88560</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1915,7 +1915,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5757120" cy="2516760"/>
+        <a:ext cx="5756760" cy="2516400"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2364,7 +2364,7 @@
       </c>
       <c r="K9" s="8"/>
       <c r="L9" s="8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="M9" s="5" t="s">
         <v>34</v>
@@ -2375,19 +2375,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>36</v>
       </c>
       <c r="D10" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>50</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>51</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>52</v>
       </c>
       <c r="G10" s="7" t="n">
         <v>5</v>
@@ -2396,10 +2396,10 @@
         <v>20</v>
       </c>
       <c r="I10" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="J10" s="7" t="s">
         <v>53</v>
-      </c>
-      <c r="J10" s="7" t="s">
-        <v>47</v>
       </c>
       <c r="K10" s="8"/>
       <c r="L10" s="8" t="s">
@@ -2435,10 +2435,10 @@
         <v>20</v>
       </c>
       <c r="I11" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="J11" s="7" t="s">
         <v>53</v>
-      </c>
-      <c r="J11" s="7" t="s">
-        <v>41</v>
       </c>
       <c r="K11" s="8"/>
       <c r="L11" s="8" t="s">
@@ -2477,7 +2477,7 @@
         <v>67</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8" t="s">
@@ -2516,7 +2516,7 @@
         <v>67</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8" t="s">
@@ -2555,7 +2555,7 @@
         <v>78</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8" t="s">
@@ -2594,7 +2594,7 @@
         <v>78</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8" t="s">
@@ -2633,7 +2633,7 @@
         <v>78</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8" t="s">
@@ -2672,7 +2672,7 @@
         <v>78</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K17" s="8"/>
       <c r="L17" s="8" t="s">
@@ -2711,7 +2711,7 @@
         <v>78</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8" t="s">
@@ -2750,7 +2750,7 @@
         <v>78</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
@@ -2789,7 +2789,7 @@
         <v>78</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
@@ -2828,7 +2828,7 @@
         <v>78</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8" t="s">
@@ -2867,7 +2867,7 @@
         <v>78</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
@@ -2906,7 +2906,7 @@
         <v>78</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8" t="s">
@@ -2945,7 +2945,7 @@
         <v>78</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
@@ -2984,7 +2984,7 @@
         <v>78</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
@@ -3023,7 +3023,7 @@
         <v>78</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
@@ -3062,7 +3062,7 @@
         <v>78</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
@@ -3101,7 +3101,7 @@
         <v>78</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8" t="s">
@@ -3140,7 +3140,7 @@
         <v>78</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8" t="s">
@@ -3179,7 +3179,7 @@
         <v>78</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8" t="s">
@@ -3218,7 +3218,7 @@
         <v>78</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
@@ -3255,7 +3255,7 @@
         <v>78</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
@@ -3292,7 +3292,7 @@
         <v>78</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K33" s="8"/>
       <c r="L33" s="8"/>
@@ -3329,7 +3329,7 @@
         <v>78</v>
       </c>
       <c r="J34" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
@@ -3366,7 +3366,7 @@
         <v>78</v>
       </c>
       <c r="J35" s="7" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
       <c r="K35" s="8"/>
       <c r="L35" s="8"/>
@@ -3629,7 +3629,7 @@
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B8" s="14" t="s">
         <v>208</v>

</xml_diff>

<commit_message>
Sprint Planning do Sprint 2: US31 antecipada e ponto 14 decidido
- US29 e US30 feitas antes do sprint: entra a US31 (5 SP), antecipada do
  Sprint 3 (decisão do PO). Sprint 2: 13 SP (8 já feitos); Sprint 3: US05,
  5 SP, a completar no fim do Sprint 2
- Ponto 14 decidido (opção a): protótipo usado pela equipa e na
  demonstração, com aviso de 18+; requisitos 1.5, spike e docs/US29
- Excel (sprints, objetivos e notas), PROJETO.md, registo de IA; issue #27

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015vDh8NssB4QRgbuJ248CJh
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="252">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="256">
   <si>
     <t xml:space="preserve">Product Backlog — Recomendador de UCs Opcionais</t>
   </si>
@@ -263,13 +263,10 @@
 • O utilizador pode mudar de curso, o que cria uma nova decisão.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sprint 3</t>
-  </si>
-  <si>
     <t xml:space="preserve">Por fazer</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: story nova (nova visão do produto, sugestão do docente). 14/10: mantém-se no Sprint 3; a escolha parte das sugestões da US30.</t>
+    <t xml:space="preserve">Replaneamento de 13/10: story nova (nova visão do produto, sugestão do docente). 14/10: mantém-se no Sprint 3; a escolha parte das sugestões da US30. 20/10 (Sprint Planning): antecipada para o Sprint 2, porque a US29 e a US30 foram feitas antes de o sprint começar; é ela que dá sentido às sugestões.</t>
   </si>
   <si>
     <t xml:space="preserve">US05</t>
@@ -288,6 +285,9 @@
 • Ficha de cada curso com descrição, saídas profissionais, vagas, nota do último colocado e ligação à fonte.
 • Comparação de até 3 cursos lado a lado.
 • Funciona sem sessão iniciada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 3</t>
   </si>
   <si>
     <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11. 14/10: trabalho antecipado no PR #14 — pesquisa de cursos reais na página de apresentação (app/catalogo/, dados da DGES lidos do CSV). Falta: filtros por área/instituição/localidade, ficha completa do curso e comparação de até 3 cursos. 14/10: Sprint 2 → Sprint 3, para o LLM entrar no Sprint 2 com a velocidade real (10 SP). 20/10: estado volta a «Por fazer» (não fica trabalho em curso num sprint que ainda não começou); a pesquisa de 14/10 e a página /cursos/ (US30) contam como parte já entregue.</t>
@@ -774,16 +774,13 @@
     <t xml:space="preserve">US01, US02, US03</t>
   </si>
   <si>
-    <t xml:space="preserve">Uma pessoa indecisa conversa com o assistente (LLM), que lhe faz perguntas e lhe sugere 2 a 3 cursos do catálogo com explicação.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US29, US30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O utilizador escolhe um curso sugerido (fica registado no percurso) e consulta e compara cursos de várias instituições.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US31, US05</t>
+    <t xml:space="preserve">Uma pessoa indecisa conversa com o assistente (LLM), recebe 2 a 3 cursos do catálogo com explicação e escolhe um, ficando a decisão registada no percurso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US29, US30, US31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uma pessoa indecisa consulta e compara cursos de várias instituições (a completar no fim do Sprint 2).</t>
   </si>
   <si>
     <t xml:space="preserve">Quem já é aluno regista as UCs que concluiu e avalia as opcionais que fez, com as avaliações pseudonimizadas desde o início.</t>
@@ -883,6 +880,21 @@
   </si>
   <si>
     <t xml:space="preserve">• Por decidir antes do Sprint 2: idade mínima e plano do Gemini (os termos excluem menores de 18 e o plano gratuito com utilizadores no EEE).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint Planning do Sprint 2 (20/10/2026, decisão do PO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• A US29 e a US30 (8 SP) foram feitas antes de o sprint começar (PR #19, #20 e #22 a #24). Para o sprint ter trabalho novo, entra a US31 (5 SP), antecipada do Sprint 3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• O Sprint 2 fica com 13 SP planeados, acima da velocidade (10), mas só 5 SP são trabalho novo. O Sprint 3 fica com a US05 (5 SP) e 5 SP por planear: rever no fim do Sprint 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Ponto 14 decidido: o OptaBem é um protótipo usado pela equipa e na demonstração, com aviso de 18+ na conversa; fica escrito no relatório.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Servidor Ollama da faculdade testado e posto de parte: lento e não obedece ao pedido de sugestão (PR #25 e #26; 05-spike-llm.md, secção 7). Fica o Gemini.</t>
   </si>
   <si>
     <t xml:space="preserve">Resumo por prioridade (MoSCoW)</t>
@@ -1621,10 +1633,10 @@
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>8</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>10</c:v>
+                  <c:v>5</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>10</c:v>
@@ -1729,11 +1741,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="40819930"/>
-        <c:axId val="97489759"/>
+        <c:axId val="77687915"/>
+        <c:axId val="438351"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="40819930"/>
+        <c:axId val="77687915"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1764,7 +1776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97489759"/>
+        <c:crossAx val="438351"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1772,7 +1784,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="97489759"/>
+        <c:axId val="438351"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1837,7 +1849,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="40819930"/>
+        <c:crossAx val="77687915"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1904,9 +1916,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2091600</xdr:colOff>
+      <xdr:colOff>2091240</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>88560</xdr:rowOff>
+      <xdr:rowOff>88200</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1915,7 +1927,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5756760" cy="2516400"/>
+        <a:ext cx="5756400" cy="2516040"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2396,14 +2408,14 @@
         <v>20</v>
       </c>
       <c r="I10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="J10" s="7" t="s">
         <v>52</v>
-      </c>
-      <c r="J10" s="7" t="s">
-        <v>53</v>
       </c>
       <c r="K10" s="8"/>
       <c r="L10" s="8" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M10" s="5" t="s">
         <v>34</v>
@@ -2414,19 +2426,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="E11" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>59</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>5</v>
@@ -2435,10 +2447,10 @@
         <v>20</v>
       </c>
       <c r="I11" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="J11" s="7" t="s">
         <v>52</v>
-      </c>
-      <c r="J11" s="7" t="s">
-        <v>53</v>
       </c>
       <c r="K11" s="8"/>
       <c r="L11" s="8" t="s">
@@ -2477,14 +2489,14 @@
         <v>67</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8" t="s">
         <v>68</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2516,7 +2528,7 @@
         <v>67</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8" t="s">
@@ -2534,7 +2546,7 @@
         <v>61</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>74</v>
@@ -2555,7 +2567,7 @@
         <v>78</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8" t="s">
@@ -2594,7 +2606,7 @@
         <v>78</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8" t="s">
@@ -2633,7 +2645,7 @@
         <v>78</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8" t="s">
@@ -2672,7 +2684,7 @@
         <v>78</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K17" s="8"/>
       <c r="L17" s="8" t="s">
@@ -2711,7 +2723,7 @@
         <v>78</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8" t="s">
@@ -2750,7 +2762,7 @@
         <v>78</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
@@ -2789,7 +2801,7 @@
         <v>78</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
@@ -2828,7 +2840,7 @@
         <v>78</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8" t="s">
@@ -2867,7 +2879,7 @@
         <v>78</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
@@ -2906,7 +2918,7 @@
         <v>78</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8" t="s">
@@ -2945,7 +2957,7 @@
         <v>78</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
@@ -2984,7 +2996,7 @@
         <v>78</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
@@ -3023,7 +3035,7 @@
         <v>78</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
@@ -3062,7 +3074,7 @@
         <v>78</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
@@ -3101,7 +3113,7 @@
         <v>78</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8" t="s">
@@ -3140,7 +3152,7 @@
         <v>78</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8" t="s">
@@ -3179,7 +3191,7 @@
         <v>78</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8" t="s">
@@ -3218,7 +3230,7 @@
         <v>78</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
@@ -3255,7 +3267,7 @@
         <v>78</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
@@ -3292,7 +3304,7 @@
         <v>78</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K33" s="8"/>
       <c r="L33" s="8"/>
@@ -3329,7 +3341,7 @@
         <v>78</v>
       </c>
       <c r="J34" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
@@ -3366,7 +3378,7 @@
         <v>78</v>
       </c>
       <c r="J35" s="7" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K35" s="8"/>
       <c r="L35" s="8"/>
@@ -3508,7 +3520,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -3608,7 +3620,7 @@
       </c>
       <c r="D7" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A7,'Product Backlog'!$G$5:$G$36)</f>
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="E7" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A7,'Product Backlog'!$J$5:$J$36,"Feito")</f>
@@ -3620,26 +3632,26 @@
       </c>
       <c r="G7" s="16" t="n">
         <f aca="false">$C$3-D7</f>
-        <v>2</v>
+        <v>-3</v>
       </c>
       <c r="H7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A7)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="B8" s="14" t="s">
         <v>208</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>209</v>
+        <v>54</v>
       </c>
       <c r="D8" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$G$5:$G$36)</f>
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$J$5:$J$36,"Feito")</f>
@@ -3651,11 +3663,11 @@
       </c>
       <c r="G8" s="16" t="n">
         <f aca="false">$C$3-D8</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A8)</f>
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3663,10 +3675,10 @@
         <v>67</v>
       </c>
       <c r="B9" s="14" t="s">
+        <v>209</v>
+      </c>
+      <c r="C9" s="14" t="s">
         <v>210</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>211</v>
       </c>
       <c r="D9" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A9,'Product Backlog'!$G$5:$G$36)</f>
@@ -3694,10 +3706,10 @@
         <v>78</v>
       </c>
       <c r="B10" s="14" t="s">
+        <v>211</v>
+      </c>
+      <c r="C10" s="14" t="s">
         <v>212</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>213</v>
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A10,'Product Backlog'!$G$5:$G$36)</f>
@@ -3721,7 +3733,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
@@ -3745,142 +3757,167 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="24" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="24" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="24" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="23" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="24" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="24" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="24" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="24" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="23" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="24" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="24" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="24" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="24" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="24" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="24" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="23" t="s">
         <v>242</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="24" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A62" s="24" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="24" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="24" t="s">
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -3913,24 +3950,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>245</v>
+        <v>249</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>203</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>246</v>
+        <v>250</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>247</v>
+        <v>251</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3938,7 +3975,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="C5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A5)</f>
@@ -3958,7 +3995,7 @@
         <v>77</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>249</v>
+        <v>253</v>
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A6)</f>
@@ -3978,7 +4015,7 @@
         <v>163</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>250</v>
+        <v>254</v>
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A7)</f>
@@ -3998,7 +4035,7 @@
         <v>183</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>251</v>
+        <v>255</v>
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A8)</f>
@@ -4015,7 +4052,7 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>

</xml_diff>

<commit_message>
US31: escolher curso e linha do tempo do percurso
- «Escolher este curso» nos cursos sugeridos e, com sessão, em /cursos/;
  página de confirmação: só o POST regista (RN10); só cursos do catálogo
- Tabela decisoes: data, curso e instituição, cursos sugeridos nessa
  altura e origem (sugestão ou catálogo) (RF35)
- O curso do perfil é a decisão mais recente (RF03); a página inicial
  mostra-o e o percurso passa a «com curso»
- /percurso/: linha do tempo, da mais recente para a mais antiga; mudar
  de curso cria uma decisão nova; o mesmo curso não
- Depois de escolher, a conversa com o LLM é apagada (ponto 15, PO)
- app/percurso.py passa a pacote app/percurso/ (State em __init__.py)
- tests/test_escolha.py (20 testes, 275 no total); docs/US31 com
  requisitos, use case, BPMN e diagramas; requisitos 1.6, 03, guia,
  PROJETO.md, Excel e registo de IA. Refs #27

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015vDh8NssB4QRgbuJ248CJh
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -263,10 +263,7 @@
 • O utilizador pode mudar de curso, o que cria uma nova decisão.</t>
   </si>
   <si>
-    <t xml:space="preserve">Por fazer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 13/10: story nova (nova visão do produto, sugestão do docente). 14/10: mantém-se no Sprint 3; a escolha parte das sugestões da US30. 20/10 (Sprint Planning): antecipada para o Sprint 2, porque a US29 e a US30 foram feitas antes de o sprint começar; é ela que dá sentido às sugestões.</t>
+    <t xml:space="preserve">Replaneamento de 13/10: story nova (nova visão do produto, sugestão do docente). 14/10: mantém-se no Sprint 3; a escolha parte das sugestões da US30. 20/10 (Sprint Planning): antecipada para o Sprint 2, porque a US29 e a US30 foram feitas antes de o sprint começar; é ela que dá sentido às sugestões. 20/10: feita (PR da US31, à espera de revisão); docs/US31/, issue #27. Depois de escolher, a conversa com o LLM é apagada (ponto 15, decisão do PO).</t>
   </si>
   <si>
     <t xml:space="preserve">US05</t>
@@ -288,6 +285,9 @@
   </si>
   <si>
     <t xml:space="preserve">Sprint 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por fazer</t>
   </si>
   <si>
     <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11. 14/10: trabalho antecipado no PR #14 — pesquisa de cursos reais na página de apresentação (app/catalogo/, dados da DGES lidos do CSV). Falta: filtros por área/instituição/localidade, ficha completa do curso e comparação de até 3 cursos. 14/10: Sprint 2 → Sprint 3, para o LLM entrar no Sprint 2 com a velocidade real (10 SP). 20/10: estado volta a «Por fazer» (não fica trabalho em curso num sprint que ainda não começou); a pesquisa de 14/10 e a página /cursos/ (US30) contam como parte já entregue.</t>
@@ -1741,11 +1741,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="77687915"/>
-        <c:axId val="438351"/>
+        <c:axId val="46601744"/>
+        <c:axId val="56421148"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="77687915"/>
+        <c:axId val="46601744"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1776,7 +1776,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="438351"/>
+        <c:crossAx val="56421148"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1784,7 +1784,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="438351"/>
+        <c:axId val="56421148"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1849,7 +1849,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77687915"/>
+        <c:crossAx val="46601744"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1916,9 +1916,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2091240</xdr:colOff>
+      <xdr:colOff>2090880</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>88200</xdr:rowOff>
+      <xdr:rowOff>87840</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1927,7 +1927,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5756400" cy="2516040"/>
+        <a:ext cx="5756040" cy="2515680"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2411,11 +2411,11 @@
         <v>40</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="K10" s="8"/>
       <c r="L10" s="8" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="M10" s="5" t="s">
         <v>34</v>
@@ -2426,19 +2426,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="E11" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>57</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>58</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>5</v>
@@ -2447,10 +2447,10 @@
         <v>20</v>
       </c>
       <c r="I11" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="J11" s="7" t="s">
         <v>59</v>
-      </c>
-      <c r="J11" s="7" t="s">
-        <v>52</v>
       </c>
       <c r="K11" s="8"/>
       <c r="L11" s="8" t="s">
@@ -2489,14 +2489,14 @@
         <v>67</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8" t="s">
         <v>68</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2528,7 +2528,7 @@
         <v>67</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8" t="s">
@@ -2546,7 +2546,7 @@
         <v>61</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>74</v>
@@ -2567,7 +2567,7 @@
         <v>78</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8" t="s">
@@ -2606,7 +2606,7 @@
         <v>78</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8" t="s">
@@ -2645,7 +2645,7 @@
         <v>78</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8" t="s">
@@ -2684,7 +2684,7 @@
         <v>78</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K17" s="8"/>
       <c r="L17" s="8" t="s">
@@ -2723,7 +2723,7 @@
         <v>78</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8" t="s">
@@ -2762,7 +2762,7 @@
         <v>78</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
@@ -2801,7 +2801,7 @@
         <v>78</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
@@ -2840,7 +2840,7 @@
         <v>78</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8" t="s">
@@ -2879,7 +2879,7 @@
         <v>78</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
@@ -2918,7 +2918,7 @@
         <v>78</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8" t="s">
@@ -2957,7 +2957,7 @@
         <v>78</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
@@ -2996,7 +2996,7 @@
         <v>78</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
@@ -3035,7 +3035,7 @@
         <v>78</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
@@ -3074,7 +3074,7 @@
         <v>78</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
@@ -3113,7 +3113,7 @@
         <v>78</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8" t="s">
@@ -3152,7 +3152,7 @@
         <v>78</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8" t="s">
@@ -3191,7 +3191,7 @@
         <v>78</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8" t="s">
@@ -3230,7 +3230,7 @@
         <v>78</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
@@ -3267,7 +3267,7 @@
         <v>78</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
@@ -3304,7 +3304,7 @@
         <v>78</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K33" s="8"/>
       <c r="L33" s="8"/>
@@ -3341,7 +3341,7 @@
         <v>78</v>
       </c>
       <c r="J34" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
@@ -3378,7 +3378,7 @@
         <v>78</v>
       </c>
       <c r="J35" s="7" t="s">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="K35" s="8"/>
       <c r="L35" s="8"/>
@@ -3641,13 +3641,13 @@
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B8" s="14" t="s">
         <v>208</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D8" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$G$5:$G$36)</f>

</xml_diff>

<commit_message>
Fecho do Sprint 2: US29, US30 e US31 aceites na Sprint Review
Estado «Feito» e notas no Excel (13 de 13 SP), PROJETO.md com a Sprint
Review de 22/10 e a decisão dos PO (cursos no centro até 05/11; opcionais
em segundo plano), páginas das stories, guia do código e registo de uso
de IA. Sem alterações de código.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014RHhrBcR4DQAiiEiK69qYD
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="255">
   <si>
     <t xml:space="preserve">Product Backlog — Recomendador de UCs Opcionais</t>
   </si>
@@ -222,10 +222,7 @@
     <t xml:space="preserve">Sprint 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Em curso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 13/10: story nova (questionário de perguntas fixas). 14/10: reescrita por decisão do PO — as perguntas deixam de ser fixas e o LLM conduz a conversa; absorve a US32. 3 → 5 SP (página de conversa, estado entre pedidos, erros do fornecedor). Base técnica feita no spike (PR #17: app/llm, app/orientacao). Antes de começar: decisão do PO sobre idade e plano do Gemini (docs/geral/05-spike-llm.md, secção 5). Atenção: a conversa não cabe no cookie de sessão (4 KB); tem de ficar no servidor. 14/10: feita antes do Sprint 2 por decisão do PO (PR #19), à espera de revisão; docs/US29/.</t>
+    <t xml:space="preserve">Replaneamento de 13/10: story nova (questionário de perguntas fixas). 14/10: reescrita por decisão do PO — as perguntas deixam de ser fixas e o LLM conduz a conversa; absorve a US32. 3 → 5 SP (página de conversa, estado entre pedidos, erros do fornecedor). Base técnica feita no spike (PR #17: app/llm, app/orientacao). Antes de começar: decisão do PO sobre idade e plano do Gemini (docs/geral/05-spike-llm.md, secção 5). Atenção: a conversa não cabe no cookie de sessão (4 KB); tem de ficar no servidor. 14/10: feita antes do Sprint 2 por decisão do PO (PR #19), à espera de revisão; docs/US29/. 22/10: aceite na Sprint Review do Sprint 2 (percurso completo testado pelos PO com o Gemini real, também noutro computador); fica Feito.</t>
   </si>
   <si>
     <t xml:space="preserve">US30</t>
@@ -244,7 +241,7 @@
 • Os testes usam o LLM falso, incluindo respostas com cursos inventados.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: story nova (sugestão a partir do questionário). 14/10: passa a ser o fim da conversa da US29 e passa do Sprint 3 para o Sprint 2 (decisão do PO). 8 → 3 SP: o fornecedor configurável, a validação contra o catálogo e os testes sem rede foram feitos no spike (PR #17).</t>
+    <t xml:space="preserve">Replaneamento de 13/10: story nova (sugestão a partir do questionário). 14/10: passa a ser o fim da conversa da US29 e passa do Sprint 3 para o Sprint 2 (decisão do PO). 8 → 3 SP: o fornecedor configurável, a validação contra o catálogo e os testes sem rede foram feitos no spike (PR #17). 22/10: aceite na Sprint Review do Sprint 2 (percurso completo testado pelos PO com o Gemini real, também noutro computador); fica Feito.</t>
   </si>
   <si>
     <t xml:space="preserve">US31</t>
@@ -263,7 +260,7 @@
 • O utilizador pode mudar de curso, o que cria uma nova decisão.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: story nova (nova visão do produto, sugestão do docente). 14/10: mantém-se no Sprint 3; a escolha parte das sugestões da US30. 20/10 (Sprint Planning): antecipada para o Sprint 2, porque a US29 e a US30 foram feitas antes de o sprint começar; é ela que dá sentido às sugestões. 20/10: feita (PR da US31, à espera de revisão); docs/US31/, issue #27. Depois de escolher, a conversa com o LLM é apagada (ponto 15, decisão do PO).</t>
+    <t xml:space="preserve">Replaneamento de 13/10: story nova (nova visão do produto, sugestão do docente). 14/10: mantém-se no Sprint 3; a escolha parte das sugestões da US30. 20/10 (Sprint Planning): antecipada para o Sprint 2, porque a US29 e a US30 foram feitas antes de o sprint começar; é ela que dá sentido às sugestões. 20/10: feita (PR da US31, à espera de revisão); docs/US31/, issue #27. Depois de escolher, a conversa com o LLM é apagada (ponto 15, decisão do PO). 22/10: aceite na Sprint Review do Sprint 2 (percurso completo testado pelos PO com o Gemini real, também noutro computador); fica Feito.</t>
   </si>
   <si>
     <t xml:space="preserve">US05</t>
@@ -1277,7 +1274,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="22">
+  <dxfs count="21">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1369,14 +1366,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1727,7 +1716,7 @@
                   <c:v>10</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0</c:v>
+                  <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="2">
                   <c:v>0</c:v>
@@ -1741,11 +1730,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="46601744"/>
-        <c:axId val="56421148"/>
+        <c:axId val="85281332"/>
+        <c:axId val="13198070"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="46601744"/>
+        <c:axId val="85281332"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1776,7 +1765,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="56421148"/>
+        <c:crossAx val="13198070"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1784,7 +1773,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="56421148"/>
+        <c:axId val="13198070"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1849,7 +1838,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="46601744"/>
+        <c:crossAx val="85281332"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1916,9 +1905,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2090880</xdr:colOff>
+      <xdr:colOff>2090520</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>87840</xdr:rowOff>
+      <xdr:rowOff>87480</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1927,7 +1916,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5756040" cy="2515680"/>
+        <a:ext cx="5755680" cy="2515320"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2333,11 +2322,11 @@
         <v>40</v>
       </c>
       <c r="J8" s="7" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="K8" s="8"/>
       <c r="L8" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="M8" s="5" t="s">
         <v>34</v>
@@ -2348,19 +2337,19 @@
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>36</v>
       </c>
       <c r="D9" s="6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="E9" s="6" t="s">
+      <c r="F9" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>46</v>
       </c>
       <c r="G9" s="7" t="n">
         <v>3</v>
@@ -2372,11 +2361,11 @@
         <v>40</v>
       </c>
       <c r="J9" s="7" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="K9" s="8"/>
       <c r="L9" s="8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="M9" s="5" t="s">
         <v>34</v>
@@ -2387,19 +2376,19 @@
         <v>6</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>36</v>
       </c>
       <c r="D10" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="E10" s="6" t="s">
+      <c r="F10" s="6" t="s">
         <v>50</v>
-      </c>
-      <c r="F10" s="6" t="s">
-        <v>51</v>
       </c>
       <c r="G10" s="7" t="n">
         <v>5</v>
@@ -2411,11 +2400,11 @@
         <v>40</v>
       </c>
       <c r="J10" s="7" t="s">
-        <v>41</v>
+        <v>22</v>
       </c>
       <c r="K10" s="8"/>
       <c r="L10" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="M10" s="5" t="s">
         <v>34</v>
@@ -2426,19 +2415,19 @@
         <v>7</v>
       </c>
       <c r="B11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="D11" s="6" t="s">
+      <c r="E11" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="E11" s="6" t="s">
+      <c r="F11" s="6" t="s">
         <v>56</v>
-      </c>
-      <c r="F11" s="6" t="s">
-        <v>57</v>
       </c>
       <c r="G11" s="7" t="n">
         <v>5</v>
@@ -2447,17 +2436,17 @@
         <v>20</v>
       </c>
       <c r="I11" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="J11" s="7" t="s">
         <v>58</v>
-      </c>
-      <c r="J11" s="7" t="s">
-        <v>59</v>
       </c>
       <c r="K11" s="8"/>
       <c r="L11" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="M11" s="5" t="s">
         <v>60</v>
-      </c>
-      <c r="M11" s="5" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2465,19 +2454,19 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="D12" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="E12" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="F12" s="6" t="s">
         <v>65</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>66</v>
       </c>
       <c r="G12" s="7" t="n">
         <v>5</v>
@@ -2486,17 +2475,17 @@
         <v>20</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2504,19 +2493,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D13" s="6" t="s">
+      <c r="E13" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="F13" s="6" t="s">
         <v>71</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>72</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>5</v>
@@ -2525,17 +2514,17 @@
         <v>20</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2543,35 +2532,35 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D14" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="E14" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="6" t="s">
         <v>75</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>76</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H14" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I14" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I14" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J14" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="M14" s="5" t="s">
         <v>29</v>
@@ -2582,38 +2571,38 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="E15" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>84</v>
       </c>
       <c r="G15" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H15" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I15" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I15" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J15" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2621,38 +2610,38 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="E16" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>89</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>90</v>
       </c>
       <c r="G16" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H16" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I16" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I16" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J16" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2660,38 +2649,38 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="C17" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D17" s="6" t="s">
+      <c r="E17" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="F17" s="6" t="s">
         <v>94</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>95</v>
       </c>
       <c r="G17" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H17" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I17" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I17" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J17" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K17" s="8"/>
       <c r="L17" s="8" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2699,38 +2688,38 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
+        <v>96</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="E18" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="F18" s="6" t="s">
         <v>100</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>101</v>
       </c>
       <c r="G18" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H18" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I18" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I18" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J18" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="M18" s="5" t="s">
         <v>102</v>
-      </c>
-      <c r="M18" s="5" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2738,38 +2727,38 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="D19" s="6" t="s">
+      <c r="E19" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="F19" s="6" t="s">
         <v>106</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>107</v>
       </c>
       <c r="G19" s="7" t="n">
         <v>8</v>
       </c>
       <c r="H19" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I19" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I19" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J19" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2777,38 +2766,38 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="E20" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="F20" s="6" t="s">
         <v>111</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>112</v>
       </c>
       <c r="G20" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H20" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I20" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I20" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J20" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2816,38 +2805,38 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="E21" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="F21" s="6" t="s">
         <v>117</v>
-      </c>
-      <c r="F21" s="6" t="s">
-        <v>118</v>
       </c>
       <c r="G21" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H21" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I21" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I21" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J21" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="M21" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2855,38 +2844,38 @@
         <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D22" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="E22" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="F22" s="6" t="s">
         <v>121</v>
-      </c>
-      <c r="F22" s="6" t="s">
-        <v>122</v>
       </c>
       <c r="G22" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H22" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I22" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I22" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J22" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
+        <v>122</v>
+      </c>
+      <c r="M22" s="5" t="s">
         <v>123</v>
-      </c>
-      <c r="M22" s="5" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2894,38 +2883,38 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="D23" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="E23" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="F23" s="6" t="s">
         <v>128</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>129</v>
       </c>
       <c r="G23" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H23" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I23" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I23" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J23" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8" t="s">
+        <v>129</v>
+      </c>
+      <c r="M23" s="5" t="s">
         <v>130</v>
-      </c>
-      <c r="M23" s="5" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2933,38 +2922,38 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="D24" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="C24" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="D24" s="6" t="s">
+      <c r="E24" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="F24" s="6" t="s">
         <v>134</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>135</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H24" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I24" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I24" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J24" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2972,38 +2961,38 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="C25" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D25" s="6" t="s">
+      <c r="E25" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="F25" s="6" t="s">
         <v>139</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>140</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H25" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I25" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I25" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J25" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3011,38 +3000,38 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="C26" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="D26" s="6" t="s">
+      <c r="E26" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="F26" s="6" t="s">
         <v>143</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>144</v>
       </c>
       <c r="G26" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H26" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I26" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I26" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J26" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3050,38 +3039,38 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D27" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="E27" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="F27" s="6" t="s">
         <v>147</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>148</v>
       </c>
       <c r="G27" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H27" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I27" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I27" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J27" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3089,38 +3078,38 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D28" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="E28" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="F28" s="6" t="s">
         <v>150</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>151</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H28" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I28" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I28" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J28" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3128,38 +3117,38 @@
         <v>25</v>
       </c>
       <c r="B29" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="D29" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="E29" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="F29" s="6" t="s">
         <v>156</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>157</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H29" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I29" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="I29" s="7" t="s">
-        <v>78</v>
-      </c>
       <c r="J29" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="M29" s="5" t="s">
         <v>158</v>
-      </c>
-      <c r="M29" s="5" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3167,38 +3156,38 @@
         <v>26</v>
       </c>
       <c r="B30" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D30" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="C30" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="D30" s="6" t="s">
+      <c r="E30" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="F30" s="6" t="s">
         <v>161</v>
-      </c>
-      <c r="F30" s="6" t="s">
-        <v>162</v>
       </c>
       <c r="G30" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3206,36 +3195,36 @@
         <v>27</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D31" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="E31" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="F31" s="6" t="s">
         <v>166</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>167</v>
       </c>
       <c r="G31" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
       <c r="M31" s="5" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3243,36 +3232,36 @@
         <v>28</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D32" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="E32" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="F32" s="6" t="s">
         <v>169</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>170</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
       <c r="M32" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3280,36 +3269,36 @@
         <v>29</v>
       </c>
       <c r="B33" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D33" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="C33" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="D33" s="6" t="s">
+      <c r="E33" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="F33" s="6" t="s">
         <v>173</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>174</v>
       </c>
       <c r="G33" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I33" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K33" s="8"/>
       <c r="L33" s="8"/>
       <c r="M33" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3317,36 +3306,36 @@
         <v>30</v>
       </c>
       <c r="B34" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D34" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="C34" s="5" t="s">
-        <v>109</v>
-      </c>
-      <c r="D34" s="6" t="s">
+      <c r="E34" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="E34" s="6" t="s">
+      <c r="F34" s="6" t="s">
         <v>177</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>178</v>
       </c>
       <c r="G34" s="7" t="n">
         <v>8</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J34" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
       <c r="M34" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3354,36 +3343,36 @@
         <v>31</v>
       </c>
       <c r="B35" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="D35" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="C35" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="D35" s="6" t="s">
+      <c r="E35" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="F35" s="6" t="s">
         <v>181</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>182</v>
       </c>
       <c r="G35" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I35" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J35" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="K35" s="8"/>
       <c r="L35" s="8"/>
       <c r="M35" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3391,39 +3380,39 @@
         <v>32</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>36</v>
       </c>
       <c r="D36" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="E36" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="F36" s="6" t="s">
         <v>186</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>187</v>
       </c>
       <c r="G36" s="7"/>
       <c r="H36" s="5"/>
       <c r="I36" s="7" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J36" s="7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K36" s="8"/>
       <c r="L36" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="M36" s="5" t="s">
         <v>189</v>
-      </c>
-      <c r="M36" s="5" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F37" s="9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G37" s="9" t="n">
         <f aca="false">SUM(G5:G36)</f>
@@ -3432,56 +3421,56 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F38" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G38" s="9" t="n">
         <f aca="false">SUMIF(J5:J36,"Feito",G5:G36)</f>
-        <v>10</v>
+        <v>23</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F39" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:M36"/>
   <conditionalFormatting sqref="J5:J36">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>"Feito"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Em curso"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:H36">
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>"Must"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Should"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Could"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>"Won't"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5:I36">
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Sprint 1"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Sprint 2"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Sprint 3"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"Sprint 4"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
+    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
       <formula>"Backlog"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3535,17 +3524,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>10</v>
@@ -3556,25 +3545,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="H5" s="4" t="s">
         <v>202</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3582,10 +3571,10 @@
         <v>21</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>204</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>205</v>
       </c>
       <c r="D6" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A6,'Product Backlog'!$G$5:$G$36)</f>
@@ -3613,10 +3602,10 @@
         <v>40</v>
       </c>
       <c r="B7" s="14" t="s">
+        <v>205</v>
+      </c>
+      <c r="C7" s="14" t="s">
         <v>206</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>207</v>
       </c>
       <c r="D7" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A7,'Product Backlog'!$G$5:$G$36)</f>
@@ -3624,11 +3613,11 @@
       </c>
       <c r="E7" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A7,'Product Backlog'!$J$5:$J$36,"Feito")</f>
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="F7" s="15" t="n">
         <f aca="false">IF(D7=0,0,E7/D7)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" s="16" t="n">
         <f aca="false">$C$3-D7</f>
@@ -3641,13 +3630,13 @@
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D8" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$G$5:$G$36)</f>
@@ -3672,13 +3661,13 @@
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B9" s="14" t="s">
+        <v>208</v>
+      </c>
+      <c r="C9" s="14" t="s">
         <v>209</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>210</v>
       </c>
       <c r="D9" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A9,'Product Backlog'!$G$5:$G$36)</f>
@@ -3703,13 +3692,13 @@
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B10" s="14" t="s">
+        <v>210</v>
+      </c>
+      <c r="C10" s="14" t="s">
         <v>211</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>212</v>
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A10,'Product Backlog'!$G$5:$G$36)</f>
@@ -3733,7 +3722,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
@@ -3743,11 +3732,11 @@
       </c>
       <c r="E11" s="21" t="n">
         <f aca="false">SUM(E6:E10)</f>
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="F11" s="22" t="n">
         <f aca="false">IF(D11=0,0,E11/D11)</f>
-        <v>0.0793650793650794</v>
+        <v>0.182539682539683</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21" t="n">
@@ -3757,167 +3746,167 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="24" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="24" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="24" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="23" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="24" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="24" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="24" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="24" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="23" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="24" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="24" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="24" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="24" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="24" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="24" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="23" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="24" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="24" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="24" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="24" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -3950,24 +3939,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
+        <v>247</v>
+      </c>
+      <c r="B4" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="C4" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>249</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>250</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>251</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3975,7 +3964,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="C5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A5)</f>
@@ -3992,10 +3981,10 @@
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A6)</f>
@@ -4012,10 +4001,10 @@
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A7)</f>
@@ -4032,10 +4021,10 @@
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A8)</f>
@@ -4052,7 +4041,7 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>

</xml_diff>

<commit_message>
Sprint Planning do Sprint 3 (22/10): US05 e US17; opcionais no backlog
Sprints de uma semana até à entrega de 05/11. US17 sobe do backlog e passa
a Must; US06 e US07 saem do Sprint 4 para o backlog (Must → Should).
Sprint 4 com uma story nova a decidir com o docente. Excel, PROJETO.md,
guia do código e registo de uso de IA. Sem alterações de código.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014RHhrBcR4DQAiiEiK69qYD
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="255">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="264">
   <si>
     <t xml:space="preserve">Product Backlog — Recomendador de UCs Opcionais</t>
   </si>
@@ -287,7 +287,7 @@
     <t xml:space="preserve">Por fazer</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11. 14/10: trabalho antecipado no PR #14 — pesquisa de cursos reais na página de apresentação (app/catalogo/, dados da DGES lidos do CSV). Falta: filtros por área/instituição/localidade, ficha completa do curso e comparação de até 3 cursos. 14/10: Sprint 2 → Sprint 3, para o LLM entrar no Sprint 2 com a velocidade real (10 SP). 20/10: estado volta a «Por fazer» (não fica trabalho em curso num sprint que ainda não começou); a pesquisa de 14/10 e a página /cursos/ (US30) contam como parte já entregue.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11. 14/10: trabalho antecipado no PR #14 — pesquisa de cursos reais na página de apresentação (app/catalogo/, dados da DGES lidos do CSV). Falta: filtros por área/instituição/localidade, ficha completa do curso e comparação de até 3 cursos. 14/10: Sprint 2 → Sprint 3, para o LLM entrar no Sprint 2 com a velocidade real (10 SP). 20/10: estado volta a «Por fazer» (não fica trabalho em curso num sprint que ainda não começou); a pesquisa de 14/10 e a página /cursos/ (US30) contam como parte já entregue. 22/10 (Sprint Planning do Sprint 3): entra no Sprint 3 com a US17.</t>
   </si>
   <si>
     <t xml:space="preserve">US04</t>
@@ -311,10 +311,13 @@
 • O aluno pode remover um registo.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sprint 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4; inclui a importação das UCs; 3 → 5 SP. 14/10: mantém-se no Sprint 4.</t>
+    <t xml:space="preserve">Should</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backlog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4; inclui a importação das UCs; 3 → 5 SP. 14/10: mantém-se no Sprint 4. 22/10: Sprint 4 → Backlog, Must → Should. Decisão dos PO: até à entrega de 05/11 o centro são os cursos e as opcionais ficam em segundo plano.</t>
   </si>
   <si>
     <t xml:space="preserve">US07</t>
@@ -333,7 +336,7 @@
 • As avaliações ficam ligadas a um pseudo_id desde o início, e não ao email (ponto 2 dos requisitos); as regras de visualização e exportação ficam na US09.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4. 14/10: fica no Sprint 4 sem a US09 (velocidade de 10 SP); por isso guarda já com pseudo_id.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4. 14/10: fica no Sprint 4 sem a US09 (velocidade de 10 SP); por isso guarda já com pseudo_id. 22/10: Sprint 4 → Backlog, Must → Should. Decisão dos PO: até à entrega de 05/11 o centro são os cursos e as opcionais ficam em segundo plano.</t>
   </si>
   <si>
     <t xml:space="preserve">Importar catálogo de instituições e cursos</t>
@@ -348,13 +351,7 @@
 • Reimportar atualiza cursos existentes pelo par código de instituição + código de curso.</t>
   </si>
   <si>
-    <t xml:space="preserve">Should</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Backlog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa a importar instituições e cursos (nova visão). As UCs de cada curso entram com a US06. 14/10: Sprint 2 → Backlog, Must → Should: a aplicação já lê o catálogo do CSV (app/catalogo) e o LLM trabalha sobre ele; importar para a base de dados não muda nada para o utilizador nesta release.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa a importar instituições e cursos (nova visão). As UCs de cada curso entram com a US06. 14/10: Sprint 2 → Backlog, Must → Should: a aplicação já lê o catálogo do CSV (app/catalogo) e o LLM trabalha sobre ele; importar para a base de dados não muda nada para o utilizador nesta release. 22/10: candidata ao Sprint 4 se houver folga.</t>
   </si>
   <si>
     <t xml:space="preserve">US09</t>
@@ -545,7 +542,7 @@
 • A ação pede confirmação.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro).</t>
+    <t xml:space="preserve">Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). 22/10 (Sprint Planning do Sprint 3): Backlog → Sprint 3, Should → Must. O OptaBem já guarda conversas e decisões de pessoas, por isso exportar e apagar os dados passa a ser essencial (RGPD).</t>
   </si>
   <si>
     <t xml:space="preserve">US18</t>
@@ -577,6 +574,9 @@
 • Os alunos podem sinalizar comentários.</t>
   </si>
   <si>
+    <t xml:space="preserve">Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro).</t>
+  </si>
+  <si>
     <t xml:space="preserve">US25</t>
   </si>
   <si>
@@ -777,19 +777,25 @@
     <t xml:space="preserve">US29, US30, US31</t>
   </si>
   <si>
-    <t xml:space="preserve">Uma pessoa indecisa consulta e compara cursos de várias instituições (a completar no fim do Sprint 2).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quem já é aluno regista as UCs que concluiu e avalia as opcionais que fez, com as avaliações pseudonimizadas desde o início.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US06, US07</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fora do plano desta release; entra se houver folga.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US04, US09, US11, US08, US10, US12–US28 (US32 fundida na US29)</t>
+    <t xml:space="preserve">Uma pessoa indecisa filtra, consulta e compara cursos de várias instituições, e pode exportar ou apagar os seus dados (22/10 a 29/10).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US05, US17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">O percurso continua depois da escolha do curso: story nova a decidir com o docente (preparar o percurso ou perguntas e respostas por curso); US04 se houver folga (29/10 a 05/11; código fechado por volta de 03/11).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Story nova (a definir); US04 se houver folga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fora desta release (entrega a 05/11). As stories das opcionais ficam em segundo plano (decisão dos PO de 22/10).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US04, US06–US16, US18–US28 (US32 fundida na US29)</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -892,6 +898,27 @@
   </si>
   <si>
     <t xml:space="preserve">• Servidor Ollama da faculdade testado e posto de parte: lento e não obedece ao pedido de sugestão (PR #25 e #26; 05-spike-llm.md, secção 7). Fica o Gemini.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint Review do Sprint 2 e Sprint Planning do Sprint 3 (22/10/2026, decisão dos PO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sprint Review: US29, US30 e US31 aceites, 13 de 13 SP. O percurso completo foi testado com o Gemini real, também noutro computador.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Até à entrega de 05/11, o centro do produto são os cursos. As opcionais saíram do site (PR #33) e as suas stories passam para segundo plano: US06 e US07 saem do Sprint 4 (Must → Should).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sprints de uma semana: Sprint 3 de 22/10 a 29/10 e Sprint 4 de 29/10 a 05/11.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sprint 3: US05 (5 SP) e US17 (3 SP, sobe do Backlog e passa a Must), com 2 SP de folga.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sprint 4: uma story nova a decidir com o docente; a US04 entra se houver folga. O código fecha por volta de 03/11, para o relatório e a demonstração.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• A revisão de 22/10 (segurança do túnel, menu do aluno, textos) fica adiada por decisão do PO; o túnel é só para a equipa.</t>
   </si>
   <si>
     <t xml:space="preserve">Resumo por prioridade (MoSCoW)</t>
@@ -1274,7 +1301,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="20">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1334,14 +1361,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF8CBAD"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFEDE4F5"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1625,10 +1644,10 @@
                   <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5</c:v>
+                  <c:v>8</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>10</c:v>
+                  <c:v>0</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1730,11 +1749,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="85281332"/>
-        <c:axId val="13198070"/>
+        <c:axId val="30048100"/>
+        <c:axId val="22900469"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="85281332"/>
+        <c:axId val="30048100"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1765,7 +1784,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13198070"/>
+        <c:crossAx val="22900469"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1773,7 +1792,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="13198070"/>
+        <c:axId val="22900469"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1838,7 +1857,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85281332"/>
+        <c:crossAx val="30048100"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1905,9 +1924,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2090520</xdr:colOff>
+      <xdr:colOff>2090160</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>87480</xdr:rowOff>
+      <xdr:rowOff>87120</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1916,7 +1935,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5755680" cy="2515320"/>
+        <a:ext cx="5755320" cy="2514960"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2472,17 +2491,17 @@
         <v>5</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J12" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="M12" s="5" t="s">
         <v>52</v>
@@ -2493,35 +2512,35 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>62</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J13" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="M13" s="5" t="s">
         <v>61</v>
@@ -2538,29 +2557,29 @@
         <v>53</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J14" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="M14" s="5" t="s">
         <v>29</v>
@@ -2571,38 +2590,38 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="E15" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="6" t="s">
         <v>82</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>83</v>
       </c>
       <c r="G15" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J15" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2610,38 +2629,38 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="E16" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="G16" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J16" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2649,38 +2668,38 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>62</v>
       </c>
       <c r="D17" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="E17" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="F17" s="6" t="s">
         <v>93</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>94</v>
       </c>
       <c r="G17" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J17" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K17" s="8"/>
       <c r="L17" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2688,38 +2707,38 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="E18" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="F18" s="6" t="s">
         <v>99</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>100</v>
       </c>
       <c r="G18" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J18" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="M18" s="5" t="s">
         <v>101</v>
-      </c>
-      <c r="M18" s="5" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2727,38 +2746,38 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D19" s="6" t="s">
+      <c r="E19" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="F19" s="6" t="s">
         <v>105</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>106</v>
       </c>
       <c r="G19" s="7" t="n">
         <v>8</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J19" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2766,38 +2785,38 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="E20" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="F20" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>111</v>
       </c>
       <c r="G20" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J20" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2805,38 +2824,38 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="E21" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="F21" s="6" t="s">
         <v>116</v>
-      </c>
-      <c r="F21" s="6" t="s">
-        <v>117</v>
       </c>
       <c r="G21" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J21" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M21" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2844,38 +2863,38 @@
         <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D22" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E22" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="F22" s="6" t="s">
         <v>120</v>
-      </c>
-      <c r="F22" s="6" t="s">
-        <v>121</v>
       </c>
       <c r="G22" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J22" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="M22" s="5" t="s">
         <v>122</v>
-      </c>
-      <c r="M22" s="5" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2883,38 +2902,38 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="D23" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="E23" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="F23" s="6" t="s">
         <v>127</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>128</v>
       </c>
       <c r="G23" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J23" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="M23" s="5" t="s">
         <v>129</v>
-      </c>
-      <c r="M23" s="5" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2922,38 +2941,38 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D24" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="C24" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="D24" s="6" t="s">
+      <c r="E24" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="F24" s="6" t="s">
         <v>133</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>134</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>76</v>
+        <v>20</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>77</v>
+        <v>57</v>
       </c>
       <c r="J24" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2961,38 +2980,38 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>62</v>
       </c>
       <c r="D25" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="E25" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="F25" s="6" t="s">
         <v>138</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>139</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J25" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3000,35 +3019,35 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C26" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="D26" s="6" t="s">
+      <c r="E26" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="F26" s="6" t="s">
         <v>142</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>143</v>
       </c>
       <c r="G26" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J26" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="M26" s="5" t="s">
         <v>144</v>
@@ -3039,10 +3058,10 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>145</v>
@@ -3057,20 +3076,20 @@
         <v>2</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J27" s="7" t="s">
         <v>58</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3078,10 +3097,10 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>148</v>
@@ -3096,10 +3115,10 @@
         <v>5</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J28" s="7" t="s">
         <v>58</v>
@@ -3109,7 +3128,7 @@
         <v>151</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3135,10 +3154,10 @@
         <v>3</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J29" s="7" t="s">
         <v>58</v>
@@ -3159,7 +3178,7 @@
         <v>158</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>159</v>
@@ -3177,7 +3196,7 @@
         <v>162</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J30" s="7" t="s">
         <v>58</v>
@@ -3187,7 +3206,7 @@
         <v>163</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3195,10 +3214,10 @@
         <v>27</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>164</v>
@@ -3216,7 +3235,7 @@
         <v>162</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J31" s="7" t="s">
         <v>58</v>
@@ -3224,7 +3243,7 @@
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
       <c r="M31" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3235,7 +3254,7 @@
         <v>144</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D32" s="6" t="s">
         <v>167</v>
@@ -3253,7 +3272,7 @@
         <v>162</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J32" s="7" t="s">
         <v>58</v>
@@ -3290,7 +3309,7 @@
         <v>162</v>
       </c>
       <c r="I33" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J33" s="7" t="s">
         <v>58</v>
@@ -3309,7 +3328,7 @@
         <v>174</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D34" s="6" t="s">
         <v>175</v>
@@ -3327,7 +3346,7 @@
         <v>162</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J34" s="7" t="s">
         <v>58</v>
@@ -3335,7 +3354,7 @@
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
       <c r="M34" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3346,7 +3365,7 @@
         <v>178</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>179</v>
@@ -3364,7 +3383,7 @@
         <v>182</v>
       </c>
       <c r="I35" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J35" s="7" t="s">
         <v>58</v>
@@ -3397,7 +3416,7 @@
       <c r="G36" s="7"/>
       <c r="H36" s="5"/>
       <c r="I36" s="7" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="J36" s="7" t="s">
         <v>187</v>
@@ -3436,41 +3455,41 @@
   </sheetData>
   <autoFilter ref="A4:M36"/>
   <conditionalFormatting sqref="J5:J36">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>"Feito"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>"Em curso"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:H36">
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Must"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>"Should"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Could"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Won't"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5:I36">
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>"Sprint 1"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Sprint 2"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>"Sprint 3"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Sprint 4"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"Backlog"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3509,7 +3528,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H64"/>
+  <dimension ref="A1:H72"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -3636,11 +3655,11 @@
         <v>207</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>52</v>
+        <v>208</v>
       </c>
       <c r="D8" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$G$5:$G$36)</f>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$J$5:$J$36,"Feito")</f>
@@ -3652,26 +3671,26 @@
       </c>
       <c r="G8" s="16" t="n">
         <f aca="false">$C$3-D8</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A8)</f>
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>66</v>
+        <v>209</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D9" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A9,'Product Backlog'!$G$5:$G$36)</f>
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E9" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A9,'Product Backlog'!$J$5:$J$36,"Feito")</f>
@@ -3683,26 +3702,26 @@
       </c>
       <c r="G9" s="16" t="n">
         <f aca="false">$C$3-D9</f>
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A9)</f>
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>77</v>
+        <v>67</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A10,'Product Backlog'!$G$5:$G$36)</f>
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="E10" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A10,'Product Backlog'!$J$5:$J$36,"Feito")</f>
@@ -3717,12 +3736,12 @@
       </c>
       <c r="H10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A10)</f>
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
@@ -3746,167 +3765,202 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="24" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="24" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="24" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="23" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="24" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="24" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="24" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="24" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="23" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="24" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="24" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="24" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="24" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="24" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="24" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="23" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="24" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="24" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="24" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="24" t="s">
-        <v>245</v>
+        <v>247</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="23" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="24" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="24" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="24" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A70" s="24" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A71" s="24" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A72" s="24" t="s">
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -3939,24 +3993,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>202</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3964,39 +4018,39 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
       <c r="C5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A5)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D5" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$H$5:$H$36,A5,'Product Backlog'!$G$5:$G$36)</f>
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="E5" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D5/SUM($D$5:$D$8))</f>
-        <v>0.301587301587302</v>
+        <v>0.246031746031746</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A6)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D6" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$H$5:$H$36,A6,'Product Backlog'!$G$5:$G$36)</f>
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="E6" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D6/SUM($D$5:$D$8))</f>
-        <v>0.5</v>
+        <v>0.555555555555556</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4004,7 +4058,7 @@
         <v>162</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A7)</f>
@@ -4024,7 +4078,7 @@
         <v>182</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A8)</f>
@@ -4041,7 +4095,7 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>

</xml_diff>

<commit_message>
US05: consultar e comparar cursos
Filtros por área, instituição e localidade em /cursos/ (GET, sem
JavaScript), ficha completa de cada curso em /cursos/<curso> e comparação
de 2 ou 3 cursos lado a lado em /cursos/comparar. Tudo sem sessão; com
sessão aparece «Escolher este curso» (US31). O nome do curso passa a
levar à ficha em todas as fichas resumidas. O campo de pesquisa e as
listas de escolha ganham estilo. 20 testes novos (297 no total).
Documentação em docs/US05/ com diagramas gerados por script.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014RHhrBcR4DQAiiEiK69qYD
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="264">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="265">
   <si>
     <t xml:space="preserve">Product Backlog — Recomendador de UCs Opcionais</t>
   </si>
@@ -284,10 +284,10 @@
     <t xml:space="preserve">Sprint 3</t>
   </si>
   <si>
-    <t xml:space="preserve">Por fazer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11. 14/10: trabalho antecipado no PR #14 — pesquisa de cursos reais na página de apresentação (app/catalogo/, dados da DGES lidos do CSV). Falta: filtros por área/instituição/localidade, ficha completa do curso e comparação de até 3 cursos. 14/10: Sprint 2 → Sprint 3, para o LLM entrar no Sprint 2 com a velocidade real (10 SP). 20/10: estado volta a «Por fazer» (não fica trabalho em curso num sprint que ainda não começou); a pesquisa de 14/10 e a página /cursos/ (US30) contam como parte já entregue. 22/10 (Sprint Planning do Sprint 3): entra no Sprint 3 com a US17.</t>
+    <t xml:space="preserve">Em curso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11. 14/10: trabalho antecipado no PR #14 — pesquisa de cursos reais na página de apresentação (app/catalogo/, dados da DGES lidos do CSV). Falta: filtros por área/instituição/localidade, ficha completa do curso e comparação de até 3 cursos. 14/10: Sprint 2 → Sprint 3, para o LLM entrar no Sprint 2 com a velocidade real (10 SP). 20/10: estado volta a «Por fazer» (não fica trabalho em curso num sprint que ainda não começou); a pesquisa de 14/10 e a página /cursos/ (US30) contam como parte já entregue. 22/10 (Sprint Planning do Sprint 3): entra no Sprint 3 com a US17. 22/10: feita (PR da US05, à espera de revisão): filtros, ficha completa e comparação de até 3 cursos; docs/US05/, issue #12.</t>
   </si>
   <si>
     <t xml:space="preserve">US04</t>
@@ -315,6 +315,9 @@
   </si>
   <si>
     <t xml:space="preserve">Backlog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por fazer</t>
   </si>
   <si>
     <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4; inclui a importação das UCs; 3 → 5 SP. 14/10: mantém-se no Sprint 4. 22/10: Sprint 4 → Backlog, Must → Should. Decisão dos PO: até à entrega de 05/11 o centro são os cursos e as opcionais ficam em segundo plano.</t>
@@ -1301,7 +1304,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="21">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1385,6 +1388,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1749,11 +1760,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="30048100"/>
-        <c:axId val="22900469"/>
+        <c:axId val="45675012"/>
+        <c:axId val="86147293"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="30048100"/>
+        <c:axId val="45675012"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1784,7 +1795,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22900469"/>
+        <c:crossAx val="86147293"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1792,7 +1803,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="22900469"/>
+        <c:axId val="86147293"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1857,7 +1868,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30048100"/>
+        <c:crossAx val="45675012"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1924,9 +1935,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2090160</xdr:colOff>
+      <xdr:colOff>2089800</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>87120</xdr:rowOff>
+      <xdr:rowOff>86760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1935,7 +1946,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5755320" cy="2514960"/>
+        <a:ext cx="5754960" cy="2514600"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2497,11 +2508,11 @@
         <v>67</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="M12" s="5" t="s">
         <v>52</v>
@@ -2512,19 +2523,19 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>62</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>5</v>
@@ -2536,11 +2547,11 @@
         <v>67</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="M13" s="5" t="s">
         <v>61</v>
@@ -2557,13 +2568,13 @@
         <v>53</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>5</v>
@@ -2575,11 +2586,11 @@
         <v>67</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="M14" s="5" t="s">
         <v>29</v>
@@ -2590,19 +2601,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G15" s="7" t="n">
         <v>5</v>
@@ -2614,14 +2625,14 @@
         <v>67</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2629,19 +2640,19 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="G16" s="7" t="n">
         <v>3</v>
@@ -2653,14 +2664,14 @@
         <v>67</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2668,19 +2679,19 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>62</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G17" s="7" t="n">
         <v>3</v>
@@ -2692,14 +2703,14 @@
         <v>67</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K17" s="8"/>
       <c r="L17" s="8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2707,19 +2718,19 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G18" s="7" t="n">
         <v>5</v>
@@ -2731,14 +2742,14 @@
         <v>67</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2746,19 +2757,19 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G19" s="7" t="n">
         <v>8</v>
@@ -2770,14 +2781,14 @@
         <v>67</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2785,19 +2796,19 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G20" s="7" t="n">
         <v>2</v>
@@ -2809,14 +2820,14 @@
         <v>67</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2824,19 +2835,19 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G21" s="7" t="n">
         <v>5</v>
@@ -2848,14 +2859,14 @@
         <v>67</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="M21" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2863,19 +2874,19 @@
         <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="G22" s="7" t="n">
         <v>5</v>
@@ -2887,14 +2898,14 @@
         <v>67</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2902,19 +2913,19 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G23" s="7" t="n">
         <v>3</v>
@@ -2926,14 +2937,14 @@
         <v>67</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="M23" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2941,19 +2952,19 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>3</v>
@@ -2965,14 +2976,14 @@
         <v>57</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2980,19 +2991,19 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>62</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>3</v>
@@ -3004,14 +3015,14 @@
         <v>67</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3019,19 +3030,19 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G26" s="7" t="n">
         <v>3</v>
@@ -3043,14 +3054,14 @@
         <v>67</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3058,19 +3069,19 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G27" s="7" t="n">
         <v>2</v>
@@ -3082,14 +3093,14 @@
         <v>67</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3097,19 +3108,19 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>5</v>
@@ -3121,14 +3132,14 @@
         <v>67</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3136,19 +3147,19 @@
         <v>25</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>3</v>
@@ -3160,14 +3171,14 @@
         <v>67</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="M29" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3175,38 +3186,38 @@
         <v>26</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="G30" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I30" s="7" t="s">
         <v>67</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3214,36 +3225,36 @@
         <v>27</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G31" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I31" s="7" t="s">
         <v>67</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
       <c r="M31" s="5" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3251,36 +3262,36 @@
         <v>28</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I32" s="7" t="s">
         <v>67</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
       <c r="M32" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3288,36 +3299,36 @@
         <v>29</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="G33" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I33" s="7" t="s">
         <v>67</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K33" s="8"/>
       <c r="L33" s="8"/>
       <c r="M33" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3325,36 +3336,36 @@
         <v>30</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="G34" s="7" t="n">
         <v>8</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="I34" s="7" t="s">
         <v>67</v>
       </c>
       <c r="J34" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
       <c r="M34" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3362,36 +3373,36 @@
         <v>31</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G35" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="I35" s="7" t="s">
         <v>67</v>
       </c>
       <c r="J35" s="7" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="K35" s="8"/>
       <c r="L35" s="8"/>
       <c r="M35" s="5" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3399,19 +3410,19 @@
         <v>32</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>36</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="G36" s="7"/>
       <c r="H36" s="5"/>
@@ -3419,19 +3430,19 @@
         <v>67</v>
       </c>
       <c r="J36" s="7" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="K36" s="8"/>
       <c r="L36" s="8" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="M36" s="5" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F37" s="9" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G37" s="9" t="n">
         <f aca="false">SUM(G5:G36)</f>
@@ -3440,7 +3451,7 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F38" s="9" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="G38" s="9" t="n">
         <f aca="false">SUMIF(J5:J36,"Feito",G5:G36)</f>
@@ -3449,47 +3460,47 @@
     </row>
     <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F39" s="10" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:M36"/>
   <conditionalFormatting sqref="J5:J36">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>"Feito"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Em curso"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:H36">
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>"Must"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Should"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Could"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>"Won't"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5:I36">
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Sprint 1"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Sprint 2"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Sprint 3"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"Sprint 4"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
       <formula>"Backlog"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3543,17 +3554,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>10</v>
@@ -3564,25 +3575,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3590,10 +3601,10 @@
         <v>21</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D6" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A6,'Product Backlog'!$G$5:$G$36)</f>
@@ -3621,10 +3632,10 @@
         <v>40</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D7" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A7,'Product Backlog'!$G$5:$G$36)</f>
@@ -3652,10 +3663,10 @@
         <v>57</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D8" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$G$5:$G$36)</f>
@@ -3680,13 +3691,13 @@
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D9" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A9,'Product Backlog'!$G$5:$G$36)</f>
@@ -3714,10 +3725,10 @@
         <v>67</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A10,'Product Backlog'!$G$5:$G$36)</f>
@@ -3741,7 +3752,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
@@ -3765,202 +3776,202 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="24" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="24" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="24" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="23" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="24" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="24" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="24" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="24" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="23" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="24" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="24" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="24" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="24" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="24" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="24" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="23" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="24" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="24" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="24" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="24" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="23" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="24" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="24" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="24" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="24" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="24" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="24" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
   </sheetData>
@@ -3993,24 +4004,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4018,7 +4029,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A5)</f>
@@ -4038,7 +4049,7 @@
         <v>66</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A6)</f>
@@ -4055,10 +4066,10 @@
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A7)</f>
@@ -4075,10 +4086,10 @@
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A8)</f>
@@ -4095,7 +4106,7 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>

</xml_diff>

<commit_message>
US17: apagar a minha conta (âmbito reduzido a 22/10); guia do túnel
Ligação «Apagar a minha conta e todos os meus dados» no fim do início;
página que diz o que se perde e pede a palavra-passe; apaga a conta, a
conversa, as decisões e os pedidos ao LLM (ON DELETE CASCADE), termina a
sessão e avisa na apresentação. A exportação fica no backlog (decisão do
PO). Política de privacidade provisória corrigida. 12 testes (330 no
total). docs/US17/, requisitos 1.7 (RF17, ponto 11), Excel e issue #34.

Guia do túnel 1.2: o exemplo do .env deixa de ter comentários na mesma
linha, que o arrancar.ps1 lia como parte do valor.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014RHhrBcR4DQAiiEiK69qYD
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -534,18 +534,18 @@
     <t xml:space="preserve">US17</t>
   </si>
   <si>
-    <t xml:space="preserve">Exportar e apagar dados</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como aluno, quero exportar ou apagar todos os meus dados, para exercer os meus direitos de privacidade.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Exportação em JSON/CSV.
-• Apagar remove conta, percurso e avaliações.
-• A ação pede confirmação.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). 22/10 (Sprint Planning do Sprint 3): Backlog → Sprint 3, Should → Must. O OptaBem já guarda conversas e decisões de pessoas, por isso exportar e apagar os dados passa a ser essencial (RGPD).</t>
+    <t xml:space="preserve">Apagar a minha conta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como aluno, quero apagar a minha conta e todos os meus dados, para exercer o meu direito ao apagamento.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Apagar remove a conta, a conversa de orientação, as decisões do percurso e os pedidos ao LLM.
+• A ação pede confirmação (palavra-passe).
+• A sessão termina e a página confirma que os dados foram apagados.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). 22/10 (Sprint Planning do Sprint 3): Backlog → Sprint 3, Should → Must. O OptaBem já guarda conversas e decisões de pessoas, por isso exportar e apagar os dados passa a ser essencial (RGPD). 22/10 (decisão do PO): âmbito reduzido ao apagamento da conta; a exportação fica no backlog (RF17). 3 → 2 SP. Feita (PR da US17, à espera de revisão); docs/US17/, issue #34.</t>
   </si>
   <si>
     <t xml:space="preserve">US18</t>
@@ -780,7 +780,7 @@
     <t xml:space="preserve">US29, US30, US31</t>
   </si>
   <si>
-    <t xml:space="preserve">Uma pessoa indecisa filtra, consulta e compara cursos de várias instituições, e pode exportar ou apagar os seus dados (22/10 a 29/10).</t>
+    <t xml:space="preserve">Uma pessoa indecisa filtra, consulta e compara cursos de várias instituições, e pode apagar a sua conta e todos os seus dados (22/10 a 29/10).</t>
   </si>
   <si>
     <t xml:space="preserve">US05, US17</t>
@@ -1655,7 +1655,7 @@
                   <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>8</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1760,11 +1760,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="45675012"/>
-        <c:axId val="86147293"/>
+        <c:axId val="60132693"/>
+        <c:axId val="86059893"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="45675012"/>
+        <c:axId val="60132693"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1795,7 +1795,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86147293"/>
+        <c:crossAx val="86059893"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1803,7 +1803,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="86147293"/>
+        <c:axId val="86059893"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1868,7 +1868,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="45675012"/>
+        <c:crossAx val="60132693"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1935,9 +1935,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2089800</xdr:colOff>
+      <xdr:colOff>2089440</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>86760</xdr:rowOff>
+      <xdr:rowOff>86400</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1946,7 +1946,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5754960" cy="2514600"/>
+        <a:ext cx="5754600" cy="2514240"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2967,7 +2967,7 @@
         <v>134</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H24" s="5" t="s">
         <v>20</v>
@@ -2976,7 +2976,7 @@
         <v>57</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
@@ -3446,7 +3446,7 @@
       </c>
       <c r="G37" s="9" t="n">
         <f aca="false">SUM(G5:G36)</f>
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3670,7 +3670,7 @@
       </c>
       <c r="D8" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$G$5:$G$36)</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$J$5:$J$36,"Feito")</f>
@@ -3682,7 +3682,7 @@
       </c>
       <c r="G8" s="16" t="n">
         <f aca="false">$C$3-D8</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A8)</f>
@@ -3758,7 +3758,7 @@
       <c r="C11" s="20"/>
       <c r="D11" s="21" t="n">
         <f aca="false">SUM(D6:D10)</f>
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E11" s="21" t="n">
         <f aca="false">SUM(E6:E10)</f>
@@ -3766,7 +3766,7 @@
       </c>
       <c r="F11" s="22" t="n">
         <f aca="false">IF(D11=0,0,E11/D11)</f>
-        <v>0.182539682539683</v>
+        <v>0.184</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21" t="n">
@@ -4037,11 +4037,11 @@
       </c>
       <c r="D5" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$H$5:$H$36,A5,'Product Backlog'!$G$5:$G$36)</f>
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E5" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D5/SUM($D$5:$D$8))</f>
-        <v>0.246031746031746</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="E6" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D6/SUM($D$5:$D$8))</f>
-        <v>0.555555555555556</v>
+        <v>0.56</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4081,7 +4081,7 @@
       </c>
       <c r="E7" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D7/SUM($D$5:$D$8))</f>
-        <v>0.174603174603175</v>
+        <v>0.176</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="E8" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D8/SUM($D$5:$D$8))</f>
-        <v>0.0238095238095238</v>
+        <v>0.024</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="D9" s="27" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fecho do Sprint 3: US05 e US17 aceites na Sprint Review
Estado «Feito» da US05 e da US17 no Excel (Sprint 3: 7 de 7 SP) e
notas da Sprint Review; PROJETO.md, docs/US05 e docs/US17, guia do
código e registo de uso de IA. O teste test_apaga_a_conta_e_todos_os_dados
dependia da data em que corria (falhava a 23/10) e passa a usar um dia
passado fixo. Sem alterações ao código da aplicação.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Pxqp9zSSYM9cG9Z8Qdyym4
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="269">
   <si>
     <t xml:space="preserve">Product Backlog — Recomendador de UCs Opcionais</t>
   </si>
@@ -284,10 +284,7 @@
     <t xml:space="preserve">Sprint 3</t>
   </si>
   <si>
-    <t xml:space="preserve">Em curso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11. 14/10: trabalho antecipado no PR #14 — pesquisa de cursos reais na página de apresentação (app/catalogo/, dados da DGES lidos do CSV). Falta: filtros por área/instituição/localidade, ficha completa do curso e comparação de até 3 cursos. 14/10: Sprint 2 → Sprint 3, para o LLM entrar no Sprint 2 com a velocidade real (10 SP). 20/10: estado volta a «Por fazer» (não fica trabalho em curso num sprint que ainda não começou); a pesquisa de 14/10 e a página /cursos/ (US30) contam como parte já entregue. 22/10 (Sprint Planning do Sprint 3): entra no Sprint 3 com a US17. 22/10: feita (PR da US05, à espera de revisão): filtros, ficha completa e comparação de até 3 cursos; docs/US05/, issue #12.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11. 14/10: trabalho antecipado no PR #14 — pesquisa de cursos reais na página de apresentação (app/catalogo/, dados da DGES lidos do CSV). Falta: filtros por área/instituição/localidade, ficha completa do curso e comparação de até 3 cursos. 14/10: Sprint 2 → Sprint 3, para o LLM entrar no Sprint 2 com a velocidade real (10 SP). 20/10: estado volta a «Por fazer» (não fica trabalho em curso num sprint que ainda não começou); a pesquisa de 14/10 e a página /cursos/ (US30) contam como parte já entregue. 22/10 (Sprint Planning do Sprint 3): entra no Sprint 3 com a US17. 22/10: feita (PR da US05, à espera de revisão): filtros, ficha completa e comparação de até 3 cursos; docs/US05/, issue #12. 23/10: aceite na Sprint Review do Sprint 3 (testada pelos PO); fica Feito.</t>
   </si>
   <si>
     <t xml:space="preserve">US04</t>
@@ -545,7 +542,7 @@
 • A sessão termina e a página confirma que os dados foram apagados.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). 22/10 (Sprint Planning do Sprint 3): Backlog → Sprint 3, Should → Must. O OptaBem já guarda conversas e decisões de pessoas, por isso exportar e apagar os dados passa a ser essencial (RGPD). 22/10 (decisão do PO): âmbito reduzido ao apagamento da conta; a exportação fica no backlog (RF17). 3 → 2 SP. Feita (PR da US17, à espera de revisão); docs/US17/, issue #34.</t>
+    <t xml:space="preserve">Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). 22/10 (Sprint Planning do Sprint 3): Backlog → Sprint 3, Should → Must. O OptaBem já guarda conversas e decisões de pessoas, por isso exportar e apagar os dados passa a ser essencial (RGPD). 22/10 (decisão do PO): âmbito reduzido ao apagamento da conta; a exportação fica no backlog (RF17). 3 → 2 SP. Feita (PR da US17, à espera de revisão); docs/US17/, issue #34. 23/10: aceite na Sprint Review do Sprint 3 (testada pelos PO); fica Feito.</t>
   </si>
   <si>
     <t xml:space="preserve">US18</t>
@@ -780,7 +777,7 @@
     <t xml:space="preserve">US29, US30, US31</t>
   </si>
   <si>
-    <t xml:space="preserve">Uma pessoa indecisa filtra, consulta e compara cursos de várias instituições, e pode apagar a sua conta e todos os seus dados (22/10 a 29/10).</t>
+    <t xml:space="preserve">Uma pessoa indecisa filtra, consulta e compara cursos de várias instituições, e pode apagar a sua conta e todos os seus dados (22/10 a 29/10; concluído a 23/10).</t>
   </si>
   <si>
     <t xml:space="preserve">US05, US17</t>
@@ -922,6 +919,21 @@
   </si>
   <si>
     <t xml:space="preserve">• A revisão de 22/10 (segurança do túnel, menu do aluno, textos) fica adiada por decisão do PO; o túnel é só para a equipa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint Review do Sprint 3 (23/10/2026, decisão dos PO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US05 e US17 aceites, 7 de 7 SP. As duas stories foram testadas pelos PO (filtros, ficha, comparação e apagar a conta).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• O sprint fecha antes de 29/10 porque o objetivo foi cumprido. Entrou também, sem story, o menu fixo no topo (PR #40).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• No fecho, um teste da US17 que dependia da data em que corria foi corrigido (sem mudanças no código da aplicação).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sprint 4 por planear: a story nova fica a decidir com o docente.</t>
   </si>
   <si>
     <t xml:space="preserve">Resumo por prioridade (MoSCoW)</t>
@@ -1187,111 +1199,111 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1304,7 +1316,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="20">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1388,14 +1400,6 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1749,7 +1753,7 @@
                   <c:v>13</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0</c:v>
+                  <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0</c:v>
@@ -1760,11 +1764,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="60132693"/>
-        <c:axId val="86059893"/>
+        <c:axId val="71063653"/>
+        <c:axId val="6152493"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="60132693"/>
+        <c:axId val="71063653"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1795,7 +1799,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="86059893"/>
+        <c:crossAx val="6152493"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1803,7 +1807,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="86059893"/>
+        <c:axId val="6152493"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1868,7 +1872,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60132693"/>
+        <c:crossAx val="71063653"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1935,9 +1939,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2089440</xdr:colOff>
+      <xdr:colOff>2089080</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>86400</xdr:rowOff>
+      <xdr:rowOff>86040</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1946,7 +1950,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5754600" cy="2514240"/>
+        <a:ext cx="5754240" cy="2513880"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2469,14 +2473,14 @@
         <v>57</v>
       </c>
       <c r="J11" s="7" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
       <c r="K11" s="8"/>
       <c r="L11" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="M11" s="5" t="s">
         <v>59</v>
-      </c>
-      <c r="M11" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2484,35 +2488,35 @@
         <v>8</v>
       </c>
       <c r="B12" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="D12" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="E12" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="F12" s="6" t="s">
         <v>64</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>65</v>
       </c>
       <c r="G12" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H12" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I12" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I12" s="7" t="s">
+      <c r="J12" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J12" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="M12" s="5" t="s">
         <v>52</v>
@@ -2523,38 +2527,38 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D13" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="D13" s="6" t="s">
+      <c r="E13" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="F13" s="6" t="s">
         <v>72</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>73</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H13" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I13" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I13" s="7" t="s">
+      <c r="J13" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J13" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2562,35 +2566,35 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>53</v>
       </c>
       <c r="D14" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E14" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>77</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H14" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I14" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I14" s="7" t="s">
+      <c r="J14" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J14" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="M14" s="5" t="s">
         <v>29</v>
@@ -2601,38 +2605,38 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="D15" s="6" t="s">
+      <c r="E15" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="6" t="s">
         <v>82</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>83</v>
       </c>
       <c r="G15" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H15" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I15" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I15" s="7" t="s">
+      <c r="J15" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J15" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2640,38 +2644,38 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="E16" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>89</v>
       </c>
       <c r="G16" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H16" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I16" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I16" s="7" t="s">
+      <c r="J16" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J16" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2679,38 +2683,38 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C17" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="D17" s="6" t="s">
+      <c r="E17" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="F17" s="6" t="s">
         <v>93</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>94</v>
       </c>
       <c r="G17" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H17" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I17" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I17" s="7" t="s">
+      <c r="J17" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J17" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K17" s="8"/>
       <c r="L17" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2718,38 +2722,38 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="D18" s="6" t="s">
+      <c r="E18" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="F18" s="6" t="s">
         <v>99</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>100</v>
       </c>
       <c r="G18" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H18" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I18" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I18" s="7" t="s">
+      <c r="J18" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J18" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="M18" s="5" t="s">
         <v>101</v>
-      </c>
-      <c r="M18" s="5" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2757,38 +2761,38 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="D19" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C19" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="D19" s="6" t="s">
+      <c r="E19" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="F19" s="6" t="s">
         <v>105</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>106</v>
       </c>
       <c r="G19" s="7" t="n">
         <v>8</v>
       </c>
       <c r="H19" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I19" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I19" s="7" t="s">
+      <c r="J19" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J19" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2796,38 +2800,38 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="D20" s="6" t="s">
+      <c r="E20" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="E20" s="6" t="s">
+      <c r="F20" s="6" t="s">
         <v>110</v>
-      </c>
-      <c r="F20" s="6" t="s">
-        <v>111</v>
       </c>
       <c r="G20" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H20" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I20" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I20" s="7" t="s">
+      <c r="J20" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J20" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2835,38 +2839,38 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="D21" s="6" t="s">
+      <c r="E21" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="E21" s="6" t="s">
+      <c r="F21" s="6" t="s">
         <v>116</v>
-      </c>
-      <c r="F21" s="6" t="s">
-        <v>117</v>
       </c>
       <c r="G21" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H21" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I21" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I21" s="7" t="s">
+      <c r="J21" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J21" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="M21" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2874,38 +2878,38 @@
         <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D22" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="E22" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="E22" s="6" t="s">
+      <c r="F22" s="6" t="s">
         <v>120</v>
-      </c>
-      <c r="F22" s="6" t="s">
-        <v>121</v>
       </c>
       <c r="G22" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H22" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I22" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I22" s="7" t="s">
+      <c r="J22" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J22" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
+        <v>121</v>
+      </c>
+      <c r="M22" s="5" t="s">
         <v>122</v>
-      </c>
-      <c r="M22" s="5" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2913,38 +2917,38 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>124</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="D23" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="E23" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="F23" s="6" t="s">
         <v>127</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>128</v>
       </c>
       <c r="G23" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H23" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I23" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I23" s="7" t="s">
+      <c r="J23" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J23" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8" t="s">
+        <v>128</v>
+      </c>
+      <c r="M23" s="5" t="s">
         <v>129</v>
-      </c>
-      <c r="M23" s="5" t="s">
-        <v>130</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2952,19 +2956,19 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D24" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="C24" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="D24" s="6" t="s">
+      <c r="E24" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="E24" s="6" t="s">
+      <c r="F24" s="6" t="s">
         <v>133</v>
-      </c>
-      <c r="F24" s="6" t="s">
-        <v>134</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>2</v>
@@ -2976,14 +2980,14 @@
         <v>57</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2991,38 +2995,38 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
+        <v>135</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="C25" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="D25" s="6" t="s">
+      <c r="E25" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="E25" s="6" t="s">
+      <c r="F25" s="6" t="s">
         <v>138</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>139</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H25" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I25" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I25" s="7" t="s">
+      <c r="J25" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J25" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3030,38 +3034,38 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D26" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C26" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="D26" s="6" t="s">
+      <c r="E26" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="F26" s="6" t="s">
         <v>142</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>143</v>
       </c>
       <c r="G26" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H26" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I26" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I26" s="7" t="s">
+      <c r="J26" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J26" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="M26" s="5" t="s">
         <v>144</v>
-      </c>
-      <c r="M26" s="5" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3069,38 +3073,38 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D27" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="E27" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="E27" s="6" t="s">
+      <c r="F27" s="6" t="s">
         <v>147</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>148</v>
       </c>
       <c r="G27" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H27" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I27" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I27" s="7" t="s">
+      <c r="J27" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J27" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3108,38 +3112,38 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D28" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="E28" s="6" t="s">
         <v>149</v>
       </c>
-      <c r="E28" s="6" t="s">
+      <c r="F28" s="6" t="s">
         <v>150</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>151</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H28" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I28" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I28" s="7" t="s">
+      <c r="J28" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J28" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3147,38 +3151,38 @@
         <v>25</v>
       </c>
       <c r="B29" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="D29" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="E29" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="F29" s="6" t="s">
         <v>156</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>157</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H29" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I29" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="I29" s="7" t="s">
+      <c r="J29" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J29" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8" t="s">
+        <v>157</v>
+      </c>
+      <c r="M29" s="5" t="s">
         <v>158</v>
-      </c>
-      <c r="M29" s="5" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3186,38 +3190,38 @@
         <v>26</v>
       </c>
       <c r="B30" s="5" t="s">
+        <v>158</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="D30" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="C30" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D30" s="6" t="s">
+      <c r="E30" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="F30" s="6" t="s">
         <v>161</v>
-      </c>
-      <c r="F30" s="6" t="s">
-        <v>162</v>
       </c>
       <c r="G30" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I30" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="J30" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J30" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3225,36 +3229,36 @@
         <v>27</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D31" s="6" t="s">
+        <v>164</v>
+      </c>
+      <c r="E31" s="6" t="s">
         <v>165</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="F31" s="6" t="s">
         <v>166</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>167</v>
       </c>
       <c r="G31" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I31" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="J31" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J31" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K31" s="8"/>
       <c r="L31" s="8"/>
       <c r="M31" s="5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3262,36 +3266,36 @@
         <v>28</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D32" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="E32" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="F32" s="6" t="s">
         <v>169</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>170</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I32" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="J32" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J32" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K32" s="8"/>
       <c r="L32" s="8"/>
       <c r="M32" s="5" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3299,36 +3303,36 @@
         <v>29</v>
       </c>
       <c r="B33" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="D33" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="C33" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="D33" s="6" t="s">
+      <c r="E33" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="F33" s="6" t="s">
         <v>173</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>174</v>
       </c>
       <c r="G33" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I33" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="J33" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J33" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K33" s="8"/>
       <c r="L33" s="8"/>
       <c r="M33" s="5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3336,36 +3340,36 @@
         <v>30</v>
       </c>
       <c r="B34" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="D34" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="C34" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D34" s="6" t="s">
+      <c r="E34" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="E34" s="6" t="s">
+      <c r="F34" s="6" t="s">
         <v>177</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>178</v>
       </c>
       <c r="G34" s="7" t="n">
         <v>8</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I34" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="J34" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J34" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K34" s="8"/>
       <c r="L34" s="8"/>
       <c r="M34" s="5" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3373,36 +3377,36 @@
         <v>31</v>
       </c>
       <c r="B35" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>124</v>
+      </c>
+      <c r="D35" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="C35" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="D35" s="6" t="s">
+      <c r="E35" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="E35" s="6" t="s">
+      <c r="F35" s="6" t="s">
         <v>181</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>182</v>
       </c>
       <c r="G35" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="I35" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="J35" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="J35" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="K35" s="8"/>
       <c r="L35" s="8"/>
       <c r="M35" s="5" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3410,39 +3414,39 @@
         <v>32</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>36</v>
       </c>
       <c r="D36" s="6" t="s">
+        <v>184</v>
+      </c>
+      <c r="E36" s="6" t="s">
         <v>185</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="F36" s="6" t="s">
         <v>186</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>187</v>
       </c>
       <c r="G36" s="7"/>
       <c r="H36" s="5"/>
       <c r="I36" s="7" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="J36" s="7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K36" s="8"/>
       <c r="L36" s="8" t="s">
+        <v>188</v>
+      </c>
+      <c r="M36" s="5" t="s">
         <v>189</v>
-      </c>
-      <c r="M36" s="5" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F37" s="9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G37" s="9" t="n">
         <f aca="false">SUM(G5:G36)</f>
@@ -3451,56 +3455,56 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F38" s="9" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G38" s="9" t="n">
         <f aca="false">SUMIF(J5:J36,"Feito",G5:G36)</f>
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F39" s="10" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:M36"/>
   <conditionalFormatting sqref="J5:J36">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>"Feito"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>"Em curso"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H5:H36">
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Must"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>"Should"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Could"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Won't"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5:I36">
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>"Sprint 1"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Sprint 2"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>"Sprint 3"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Sprint 4"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"Backlog"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3539,7 +3543,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -3554,17 +3558,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>10</v>
@@ -3575,25 +3579,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
+        <v>196</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>197</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="4" t="s">
         <v>198</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="E5" s="4" t="s">
         <v>199</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="F5" s="4" t="s">
         <v>200</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>201</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="H5" s="4" t="s">
         <v>202</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3601,10 +3605,10 @@
         <v>21</v>
       </c>
       <c r="B6" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="C6" s="14" t="s">
         <v>204</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>205</v>
       </c>
       <c r="D6" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A6,'Product Backlog'!$G$5:$G$36)</f>
@@ -3632,10 +3636,10 @@
         <v>40</v>
       </c>
       <c r="B7" s="14" t="s">
+        <v>205</v>
+      </c>
+      <c r="C7" s="14" t="s">
         <v>206</v>
-      </c>
-      <c r="C7" s="14" t="s">
-        <v>207</v>
       </c>
       <c r="D7" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A7,'Product Backlog'!$G$5:$G$36)</f>
@@ -3663,10 +3667,10 @@
         <v>57</v>
       </c>
       <c r="B8" s="14" t="s">
+        <v>207</v>
+      </c>
+      <c r="C8" s="14" t="s">
         <v>208</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>209</v>
       </c>
       <c r="D8" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$G$5:$G$36)</f>
@@ -3674,11 +3678,11 @@
       </c>
       <c r="E8" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$J$5:$J$36,"Feito")</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F8" s="15" t="n">
         <f aca="false">IF(D8=0,0,E8/D8)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G8" s="16" t="n">
         <f aca="false">$C$3-D8</f>
@@ -3691,13 +3695,13 @@
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
+        <v>209</v>
+      </c>
+      <c r="B9" s="14" t="s">
         <v>210</v>
       </c>
-      <c r="B9" s="14" t="s">
+      <c r="C9" s="14" t="s">
         <v>211</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>212</v>
       </c>
       <c r="D9" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A9,'Product Backlog'!$G$5:$G$36)</f>
@@ -3722,13 +3726,13 @@
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B10" s="14" t="s">
+        <v>212</v>
+      </c>
+      <c r="C10" s="14" t="s">
         <v>213</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>214</v>
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A10,'Product Backlog'!$G$5:$G$36)</f>
@@ -3752,7 +3756,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
@@ -3762,11 +3766,11 @@
       </c>
       <c r="E11" s="21" t="n">
         <f aca="false">SUM(E6:E10)</f>
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="F11" s="22" t="n">
         <f aca="false">IF(D11=0,0,E11/D11)</f>
-        <v>0.184</v>
+        <v>0.24</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21" t="n">
@@ -3776,202 +3780,227 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="24" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="24" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="24" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="23" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="24" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="24" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="24" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="24" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="23" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="24" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="24" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="24" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="24" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="24" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="24" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="23" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="24" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="24" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="24" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="24" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="23" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="24" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="24" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="24" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="24" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="24" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="24" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A74" s="23" t="s">
         <v>255</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A75" s="24" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A76" s="24" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A77" s="24" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A78" s="24" t="s">
+        <v>259</v>
       </c>
     </row>
   </sheetData>
@@ -4004,24 +4033,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>258</v>
+        <v>262</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>259</v>
+        <v>263</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>260</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4029,7 +4058,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>261</v>
+        <v>265</v>
       </c>
       <c r="C5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A5)</f>
@@ -4046,10 +4075,10 @@
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>262</v>
+        <v>266</v>
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A6)</f>
@@ -4066,10 +4095,10 @@
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A7)</f>
@@ -4086,10 +4115,10 @@
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>264</v>
+        <v>268</v>
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A8)</f>
@@ -4106,7 +4135,7 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>

</xml_diff>

<commit_message>
Replaneamento de 23/10: plano de candidatura no backlog, nos requisitos e na documentação
- Backlog: US04 reescrita (catálogo da DGES, Sprint 4, Must); US33 a US39 novas (épico E12);
  as 22 stories das opcionais passam a Won't (fase 2) e ficam no fim; US02 sem «avaliações»;
  objetivo do Sprint 4 e notas do replaneamento (18 SP planeados, acima da velocidade).
- Requisitos 1.8: módulo K (RF40 a RF43) e rastreabilidade; visão do produto.
- dados/README.md (colunas das condições de acesso), guia do código, PROJETO.md, registo de uso de IA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jr1j7KW7k7X8nu4tsEr7G3
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Product Backlog'!$4:$4</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$36</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$43</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -82,12 +82,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="420" uniqueCount="269">
-  <si>
-    <t xml:space="preserve">Product Backlog — Recomendador de UCs Opcionais</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ordenado pela ordem de trabalho (sprint e prioridade). Células a amarelo são para a equipa atualizar (Sprint, Estado, Responsável, SP, Notas). Replaneado a 14/10/2026 com a velocidade real (10 SP por sprint) e a decisão de o LLM conduzir a orientação (ver folha «Plano de sprints»). A partir de 13/10 os IDs não mudam.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="317">
+  <si>
+    <t xml:space="preserve">Product Backlog — OptaBem (orientação de curso e candidatura)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordenado pela ordem de trabalho (sprint e prioridade). Células a amarelo são para a equipa atualizar (Sprint, Estado, Responsável, SP, Notas). Replaneado a 14/10/2026 com a velocidade real (10 SP por sprint) e a decisão de o LLM conduzir a orientação (ver folha «Plano de sprints»). A partir de 13/10 os IDs não mudam. Replaneado a 23/10/2026: o plano de candidatura substitui as opcionais, que passam a Won't (fase 2).</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -156,7 +156,7 @@
     <t xml:space="preserve">Feito</t>
   </si>
   <si>
-    <t xml:space="preserve">Código, testes e documentação no GitHub (PR #1 a #3 aceites).</t>
+    <t xml:space="preserve">Código, testes e documentação no GitHub (PR #1 a #3 aceites). 23/10: o registo pede também o nome, e o OptaBem trata a pessoa por ele (PR #43; RF01.17 e RF01.18).</t>
   </si>
   <si>
     <t xml:space="preserve">US02</t>
@@ -165,7 +165,7 @@
     <t xml:space="preserve">Autenticação</t>
   </si>
   <si>
-    <t xml:space="preserve">Como aluno, quero iniciar e terminar sessão, para aceder às minhas avaliações e recomendações de forma segura.</t>
+    <t xml:space="preserve">Como aluno, quero iniciar e terminar sessão, para aceder ao meu percurso de forma segura.</t>
   </si>
   <si>
     <t xml:space="preserve">• Login com email e palavra-passe.
@@ -174,7 +174,7 @@
 • Páginas privadas redirecionam para o login.</t>
   </si>
   <si>
-    <t xml:space="preserve">Código, testes e documentação no GitHub (PR #4 e #5 aceites, com o ícone para mostrar a palavra-passe).</t>
+    <t xml:space="preserve">Código, testes e documentação no GitHub (PR #4 e #5 aceites, com o ícone para mostrar a palavra-passe). 23/10: texto da story sem «avaliações e recomendações» (eram das opcionais). Terminar sessão passa a voltar à página inicial (PR #43).</t>
   </si>
   <si>
     <t xml:space="preserve">US03</t>
@@ -260,7 +260,7 @@
 • O utilizador pode mudar de curso, o que cria uma nova decisão.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: story nova (nova visão do produto, sugestão do docente). 14/10: mantém-se no Sprint 3; a escolha parte das sugestões da US30. 20/10 (Sprint Planning): antecipada para o Sprint 2, porque a US29 e a US30 foram feitas antes de o sprint começar; é ela que dá sentido às sugestões. 20/10: feita (PR da US31, à espera de revisão); docs/US31/, issue #27. Depois de escolher, a conversa com o LLM é apagada (ponto 15, decisão do PO). 22/10: aceite na Sprint Review do Sprint 2 (percurso completo testado pelos PO com o Gemini real, também noutro computador); fica Feito.</t>
+    <t xml:space="preserve">Replaneamento de 13/10: story nova (nova visão do produto, sugestão do docente). 14/10: mantém-se no Sprint 3; a escolha parte das sugestões da US30. 20/10 (Sprint Planning): antecipada para o Sprint 2, porque a US29 e a US30 foram feitas antes de o sprint começar; é ela que dá sentido às sugestões. 20/10: feita (PR da US31, à espera de revisão); docs/US31/, issue #27. Depois de escolher, a conversa com o LLM é apagada (ponto 15, decisão do PO). 22/10: aceite na Sprint Review do Sprint 2 (percurso completo testado pelos PO com o Gemini real, também noutro computador); fica Feito. 23/10: «As minhas decisões» sai do menu (decisão do PO); continua acessível pelo início e por «A minha conta».</t>
   </si>
   <si>
     <t xml:space="preserve">US05</t>
@@ -290,6 +290,197 @@
     <t xml:space="preserve">US04</t>
   </si>
   <si>
+    <t xml:space="preserve">US17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Apagar a minha conta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como aluno, quero apagar a minha conta e todos os meus dados, para exercer o meu direito ao apagamento.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Apagar remove a conta, a conversa de orientação, as decisões do percurso e os pedidos ao LLM.
+• A ação pede confirmação (palavra-passe).
+• A sessão termina e a página confirma que os dados foram apagados.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). 22/10 (Sprint Planning do Sprint 3): Backlog → Sprint 3, Should → Must. O OptaBem já guarda conversas e decisões de pessoas, por isso exportar e apagar os dados passa a ser essencial (RGPD). 22/10 (decisão do PO): âmbito reduzido ao apagamento da conta; a exportação fica no backlog (RF17). 3 → 2 SP. Feita (PR da US17, à espera de revisão); docs/US17/, issue #34. 23/10: aceite na Sprint Review do Sprint 3 (testada pelos PO); fica Feito.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catálogo completo de licenciaturas (DGES)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como pessoa indecisa, quero procurar em todas as licenciaturas do concurso nacional, e não só numa amostra, para não deixar de fora um curso que me sirva.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Os cursos vêm das páginas públicas da DGES, por um script que corre no computador da equipa (dados/recolher_dges.py), devagar e retomável.
+• O catálogo tem as licenciaturas e mestrados integrados do concurso nacional, com vagas, nota do último colocado e condições de acesso.
+• As descrições escritas pela equipa (catálogo do MVP) mantêm-se.
+• Lista de cursos com paginação (24 por página).
+• Acima de 150 cursos, o assistente (LLM) recebe só os cursos das áreas escolhidas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Em curso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa a importar instituições e cursos (nova visão). As UCs de cada curso entram com a US06. 14/10: Sprint 2 → Backlog, Must → Should: a aplicação já lê o catálogo do CSV (app/catalogo) e o LLM trabalha sobre ele; importar para a base de dados não muda nada para o utilizador nesta release. 22/10: candidata ao Sprint 4 se houver folga. 23/10: reescrita por decisão do PO. Em vez de o administrador importar um CSV, o catálogo vem da DGES por recolha (sugestão de um colega). Ramo feature/US04-catalogo-completo: 174 cursos recolhidos, falta a recolha completa e a documentação. Backlog → Sprint 4, Should → Must; a confirmar com o docente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US33</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Condições de acesso na ficha do curso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como pessoa a escolher curso, quero ver na ficha de cada curso as provas de ingresso, a fórmula de cálculo, as classificações mínimas e os pré-requisitos, para saber o que é preciso para entrar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Dados lidos das páginas da DGES (a mesma recolha da US04).
+• Conjuntos alternativos de provas mostrados pelo nome («Basta um destes conjuntos»).
+• Fórmula (peso da média e das provas) e mínimos em pontos.
+• Um curso sem estes dados mostra a ligação à DGES.
+• Funciona sem sessão iniciada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23/10: story nova (decisão do PO: o plano de candidatura substitui as opcionais). Protótipo no PR #44 (rascunho), feito antes do sprint para o PO ver a ideia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nova</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US34</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Registar as minhas notas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como candidato, quero indicar a minha média do secundário e as notas dos exames nacionais que fiz, para o OptaBem fazer as contas por mim.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Média de 9,5 a 20 valores; exames de 0 a 200 pontos (ou de 0 a 20, convertidos).
+• Só se preenchem os exames feitos.
+• As notas podem ser mudadas e saem com a conta (US17).
+• Matemática e Matemática A contam com o mesmo exame (a confirmar pela equipa na DGES).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23/10: story nova. Protótipo no PR #44 (rascunho), feito antes do sprint para o PO ver a ideia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US35</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota de candidatura a cada curso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como candidato, quero ver a minha nota de candidatura a cada curso e a diferença para o último colocado, para perceber onde tenho hipóteses.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Nota = média do secundário × peso + provas × peso, com o conjunto de provas mais favorável.
+• Situação: acima (5 ou mais pontos), perto (menos de 5 de diferença) ou abaixo do último colocado; falta de prova e nota abaixo do mínimo assinaladas.
+• Aparece na ficha de cada curso, com sessão iniciada.
+• Aviso visível: estimativa para o contingente geral da 1.ª fase, não uma garantia.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23/10: story nova. Protótipo no PR #44 (rascunho), feito antes do sprint para o PO ver a ideia. Contas em funções puras (app/candidatura/calculos.py).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plano das 6 opções de candidatura</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como candidato, quero montar e ordenar a minha lista de até 6 opções, com avisos, para submeter na DGES uma candidatura equilibrada.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Juntar cursos a partir da ficha; no máximo 6, sem repetidos.
+• Subir, descer e retirar opções (funciona sem JavaScript).
+• Avisos: opções que não contam, nenhuma opção segura, a mais fácil em 1.º lugar, menos de 6 opções, pré-requisitos.
+• Sugestões de cursos da mesma área onde a pessoa fica acima ou perto.
+• Passo «Preparar a candidatura» no percurso do início.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Should</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23/10: story nova. Protótipo no PR #44 (rascunho), feito antes do sprint para o PO ver a ideia. O OptaBem não submete a candidatura: ajuda a prepará-la.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assistente que conhece as minhas notas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como pessoa indecisa, quero que o assistente tenha em conta as provas que fiz e a minha nota, para não me sugerir cursos a que não posso concorrer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Só com autorização da pessoa, o LLM recebe as provas feitas e um intervalo de nota (nunca a média exata, RNF12).
+• Cursos a que falta uma prova não são sugeridos, ou vêm assinalados.
+• Os testes usam o LLM falso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backlog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por fazer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23/10: story nova. Atenção: os termos do Gemini excluem menores de 18, e muitos candidatos têm 17 anos (protótipo para a equipa, ponto 14 dos requisitos).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corrigir e esconder cursos do catálogo (gestão)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como administrador, quero corrigir a descrição e as saídas profissionais de um curso, ou escondê-lo, para o catálogo não ter erros sem mexer no ficheiro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Só na área de gestão.
+• As correções ficam na base de dados, por cima dos dados da DGES (a recolha seguinte não as apaga).
+• Fica registado quem alterou e quando.
+• Sem acesso aos dados dos alunos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23/10: sugestão de um colega («editar a base de dados na área de gestão»), reescrita com uma necessidade concreta. Um editor genérico de tabelas daria aos administradores os dados pessoais dos alunos (RGPD) e seria o ponto mais perigoso do site aberto pelo túnel. Precisa do catálogo na base de dados.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Datas do concurso no percurso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como candidato, quero ver as datas das fases do concurso nacional, para não falhar prazos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Datas das 3 fases do concurso, com a ligação para a DGES.
+• O passo atual do percurso mostra o próximo prazo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Could</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23/10: story nova.</t>
+  </si>
+  <si>
     <t xml:space="preserve">US06</t>
   </si>
   <si>
@@ -308,16 +499,10 @@
 • O aluno pode remover um registo.</t>
   </si>
   <si>
-    <t xml:space="preserve">Should</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Backlog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Por fazer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4; inclui a importação das UCs; 3 → 5 SP. 14/10: mantém-se no Sprint 4. 22/10: Sprint 4 → Backlog, Must → Should. Decisão dos PO: até à entrega de 05/11 o centro são os cursos e as opcionais ficam em segundo plano.</t>
+    <t xml:space="preserve">Won't</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4; inclui a importação das UCs; 3 → 5 SP. 14/10: mantém-se no Sprint 4. 22/10: Sprint 4 → Backlog, Must → Should. Decisão dos PO: até à entrega de 05/11 o centro são os cursos e as opcionais ficam em segundo plano. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">US07</t>
@@ -336,28 +521,10 @@
 • As avaliações ficam ligadas a um pseudo_id desde o início, e não ao email (ponto 2 dos requisitos); as regras de visualização e exportação ficam na US09.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4. 14/10: fica no Sprint 4 sem a US09 (velocidade de 10 SP); por isso guarda já com pseudo_id. 22/10: Sprint 4 → Backlog, Must → Should. Decisão dos PO: até à entrega de 05/11 o centro são os cursos e as opcionais ficam em segundo plano.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Importar catálogo de instituições e cursos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como administrador, quero importar instituições e cursos a partir de um ficheiro CSV, para que o catálogo tenha várias instituições sem introduzir os dados um a um.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Aceita o formato de dados/catalogo-cursos-mvp.csv (códigos DGES, curso, instituição, área, vagas, nota do último colocado, descrição, saídas, fontes).
-• O CSV é validado (colunas obrigatórias, tipos, códigos duplicados).
-• Linhas inválidas são reportadas sem bloquear as válidas.
-• Reimportar atualiza cursos existentes pelo par código de instituição + código de curso.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa a importar instituições e cursos (nova visão). As UCs de cada curso entram com a US06. 14/10: Sprint 2 → Backlog, Must → Should: a aplicação já lê o catálogo do CSV (app/catalogo) e o LLM trabalha sobre ele; importar para a base de dados não muda nada para o utilizador nesta release. 22/10: candidata ao Sprint 4 se houver folga.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4. 14/10: fica no Sprint 4 sem a US09 (velocidade de 10 SP); por isso guarda já com pseudo_id. 22/10: Sprint 4 → Backlog, Must → Should. Decisão dos PO: até à entrega de 05/11 o centro são os cursos e as opcionais ficam em segundo plano. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">US09</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E4</t>
   </si>
   <si>
     <t xml:space="preserve">Avaliações pseudonimizadas</t>
@@ -372,7 +539,7 @@
 • Teste automático que verifica RN04.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: Sprint 2 → Sprint 4, com a US07 para as avaliações serem anónimas desde o início. 14/10: Sprint 4 → Backlog, Must → Should (velocidade de 10 SP). A US07 guarda já com pseudo_id; sem agregados (US11) a RN04 ainda não se aplica.</t>
+    <t xml:space="preserve">Replaneamento de 13/10: Sprint 2 → Sprint 4, com a US07 para as avaliações serem anónimas desde o início. 14/10: Sprint 4 → Backlog, Must → Should (velocidade de 10 SP). A US07 guarda já com pseudo_id; sem agregados (US11) a RN04 ainda não se aplica. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">US11</t>
@@ -393,7 +560,7 @@
 • Implementada como estratégia intercambiável (padrão Strategy, docs/geral/03).</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 2 para Sprint 3. Replaneamento de 13/10: Sprint 3 → Sprint 4; segue o padrão Strategy. 14/10: Sprint 4 → Backlog, Must → Should (velocidade de 10 SP). Primeira candidata se houver um Sprint 5 ou folga.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 2 para Sprint 3. Replaneamento de 13/10: Sprint 3 → Sprint 4; segue o padrão Strategy. 14/10: Sprint 4 → Backlog, Must → Should (velocidade de 10 SP). Primeira candidata se houver um Sprint 5 ou folga. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">US08</t>
@@ -410,10 +577,7 @@
 • Avaliar 10 UCs demora menos de 2 minutos.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US10</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">E9</t>
@@ -429,7 +593,7 @@
 • O motor recomenda UCs do perfil "plantado" na maioria dos casos.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 2 para Sprint 3. Replaneamento de 13/10: Sprint 3 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 2 para Sprint 3. Replaneamento de 13/10: Sprint 3 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">US20</t>
@@ -486,7 +650,7 @@
 • A explicação não revela identidades.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: Sprint 3 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release.</t>
+    <t xml:space="preserve">Replaneamento de 13/10: Sprint 3 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">Avaliação offline do motor</t>
@@ -500,16 +664,13 @@
 • Resultados guardados e comparáveis entre estratégias.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 3 para Sprint 4. Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 3 para Sprint 4. Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">US21</t>
   </si>
   <si>
     <t xml:space="preserve">US16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E10</t>
   </si>
   <si>
     <t xml:space="preserve">Períodos de avaliação</t>
@@ -522,27 +683,10 @@
 • Fora do período, o formulário de avaliação fica bloqueado com mensagem explicativa.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 3 para Sprint 4. Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro).</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 3 para Sprint 4. Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">US24</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Apagar a minha conta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como aluno, quero apagar a minha conta e todos os meus dados, para exercer o meu direito ao apagamento.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Apagar remove a conta, a conversa de orientação, as decisões do percurso e os pedidos ao LLM.
-• A ação pede confirmação (palavra-passe).
-• A sessão termina e a página confirma que os dados foram apagados.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). 22/10 (Sprint Planning do Sprint 3): Backlog → Sprint 3, Should → Must. O OptaBem já guarda conversas e decisões de pessoas, por isso exportar e apagar os dados passa a ser essencial (RGPD). 22/10 (decisão do PO): âmbito reduzido ao apagamento da conta; a exportação fica no backlog (RF17). 3 → 2 SP. Feita (PR da US17, à espera de revisão); docs/US17/, issue #34. 23/10: aceite na Sprint Review do Sprint 3 (testada pelos PO); fica Feito.</t>
   </si>
   <si>
     <t xml:space="preserve">US18</t>
@@ -574,7 +718,7 @@
 • Os alunos podem sinalizar comentários.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro).</t>
+    <t xml:space="preserve">Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">US25</t>
@@ -601,7 +745,7 @@
 • "Indiferente" mantém a ordenação original.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 3 para Backlog.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 3 para Backlog. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">US22</t>
@@ -620,7 +764,7 @@
 • A estratégia ativa muda sem reiniciar a aplicação.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 4 para Backlog. Depende do SVD (antiga US22), que também ficou fora do plano.</t>
+    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 4 para Backlog. Depende do SVD (antiga US22), que também ficou fora do plano. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">US23</t>
@@ -636,10 +780,7 @@
 • UCs com 0 vagas não aparecem, com opção "mostrar todas".</t>
   </si>
   <si>
-    <t xml:space="preserve">Could</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entra no Sprint 4 se houver folga de velocidade.</t>
+    <t xml:space="preserve">Entra no Sprint 4 se houver folga de velocidade. 23/10: Could → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">Feedback sobre recomendações</t>
@@ -650,6 +791,9 @@
   <si>
     <t xml:space="preserve">• UCs ocultas deixam de aparecer.
 • O feedback fica registado para análise.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23/10: Could → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">Painel de participação</t>
@@ -702,7 +846,7 @@
 • O aluno pode desativar lembretes.</t>
   </si>
   <si>
-    <t xml:space="preserve">Won't</t>
+    <t xml:space="preserve">23/10: Won't → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
   </si>
   <si>
     <t xml:space="preserve">US32</t>
@@ -723,19 +867,16 @@
     <t xml:space="preserve">14/10: pedido do PO para verificar a inserção de um agente LLM. No mesmo dia, o PO decidiu que o LLM conduz a conversa: a story foi fundida na US29. O ID fica, para a rastreabilidade.</t>
   </si>
   <si>
-    <t xml:space="preserve">nova</t>
-  </si>
-  <si>
     <t xml:space="preserve">Total de story points</t>
   </si>
   <si>
     <t xml:space="preserve">Story points concluídos (Estado = Feito)</t>
   </si>
   <si>
-    <t xml:space="preserve">Nota: a fatorização de matrizes (SVD, antiga US22) fica fora do plano da release. Épico E11 (novo): Orientação de curso.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plano de sprints — Recomendador de UCs Opcionais</t>
+    <t xml:space="preserve">Nota: a fatorização de matrizes (SVD, antiga US22) fica fora do plano da release. Épicos novos: E11 Orientação de curso (13/10) e E12 Candidatura (23/10). As stories das opcionais (Won't) ficam no fim, como fase 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plano de sprints — OptaBem</t>
   </si>
   <si>
     <t xml:space="preserve">Calculado a partir da folha «Product Backlog»: mudar o Sprint ou o Estado de uma story lá atualiza esta tabela.</t>
@@ -783,19 +924,16 @@
     <t xml:space="preserve">US05, US17</t>
   </si>
   <si>
-    <t xml:space="preserve">Sprint 4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">O percurso continua depois da escolha do curso: story nova a decidir com o docente (preparar o percurso ou perguntas e respostas por curso); US04 se houver folga (29/10 a 05/11; código fechado por volta de 03/11).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Story nova (a definir); US04 se houver folga</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fora desta release (entrega a 05/11). As stories das opcionais ficam em segundo plano (decisão dos PO de 22/10).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US04, US06–US16, US18–US28 (US32 fundida na US29)</t>
+    <t xml:space="preserve">Quem escolheu um curso prepara a candidatura: vê as condições de acesso, calcula a sua nota em cada curso e ordena as 6 opções; o catálogo passa a ter as licenciaturas da DGES (29/10 a 05/11; a confirmar com o docente).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US04, US33, US34, US35, US36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fora desta release (entrega a 05/11). As stories das opcionais passam a Won't (fase 2) a 23/10: o plano de candidatura substitui-as.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US37–US39, US06–US16, US18–US28 (US32 fundida na US29)</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -934,6 +1072,33 @@
   </si>
   <si>
     <t xml:space="preserve">• Sprint 4 por planear: a story nova fica a decidir com o docente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 23/10/2026 (decisões do PO, com o protótipo do PR #44)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• O plano de candidatura ao Concurso Nacional de Acesso substitui as opcionais: épico novo E12 com a US33 (condições de acesso), US34 (notas), US35 (nota por curso), US36 (as 6 opções), US37 (assistente com as notas) e US38 (datas do concurso).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• As 22 stories das opcionais passam a Won't (fase 2) e ficam no fim do backlog, para a rastreabilidade.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US04 reescrita: o catálogo vem da DGES por recolha, em vez de ser importado por CSV na gestão; passa a Must e entra no Sprint 4.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US39 nova (gestão do catálogo), a partir da sugestão de um colega de editar a base de dados na área de gestão; fica no Backlog (Should).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Atenção: o Sprint 4 fica com 18 SP planeados, acima da velocidade (10). O código das US33 a US36 foi feito antes do sprint (protótipo), como a US29 e a US30 no Sprint 2. Se o docente achar demais, a US36 é a primeira a sair (é Should).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sem story: o registo pede o nome, terminar sessão volta à página inicial e «As minhas decisões» sai do menu (PR #43 e #44).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Correção: o Sprint Planning de 22/10 dizia «US17 (3 SP)»; a US17 tem 2 SP (o total de 7 SP da Sprint Review está certo).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• A story do Sprint 4 tem de ser confirmada com o docente.</t>
   </si>
   <si>
     <t xml:space="preserve">Resumo por prioridade (MoSCoW)</t>
@@ -1316,7 +1481,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="22">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1383,6 +1548,14 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
+          <fgColor rgb="FFEDE4F5"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
           <fgColor rgb="FFFCE4D6"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
@@ -1400,6 +1573,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFC6EFCE"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFEB9C"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1662,7 +1843,7 @@
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1764,11 +1945,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="71063653"/>
-        <c:axId val="6152493"/>
+        <c:axId val="57761804"/>
+        <c:axId val="79428830"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="71063653"/>
+        <c:axId val="57761804"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1799,7 +1980,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="6152493"/>
+        <c:crossAx val="79428830"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1807,7 +1988,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="6152493"/>
+        <c:axId val="79428830"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1872,7 +2053,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="71063653"/>
+        <c:crossAx val="57761804"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1939,9 +2120,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2089080</xdr:colOff>
+      <xdr:colOff>2088720</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>86040</xdr:rowOff>
+      <xdr:rowOff>85680</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1950,7 +2131,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5754240" cy="2513880"/>
+        <a:ext cx="5753880" cy="2513520"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2143,7 +2324,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:M39"/>
+  <dimension ref="A1:M46"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
@@ -2327,7 +2508,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="139.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="n">
         <v>4</v>
       </c>
@@ -2366,7 +2547,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="139.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="n">
         <v>5</v>
       </c>
@@ -2503,23 +2684,23 @@
         <v>64</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="I12" s="7" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="J12" s="7" t="s">
-        <v>67</v>
+        <v>22</v>
       </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="M12" s="5" t="s">
-        <v>52</v>
+        <v>66</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2527,38 +2708,38 @@
         <v>9</v>
       </c>
       <c r="B13" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="F13" s="6" t="s">
         <v>69</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>72</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="I13" s="7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J13" s="7" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="M13" s="5" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2566,38 +2747,38 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>59</v>
+        <v>73</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="I14" s="7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J14" s="7" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="M14" s="5" t="s">
-        <v>29</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2605,38 +2786,38 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="I15" s="7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J15" s="7" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2644,10 +2825,10 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>85</v>
+        <v>74</v>
       </c>
       <c r="D16" s="6" t="s">
         <v>86</v>
@@ -2662,20 +2843,20 @@
         <v>3</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>65</v>
+        <v>20</v>
       </c>
       <c r="I16" s="7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J16" s="7" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8" t="s">
         <v>89</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2686,7 +2867,7 @@
         <v>90</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>91</v>
@@ -2698,23 +2879,23 @@
         <v>93</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="I17" s="7" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="K17" s="8"/>
       <c r="L17" s="8" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>69</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2722,10 +2903,10 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>96</v>
+        <v>74</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>97</v>
@@ -2737,23 +2918,23 @@
         <v>99</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>101</v>
+        <v>79</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2761,38 +2942,38 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>85</v>
+        <v>104</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>102</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2800,38 +2981,38 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>107</v>
+        <v>74</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G20" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>65</v>
+        <v>113</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>111</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2839,38 +3020,38 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="G21" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="M21" s="5" t="s">
-        <v>106</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2878,38 +3059,38 @@
         <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>96</v>
+        <v>116</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="G22" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2917,38 +3098,38 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>124</v>
+        <v>61</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="M23" s="5" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2956,38 +3137,38 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>79</v>
+        <v>133</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>57</v>
+        <v>100</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>22</v>
+        <v>101</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>95</v>
+        <v>132</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2995,38 +3176,38 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>61</v>
+        <v>116</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
-        <v>128</v>
+        <v>142</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>90</v>
+        <v>122</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3034,38 +3215,38 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>139</v>
+        <v>66</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>124</v>
+        <v>143</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3073,38 +3254,38 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="G27" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="H27" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="J27" s="7" t="s">
         <v>101</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="G27" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="I27" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="J27" s="7" t="s">
-        <v>67</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>123</v>
+        <v>149</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3112,38 +3293,38 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>122</v>
+        <v>153</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>107</v>
+        <v>154</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="G28" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>112</v>
+        <v>158</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3151,38 +3332,38 @@
         <v>25</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="G29" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>65</v>
+        <v>120</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="M29" s="5" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3193,35 +3374,35 @@
         <v>158</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>107</v>
+        <v>143</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="G30" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>162</v>
+        <v>120</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>130</v>
+        <v>169</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3229,36 +3410,38 @@
         <v>27</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>129</v>
+        <v>170</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>113</v>
+        <v>104</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="G31" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>162</v>
+        <v>120</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="K31" s="8"/>
-      <c r="L31" s="8"/>
+      <c r="L31" s="8" t="s">
+        <v>174</v>
+      </c>
       <c r="M31" s="5" t="s">
-        <v>139</v>
+        <v>175</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3266,36 +3449,38 @@
         <v>28</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>144</v>
+        <v>176</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>167</v>
+        <v>177</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>168</v>
+        <v>178</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>169</v>
+        <v>179</v>
       </c>
       <c r="G32" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>162</v>
+        <v>120</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="K32" s="8"/>
-      <c r="L32" s="8"/>
+      <c r="L32" s="8" t="s">
+        <v>174</v>
+      </c>
       <c r="M32" s="5" t="s">
-        <v>170</v>
+        <v>138</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3303,36 +3488,38 @@
         <v>29</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>153</v>
+        <v>104</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>171</v>
+        <v>181</v>
       </c>
       <c r="E33" s="6" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="G33" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>162</v>
+        <v>120</v>
       </c>
       <c r="I33" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="K33" s="8"/>
-      <c r="L33" s="8"/>
+      <c r="L33" s="8" t="s">
+        <v>184</v>
+      </c>
       <c r="M33" s="5" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3340,36 +3527,38 @@
         <v>30</v>
       </c>
       <c r="B34" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="C34" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="D34" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>188</v>
+      </c>
+      <c r="G34" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="I34" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="J34" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="K34" s="8"/>
+      <c r="L34" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="C34" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>175</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="G34" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H34" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="I34" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="J34" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="K34" s="8"/>
-      <c r="L34" s="8"/>
       <c r="M34" s="5" t="s">
-        <v>135</v>
+        <v>170</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3377,151 +3566,426 @@
         <v>31</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>178</v>
+        <v>169</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>179</v>
+        <v>189</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="F35" s="6" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>182</v>
+        <v>120</v>
       </c>
       <c r="I35" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J35" s="7" t="s">
-        <v>67</v>
+        <v>101</v>
       </c>
       <c r="K35" s="8"/>
-      <c r="L35" s="8"/>
+      <c r="L35" s="8" t="s">
+        <v>192</v>
+      </c>
       <c r="M35" s="5" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="60" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="n">
         <v>32</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>183</v>
+        <v>193</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>36</v>
+        <v>194</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>186</v>
-      </c>
-      <c r="G36" s="7"/>
-      <c r="H36" s="5"/>
+        <v>197</v>
+      </c>
+      <c r="G36" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H36" s="5" t="s">
+        <v>120</v>
+      </c>
       <c r="I36" s="7" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="J36" s="7" t="s">
-        <v>187</v>
+        <v>101</v>
       </c>
       <c r="K36" s="8"/>
       <c r="L36" s="8" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="M36" s="5" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F37" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="G37" s="9" t="n">
-        <f aca="false">SUM(G5:G36)</f>
-        <v>125</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F38" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="G38" s="9" t="n">
-        <f aca="false">SUMIF(J5:J36,"Feito",G5:G36)</f>
+        <v>199</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="5" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="E37" s="6" t="s">
+        <v>201</v>
+      </c>
+      <c r="F37" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="G37" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H37" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="I37" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="J37" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="K37" s="8"/>
+      <c r="L37" s="8" t="s">
+        <v>203</v>
+      </c>
+      <c r="M37" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="5" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>160</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>204</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>205</v>
+      </c>
+      <c r="F38" s="6" t="s">
+        <v>206</v>
+      </c>
+      <c r="G38" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="I38" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="J38" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="K38" s="8"/>
+      <c r="L38" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="M38" s="5" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="5" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>208</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="F39" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="G39" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H39" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="I39" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="J39" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="K39" s="8"/>
+      <c r="L39" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="M39" s="5" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>194</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>212</v>
+      </c>
+      <c r="E40" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="F40" s="6" t="s">
+        <v>214</v>
+      </c>
+      <c r="G40" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H40" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="I40" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="J40" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="K40" s="8"/>
+      <c r="L40" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="M40" s="5" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>215</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>217</v>
+      </c>
+      <c r="F41" s="6" t="s">
+        <v>218</v>
+      </c>
+      <c r="G41" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="H41" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="I41" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="J41" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="K41" s="8"/>
+      <c r="L41" s="8" t="s">
+        <v>207</v>
+      </c>
+      <c r="M41" s="5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="D42" s="6" t="s">
+        <v>220</v>
+      </c>
+      <c r="E42" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="F42" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="G42" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H42" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="I42" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="J42" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="K42" s="8"/>
+      <c r="L42" s="8" t="s">
+        <v>223</v>
+      </c>
+      <c r="M42" s="5" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="5" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>224</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D43" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="E43" s="6" t="s">
+        <v>226</v>
+      </c>
+      <c r="F43" s="6" t="s">
+        <v>227</v>
+      </c>
+      <c r="G43" s="7"/>
+      <c r="H43" s="5"/>
+      <c r="I43" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="J43" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="K43" s="8"/>
+      <c r="L43" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="M43" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F44" s="9" t="s">
+        <v>230</v>
+      </c>
+      <c r="G44" s="9" t="n">
+        <f aca="false">SUM(G5:G43)</f>
+        <v>148</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F45" s="9" t="s">
+        <v>231</v>
+      </c>
+      <c r="G45" s="9" t="n">
+        <f aca="false">SUMIF(J5:J43,"Feito",G5:G43)</f>
         <v>30</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F39" s="10" t="s">
-        <v>192</v>
+    <row r="46" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F46" s="10" t="s">
+        <v>232</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:M36"/>
-  <conditionalFormatting sqref="J5:J36">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
+  <autoFilter ref="A4:M43"/>
+  <conditionalFormatting sqref="J5:J43">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Feito"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>"Em curso"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H36">
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+  <conditionalFormatting sqref="H5:H43">
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Must"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Should"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>"Could"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Won't"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I36">
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+  <conditionalFormatting sqref="I5:I43">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Sprint 1"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>"Sprint 2"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"Sprint 3"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
       <formula>"Sprint 4"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
       <formula>"Backlog"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G36" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G43" type="list">
       <formula1>"1,2,3,5,8,13,21"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H36" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H43" type="list">
       <formula1>"Must,Should,Could,Won't"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I36" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I43" type="list">
       <formula1>"Sprint 1,Sprint 2,Sprint 3,Sprint 4,Backlog"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J36" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J43" type="list">
       <formula1>"Por fazer,Em curso,Feito,Fundida"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3543,7 +4007,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:H88"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -3558,17 +4022,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>193</v>
+        <v>233</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>194</v>
+        <v>234</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>195</v>
+        <v>235</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>10</v>
@@ -3579,25 +4043,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>196</v>
+        <v>236</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>197</v>
+        <v>237</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>198</v>
+        <v>238</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>199</v>
+        <v>239</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>201</v>
+        <v>241</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>202</v>
+        <v>242</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3605,17 +4069,17 @@
         <v>21</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>203</v>
+        <v>243</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>204</v>
+        <v>244</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A6,'Product Backlog'!$G$5:$G$36)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$43,$A6,'Product Backlog'!$G$5:$G$43)</f>
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A6,'Product Backlog'!$J$5:$J$36,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$43,'Product Backlog'!$I$5:$I$43,$A6,'Product Backlog'!$J$5:$J$43,"Feito")</f>
         <v>10</v>
       </c>
       <c r="F6" s="15" t="n">
@@ -3627,7 +4091,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A6)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$43,$A6)</f>
         <v>3</v>
       </c>
     </row>
@@ -3636,17 +4100,17 @@
         <v>40</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>205</v>
+        <v>245</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>206</v>
+        <v>246</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A7,'Product Backlog'!$G$5:$G$36)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$43,$A7,'Product Backlog'!$G$5:$G$43)</f>
         <v>13</v>
       </c>
       <c r="E7" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A7,'Product Backlog'!$J$5:$J$36,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$43,'Product Backlog'!$I$5:$I$43,$A7,'Product Backlog'!$J$5:$J$43,"Feito")</f>
         <v>13</v>
       </c>
       <c r="F7" s="15" t="n">
@@ -3658,7 +4122,7 @@
         <v>-3</v>
       </c>
       <c r="H7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A7)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$43,$A7)</f>
         <v>3</v>
       </c>
     </row>
@@ -3667,17 +4131,17 @@
         <v>57</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>207</v>
+        <v>247</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>208</v>
+        <v>248</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$G$5:$G$36)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$43,$A8,'Product Backlog'!$G$5:$G$43)</f>
         <v>7</v>
       </c>
       <c r="E8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A8,'Product Backlog'!$J$5:$J$36,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$43,'Product Backlog'!$I$5:$I$43,$A8,'Product Backlog'!$J$5:$J$43,"Feito")</f>
         <v>7</v>
       </c>
       <c r="F8" s="15" t="n">
@@ -3689,26 +4153,26 @@
         <v>3</v>
       </c>
       <c r="H8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A8)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$43,$A8)</f>
         <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>209</v>
+        <v>70</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>210</v>
+        <v>249</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>211</v>
+        <v>250</v>
       </c>
       <c r="D9" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A9,'Product Backlog'!$G$5:$G$36)</f>
-        <v>0</v>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$43,$A9,'Product Backlog'!$G$5:$G$43)</f>
+        <v>18</v>
       </c>
       <c r="E9" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A9,'Product Backlog'!$J$5:$J$36,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$43,'Product Backlog'!$I$5:$I$43,$A9,'Product Backlog'!$J$5:$J$43,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F9" s="15" t="n">
@@ -3717,29 +4181,29 @@
       </c>
       <c r="G9" s="16" t="n">
         <f aca="false">$C$3-D9</f>
-        <v>10</v>
+        <v>-8</v>
       </c>
       <c r="H9" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A9)</f>
-        <v>0</v>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$43,$A9)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>66</v>
+        <v>100</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>212</v>
+        <v>251</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>213</v>
+        <v>252</v>
       </c>
       <c r="D10" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$36,$A10,'Product Backlog'!$G$5:$G$36)</f>
-        <v>95</v>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$43,$A10,'Product Backlog'!$G$5:$G$43)</f>
+        <v>100</v>
       </c>
       <c r="E10" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$36,'Product Backlog'!$I$5:$I$36,$A10,'Product Backlog'!$J$5:$J$36,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$43,'Product Backlog'!$I$5:$I$43,$A10,'Product Backlog'!$J$5:$J$43,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F10" s="15" t="n">
@@ -3750,19 +4214,19 @@
         <v>34</v>
       </c>
       <c r="H10" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$36,$A10)</f>
-        <v>24</v>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$43,$A10)</f>
+        <v>26</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>214</v>
+        <v>253</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
       <c r="D11" s="21" t="n">
         <f aca="false">SUM(D6:D10)</f>
-        <v>125</v>
+        <v>148</v>
       </c>
       <c r="E11" s="21" t="n">
         <f aca="false">SUM(E6:E10)</f>
@@ -3770,237 +4234,282 @@
       </c>
       <c r="F11" s="22" t="n">
         <f aca="false">IF(D11=0,0,E11/D11)</f>
-        <v>0.24</v>
+        <v>0.202702702702703</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21" t="n">
         <f aca="false">SUM(H6:H10)</f>
-        <v>32</v>
+        <v>39</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>215</v>
+        <v>254</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>216</v>
+        <v>255</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>217</v>
+        <v>256</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>218</v>
+        <v>257</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>219</v>
+        <v>258</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>220</v>
+        <v>259</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>221</v>
+        <v>260</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>222</v>
+        <v>261</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>223</v>
+        <v>262</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
-        <v>224</v>
+        <v>263</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>225</v>
+        <v>264</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
-        <v>226</v>
+        <v>265</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>227</v>
+        <v>266</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="24" t="s">
-        <v>228</v>
+        <v>267</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="24" t="s">
-        <v>229</v>
+        <v>268</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="24" t="s">
-        <v>230</v>
+        <v>269</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="23" t="s">
-        <v>231</v>
+        <v>270</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="24" t="s">
-        <v>232</v>
+        <v>271</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="24" t="s">
-        <v>233</v>
+        <v>272</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="24" t="s">
-        <v>234</v>
+        <v>273</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="24" t="s">
-        <v>235</v>
+        <v>274</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="23" t="s">
-        <v>236</v>
+        <v>275</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="24" t="s">
-        <v>237</v>
+        <v>276</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="24" t="s">
-        <v>238</v>
+        <v>277</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="24" t="s">
-        <v>239</v>
+        <v>278</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="24" t="s">
-        <v>240</v>
+        <v>279</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="24" t="s">
-        <v>241</v>
+        <v>280</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="24" t="s">
-        <v>242</v>
+        <v>281</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="23" t="s">
-        <v>243</v>
+        <v>282</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="24" t="s">
-        <v>244</v>
+        <v>283</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="24" t="s">
-        <v>245</v>
+        <v>284</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="24" t="s">
-        <v>246</v>
+        <v>285</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="24" t="s">
-        <v>247</v>
+        <v>286</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="23" t="s">
-        <v>248</v>
+        <v>287</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="24" t="s">
-        <v>249</v>
+        <v>288</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="24" t="s">
-        <v>250</v>
+        <v>289</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="24" t="s">
-        <v>251</v>
+        <v>290</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="24" t="s">
-        <v>252</v>
+        <v>291</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="24" t="s">
-        <v>253</v>
+        <v>292</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="24" t="s">
-        <v>254</v>
+        <v>293</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="23" t="s">
-        <v>255</v>
+        <v>294</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="24" t="s">
-        <v>256</v>
+        <v>295</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="24" t="s">
-        <v>257</v>
+        <v>296</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="24" t="s">
-        <v>258</v>
+        <v>297</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="24" t="s">
-        <v>259</v>
+        <v>298</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="23" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A81" s="24" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A82" s="24" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A83" s="24" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A84" s="24" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A85" s="24" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A86" s="24" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="24" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="24" t="s">
+        <v>307</v>
       </c>
     </row>
   </sheetData>
@@ -4033,24 +4542,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>260</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>261</v>
+        <v>309</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>262</v>
+        <v>310</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>202</v>
+        <v>242</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>263</v>
+        <v>311</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>264</v>
+        <v>312</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4058,92 +4567,92 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>265</v>
+        <v>313</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A5)</f>
-        <v>8</v>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$43,A5)</f>
+        <v>12</v>
       </c>
       <c r="D5" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$36,A5,'Product Backlog'!$G$5:$G$36)</f>
-        <v>30</v>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$43,A5,'Product Backlog'!$G$5:$G$43)</f>
+        <v>43</v>
       </c>
       <c r="E5" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D5/SUM($D$5:$D$8))</f>
-        <v>0.24</v>
+        <v>0.290540540540541</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>65</v>
+        <v>94</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>266</v>
+        <v>314</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A6)</f>
-        <v>17</v>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$43,A6)</f>
+        <v>3</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$36,A6,'Product Backlog'!$G$5:$G$36)</f>
-        <v>70</v>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$43,A6,'Product Backlog'!$G$5:$G$43)</f>
+        <v>13</v>
       </c>
       <c r="E6" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D6/SUM($D$5:$D$8))</f>
-        <v>0.56</v>
+        <v>0.0878378378378378</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>162</v>
+        <v>113</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>267</v>
+        <v>315</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A7)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$43,A7)</f>
+        <v>1</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$36,A7,'Product Backlog'!$G$5:$G$36)</f>
-        <v>22</v>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$43,A7,'Product Backlog'!$G$5:$G$43)</f>
+        <v>2</v>
       </c>
       <c r="E7" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D7/SUM($D$5:$D$8))</f>
-        <v>0.176</v>
+        <v>0.0135135135135135</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>182</v>
+        <v>120</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>268</v>
+        <v>316</v>
       </c>
       <c r="C8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$36,A8)</f>
-        <v>1</v>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$43,A8)</f>
+        <v>22</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$36,A8,'Product Backlog'!$G$5:$G$36)</f>
-        <v>3</v>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$43,A8,'Product Backlog'!$G$5:$G$43)</f>
+        <v>90</v>
       </c>
       <c r="E8" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D8/SUM($D$5:$D$8))</f>
-        <v>0.024</v>
+        <v>0.608108108108108</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>214</v>
+        <v>253</v>
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="D9" s="27" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>125</v>
+        <v>148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Quanto preciso no exame, tendência do último colocado, procura do curso e partilhar o plano (US40 a US43)
- Ficha do curso: nota necessária nas provas em falta (conjunto mais fácil, mínimos, aviso
  quando nem 200 chegam), último colocado 2023–2025 com «A subir/A descer/Estável» e procura
  em 2025 (candidatos, 1.ª opção, vagas, colocados).
- Plano: tendência em cada opção e «Precisa de X em Y» nas opções a que falta uma prova.
- Partilhar o plano: ligação só de leitura com código aleatório, sem email, média nem exames;
  «Deixar de partilhar» invalida-a. Coluna planos_candidatura.partilha (migração automática).
- Recolha da DGES: tabela de estatísticas da 1.ª fase (6 colunas novas no CSV).
- Backlog (US40–US43, Sprint 4 com 27 SP), requisitos RF44–RF47, documentação e registo de IA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jr1j7KW7k7X8nu4tsEr7G3
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Product Backlog'!$4:$4</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$43</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$47</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="504" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="338">
   <si>
     <t xml:space="preserve">Product Backlog — OptaBem (orientação de curso e candidatura)</t>
   </si>
@@ -418,6 +418,73 @@
     <t xml:space="preserve">23/10: story nova. Protótipo no PR #44 (rascunho), feito antes do sprint para o PO ver a ideia. O OptaBem não submete a candidatura: ajuda a prepará-la.</t>
   </si>
   <si>
+    <t xml:space="preserve">US40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quanto preciso no exame?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como candidato, quero saber que nota preciso nos exames que ainda não fiz para chegar ao último colocado de um curso, para saber quanto tenho de estudar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Na ficha do curso, com a média do secundário indicada.
+• Usa os exames já feitos e escolhe o conjunto de provas em que é mais fácil lá chegar.
+• Respeita o mínimo de cada prova; sem último colocado, usa a nota mínima do curso.
+• Diz quando nem 200 pontos chegam.
+• No plano, as opções a que falta uma prova mostram quanto precisa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23/10: story nova (ideia proposta pelo Claude e aceite pelo PO). Feita no PR #44 a pedido do PO, antes do sprint.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tendência do último colocado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como candidato, quero ver como a nota do último colocado mudou de 2023 a 2025, para perceber se um curso está a ficar mais difícil de entrar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Notas da 1.ª fase de 2023, 2024 e 2025 (DGES) na ficha do curso.
+• Etiqueta «A subir», «A descer» ou «Estável» (3 pontos de margem entre o primeiro e o último ano).
+• A etiqueta aparece também em cada opção do plano.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Procura do curso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como candidato, quero ver quantas pessoas concorreram a um curso e quantas o puseram em 1.ª opção, para perceber o risco da minha escolha.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Candidatos, candidatos em 1.ª opção, vagas e colocados da 1.ª fase de 2025 (DGES), na ficha do curso.
+• Etiqueta: «Sobraram vagas», «Muito procurado» (1,5 ou mais em 1.ª opção por vaga), «Procurado» (0,75 a 1,5) ou «Pouco escolhido em 1.ª opção».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partilhar o plano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como candidato, quero partilhar o meu plano com quem me ajuda a decidir (pais, explicador), com uma ligação só de leitura, para pedir opinião sem dar a minha palavra-passe.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Ligação com um código aleatório; quem a tem vê o plano sem iniciar sessão.
+• Mostra o primeiro nome, as opções, a nota de candidatura e a situação; nunca o email, a média nem os exames.
+• «Deixar de partilhar» invalida a ligação de imediato.
+• A página não é indexada pelos motores de pesquisa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Could</t>
+  </si>
+  <si>
+    <t xml:space="preserve">23/10: story nova (ideia proposta pelo Claude e aceite pelo PO). Feita no PR #44 a pedido do PO, antes do sprint. RGPD: a pessoa escolhe partilhar; política de privacidade provisória atualizada.</t>
+  </si>
+  <si>
     <t xml:space="preserve">US37</t>
   </si>
   <si>
@@ -473,9 +540,6 @@
   <si>
     <t xml:space="preserve">• Datas das 3 fases do concurso, com a ligação para a DGES.
 • O passo atual do percurso mostra o próximo prazo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Could</t>
   </si>
   <si>
     <t xml:space="preserve">23/10: story nova.</t>
@@ -924,10 +988,10 @@
     <t xml:space="preserve">US05, US17</t>
   </si>
   <si>
-    <t xml:space="preserve">Quem escolheu um curso prepara a candidatura: vê as condições de acesso, calcula a sua nota em cada curso e ordena as 6 opções; o catálogo passa a ter as licenciaturas da DGES (29/10 a 05/11; a confirmar com o docente).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US04, US33, US34, US35, US36</t>
+    <t xml:space="preserve">Quem escolheu um curso prepara a candidatura: vê as condições de acesso, a tendência e a procura de cada curso, calcula a sua nota e quanto precisa nos exames, ordena as 6 opções e pode partilhar o plano; o catálogo passa a ter as licenciaturas da DGES (29/10 a 05/11; a confirmar com o docente).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US04, US33–US36, US40–US43</t>
   </si>
   <si>
     <t xml:space="preserve">Fora desta release (entrega a 05/11). As stories das opcionais passam a Won't (fase 2) a 23/10: o plano de candidatura substitui-as.</t>
@@ -1099,6 +1163,15 @@
   </si>
   <si>
     <t xml:space="preserve">• A story do Sprint 4 tem de ser confirmada com o docente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• (23/10, mais tarde) Stories novas US40 a US43, propostas pelo Claude e aceites pelo PO: quanto preciso no exame, tendência do último colocado, procura do curso e partilhar o plano. Feitas no PR #44.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Atenção: com elas, o Sprint 4 fica com 27 SP planeados para uma velocidade de 10. Quase todo o código já está feito (protótipo), mas a documentação de cada story (requisitos, use case, BPMN) não. Se o docente achar demais, saem primeiro a US43 (Could) e depois a US36, US40, US41 e US42 (Should).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sem story: a gestão passa a ativar contas por confirmar, enquanto o site não envia emails reais (PR #43).</t>
   </si>
   <si>
     <t xml:space="preserve">Resumo por prioridade (MoSCoW)</t>
@@ -1843,7 +1916,7 @@
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>18</c:v>
+                  <c:v>27</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1945,11 +2018,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="57761804"/>
-        <c:axId val="79428830"/>
+        <c:axId val="60156413"/>
+        <c:axId val="87388493"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="57761804"/>
+        <c:axId val="60156413"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1980,7 +2053,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79428830"/>
+        <c:crossAx val="87388493"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1988,7 +2061,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="79428830"/>
+        <c:axId val="87388493"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2053,7 +2126,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="57761804"/>
+        <c:crossAx val="60156413"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2120,9 +2193,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2088720</xdr:colOff>
+      <xdr:colOff>2088360</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>85680</xdr:rowOff>
+      <xdr:rowOff>85320</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2131,7 +2204,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5753880" cy="2513520"/>
+        <a:ext cx="5753520" cy="2513160"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2324,7 +2397,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:M46"/>
+  <dimension ref="A1:M50"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
@@ -2918,20 +2991,20 @@
         <v>99</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>94</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="J18" s="7" t="s">
-        <v>101</v>
+        <v>71</v>
       </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="M18" s="5" t="s">
         <v>79</v>
@@ -2942,35 +3015,35 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="E19" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="F19" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="D19" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>107</v>
-      </c>
       <c r="G19" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>94</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="J19" s="7" t="s">
-        <v>101</v>
+        <v>71</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="M19" s="5" t="s">
         <v>79</v>
@@ -2981,35 +3054,35 @@
         <v>16</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>74</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G20" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="J20" s="7" t="s">
-        <v>101</v>
+        <v>71</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="M20" s="5" t="s">
         <v>79</v>
@@ -3020,38 +3093,38 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>116</v>
+        <v>74</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="G21" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="J21" s="7" t="s">
-        <v>101</v>
+        <v>71</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="M21" s="5" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3059,38 +3132,38 @@
         <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="C22" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D22" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="D22" s="6" t="s">
-        <v>123</v>
-      </c>
       <c r="E22" s="6" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H22" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="I22" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J22" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I22" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J22" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>115</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3098,38 +3171,38 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>61</v>
+        <v>123</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="G23" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H23" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="I23" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J23" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I23" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J23" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="M23" s="5" t="s">
-        <v>127</v>
+        <v>79</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3137,38 +3210,38 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>133</v>
+        <v>74</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H24" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="I24" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J24" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I24" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J24" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>132</v>
+        <v>79</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3176,38 +3249,38 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="G25" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H25" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="C25" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>140</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="G25" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H25" s="5" t="s">
+      <c r="I25" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J25" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J25" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>122</v>
+        <v>52</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3215,38 +3288,38 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>66</v>
+        <v>140</v>
       </c>
       <c r="C26" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="F26" s="6" t="s">
         <v>143</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="F26" s="6" t="s">
-        <v>146</v>
       </c>
       <c r="G26" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H26" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I26" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J26" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I26" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J26" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3254,38 +3327,38 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>133</v>
+        <v>61</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="H27" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I27" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J27" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I27" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J27" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3293,38 +3366,38 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
+        <v>150</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="E28" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="F28" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="D28" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>157</v>
-      </c>
       <c r="G28" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H28" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I28" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J28" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I28" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J28" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3332,38 +3405,38 @@
         <v>25</v>
       </c>
       <c r="B29" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>157</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="F29" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="C29" s="5" t="s">
-        <v>160</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>163</v>
-      </c>
       <c r="G29" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H29" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J29" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I29" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J29" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="M29" s="5" t="s">
-        <v>153</v>
+        <v>140</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3371,38 +3444,38 @@
         <v>26</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>158</v>
+        <v>66</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>143</v>
+        <v>161</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="G30" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H30" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I30" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J30" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I30" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J30" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3410,38 +3483,38 @@
         <v>27</v>
       </c>
       <c r="B31" s="5" t="s">
+        <v>167</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>151</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="F31" s="6" t="s">
         <v>170</v>
       </c>
-      <c r="C31" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>173</v>
-      </c>
       <c r="G31" s="7" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="H31" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I31" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J31" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I31" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J31" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K31" s="8"/>
       <c r="L31" s="8" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="M31" s="5" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3449,38 +3522,38 @@
         <v>28</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>116</v>
+        <v>172</v>
       </c>
       <c r="D32" s="6" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="F32" s="6" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="G32" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H32" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I32" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J32" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I32" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J32" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K32" s="8"/>
       <c r="L32" s="8" t="s">
-        <v>174</v>
+        <v>165</v>
       </c>
       <c r="M32" s="5" t="s">
-        <v>138</v>
+        <v>176</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3488,38 +3561,38 @@
         <v>29</v>
       </c>
       <c r="B33" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="E33" s="6" t="s">
         <v>180</v>
       </c>
-      <c r="C33" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="D33" s="6" t="s">
+      <c r="F33" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="E33" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>183</v>
-      </c>
       <c r="G33" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H33" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I33" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J33" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I33" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J33" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K33" s="8"/>
       <c r="L33" s="8" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="M33" s="5" t="s">
-        <v>185</v>
+        <v>171</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3527,38 +3600,38 @@
         <v>30</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>148</v>
+        <v>176</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="F34" s="6" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="G34" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H34" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I34" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J34" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I34" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J34" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K34" s="8"/>
       <c r="L34" s="8" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="M34" s="5" t="s">
-        <v>170</v>
+        <v>187</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3566,10 +3639,10 @@
         <v>31</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>169</v>
+        <v>188</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>154</v>
+        <v>123</v>
       </c>
       <c r="D35" s="6" t="s">
         <v>189</v>
@@ -3581,23 +3654,23 @@
         <v>191</v>
       </c>
       <c r="G35" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H35" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I35" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J35" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I35" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J35" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K35" s="8"/>
       <c r="L35" s="8" t="s">
         <v>192</v>
       </c>
       <c r="M35" s="5" t="s">
-        <v>159</v>
+        <v>193</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3605,10 +3678,10 @@
         <v>32</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>194</v>
+        <v>134</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>195</v>
@@ -3623,20 +3696,20 @@
         <v>3</v>
       </c>
       <c r="H36" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I36" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J36" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I36" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J36" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K36" s="8"/>
       <c r="L36" s="8" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="M36" s="5" t="s">
-        <v>199</v>
+        <v>156</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3644,38 +3717,38 @@
         <v>33</v>
       </c>
       <c r="B37" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D37" s="6" t="s">
         <v>199</v>
       </c>
-      <c r="C37" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="D37" s="6" t="s">
+      <c r="E37" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="E37" s="6" t="s">
+      <c r="F37" s="6" t="s">
         <v>201</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>202</v>
       </c>
       <c r="G37" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H37" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I37" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J37" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I37" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J37" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K37" s="8"/>
       <c r="L37" s="8" t="s">
+        <v>202</v>
+      </c>
+      <c r="M37" s="5" t="s">
         <v>203</v>
-      </c>
-      <c r="M37" s="5" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3683,10 +3756,10 @@
         <v>34</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>175</v>
+        <v>166</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="D38" s="6" t="s">
         <v>204</v>
@@ -3698,23 +3771,23 @@
         <v>206</v>
       </c>
       <c r="G38" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H38" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I38" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J38" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I38" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J38" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K38" s="8"/>
       <c r="L38" s="8" t="s">
-        <v>207</v>
+        <v>192</v>
       </c>
       <c r="M38" s="5" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3722,38 +3795,38 @@
         <v>35</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>104</v>
+        <v>172</v>
       </c>
       <c r="D39" s="6" t="s">
+        <v>207</v>
+      </c>
+      <c r="E39" s="6" t="s">
         <v>208</v>
       </c>
-      <c r="E39" s="6" t="s">
+      <c r="F39" s="6" t="s">
         <v>209</v>
       </c>
-      <c r="F39" s="6" t="s">
-        <v>210</v>
-      </c>
       <c r="G39" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H39" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I39" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J39" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I39" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J39" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K39" s="8"/>
       <c r="L39" s="8" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="M39" s="5" t="s">
-        <v>211</v>
+        <v>177</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3764,35 +3837,35 @@
         <v>211</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>194</v>
+        <v>212</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G40" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H40" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I40" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J40" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I40" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J40" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K40" s="8"/>
       <c r="L40" s="8" t="s">
-        <v>207</v>
+        <v>216</v>
       </c>
       <c r="M40" s="5" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3800,38 +3873,38 @@
         <v>37</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>154</v>
+        <v>172</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="E41" s="6" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="G41" s="7" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H41" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I41" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J41" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I41" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J41" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K41" s="8"/>
       <c r="L41" s="8" t="s">
-        <v>207</v>
+        <v>221</v>
       </c>
       <c r="M41" s="5" t="s">
-        <v>176</v>
+        <v>60</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3839,38 +3912,38 @@
         <v>38</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>219</v>
+        <v>193</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>104</v>
+        <v>178</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F42" s="6" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="G42" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H42" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I42" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J42" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="I42" s="7" t="s">
-        <v>100</v>
-      </c>
-      <c r="J42" s="7" t="s">
-        <v>101</v>
       </c>
       <c r="K42" s="8"/>
       <c r="L42" s="8" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="M42" s="5" t="s">
-        <v>219</v>
+        <v>198</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3878,62 +3951,218 @@
         <v>39</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>224</v>
+        <v>203</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>36</v>
+        <v>123</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F43" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="G43" s="7"/>
-      <c r="H43" s="5"/>
+        <v>228</v>
+      </c>
+      <c r="G43" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H43" s="5" t="s">
+        <v>138</v>
+      </c>
       <c r="I43" s="7" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="J43" s="7" t="s">
-        <v>228</v>
+        <v>120</v>
       </c>
       <c r="K43" s="8"/>
       <c r="L43" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="M43" s="5" t="s">
         <v>229</v>
       </c>
-      <c r="M43" s="5" t="s">
+    </row>
+    <row r="44" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="5" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>212</v>
+      </c>
+      <c r="D44" s="6" t="s">
+        <v>230</v>
+      </c>
+      <c r="E44" s="6" t="s">
+        <v>231</v>
+      </c>
+      <c r="F44" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="G44" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="H44" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I44" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J44" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="K44" s="8"/>
+      <c r="L44" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="M44" s="5" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="5" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="D45" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="E45" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="F45" s="6" t="s">
+        <v>236</v>
+      </c>
+      <c r="G45" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="H45" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I45" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J45" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="K45" s="8"/>
+      <c r="L45" s="8" t="s">
+        <v>225</v>
+      </c>
+      <c r="M45" s="5" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="C46" s="5" t="s">
+        <v>123</v>
+      </c>
+      <c r="D46" s="6" t="s">
+        <v>238</v>
+      </c>
+      <c r="E46" s="6" t="s">
+        <v>239</v>
+      </c>
+      <c r="F46" s="6" t="s">
+        <v>240</v>
+      </c>
+      <c r="G46" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H46" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="I46" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J46" s="7" t="s">
+        <v>120</v>
+      </c>
+      <c r="K46" s="8"/>
+      <c r="L46" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="M46" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="5" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D47" s="6" t="s">
+        <v>243</v>
+      </c>
+      <c r="E47" s="6" t="s">
+        <v>244</v>
+      </c>
+      <c r="F47" s="6" t="s">
+        <v>245</v>
+      </c>
+      <c r="G47" s="7"/>
+      <c r="H47" s="5"/>
+      <c r="I47" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="J47" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="K47" s="8"/>
+      <c r="L47" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="M47" s="5" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F44" s="9" t="s">
-        <v>230</v>
-      </c>
-      <c r="G44" s="9" t="n">
-        <f aca="false">SUM(G5:G43)</f>
-        <v>148</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F45" s="9" t="s">
-        <v>231</v>
-      </c>
-      <c r="G45" s="9" t="n">
-        <f aca="false">SUMIF(J5:J43,"Feito",G5:G43)</f>
+    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F48" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="G48" s="9" t="n">
+        <f aca="false">SUM(G5:G47)</f>
+        <v>157</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F49" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="G49" s="9" t="n">
+        <f aca="false">SUMIF(J5:J47,"Feito",G5:G47)</f>
         <v>30</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F46" s="10" t="s">
-        <v>232</v>
+    <row r="50" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F50" s="10" t="s">
+        <v>250</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:M43"/>
-  <conditionalFormatting sqref="J5:J43">
+  <autoFilter ref="A4:M47"/>
+  <conditionalFormatting sqref="J5:J47">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Feito"</formula>
     </cfRule>
@@ -3941,7 +4170,7 @@
       <formula>"Em curso"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H43">
+  <conditionalFormatting sqref="H5:H47">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Must"</formula>
     </cfRule>
@@ -3955,7 +4184,7 @@
       <formula>"Won't"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I43">
+  <conditionalFormatting sqref="I5:I47">
     <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Sprint 1"</formula>
     </cfRule>
@@ -3973,19 +4202,19 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G43" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G47" type="list">
       <formula1>"1,2,3,5,8,13,21"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H43" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H47" type="list">
       <formula1>"Must,Should,Could,Won't"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I43" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I47" type="list">
       <formula1>"Sprint 1,Sprint 2,Sprint 3,Sprint 4,Backlog"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J43" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J47" type="list">
       <formula1>"Por fazer,Em curso,Feito,Fundida"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4007,7 +4236,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H88"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -4022,17 +4251,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>233</v>
+        <v>251</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>234</v>
+        <v>252</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>235</v>
+        <v>253</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>10</v>
@@ -4043,25 +4272,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>236</v>
+        <v>254</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>237</v>
+        <v>255</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>238</v>
+        <v>256</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>239</v>
+        <v>257</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>240</v>
+        <v>258</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>241</v>
+        <v>259</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>242</v>
+        <v>260</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4069,17 +4298,17 @@
         <v>21</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>243</v>
+        <v>261</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>244</v>
+        <v>262</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$43,$A6,'Product Backlog'!$G$5:$G$43)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$47,$A6,'Product Backlog'!$G$5:$G$47)</f>
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$43,'Product Backlog'!$I$5:$I$43,$A6,'Product Backlog'!$J$5:$J$43,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$47,'Product Backlog'!$I$5:$I$47,$A6,'Product Backlog'!$J$5:$J$47,"Feito")</f>
         <v>10</v>
       </c>
       <c r="F6" s="15" t="n">
@@ -4091,7 +4320,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$43,$A6)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$47,$A6)</f>
         <v>3</v>
       </c>
     </row>
@@ -4100,17 +4329,17 @@
         <v>40</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>245</v>
+        <v>263</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>246</v>
+        <v>264</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$43,$A7,'Product Backlog'!$G$5:$G$43)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$47,$A7,'Product Backlog'!$G$5:$G$47)</f>
         <v>13</v>
       </c>
       <c r="E7" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$43,'Product Backlog'!$I$5:$I$43,$A7,'Product Backlog'!$J$5:$J$43,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$47,'Product Backlog'!$I$5:$I$47,$A7,'Product Backlog'!$J$5:$J$47,"Feito")</f>
         <v>13</v>
       </c>
       <c r="F7" s="15" t="n">
@@ -4122,7 +4351,7 @@
         <v>-3</v>
       </c>
       <c r="H7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$43,$A7)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$47,$A7)</f>
         <v>3</v>
       </c>
     </row>
@@ -4131,17 +4360,17 @@
         <v>57</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>247</v>
+        <v>265</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>248</v>
+        <v>266</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$43,$A8,'Product Backlog'!$G$5:$G$43)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$47,$A8,'Product Backlog'!$G$5:$G$47)</f>
         <v>7</v>
       </c>
       <c r="E8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$43,'Product Backlog'!$I$5:$I$43,$A8,'Product Backlog'!$J$5:$J$43,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$47,'Product Backlog'!$I$5:$I$47,$A8,'Product Backlog'!$J$5:$J$47,"Feito")</f>
         <v>7</v>
       </c>
       <c r="F8" s="15" t="n">
@@ -4153,7 +4382,7 @@
         <v>3</v>
       </c>
       <c r="H8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$43,$A8)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$47,$A8)</f>
         <v>2</v>
       </c>
     </row>
@@ -4162,17 +4391,17 @@
         <v>70</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>249</v>
+        <v>267</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>250</v>
+        <v>268</v>
       </c>
       <c r="D9" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$43,$A9,'Product Backlog'!$G$5:$G$43)</f>
-        <v>18</v>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$47,$A9,'Product Backlog'!$G$5:$G$47)</f>
+        <v>27</v>
       </c>
       <c r="E9" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$43,'Product Backlog'!$I$5:$I$43,$A9,'Product Backlog'!$J$5:$J$43,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$47,'Product Backlog'!$I$5:$I$47,$A9,'Product Backlog'!$J$5:$J$47,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F9" s="15" t="n">
@@ -4181,29 +4410,29 @@
       </c>
       <c r="G9" s="16" t="n">
         <f aca="false">$C$3-D9</f>
-        <v>-8</v>
+        <v>-17</v>
       </c>
       <c r="H9" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$43,$A9)</f>
-        <v>5</v>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$47,$A9)</f>
+        <v>9</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" s="14" t="s">
+        <v>269</v>
+      </c>
+      <c r="C10" s="14" t="s">
+        <v>270</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$47,$A10,'Product Backlog'!$G$5:$G$47)</f>
         <v>100</v>
       </c>
-      <c r="B10" s="14" t="s">
-        <v>251</v>
-      </c>
-      <c r="C10" s="14" t="s">
-        <v>252</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$43,$A10,'Product Backlog'!$G$5:$G$43)</f>
-        <v>100</v>
-      </c>
       <c r="E10" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$43,'Product Backlog'!$I$5:$I$43,$A10,'Product Backlog'!$J$5:$J$43,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$47,'Product Backlog'!$I$5:$I$47,$A10,'Product Backlog'!$J$5:$J$47,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F10" s="15" t="n">
@@ -4214,19 +4443,19 @@
         <v>34</v>
       </c>
       <c r="H10" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$43,$A10)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$47,$A10)</f>
         <v>26</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>253</v>
+        <v>271</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
       <c r="D11" s="21" t="n">
         <f aca="false">SUM(D6:D10)</f>
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="E11" s="21" t="n">
         <f aca="false">SUM(E6:E10)</f>
@@ -4234,282 +4463,297 @@
       </c>
       <c r="F11" s="22" t="n">
         <f aca="false">IF(D11=0,0,E11/D11)</f>
-        <v>0.202702702702703</v>
+        <v>0.191082802547771</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21" t="n">
         <f aca="false">SUM(H6:H10)</f>
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>254</v>
+        <v>272</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>255</v>
+        <v>273</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>256</v>
+        <v>274</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>257</v>
+        <v>275</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>258</v>
+        <v>276</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>259</v>
+        <v>277</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>260</v>
+        <v>278</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>261</v>
+        <v>279</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>262</v>
+        <v>280</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
-        <v>263</v>
+        <v>281</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>264</v>
+        <v>282</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
-        <v>265</v>
+        <v>283</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>266</v>
+        <v>284</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="24" t="s">
-        <v>267</v>
+        <v>285</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="24" t="s">
-        <v>268</v>
+        <v>286</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="24" t="s">
-        <v>269</v>
+        <v>287</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="23" t="s">
-        <v>270</v>
+        <v>288</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="24" t="s">
-        <v>271</v>
+        <v>289</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="24" t="s">
-        <v>272</v>
+        <v>290</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="24" t="s">
-        <v>273</v>
+        <v>291</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="24" t="s">
-        <v>274</v>
+        <v>292</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="23" t="s">
-        <v>275</v>
+        <v>293</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="24" t="s">
-        <v>276</v>
+        <v>294</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="24" t="s">
-        <v>277</v>
+        <v>295</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="24" t="s">
-        <v>278</v>
+        <v>296</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="24" t="s">
-        <v>279</v>
+        <v>297</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="24" t="s">
-        <v>280</v>
+        <v>298</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="24" t="s">
-        <v>281</v>
+        <v>299</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="23" t="s">
-        <v>282</v>
+        <v>300</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="24" t="s">
-        <v>283</v>
+        <v>301</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="24" t="s">
-        <v>284</v>
+        <v>302</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="24" t="s">
-        <v>285</v>
+        <v>303</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="24" t="s">
-        <v>286</v>
+        <v>304</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="23" t="s">
-        <v>287</v>
+        <v>305</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="24" t="s">
-        <v>288</v>
+        <v>306</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="24" t="s">
-        <v>289</v>
+        <v>307</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="24" t="s">
-        <v>290</v>
+        <v>308</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="24" t="s">
-        <v>291</v>
+        <v>309</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="24" t="s">
-        <v>292</v>
+        <v>310</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="24" t="s">
-        <v>293</v>
+        <v>311</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="23" t="s">
-        <v>294</v>
+        <v>312</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="24" t="s">
-        <v>295</v>
+        <v>313</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="24" t="s">
-        <v>296</v>
+        <v>314</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="24" t="s">
-        <v>297</v>
+        <v>315</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="24" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="23" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="24" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="24" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="24" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="24" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="24" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="24" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="24" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="24" t="s">
-        <v>307</v>
+        <v>325</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A89" s="24" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A90" s="24" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A91" s="24" t="s">
+        <v>328</v>
       </c>
     </row>
   </sheetData>
@@ -4542,24 +4786,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>308</v>
+        <v>329</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>309</v>
+        <v>330</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>310</v>
+        <v>331</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>242</v>
+        <v>260</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>311</v>
+        <v>332</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>312</v>
+        <v>333</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4567,19 +4811,19 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>313</v>
+        <v>334</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$43,A5)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$47,A5)</f>
         <v>12</v>
       </c>
       <c r="D5" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$43,A5,'Product Backlog'!$G$5:$G$43)</f>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$47,A5,'Product Backlog'!$G$5:$G$47)</f>
         <v>43</v>
       </c>
       <c r="E5" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D5/SUM($D$5:$D$8))</f>
-        <v>0.290540540540541</v>
+        <v>0.273885350318471</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4587,19 +4831,19 @@
         <v>94</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>314</v>
+        <v>335</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$43,A6)</f>
-        <v>3</v>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$47,A6)</f>
+        <v>6</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$43,A6,'Product Backlog'!$G$5:$G$43)</f>
-        <v>13</v>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$47,A6,'Product Backlog'!$G$5:$G$47)</f>
+        <v>19</v>
       </c>
       <c r="E6" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D6/SUM($D$5:$D$8))</f>
-        <v>0.0878378378378378</v>
+        <v>0.121019108280255</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4607,52 +4851,52 @@
         <v>113</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>315</v>
+        <v>336</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$43,A7)</f>
-        <v>1</v>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$47,A7)</f>
+        <v>2</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$43,A7,'Product Backlog'!$G$5:$G$43)</f>
-        <v>2</v>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$47,A7,'Product Backlog'!$G$5:$G$47)</f>
+        <v>5</v>
       </c>
       <c r="E7" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D7/SUM($D$5:$D$8))</f>
-        <v>0.0135135135135135</v>
+        <v>0.0318471337579618</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>120</v>
+        <v>138</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>316</v>
+        <v>337</v>
       </c>
       <c r="C8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$43,A8)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$47,A8)</f>
         <v>22</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$43,A8,'Product Backlog'!$G$5:$G$43)</f>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$47,A8,'Product Backlog'!$G$5:$G$47)</f>
         <v>90</v>
       </c>
       <c r="E8" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D8/SUM($D$5:$D$8))</f>
-        <v>0.608108108108108</v>
+        <v>0.573248407643312</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>253</v>
+        <v>271</v>
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="D9" s="27" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>148</v>
+        <v>157</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Que exames me abrem mais portas (US44) e plano B da 2.ª fase (US45)
- Plano: combinações de até 3 exames que dão para mais opções (só as mínimas; diz para que
  opções não dão e que exames já fez) e cursos das mesmas áreas com vagas na 2.ª fase de 2025
  a que a nota chegava.
- Recolha da DGES: vagas, colocados e último colocado da 2.ª fase (3 colunas novas no CSV).
- Backlog (US44, US45; Sprint 4 com 32 SP e nota sobre quando fecha um sprint), RF48 e RF49,
  documentação e registo de uso de IA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jr1j7KW7k7X8nu4tsEr7G3
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Product Backlog'!$4:$4</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$47</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$49</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="349">
   <si>
     <t xml:space="preserve">Product Backlog — OptaBem (orientação de curso e candidatura)</t>
   </si>
@@ -485,6 +485,35 @@
     <t xml:space="preserve">23/10: story nova (ideia proposta pelo Claude e aceite pelo PO). Feita no PR #44 a pedido do PO, antes do sprint. RGPD: a pessoa escolhe partilhar; política de privacidade provisória atualizada.</t>
   </si>
   <si>
+    <t xml:space="preserve">US44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Que exames me abrem mais portas?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como candidato, quero saber que combinação de exames nacionais me deixa concorrer a mais cursos do meu plano, para decidir que exames fazer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Combinações de até 3 exames, a partir dos conjuntos de provas das opções do plano (2 ou mais opções).
+• Mostra as 3 melhores: a que serve para mais opções primeiro, depois a com menos exames.
+• Diz para que opções não dá e que exames da combinação a pessoa já fez.
+• Matemática e Matemática A contam como o mesmo exame.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plano B: 2.ª fase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como candidato, quero ver cursos das áreas do meu plano que tiveram vagas na 2.ª fase e a que a minha nota chegava, para ter uma alternativa se não entrar na 1.ª fase.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Vagas, colocados e último colocado da 2.ª fase de 2025 (DGES).
+• Só cursos fora do plano, das mesmas áreas, onde a nota da pessoa chegava ao último colocado da 2.ª fase (ou, sem essa nota, onde sobraram vagas).
+• Aviso: as vagas da 2.ª fase são as que sobram da 1.ª e mudam todos os anos.</t>
+  </si>
+  <si>
     <t xml:space="preserve">US37</t>
   </si>
   <si>
@@ -988,10 +1017,10 @@
     <t xml:space="preserve">US05, US17</t>
   </si>
   <si>
-    <t xml:space="preserve">Quem escolheu um curso prepara a candidatura: vê as condições de acesso, a tendência e a procura de cada curso, calcula a sua nota e quanto precisa nos exames, ordena as 6 opções e pode partilhar o plano; o catálogo passa a ter as licenciaturas da DGES (29/10 a 05/11; a confirmar com o docente).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US04, US33–US36, US40–US43</t>
+    <t xml:space="preserve">Quem escolheu um curso prepara a candidatura: vê as condições de acesso, a tendência e a procura de cada curso, calcula a sua nota e quanto precisa nos exames, descobre que exames lhe abrem mais portas, ordena as 6 opções, tem um plano B para a 2.ª fase e pode partilhar o plano; o catálogo passa a ter as licenciaturas da DGES (29/10 a 05/11; a confirmar com o docente).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US04, US33–US36, US40–US45</t>
   </si>
   <si>
     <t xml:space="preserve">Fora desta release (entrega a 05/11). As stories das opcionais passam a Won't (fase 2) a 23/10: o plano de candidatura substitui-as.</t>
@@ -1172,6 +1201,15 @@
   </si>
   <si>
     <t xml:space="preserve">• Sem story: a gestão passa a ativar contas por confirmar, enquanto o site não envia emails reais (PR #43).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• (23/10, ao fim do dia) Stories novas US44 (que exames me abrem mais portas) e US45 (plano B: 2.ª fase), propostas pelo Claude e escolhidas pelo PO. Feitas no PR #44.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• O Sprint 4 fica com 32 SP planeados para uma velocidade de 10. Isto não é um planeamento realista em Scrum: o código foi feito antes do sprint, como protótipo. No Sprint Planning de 29/10, os PO e o docente decidem que stories entram; as restantes voltam ao Backlog com o código já feito.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Esclarecimento: o Sprint 4 ainda não começou (29/10 a 05/11). Um sprint fecha na Sprint Review, no fim do tempo marcado; aceitar um PR é o que faz uma story contar como Feita.</t>
   </si>
   <si>
     <t xml:space="preserve">Resumo por prioridade (MoSCoW)</t>
@@ -1916,7 +1954,7 @@
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>27</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2018,11 +2056,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="60156413"/>
-        <c:axId val="87388493"/>
+        <c:axId val="16294996"/>
+        <c:axId val="95851061"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="60156413"/>
+        <c:axId val="16294996"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2053,7 +2091,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87388493"/>
+        <c:crossAx val="95851061"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2061,7 +2099,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="87388493"/>
+        <c:axId val="95851061"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2126,7 +2164,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60156413"/>
+        <c:crossAx val="16294996"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2193,9 +2231,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2088360</xdr:colOff>
+      <xdr:colOff>2088000</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>85320</xdr:rowOff>
+      <xdr:rowOff>84960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2204,7 +2242,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5753520" cy="2513160"/>
+        <a:ext cx="5753160" cy="2512800"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2397,7 +2435,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:M50"/>
+  <dimension ref="A1:M52"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="4"/>
@@ -3153,14 +3191,14 @@
         <v>94</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>119</v>
+        <v>70</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>120</v>
+        <v>71</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
-        <v>121</v>
+        <v>100</v>
       </c>
       <c r="M22" s="5" t="s">
         <v>79</v>
@@ -3171,35 +3209,35 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
+        <v>119</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="F23" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="C23" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="F23" s="6" t="s">
-        <v>126</v>
-      </c>
       <c r="G23" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>94</v>
+        <v>113</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>119</v>
+        <v>70</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>120</v>
+        <v>71</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8" t="s">
-        <v>127</v>
+        <v>100</v>
       </c>
       <c r="M23" s="5" t="s">
         <v>79</v>
@@ -3210,35 +3248,35 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>74</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="M24" s="5" t="s">
         <v>79</v>
@@ -3249,38 +3287,38 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="E25" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="F25" s="6" t="s">
         <v>134</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>137</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>138</v>
+        <v>94</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>52</v>
+        <v>79</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3288,38 +3326,38 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>134</v>
+        <v>74</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>138</v>
+        <v>113</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>133</v>
+        <v>79</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3327,38 +3365,38 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="F27" s="6" t="s">
         <v>145</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>148</v>
       </c>
       <c r="G27" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>145</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3366,38 +3404,38 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="D28" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="E28" s="6" t="s">
         <v>150</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="F28" s="6" t="s">
         <v>151</v>
       </c>
-      <c r="D28" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="F28" s="6" t="s">
-        <v>154</v>
-      </c>
       <c r="G28" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3405,38 +3443,38 @@
         <v>25</v>
       </c>
       <c r="B29" s="5" t="s">
+        <v>153</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="F29" s="6" t="s">
         <v>156</v>
       </c>
-      <c r="C29" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>157</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>159</v>
-      </c>
       <c r="G29" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="M29" s="5" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3444,38 +3482,38 @@
         <v>26</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>66</v>
+        <v>158</v>
       </c>
       <c r="C30" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="D30" s="6" t="s">
+        <v>160</v>
+      </c>
+      <c r="E30" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="F30" s="6" t="s">
         <v>162</v>
       </c>
-      <c r="E30" s="6" t="s">
-        <v>163</v>
-      </c>
-      <c r="F30" s="6" t="s">
-        <v>164</v>
-      </c>
       <c r="G30" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I30" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K30" s="8"/>
       <c r="L30" s="8" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="M30" s="5" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3483,38 +3521,38 @@
         <v>27</v>
       </c>
       <c r="B31" s="5" t="s">
+        <v>164</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>142</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>165</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>166</v>
+      </c>
+      <c r="F31" s="6" t="s">
         <v>167</v>
       </c>
-      <c r="C31" s="5" t="s">
-        <v>151</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>168</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>169</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>170</v>
-      </c>
       <c r="G31" s="7" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K31" s="8"/>
       <c r="L31" s="8" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="M31" s="5" t="s">
-        <v>167</v>
+        <v>148</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3522,38 +3560,38 @@
         <v>28</v>
       </c>
       <c r="B32" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="D32" s="6" t="s">
+        <v>170</v>
+      </c>
+      <c r="E32" s="6" t="s">
         <v>171</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="F32" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="D32" s="6" t="s">
-        <v>173</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>174</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>175</v>
-      </c>
       <c r="G32" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K32" s="8"/>
       <c r="L32" s="8" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="M32" s="5" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3561,38 +3599,38 @@
         <v>29</v>
       </c>
       <c r="B33" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="C33" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>176</v>
+      </c>
+      <c r="E33" s="6" t="s">
         <v>177</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="F33" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="D33" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>180</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>181</v>
-      </c>
       <c r="G33" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I33" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K33" s="8"/>
       <c r="L33" s="8" t="s">
-        <v>182</v>
+        <v>173</v>
       </c>
       <c r="M33" s="5" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3600,38 +3638,38 @@
         <v>30</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>161</v>
+        <v>180</v>
       </c>
       <c r="D34" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="F34" s="6" t="s">
         <v>183</v>
       </c>
-      <c r="E34" s="6" t="s">
-        <v>184</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>185</v>
-      </c>
       <c r="G34" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I34" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J34" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K34" s="8"/>
       <c r="L34" s="8" t="s">
-        <v>186</v>
+        <v>173</v>
       </c>
       <c r="M34" s="5" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3639,38 +3677,38 @@
         <v>31</v>
       </c>
       <c r="B35" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="C35" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="D35" s="6" t="s">
+        <v>187</v>
+      </c>
+      <c r="E35" s="6" t="s">
         <v>188</v>
       </c>
-      <c r="C35" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="D35" s="6" t="s">
+      <c r="F35" s="6" t="s">
         <v>189</v>
       </c>
-      <c r="E35" s="6" t="s">
-        <v>190</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>191</v>
-      </c>
       <c r="G35" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I35" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J35" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K35" s="8"/>
       <c r="L35" s="8" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="M35" s="5" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3678,38 +3716,38 @@
         <v>32</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>134</v>
+        <v>169</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="G36" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I36" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J36" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K36" s="8"/>
       <c r="L36" s="8" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="M36" s="5" t="s">
-        <v>156</v>
+        <v>195</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3717,38 +3755,38 @@
         <v>33</v>
       </c>
       <c r="B37" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="C37" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>197</v>
+      </c>
+      <c r="E37" s="6" t="s">
         <v>198</v>
       </c>
-      <c r="C37" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="D37" s="6" t="s">
+      <c r="F37" s="6" t="s">
         <v>199</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>200</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>201</v>
       </c>
       <c r="G37" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I37" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J37" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K37" s="8"/>
       <c r="L37" s="8" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="M37" s="5" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3756,38 +3794,38 @@
         <v>34</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>166</v>
+        <v>202</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>172</v>
+        <v>142</v>
       </c>
       <c r="D38" s="6" t="s">
+        <v>203</v>
+      </c>
+      <c r="E38" s="6" t="s">
         <v>204</v>
       </c>
-      <c r="E38" s="6" t="s">
+      <c r="F38" s="6" t="s">
         <v>205</v>
       </c>
-      <c r="F38" s="6" t="s">
-        <v>206</v>
-      </c>
       <c r="G38" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H38" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I38" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J38" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K38" s="8"/>
       <c r="L38" s="8" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="M38" s="5" t="s">
-        <v>188</v>
+        <v>164</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3795,10 +3833,10 @@
         <v>35</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>187</v>
+        <v>206</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>172</v>
+        <v>131</v>
       </c>
       <c r="D39" s="6" t="s">
         <v>207</v>
@@ -3810,23 +3848,23 @@
         <v>209</v>
       </c>
       <c r="G39" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H39" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I39" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J39" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K39" s="8"/>
       <c r="L39" s="8" t="s">
         <v>210</v>
       </c>
       <c r="M39" s="5" t="s">
-        <v>177</v>
+        <v>211</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3834,38 +3872,38 @@
         <v>36</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>211</v>
+        <v>174</v>
       </c>
       <c r="C40" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D40" s="6" t="s">
         <v>212</v>
       </c>
-      <c r="D40" s="6" t="s">
+      <c r="E40" s="6" t="s">
         <v>213</v>
       </c>
-      <c r="E40" s="6" t="s">
+      <c r="F40" s="6" t="s">
         <v>214</v>
       </c>
-      <c r="F40" s="6" t="s">
-        <v>215</v>
-      </c>
       <c r="G40" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H40" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I40" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J40" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K40" s="8"/>
       <c r="L40" s="8" t="s">
-        <v>216</v>
+        <v>200</v>
       </c>
       <c r="M40" s="5" t="s">
-        <v>217</v>
+        <v>196</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3873,38 +3911,38 @@
         <v>37</v>
       </c>
       <c r="B41" s="5" t="s">
+        <v>195</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D41" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="E41" s="6" t="s">
+        <v>216</v>
+      </c>
+      <c r="F41" s="6" t="s">
         <v>217</v>
       </c>
-      <c r="C41" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>218</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>219</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>220</v>
-      </c>
       <c r="G41" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H41" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I41" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J41" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K41" s="8"/>
       <c r="L41" s="8" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="M41" s="5" t="s">
-        <v>60</v>
+        <v>185</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3912,38 +3950,38 @@
         <v>38</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>178</v>
+        <v>220</v>
       </c>
       <c r="D42" s="6" t="s">
+        <v>221</v>
+      </c>
+      <c r="E42" s="6" t="s">
         <v>222</v>
       </c>
-      <c r="E42" s="6" t="s">
+      <c r="F42" s="6" t="s">
         <v>223</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>224</v>
       </c>
       <c r="G42" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H42" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I42" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J42" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K42" s="8"/>
       <c r="L42" s="8" t="s">
+        <v>224</v>
+      </c>
+      <c r="M42" s="5" t="s">
         <v>225</v>
-      </c>
-      <c r="M42" s="5" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3951,10 +3989,10 @@
         <v>39</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>123</v>
+        <v>180</v>
       </c>
       <c r="D43" s="6" t="s">
         <v>226</v>
@@ -3969,20 +4007,20 @@
         <v>3</v>
       </c>
       <c r="H43" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I43" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J43" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K43" s="8"/>
       <c r="L43" s="8" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="M43" s="5" t="s">
-        <v>229</v>
+        <v>60</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3990,10 +4028,10 @@
         <v>40</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>229</v>
+        <v>201</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>212</v>
+        <v>186</v>
       </c>
       <c r="D44" s="6" t="s">
         <v>230</v>
@@ -4005,23 +4043,23 @@
         <v>232</v>
       </c>
       <c r="G44" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H44" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I44" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J44" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K44" s="8"/>
       <c r="L44" s="8" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="M44" s="5" t="s">
-        <v>233</v>
+        <v>206</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4029,10 +4067,10 @@
         <v>41</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>233</v>
+        <v>211</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>172</v>
+        <v>131</v>
       </c>
       <c r="D45" s="6" t="s">
         <v>234</v>
@@ -4044,23 +4082,23 @@
         <v>236</v>
       </c>
       <c r="G45" s="7" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="H45" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I45" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J45" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K45" s="8"/>
       <c r="L45" s="8" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="M45" s="5" t="s">
-        <v>194</v>
+        <v>237</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4071,7 +4109,7 @@
         <v>237</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>123</v>
+        <v>220</v>
       </c>
       <c r="D46" s="6" t="s">
         <v>238</v>
@@ -4083,23 +4121,23 @@
         <v>240</v>
       </c>
       <c r="G46" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H46" s="5" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="I46" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J46" s="7" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K46" s="8"/>
       <c r="L46" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="M46" s="5" t="s">
         <v>241</v>
-      </c>
-      <c r="M46" s="5" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4107,62 +4145,140 @@
         <v>43</v>
       </c>
       <c r="B47" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="C47" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="D47" s="6" t="s">
         <v>242</v>
       </c>
-      <c r="C47" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D47" s="6" t="s">
+      <c r="E47" s="6" t="s">
         <v>243</v>
       </c>
-      <c r="E47" s="6" t="s">
+      <c r="F47" s="6" t="s">
         <v>244</v>
       </c>
-      <c r="F47" s="6" t="s">
-        <v>245</v>
-      </c>
-      <c r="G47" s="7"/>
-      <c r="H47" s="5"/>
+      <c r="G47" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="H47" s="5" t="s">
+        <v>146</v>
+      </c>
       <c r="I47" s="7" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="J47" s="7" t="s">
-        <v>246</v>
+        <v>128</v>
       </c>
       <c r="K47" s="8"/>
       <c r="L47" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="M47" s="5" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="5" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="D48" s="6" t="s">
+        <v>246</v>
+      </c>
+      <c r="E48" s="6" t="s">
         <v>247</v>
       </c>
-      <c r="M47" s="5" t="s">
+      <c r="F48" s="6" t="s">
+        <v>248</v>
+      </c>
+      <c r="G48" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H48" s="5" t="s">
+        <v>146</v>
+      </c>
+      <c r="I48" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="J48" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="K48" s="8"/>
+      <c r="L48" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="M48" s="5" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="5" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D49" s="6" t="s">
+        <v>251</v>
+      </c>
+      <c r="E49" s="6" t="s">
+        <v>252</v>
+      </c>
+      <c r="F49" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="G49" s="7"/>
+      <c r="H49" s="5"/>
+      <c r="I49" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="J49" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="K49" s="8"/>
+      <c r="L49" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="M49" s="5" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F48" s="9" t="s">
-        <v>248</v>
-      </c>
-      <c r="G48" s="9" t="n">
-        <f aca="false">SUM(G5:G47)</f>
-        <v>157</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F49" s="9" t="s">
-        <v>249</v>
-      </c>
-      <c r="G49" s="9" t="n">
-        <f aca="false">SUMIF(J5:J47,"Feito",G5:G47)</f>
+    <row r="50" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F50" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="G50" s="9" t="n">
+        <f aca="false">SUM(G5:G49)</f>
+        <v>162</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F51" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="G51" s="9" t="n">
+        <f aca="false">SUMIF(J5:J49,"Feito",G5:G49)</f>
         <v>30</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F50" s="10" t="s">
-        <v>250</v>
+    <row r="52" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F52" s="10" t="s">
+        <v>258</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:M47"/>
-  <conditionalFormatting sqref="J5:J47">
+  <autoFilter ref="A4:M49"/>
+  <conditionalFormatting sqref="J5:J49">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Feito"</formula>
     </cfRule>
@@ -4170,7 +4286,7 @@
       <formula>"Em curso"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H47">
+  <conditionalFormatting sqref="H5:H49">
     <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Must"</formula>
     </cfRule>
@@ -4184,7 +4300,7 @@
       <formula>"Won't"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I47">
+  <conditionalFormatting sqref="I5:I49">
     <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Sprint 1"</formula>
     </cfRule>
@@ -4202,19 +4318,19 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G47" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G49" type="list">
       <formula1>"1,2,3,5,8,13,21"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H47" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H49" type="list">
       <formula1>"Must,Should,Could,Won't"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I47" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I49" type="list">
       <formula1>"Sprint 1,Sprint 2,Sprint 3,Sprint 4,Backlog"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J47" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J49" type="list">
       <formula1>"Por fazer,Em curso,Feito,Fundida"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -4236,7 +4352,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H91"/>
+  <dimension ref="A1:H94"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -4251,17 +4367,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>251</v>
+        <v>259</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>252</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>253</v>
+        <v>261</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>10</v>
@@ -4272,25 +4388,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>254</v>
+        <v>262</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>255</v>
+        <v>263</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>256</v>
+        <v>264</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>257</v>
+        <v>265</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>258</v>
+        <v>266</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>259</v>
+        <v>267</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4298,17 +4414,17 @@
         <v>21</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>261</v>
+        <v>269</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$47,$A6,'Product Backlog'!$G$5:$G$47)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$49,$A6,'Product Backlog'!$G$5:$G$49)</f>
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$47,'Product Backlog'!$I$5:$I$47,$A6,'Product Backlog'!$J$5:$J$47,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$49,'Product Backlog'!$I$5:$I$49,$A6,'Product Backlog'!$J$5:$J$49,"Feito")</f>
         <v>10</v>
       </c>
       <c r="F6" s="15" t="n">
@@ -4320,7 +4436,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$47,$A6)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$49,$A6)</f>
         <v>3</v>
       </c>
     </row>
@@ -4329,17 +4445,17 @@
         <v>40</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>263</v>
+        <v>271</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>264</v>
+        <v>272</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$47,$A7,'Product Backlog'!$G$5:$G$47)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$49,$A7,'Product Backlog'!$G$5:$G$49)</f>
         <v>13</v>
       </c>
       <c r="E7" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$47,'Product Backlog'!$I$5:$I$47,$A7,'Product Backlog'!$J$5:$J$47,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$49,'Product Backlog'!$I$5:$I$49,$A7,'Product Backlog'!$J$5:$J$49,"Feito")</f>
         <v>13</v>
       </c>
       <c r="F7" s="15" t="n">
@@ -4351,7 +4467,7 @@
         <v>-3</v>
       </c>
       <c r="H7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$47,$A7)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$49,$A7)</f>
         <v>3</v>
       </c>
     </row>
@@ -4360,17 +4476,17 @@
         <v>57</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>265</v>
+        <v>273</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$47,$A8,'Product Backlog'!$G$5:$G$47)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$49,$A8,'Product Backlog'!$G$5:$G$49)</f>
         <v>7</v>
       </c>
       <c r="E8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$47,'Product Backlog'!$I$5:$I$47,$A8,'Product Backlog'!$J$5:$J$47,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$49,'Product Backlog'!$I$5:$I$49,$A8,'Product Backlog'!$J$5:$J$49,"Feito")</f>
         <v>7</v>
       </c>
       <c r="F8" s="15" t="n">
@@ -4382,7 +4498,7 @@
         <v>3</v>
       </c>
       <c r="H8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$47,$A8)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$49,$A8)</f>
         <v>2</v>
       </c>
     </row>
@@ -4391,17 +4507,17 @@
         <v>70</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>267</v>
+        <v>275</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="D9" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$47,$A9,'Product Backlog'!$G$5:$G$47)</f>
-        <v>27</v>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$49,$A9,'Product Backlog'!$G$5:$G$49)</f>
+        <v>32</v>
       </c>
       <c r="E9" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$47,'Product Backlog'!$I$5:$I$47,$A9,'Product Backlog'!$J$5:$J$47,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$49,'Product Backlog'!$I$5:$I$49,$A9,'Product Backlog'!$J$5:$J$49,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F9" s="15" t="n">
@@ -4410,29 +4526,29 @@
       </c>
       <c r="G9" s="16" t="n">
         <f aca="false">$C$3-D9</f>
-        <v>-17</v>
+        <v>-22</v>
       </c>
       <c r="H9" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$47,$A9)</f>
-        <v>9</v>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$49,$A9)</f>
+        <v>11</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>270</v>
+        <v>278</v>
       </c>
       <c r="D10" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$47,$A10,'Product Backlog'!$G$5:$G$47)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$49,$A10,'Product Backlog'!$G$5:$G$49)</f>
         <v>100</v>
       </c>
       <c r="E10" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$47,'Product Backlog'!$I$5:$I$47,$A10,'Product Backlog'!$J$5:$J$47,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$49,'Product Backlog'!$I$5:$I$49,$A10,'Product Backlog'!$J$5:$J$49,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F10" s="15" t="n">
@@ -4443,19 +4559,19 @@
         <v>34</v>
       </c>
       <c r="H10" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$47,$A10)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$49,$A10)</f>
         <v>26</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
       <c r="D11" s="21" t="n">
         <f aca="false">SUM(D6:D10)</f>
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="E11" s="21" t="n">
         <f aca="false">SUM(E6:E10)</f>
@@ -4463,297 +4579,312 @@
       </c>
       <c r="F11" s="22" t="n">
         <f aca="false">IF(D11=0,0,E11/D11)</f>
-        <v>0.191082802547771</v>
+        <v>0.185185185185185</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21" t="n">
         <f aca="false">SUM(H6:H10)</f>
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>273</v>
+        <v>281</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>274</v>
+        <v>282</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>275</v>
+        <v>283</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>276</v>
+        <v>284</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>277</v>
+        <v>285</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>278</v>
+        <v>286</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>279</v>
+        <v>287</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>280</v>
+        <v>288</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
-        <v>281</v>
+        <v>289</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>282</v>
+        <v>290</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>284</v>
+        <v>292</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="24" t="s">
-        <v>285</v>
+        <v>293</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="24" t="s">
-        <v>286</v>
+        <v>294</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="24" t="s">
-        <v>287</v>
+        <v>295</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="23" t="s">
-        <v>288</v>
+        <v>296</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="24" t="s">
-        <v>289</v>
+        <v>297</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="24" t="s">
-        <v>290</v>
+        <v>298</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="24" t="s">
-        <v>291</v>
+        <v>299</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="24" t="s">
-        <v>292</v>
+        <v>300</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="23" t="s">
-        <v>293</v>
+        <v>301</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="24" t="s">
-        <v>294</v>
+        <v>302</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="24" t="s">
-        <v>295</v>
+        <v>303</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="24" t="s">
-        <v>296</v>
+        <v>304</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="24" t="s">
-        <v>297</v>
+        <v>305</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="24" t="s">
-        <v>298</v>
+        <v>306</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="24" t="s">
-        <v>299</v>
+        <v>307</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="23" t="s">
-        <v>300</v>
+        <v>308</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="24" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="24" t="s">
-        <v>302</v>
+        <v>310</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="24" t="s">
-        <v>303</v>
+        <v>311</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="24" t="s">
-        <v>304</v>
+        <v>312</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="23" t="s">
-        <v>305</v>
+        <v>313</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="24" t="s">
-        <v>306</v>
+        <v>314</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="24" t="s">
-        <v>307</v>
+        <v>315</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="24" t="s">
-        <v>308</v>
+        <v>316</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="24" t="s">
-        <v>309</v>
+        <v>317</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="24" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="24" t="s">
-        <v>311</v>
+        <v>319</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="23" t="s">
-        <v>312</v>
+        <v>320</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="24" t="s">
-        <v>313</v>
+        <v>321</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="24" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="24" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="24" t="s">
-        <v>316</v>
+        <v>324</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="23" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="24" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="24" t="s">
-        <v>319</v>
+        <v>327</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="24" t="s">
-        <v>320</v>
+        <v>328</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="24" t="s">
-        <v>321</v>
+        <v>329</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="24" t="s">
-        <v>322</v>
+        <v>330</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="24" t="s">
-        <v>323</v>
+        <v>331</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="24" t="s">
-        <v>324</v>
+        <v>332</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="24" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="24" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="24" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="24" t="s">
-        <v>328</v>
+        <v>336</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A92" s="24" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A93" s="24" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A94" s="24" t="s">
+        <v>339</v>
       </c>
     </row>
   </sheetData>
@@ -4786,24 +4917,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>329</v>
+        <v>340</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>330</v>
+        <v>341</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>331</v>
+        <v>342</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>260</v>
+        <v>268</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>332</v>
+        <v>343</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>333</v>
+        <v>344</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4811,19 +4942,19 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>334</v>
+        <v>345</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$47,A5)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$49,A5)</f>
         <v>12</v>
       </c>
       <c r="D5" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$47,A5,'Product Backlog'!$G$5:$G$47)</f>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$49,A5,'Product Backlog'!$G$5:$G$49)</f>
         <v>43</v>
       </c>
       <c r="E5" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D5/SUM($D$5:$D$8))</f>
-        <v>0.273885350318471</v>
+        <v>0.265432098765432</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4831,19 +4962,19 @@
         <v>94</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>335</v>
+        <v>346</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$47,A6)</f>
-        <v>6</v>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$49,A6)</f>
+        <v>7</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$47,A6,'Product Backlog'!$G$5:$G$47)</f>
-        <v>19</v>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$49,A6,'Product Backlog'!$G$5:$G$49)</f>
+        <v>22</v>
       </c>
       <c r="E6" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D6/SUM($D$5:$D$8))</f>
-        <v>0.121019108280255</v>
+        <v>0.135802469135802</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4851,52 +4982,52 @@
         <v>113</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>336</v>
+        <v>347</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$47,A7)</f>
-        <v>2</v>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$49,A7)</f>
+        <v>3</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$47,A7,'Product Backlog'!$G$5:$G$47)</f>
-        <v>5</v>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$49,A7,'Product Backlog'!$G$5:$G$49)</f>
+        <v>7</v>
       </c>
       <c r="E7" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D7/SUM($D$5:$D$8))</f>
-        <v>0.0318471337579618</v>
+        <v>0.0432098765432099</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>337</v>
+        <v>348</v>
       </c>
       <c r="C8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$47,A8)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$49,A8)</f>
         <v>22</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$47,A8,'Product Backlog'!$G$5:$G$47)</f>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$49,A8,'Product Backlog'!$G$5:$G$49)</f>
         <v>90</v>
       </c>
       <c r="E8" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D8/SUM($D$5:$D$8))</f>
-        <v>0.573248407643312</v>
+        <v>0.555555555555556</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>271</v>
+        <v>279</v>
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D9" s="27" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Backlog reestruturado para um recomendador de cursos (autorizado pelo docente, 27/10)
- Product Backlog só com o recomendador de cursos: 24 stories, épicos E1 a E4,
  notas curtas, estado novo «Protótipo» (código feito antes do sprint).
- As 22 stories das opcionais e a US32 (fundida) passam para a folha
  «Arquivo (opcionais)», com o motivo de cada uma.
- Sprint 4 com o essencial: US04 e US33 a US36 (18 SP). As US40 a US45
  voltam ao backlog com o código pronto (PR #44).
- Stories novas: US46 (exportar os meus dados) e US47 (recuperar a
  palavra-passe).
- Requisitos 1.9: requisitos das opcionais no anexo A; RF50, RN11 e ponto 16
  novos; RNF03 a RNF08 sem o motor de opcionais.
- Visão 1.2, PROJETO.md, épico das US29 a US31, 02 e 03 alinhados;
  registo de uso de IA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VGMz7jsnoKnqj32HjKSCN6
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -11,10 +11,12 @@
     <sheet name="Product Backlog" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Plano de sprints" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Resumo MoSCoW" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Arquivo (opcionais)" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
+    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Arquivo (opcionais)'!$A$4:$H$27</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Product Backlog'!$4:$4</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$49</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$28</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -82,12 +84,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="349">
-  <si>
-    <t xml:space="preserve">Product Backlog — OptaBem (orientação de curso e candidatura)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ordenado pela ordem de trabalho (sprint e prioridade). Células a amarelo são para a equipa atualizar (Sprint, Estado, Responsável, SP, Notas). Replaneado a 14/10/2026 com a velocidade real (10 SP por sprint) e a decisão de o LLM conduzir a orientação (ver folha «Plano de sprints»). A partir de 13/10 os IDs não mudam. Replaneado a 23/10/2026: o plano de candidatura substitui as opcionais, que passam a Won't (fase 2).</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="376">
+  <si>
+    <t xml:space="preserve">Product Backlog — OptaBem (recomendador de cursos e plano de candidatura)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ordenado pela ordem de trabalho (sprint e prioridade). Células a amarelo são para a equipa atualizar (Sprint, Estado, Responsável, SP, Notas). Reestruturado a 27/10/2026, com autorização do docente: o backlog passa a ser só o de um recomendador de cursos; as stories das opcionais estão na folha «Arquivo (opcionais)». Os IDs não mudam nem são reutilizados. Estado «Protótipo» = código feito antes do sprint, ainda não aceite numa Sprint Review. Épicos: E1 Conta e privacidade · E2 Catálogo de cursos · E3 Orientação com o assistente · E4 Plano de candidatura. O histórico de replaneamentos está na folha «Plano de sprints».</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -156,7 +158,7 @@
     <t xml:space="preserve">Feito</t>
   </si>
   <si>
-    <t xml:space="preserve">Código, testes e documentação no GitHub (PR #1 a #3 aceites). 23/10: o registo pede também o nome, e o OptaBem trata a pessoa por ele (PR #43; RF01.17 e RF01.18).</t>
+    <t xml:space="preserve">Feita no Sprint 1 (PR #1 a #3). Desde 23/10 o registo pede também o nome (PR #43). docs/US01/.</t>
   </si>
   <si>
     <t xml:space="preserve">US02</t>
@@ -174,7 +176,7 @@
 • Páginas privadas redirecionam para o login.</t>
   </si>
   <si>
-    <t xml:space="preserve">Código, testes e documentação no GitHub (PR #4 e #5 aceites, com o ícone para mostrar a palavra-passe). 23/10: texto da story sem «avaliações e recomendações» (eram das opcionais). Terminar sessão passa a voltar à página inicial (PR #43).</t>
+    <t xml:space="preserve">Feita no Sprint 1 (PR #4 e #5). Terminar sessão volta à página inicial (PR #43). docs/US02/.</t>
   </si>
   <si>
     <t xml:space="preserve">US03</t>
@@ -193,7 +195,7 @@
 • Um administrador cria e remove outros administradores (não a si próprio).</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: story nova (o RF04 não tinha story). Revista pelos PO: administradores independentes e área escondida (3 → 5 SP). Código, testes e documentação no GitHub (PR #7 aceite). Revisão de 14/10 (PO): um só início de sessão para alunos e administradores, com os padrões Strategy, Chain of Responsibility e Factory (app/auth/perfis.py, PR #14).</t>
+    <t xml:space="preserve">Feita no Sprint 1 (PR #7). Um só início de sessão desde 14/10, com Strategy, Chain of Responsibility e Factory (PR #14). A gestão ativa contas por confirmar (PR #43). docs/US03/.</t>
   </si>
   <si>
     <t xml:space="preserve">—</t>
@@ -202,7 +204,7 @@
     <t xml:space="preserve">US29</t>
   </si>
   <si>
-    <t xml:space="preserve">E11</t>
+    <t xml:space="preserve">E3</t>
   </si>
   <si>
     <t xml:space="preserve">Conversa de orientação com o LLM</t>
@@ -222,7 +224,7 @@
     <t xml:space="preserve">Sprint 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: story nova (questionário de perguntas fixas). 14/10: reescrita por decisão do PO — as perguntas deixam de ser fixas e o LLM conduz a conversa; absorve a US32. 3 → 5 SP (página de conversa, estado entre pedidos, erros do fornecedor). Base técnica feita no spike (PR #17: app/llm, app/orientacao). Antes de começar: decisão do PO sobre idade e plano do Gemini (docs/geral/05-spike-llm.md, secção 5). Atenção: a conversa não cabe no cookie de sessão (4 KB); tem de ficar no servidor. 14/10: feita antes do Sprint 2 por decisão do PO (PR #19), à espera de revisão; docs/US29/. 22/10: aceite na Sprint Review do Sprint 2 (percurso completo testado pelos PO com o Gemini real, também noutro computador); fica Feito.</t>
+    <t xml:space="preserve">Feita no Sprint 2 (PR #19 e #24). Absorveu a US32 a 14/10 (issue #15). Gemini, com Groq de reserva (spike, PR #17). docs/US29/.</t>
   </si>
   <si>
     <t xml:space="preserve">US30</t>
@@ -241,7 +243,7 @@
 • Os testes usam o LLM falso, incluindo respostas com cursos inventados.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: story nova (sugestão a partir do questionário). 14/10: passa a ser o fim da conversa da US29 e passa do Sprint 3 para o Sprint 2 (decisão do PO). 8 → 3 SP: o fornecedor configurável, a validação contra o catálogo e os testes sem rede foram feitos no spike (PR #17). 22/10: aceite na Sprint Review do Sprint 2 (percurso completo testado pelos PO com o Gemini real, também noutro computador); fica Feito.</t>
+    <t xml:space="preserve">Feita no Sprint 2 (PR #22 e #23). docs/US30/.</t>
   </si>
   <si>
     <t xml:space="preserve">US31</t>
@@ -260,7 +262,7 @@
 • O utilizador pode mudar de curso, o que cria uma nova decisão.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: story nova (nova visão do produto, sugestão do docente). 14/10: mantém-se no Sprint 3; a escolha parte das sugestões da US30. 20/10 (Sprint Planning): antecipada para o Sprint 2, porque a US29 e a US30 foram feitas antes de o sprint começar; é ela que dá sentido às sugestões. 20/10: feita (PR da US31, à espera de revisão); docs/US31/, issue #27. Depois de escolher, a conversa com o LLM é apagada (ponto 15, decisão do PO). 22/10: aceite na Sprint Review do Sprint 2 (percurso completo testado pelos PO com o Gemini real, também noutro computador); fica Feito. 23/10: «As minhas decisões» sai do menu (decisão do PO); continua acessível pelo início e por «A minha conta».</t>
+    <t xml:space="preserve">Feita no Sprint 2 (issue #27). Depois da escolha, a conversa com o LLM é apagada. Fora do menu desde 23/10 (continua no início e em «A minha conta»). docs/US31/.</t>
   </si>
   <si>
     <t xml:space="preserve">US05</t>
@@ -284,16 +286,13 @@
     <t xml:space="preserve">Sprint 3</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa de opcionais para cursos (nova visão); 3 → 5 SP. A consulta de opcionais fica na US11. 14/10: trabalho antecipado no PR #14 — pesquisa de cursos reais na página de apresentação (app/catalogo/, dados da DGES lidos do CSV). Falta: filtros por área/instituição/localidade, ficha completa do curso e comparação de até 3 cursos. 14/10: Sprint 2 → Sprint 3, para o LLM entrar no Sprint 2 com a velocidade real (10 SP). 20/10: estado volta a «Por fazer» (não fica trabalho em curso num sprint que ainda não começou); a pesquisa de 14/10 e a página /cursos/ (US30) contam como parte já entregue. 22/10 (Sprint Planning do Sprint 3): entra no Sprint 3 com a US17. 22/10: feita (PR da US05, à espera de revisão): filtros, ficha completa e comparação de até 3 cursos; docs/US05/, issue #12. 23/10: aceite na Sprint Review do Sprint 3 (testada pelos PO); fica Feito.</t>
+    <t xml:space="preserve">Feita no Sprint 3 (PR #37, #38 e #42). docs/US05/.</t>
   </si>
   <si>
     <t xml:space="preserve">US04</t>
   </si>
   <si>
     <t xml:space="preserve">US17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E4</t>
   </si>
   <si>
     <t xml:space="preserve">Apagar a minha conta</t>
@@ -307,7 +306,7 @@
 • A sessão termina e a página confirma que os dados foram apagados.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). 22/10 (Sprint Planning do Sprint 3): Backlog → Sprint 3, Should → Must. O OptaBem já guarda conversas e decisões de pessoas, por isso exportar e apagar os dados passa a ser essencial (RGPD). 22/10 (decisão do PO): âmbito reduzido ao apagamento da conta; a exportação fica no backlog (RF17). 3 → 2 SP. Feita (PR da US17, à espera de revisão); docs/US17/, issue #34. 23/10: aceite na Sprint Review do Sprint 3 (testada pelos PO); fica Feito.</t>
+    <t xml:space="preserve">Feita no Sprint 3 (PR #39). Âmbito reduzido a 22/10: a exportação passou a ser a US46. docs/US17/.</t>
   </si>
   <si>
     <t xml:space="preserve">US10</t>
@@ -329,16 +328,16 @@
     <t xml:space="preserve">Sprint 4</t>
   </si>
   <si>
-    <t xml:space="preserve">Em curso</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: passa a importar instituições e cursos (nova visão). As UCs de cada curso entram com a US06. 14/10: Sprint 2 → Backlog, Must → Should: a aplicação já lê o catálogo do CSV (app/catalogo) e o LLM trabalha sobre ele; importar para a base de dados não muda nada para o utilizador nesta release. 22/10: candidata ao Sprint 4 se houver folga. 23/10: reescrita por decisão do PO. Em vez de o administrador importar um CSV, o catálogo vem da DGES por recolha (sugestão de um colega). Ramo feature/US04-catalogo-completo: 174 cursos recolhidos, falta a recolha completa e a documentação. Backlog → Sprint 4, Should → Must; a confirmar com o docente.</t>
+    <t xml:space="preserve">Protótipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protótipo no ramo feature/US04-catalogo-completo, incluído no PR #44: 174 cursos com condições de acesso. Falta a recolha completa e a documentação. Reescrita a 23/10 (antes: importar um CSV na gestão).</t>
   </si>
   <si>
     <t xml:space="preserve">US33</t>
   </si>
   <si>
-    <t xml:space="preserve">E12</t>
+    <t xml:space="preserve">E4</t>
   </si>
   <si>
     <t xml:space="preserve">Condições de acesso na ficha do curso</t>
@@ -354,7 +353,7 @@
 • Funciona sem sessão iniciada.</t>
   </si>
   <si>
-    <t xml:space="preserve">23/10: story nova (decisão do PO: o plano de candidatura substitui as opcionais). Protótipo no PR #44 (rascunho), feito antes do sprint para o PO ver a ideia.</t>
+    <t xml:space="preserve">Protótipo no PR #44, feito antes do sprint (23/10). Falta a documentação da story (requisitos, use case, BPMN).</t>
   </si>
   <si>
     <t xml:space="preserve">nova</t>
@@ -375,7 +374,7 @@
 • Matemática e Matemática A contam com o mesmo exame (a confirmar pela equipa na DGES).</t>
   </si>
   <si>
-    <t xml:space="preserve">23/10: story nova. Protótipo no PR #44 (rascunho), feito antes do sprint para o PO ver a ideia.</t>
+    <t xml:space="preserve">Protótipo no PR #44, feito antes do sprint (23/10). Falta a documentação da story (requisitos, use case, BPMN). A equipa confirma na DGES se Matemática e Matemática A contam como o mesmo exame.</t>
   </si>
   <si>
     <t xml:space="preserve">US35</t>
@@ -393,7 +392,7 @@
 • Aviso visível: estimativa para o contingente geral da 1.ª fase, não uma garantia.</t>
   </si>
   <si>
-    <t xml:space="preserve">23/10: story nova. Protótipo no PR #44 (rascunho), feito antes do sprint para o PO ver a ideia. Contas em funções puras (app/candidatura/calculos.py).</t>
+    <t xml:space="preserve">Protótipo no PR #44, feito antes do sprint (23/10). Falta a documentação da story (requisitos, use case, BPMN). Contas em app/candidatura/calculos.py.</t>
   </si>
   <si>
     <t xml:space="preserve">US36</t>
@@ -415,7 +414,7 @@
     <t xml:space="preserve">Should</t>
   </si>
   <si>
-    <t xml:space="preserve">23/10: story nova. Protótipo no PR #44 (rascunho), feito antes do sprint para o PO ver a ideia. O OptaBem não submete a candidatura: ajuda a prepará-la.</t>
+    <t xml:space="preserve">Protótipo no PR #44, feito antes do sprint (23/10). Falta a documentação da story (requisitos, use case, BPMN). O OptaBem ajuda a preparar a candidatura, não a submete. Se o Sprint 4 for demais, é a primeira a sair.</t>
   </si>
   <si>
     <t xml:space="preserve">US40</t>
@@ -434,7 +433,10 @@
 • No plano, as opções a que falta uma prova mostram quanto precisa.</t>
   </si>
   <si>
-    <t xml:space="preserve">23/10: story nova (ideia proposta pelo Claude e aceite pelo PO). Feita no PR #44 a pedido do PO, antes do sprint.</t>
+    <t xml:space="preserve">Backlog</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Código pronto no PR #44 (protótipo de 23/10, ideia proposta pelo Claude e aceite pelo PO). Fica no backlog porque o Sprint 4 já passa a velocidade; é aceite numa Sprint Review se houver folga.</t>
   </si>
   <si>
     <t xml:space="preserve">US41</t>
@@ -462,6 +464,93 @@
   <si>
     <t xml:space="preserve">• Candidatos, candidatos em 1.ª opção, vagas e colocados da 1.ª fase de 2025 (DGES), na ficha do curso.
 • Etiqueta: «Sobraram vagas», «Muito procurado» (1,5 ou mais em 1.ª opção por vaga), «Procurado» (0,75 a 1,5) ou «Pouco escolhido em 1.ª opção».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Que exames me abrem mais portas?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como candidato, quero saber que combinação de exames nacionais me deixa concorrer a mais cursos do meu plano, para decidir que exames fazer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Combinações de até 3 exames, a partir dos conjuntos de provas das opções do plano (2 ou mais opções).
+• Mostra as 3 melhores: a que serve para mais opções primeiro, depois a com menos exames.
+• Diz para que opções não dá e que exames da combinação a pessoa já fez.
+• Matemática e Matemática A contam como o mesmo exame.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assistente que conhece as minhas notas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como pessoa indecisa, quero que o assistente tenha em conta as provas que fiz e a minha nota, para não me sugerir cursos a que não posso concorrer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Só com autorização da pessoa, o LLM recebe as provas feitas e um intervalo de nota (nunca a média exata, RNF12).
+• Cursos a que falta uma prova não são sugeridos, ou vêm assinalados.
+• Os testes usam o LLM falso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Por fazer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Os termos do Gemini excluem menores de 18, e muitos candidatos têm 17 anos (ponto 14 dos requisitos).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exportar os meus dados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como utilizador, quero descarregar todos os dados que o OptaBem guarda sobre mim, para exercer o meu direito de acesso e de portabilidade.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Ficheiro JSON com a conta (sem a palavra-passe), as decisões do percurso, as notas e o plano de candidatura.
+• Pede a palavra-passe antes de descarregar.
+• Nunca inclui dados de outros utilizadores.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27/10: story nova, com a parte do RF17 que saiu da US17 a 22/10 (RNF01, RGPD).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US47</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recuperar a palavra-passe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como utilizador que se esqueceu da palavra-passe, quero receber uma ligação para definir uma nova, para não perder a conta.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Ligação de uso único, que expira ao fim de 1 hora.
+• A mensagem é a mesma quer a conta exista quer não.
+• Depois de mudar a palavra-passe, as sessões abertas terminam.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27/10: story nova, para a parte do RF02 que não tinha story. Precisa de o site enviar emails reais (hoje não envia).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US39</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corrigir e esconder cursos do catálogo (gestão)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como administrador, quero corrigir a descrição e as saídas profissionais de um curso, ou escondê-lo, para o catálogo não ter erros sem mexer no ficheiro.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Só na área de gestão.
+• As correções ficam na base de dados, por cima dos dados da DGES (a recolha seguinte não as apaga).
+• Fica registado quem alterou e quando.
+• Sem acesso aos dados dos alunos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sugestão de um colega (editar a base de dados na gestão), reescrita com uma necessidade concreta: um editor genérico de tabelas daria aos administradores os dados dos alunos. Precisa do catálogo na base de dados.</t>
   </si>
   <si>
     <t xml:space="preserve">US43</t>
@@ -482,24 +571,6 @@
     <t xml:space="preserve">Could</t>
   </si>
   <si>
-    <t xml:space="preserve">23/10: story nova (ideia proposta pelo Claude e aceite pelo PO). Feita no PR #44 a pedido do PO, antes do sprint. RGPD: a pessoa escolhe partilhar; política de privacidade provisória atualizada.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US44</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Que exames me abrem mais portas?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como candidato, quero saber que combinação de exames nacionais me deixa concorrer a mais cursos do meu plano, para decidir que exames fazer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Combinações de até 3 exames, a partir dos conjuntos de provas das opções do plano (2 ou mais opções).
-• Mostra as 3 melhores: a que serve para mais opções primeiro, depois a com menos exames.
-• Diz para que opções não dá e que exames da combinação a pessoa já fez.
-• Matemática e Matemática A contam como o mesmo exame.</t>
-  </si>
-  <si>
     <t xml:space="preserve">US45</t>
   </si>
   <si>
@@ -514,50 +585,6 @@
 • Aviso: as vagas da 2.ª fase são as que sobram da 1.ª e mudam todos os anos.</t>
   </si>
   <si>
-    <t xml:space="preserve">US37</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Assistente que conhece as minhas notas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como pessoa indecisa, quero que o assistente tenha em conta as provas que fiz e a minha nota, para não me sugerir cursos a que não posso concorrer.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Só com autorização da pessoa, o LLM recebe as provas feitas e um intervalo de nota (nunca a média exata, RNF12).
-• Cursos a que falta uma prova não são sugeridos, ou vêm assinalados.
-• Os testes usam o LLM falso.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Backlog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Por fazer</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23/10: story nova. Atenção: os termos do Gemini excluem menores de 18, e muitos candidatos têm 17 anos (protótipo para a equipa, ponto 14 dos requisitos).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US39</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corrigir e esconder cursos do catálogo (gestão)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como administrador, quero corrigir a descrição e as saídas profissionais de um curso, ou escondê-lo, para o catálogo não ter erros sem mexer no ficheiro.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Só na área de gestão.
-• As correções ficam na base de dados, por cima dos dados da DGES (a recolha seguinte não as apaga).
-• Fica registado quem alterou e quando.
-• Sem acesso aos dados dos alunos.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23/10: sugestão de um colega («editar a base de dados na área de gestão»), reescrita com uma necessidade concreta. Um editor genérico de tabelas daria aos administradores os dados pessoais dos alunos (RGPD) e seria o ponto mais perigoso do site aberto pelo túnel. Precisa do catálogo na base de dados.</t>
-  </si>
-  <si>
     <t xml:space="preserve">US38</t>
   </si>
   <si>
@@ -571,13 +598,331 @@
 • O passo atual do percurso mostra o próximo prazo.</t>
   </si>
   <si>
-    <t xml:space="preserve">23/10: story nova.</t>
+    <t xml:space="preserve">Story de 23/10, ainda sem código.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total de story points</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Story points concluídos (Estado = Feito)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota (27/10): as 22 stories das opcionais e a US32 (fundida na US29) estão na folha «Arquivo (opcionais)», com o motivo de cada uma. As US40 a US45 têm código no PR #44 mas ficam fora do Sprint 4, para o plano não passar ainda mais a velocidade.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plano de sprints — OptaBem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculado a partir da folha «Product Backlog»: mudar o Sprint ou o Estado de uma story lá atualiza esta tabela.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Velocidade por sprint (SP) — real do Sprint 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint Goal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP planeados</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP feitos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% feito</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Folga face à velocidade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nº stories</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Um aluno cria conta, entra e sai, e há um administrador com permissões próprias.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US01, US02, US03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uma pessoa indecisa conversa com o assistente (LLM), recebe 2 a 3 cursos do catálogo com explicação e escolhe um, ficando a decisão registada no percurso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US29, US30, US31</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uma pessoa indecisa filtra, consulta e compara cursos de várias instituições, e pode apagar a sua conta e todos os seus dados (22/10 a 29/10; concluído a 23/10).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US05, US17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quem escolheu um curso prepara a candidatura: vê as condições de acesso de cada curso, indica as suas notas, vê a sua nota de candidatura em cada curso e ordena as 6 opções; o catálogo passa a ter as licenciaturas da DGES (29/10 a 05/11; a confirmar com o docente).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US04, US33–US36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fora desta release, por ordem de prioridade. As US40 a US45 têm código pronto no PR #44 (protótipo). As opcionais estão na folha «Arquivo (opcionais)».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US40–US42, US44, US37, US46, US47, US39, US43, US45, US38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 07/10/2026 (decisão do Product Owner)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• O Sprint 1 tinha 24 SP planeados e a equipa concluiu 5 (registo e autenticação): o plano foi ajustado à velocidade real.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Story nova: US03 — Perfis de aluno e administrador (RF04, que não tinha story). Entra no Sprint 1 porque a importação do catálogo (US04) precisa de um administrador.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• As stories do catálogo, percurso e avaliações (US04 a US08) passam do Sprint 1 para o Sprint 2, com a pseudonimização (US09) para as avaliações serem anónimas desde o início.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• A explicação da recomendação passa para o Sprint 3; avaliação offline, períodos de avaliação, comentários e filtros para o Sprint 4.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Preferência de carga e comparação de estratégias passam para o Backlog; o SVD (antiga US22) fica fora do plano.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Escala das avaliações corrigida de 1–20 para 1–5 (igual ao resto do projeto).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• As stories foram renumeradas pela nova ordem (US01 a US28). A coluna «ID anterior» da folha «Product Backlog» mostra o número antigo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 13/10/2026 (decisão dos Product Owners, com sugestões do docente)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Nova visão do produto: o utilizador pode ainda não ter curso; o OptaBem orienta a escolha do curso e depois a das opcionais (docs/geral/00-visao-do-produto.md).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Catálogo com várias instituições: MVP com 12 instituições e 30 licenciaturas (dados/catalogo-cursos-mvp.csv, fonte DGES).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Stories novas: US29 (questionário), US30 (sugestão de cursos com LLM) e US31 (escolher curso e linha do tempo). Épico novo E11.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US04 e US05 passam a tratar instituições e cursos; US06 inclui a importação das UCs e passa para o Sprint 4.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US08, US10 e US12 a US20 passam para o Backlog; as que eram Must passam a Should nesta release.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• A partir de 13/10 os IDs ficam fixos (stories novas recebem o número seguinte). A ordem de trabalho é a deste plano.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Atenção: o plano soma 13, 13 e 18 SP; a velocidade real do Sprint 1 foi 10 SP (ponto 10 da secção 5 dos requisitos).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisão de 14/10/2026 (decisões dos Product Owners)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US03 revista: um só início de sessão para alunos e administradores (design patterns Strategy, Chain of Responsibility e Factory).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US05 começada antes do Sprint 2: pesquisa de cursos reais na página de apresentação. Os SP contam no Sprint 2, quando a story estiver completa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Story nova US32 (assistente LLM que conversa com o utilizador), no Backlog e por avaliar: decidir âmbito, custo e privacidade antes de estimar.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Redesenho visual do site (sem story própria): fica registado no PR #14 e no registo de uso de IA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 14/10/2026 (decisão do PO na issue #15)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• As perguntas deixam de ser fixas: o LLM conduz a conversa. US29 reescrita (conversa, 5 SP) e US32 fundida nela; US30 passa a ser o fim da conversa (3 SP).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Spike técnico feito antes do Sprint 2 (PR #17): Gemini e Groq atrás de ClienteLLM, testes sem rede, conclusões em docs/geral/05-spike-llm.md. Não tem SP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• O LLM passa para o Sprint 2. Velocidade ajustada à real (de 23 para 10 SP): Sprint 2 com 8 SP (2 de folga pela tecnologia nova), Sprints 3 e 4 com 10 SP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US05 passa para o Sprint 3. US04, US09 e US11 passam para o Backlog (Must → Should). A US07 guarda as avaliações com pseudo_id desde o início.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Consequência: nesta release não há recomendação de opcionais (US11). Se houver um Sprint 5, entram primeiro a US09 e a US11 (8 SP).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Por decidir antes do Sprint 2: idade mínima e plano do Gemini (os termos excluem menores de 18 e o plano gratuito com utilizadores no EEE).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint Planning do Sprint 2 (20/10/2026, decisão do PO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• A US29 e a US30 (8 SP) foram feitas antes de o sprint começar (PR #19, #20 e #22 a #24). Para o sprint ter trabalho novo, entra a US31 (5 SP), antecipada do Sprint 3.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• O Sprint 2 fica com 13 SP planeados, acima da velocidade (10), mas só 5 SP são trabalho novo. O Sprint 3 fica com a US05 (5 SP) e 5 SP por planear: rever no fim do Sprint 2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Ponto 14 decidido: o OptaBem é um protótipo usado pela equipa e na demonstração, com aviso de 18+ na conversa; fica escrito no relatório.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Servidor Ollama da faculdade testado e posto de parte: lento e não obedece ao pedido de sugestão (PR #25 e #26; 05-spike-llm.md, secção 7). Fica o Gemini.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint Review do Sprint 2 e Sprint Planning do Sprint 3 (22/10/2026, decisão dos PO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sprint Review: US29, US30 e US31 aceites, 13 de 13 SP. O percurso completo foi testado com o Gemini real, também noutro computador.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Até à entrega de 05/11, o centro do produto são os cursos. As opcionais saíram do site (PR #33) e as suas stories passam para segundo plano: US06 e US07 saem do Sprint 4 (Must → Should).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sprints de uma semana: Sprint 3 de 22/10 a 29/10 e Sprint 4 de 29/10 a 05/11.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sprint 3: US05 (5 SP) e US17 (3 SP, sobe do Backlog e passa a Must), com 2 SP de folga.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sprint 4: uma story nova a decidir com o docente; a US04 entra se houver folga. O código fecha por volta de 03/11, para o relatório e a demonstração.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• A revisão de 22/10 (segurança do túnel, menu do aluno, textos) fica adiada por decisão do PO; o túnel é só para a equipa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint Review do Sprint 3 (23/10/2026, decisão dos PO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US05 e US17 aceites, 7 de 7 SP. As duas stories foram testadas pelos PO (filtros, ficha, comparação e apagar a conta).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• O sprint fecha antes de 29/10 porque o objetivo foi cumprido. Entrou também, sem story, o menu fixo no topo (PR #40).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• No fecho, um teste da US17 que dependia da data em que corria foi corrigido (sem mudanças no código da aplicação).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sprint 4 por planear: a story nova fica a decidir com o docente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Replaneamento de 23/10/2026 (decisões do PO, com o protótipo do PR #44)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• O plano de candidatura ao Concurso Nacional de Acesso substitui as opcionais: épico novo E12 com a US33 (condições de acesso), US34 (notas), US35 (nota por curso), US36 (as 6 opções), US37 (assistente com as notas) e US38 (datas do concurso).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• As 22 stories das opcionais passam a Won't (fase 2) e ficam no fim do backlog, para a rastreabilidade.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US04 reescrita: o catálogo vem da DGES por recolha, em vez de ser importado por CSV na gestão; passa a Must e entra no Sprint 4.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US39 nova (gestão do catálogo), a partir da sugestão de um colega de editar a base de dados na área de gestão; fica no Backlog (Should).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Atenção: o Sprint 4 fica com 18 SP planeados, acima da velocidade (10). O código das US33 a US36 foi feito antes do sprint (protótipo), como a US29 e a US30 no Sprint 2. Se o docente achar demais, a US36 é a primeira a sair (é Should).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sem story: o registo pede o nome, terminar sessão volta à página inicial e «As minhas decisões» sai do menu (PR #43 e #44).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Correção: o Sprint Planning de 22/10 dizia «US17 (3 SP)»; a US17 tem 2 SP (o total de 7 SP da Sprint Review está certo).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• A story do Sprint 4 tem de ser confirmada com o docente.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• (23/10, mais tarde) Stories novas US40 a US43, propostas pelo Claude e aceites pelo PO: quanto preciso no exame, tendência do último colocado, procura do curso e partilhar o plano. Feitas no PR #44.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Atenção: com elas, o Sprint 4 fica com 27 SP planeados para uma velocidade de 10. Quase todo o código já está feito (protótipo), mas a documentação de cada story (requisitos, use case, BPMN) não. Se o docente achar demais, saem primeiro a US43 (Could) e depois a US36, US40, US41 e US42 (Should).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sem story: a gestão passa a ativar contas por confirmar, enquanto o site não envia emails reais (PR #43).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• (23/10, ao fim do dia) Stories novas US44 (que exames me abrem mais portas) e US45 (plano B: 2.ª fase), propostas pelo Claude e escolhidas pelo PO. Feitas no PR #44.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• O Sprint 4 fica com 32 SP planeados para uma velocidade de 10. Isto não é um planeamento realista em Scrum: o código foi feito antes do sprint, como protótipo. No Sprint Planning de 29/10, os PO e o docente decidem que stories entram; as restantes voltam ao Backlog com o código já feito.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Esclarecimento: o Sprint 4 ainda não começou (29/10 a 05/11). Um sprint fecha na Sprint Review, no fim do tempo marcado; aceitar um PR é o que faz uma story contar como Feita.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reestruturação de 27/10/2026 (autorizada pelo docente; decisão do PO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• O docente autorizou mudar o backlog a fundo, para corresponder a um recomendador de cursos e não de opcionais.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• As 22 stories das opcionais (US06 a US16 e US18 a US28) e a US32 (fundida na US29) saem do Product Backlog para a folha «Arquivo (opcionais)», com o motivo de cada uma. Os IDs não são reutilizados.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Épicos reorganizados: E1 Conta e privacidade, E2 Catálogo de cursos, E3 Orientação com o assistente, E4 Plano de candidatura. Os épicos antigos ficam no arquivo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Sprint 4 reduzido ao essencial: US04 e US33 a US36 (18 SP). As US40 a US45 (14 SP) voltam ao backlog com o código pronto, no estado novo «Protótipo».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Stories novas no backlog: US46 (exportar os meus dados, a parte do RF17 que saiu da US17) e US47 (recuperar a palavra-passe, a parte do RF02 sem story).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• As notas de cada story passam a dizer só o estado atual; o histórico fica nesta folha.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Atenção: mesmo assim, o Sprint 4 tem 18 SP para uma velocidade de 10. Só é defensável porque o código foi feito antes, como protótipo. A confirmar com o docente no Sprint Planning de 29/10.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resumo por prioridade (MoSCoW)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prioridade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Significado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SP total</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% do total de SP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Obrigatório para o produto fazer sentido</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Importante, mas o produto funciona sem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Desejável se houver folga</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Won't</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fora desta release</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nota (27/10): Won't fica a 0 porque as stories das opcionais (90 SP) saíram para a folha «Arquivo (opcionais)».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arquivo — stories das opcionais (fora do produto)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Até 23/10/2026 o OptaBem era também um recomendador de UCs opcionais. A 27/10, com autorização do docente, estas stories saíram do Product Backlog. Porquê: (1) o OptaBem serve quem ainda está a escolher curso, e essa pessoa não tem opcionais para escolher; (2) no ensino superior português as opcionais pesam pouco no percurso, e a decisão com consequências é a candidatura (épico E4); (3) recomendar opcionais exige avaliações de muitos alunos do mesmo curso, que um protótipo da equipa nunca teria (RN04 e RN05 deixariam quase tudo vazio); (4) não cabiam na velocidade real (10 SP por sprint). Ficam aqui para a rastreabilidade; os IDs não são reutilizados.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Épico antigo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Porque fica fora</t>
   </si>
   <si>
     <t xml:space="preserve">US06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">E3</t>
   </si>
   <si>
     <t xml:space="preserve">Registar percurso</t>
@@ -592,10 +937,7 @@
 • O aluno pode remover um registo.</t>
   </si>
   <si>
-    <t xml:space="preserve">Won't</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4; inclui a importação das UCs; 3 → 5 SP. 14/10: mantém-se no Sprint 4. 22/10: Sprint 4 → Backlog, Must → Should. Decisão dos PO: até à entrega de 05/11 o centro são os cursos e as opcionais ficam em segundo plano. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
+    <t xml:space="preserve">Pressupõe um aluno já inscrito num curso; o público do OptaBem ainda está a escolher curso.</t>
   </si>
   <si>
     <t xml:space="preserve">US07</t>
@@ -614,7 +956,7 @@
 • As avaliações ficam ligadas a um pseudo_id desde o início, e não ao email (ponto 2 dos requisitos); as regras de visualização e exportação ficam na US09.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Sprint 4. 14/10: fica no Sprint 4 sem a US09 (velocidade de 10 SP); por isso guarda já com pseudo_id. 22/10: Sprint 4 → Backlog, Must → Should. Decisão dos PO: até à entrega de 05/11 o centro são os cursos e as opcionais ficam em segundo plano. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
+    <t xml:space="preserve">Base das recomendações colaborativas; sem alunos reais do mesmo curso não há dados.</t>
   </si>
   <si>
     <t xml:space="preserve">US09</t>
@@ -632,7 +974,7 @@
 • Teste automático que verifica RN04.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: Sprint 2 → Sprint 4, com a US07 para as avaliações serem anónimas desde o início. 14/10: Sprint 4 → Backlog, Must → Should (velocidade de 10 SP). A US07 guarda já com pseudo_id; sem agregados (US11) a RN04 ainda não se aplica. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
+    <t xml:space="preserve">Só faz sentido se houver avaliações de UCs (US07).</t>
   </si>
   <si>
     <t xml:space="preserve">US11</t>
@@ -653,7 +995,7 @@
 • Implementada como estratégia intercambiável (padrão Strategy, docs/geral/03).</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 2 para Sprint 3. Replaneamento de 13/10: Sprint 3 → Sprint 4; segue o padrão Strategy. 14/10: Sprint 4 → Backlog, Must → Should (velocidade de 10 SP). Primeira candidata se houver um Sprint 5 ou folga. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
+    <t xml:space="preserve">Precisa de avaliações. O equivalente para cursos é a conversa com o assistente (US29 e US30).</t>
   </si>
   <si>
     <t xml:space="preserve">US08</t>
@@ -670,7 +1012,7 @@
 • Avaliar 10 UCs demora menos de 2 minutos.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 1 para Sprint 2. Replaneamento de 13/10: Sprint 2 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
+    <t xml:space="preserve">Só servia para alimentar o motor de recomendação de opcionais.</t>
   </si>
   <si>
     <t xml:space="preserve">E9</t>
@@ -686,10 +1028,10 @@
 • O motor recomenda UCs do perfil "plantado" na maioria dos casos.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 2 para Sprint 3. Replaneamento de 13/10: Sprint 3 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
-  </si>
-  <si>
     <t xml:space="preserve">US20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Servia para testar o motor de recomendação de opcionais.</t>
   </si>
   <si>
     <t xml:space="preserve">US12</t>
@@ -707,6 +1049,9 @@
 • Tempo de resposta &lt; 2 s (RNF03).</t>
   </si>
   <si>
+    <t xml:space="preserve">Precisa de muitos alunos com avaliações em comum (RN05); inviável numa demonstração.</t>
+  </si>
+  <si>
     <t xml:space="preserve">US13</t>
   </si>
   <si>
@@ -724,6 +1069,9 @@
   </si>
   <si>
     <t xml:space="preserve">US15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Regra do motor de opcionais.</t>
   </si>
   <si>
     <t xml:space="preserve">US14</t>
@@ -743,7 +1091,7 @@
 • A explicação não revela identidades.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: Sprint 3 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
+    <t xml:space="preserve">A explicação das sugestões de curso já existe (US30).</t>
   </si>
   <si>
     <t xml:space="preserve">Avaliação offline do motor</t>
@@ -757,13 +1105,16 @@
 • Resultados guardados e comparáveis entre estratégias.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 3 para Sprint 4. Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). Replaneamento de 13/10: Must → Should nesta release. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
-  </si>
-  <si>
     <t xml:space="preserve">US21</t>
   </si>
   <si>
+    <t xml:space="preserve">Mede um motor de recomendação que não existe.</t>
+  </si>
+  <si>
     <t xml:space="preserve">US16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E10</t>
   </si>
   <si>
     <t xml:space="preserve">Períodos de avaliação</t>
@@ -776,10 +1127,10 @@
 • Fora do período, o formulário de avaliação fica bloqueado com mensagem explicativa.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 3 para Sprint 4. Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
-  </si>
-  <si>
     <t xml:space="preserve">US24</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depende das avaliações de UCs.</t>
   </si>
   <si>
     <t xml:space="preserve">US18</t>
@@ -811,10 +1162,10 @@
 • Os alunos podem sinalizar comentários.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 13/10: Sprint 4 → Backlog (nova visão: orientação de curso primeiro). 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
-  </si>
-  <si>
     <t xml:space="preserve">US25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depende dos comentários (US18).</t>
   </si>
   <si>
     <t xml:space="preserve">Filtrar por semestre e ECTS</t>
@@ -825,6 +1176,9 @@
   <si>
     <t xml:space="preserve">• Filtros combináveis.
 • A lista atualiza sem perder a ordenação da recomendação.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtro das recomendações de opcionais; os cursos têm filtros próprios (US05).</t>
   </si>
   <si>
     <t xml:space="preserve">Preferência de carga de trabalho</t>
@@ -838,7 +1192,7 @@
 • "Indiferente" mantém a ordenação original.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 3 para Backlog. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
+    <t xml:space="preserve">Ajuste do motor de opcionais.</t>
   </si>
   <si>
     <t xml:space="preserve">US22</t>
@@ -857,10 +1211,10 @@
 • A estratégia ativa muda sem reiniciar a aplicação.</t>
   </si>
   <si>
-    <t xml:space="preserve">Replaneamento de 07/10: passou de Sprint 4 para Backlog. Depende do SVD (antiga US22), que também ficou fora do plano. 23/10: Should → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
-  </si>
-  <si>
     <t xml:space="preserve">US23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Depende de várias estratégias do motor, incluindo o SVD, que já estava fora do plano.</t>
   </si>
   <si>
     <t xml:space="preserve">Esconder UCs sem vagas</t>
@@ -873,7 +1227,7 @@
 • UCs com 0 vagas não aparecem, com opção "mostrar todas".</t>
   </si>
   <si>
-    <t xml:space="preserve">Entra no Sprint 4 se houver folga de velocidade. 23/10: Could → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
+    <t xml:space="preserve">As vagas das UCs mudam a cada semestre e não há fonte pública.</t>
   </si>
   <si>
     <t xml:space="preserve">Feedback sobre recomendações</t>
@@ -886,7 +1240,7 @@
 • O feedback fica registado para análise.</t>
   </si>
   <si>
-    <t xml:space="preserve">23/10: Could → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
+    <t xml:space="preserve">Feedback sobre recomendações de opcionais.</t>
   </si>
   <si>
     <t xml:space="preserve">Painel de participação</t>
@@ -902,6 +1256,9 @@
     <t xml:space="preserve">US26</t>
   </si>
   <si>
+    <t xml:space="preserve">Mede a participação nas avaliações de UCs.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Filtragem baseada em itens</t>
   </si>
   <si>
@@ -913,6 +1270,9 @@
   </si>
   <si>
     <t xml:space="preserve">US27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Precisa de avaliações e não tinha requisito associado.</t>
   </si>
   <si>
     <t xml:space="preserve">Evitar conflitos de horário</t>
@@ -926,6 +1286,9 @@
 • O administrador importa horários das UCs.</t>
   </si>
   <si>
+    <t xml:space="preserve">Os horários das UCs não são públicos de forma uniforme; 8 SP para um caso raro.</t>
+  </si>
+  <si>
     <t xml:space="preserve">US28</t>
   </si>
   <si>
@@ -939,12 +1302,15 @@
 • O aluno pode desativar lembretes.</t>
   </si>
   <si>
-    <t xml:space="preserve">23/10: Won't → Won't. Fase 2 (opcionais), fora desta release: o plano de candidatura substitui as opcionais (decisão do PO). Fica para rastreabilidade.</t>
+    <t xml:space="preserve">Depende dos períodos de avaliação e não tinha requisito associado.</t>
   </si>
   <si>
     <t xml:space="preserve">US32</t>
   </si>
   <si>
+    <t xml:space="preserve">E11</t>
+  </si>
+  <si>
     <t xml:space="preserve">Assistente LLM que conversa com o utilizador</t>
   </si>
   <si>
@@ -954,289 +1320,10 @@
     <t xml:space="preserve">• Fundida na US29 a 14/10/2026 (decisão do PO na issue #15): a conversa com o assistente passa a ser a própria orientação. A sugestão de cursos é a US30.</t>
   </si>
   <si>
-    <t xml:space="preserve">Fundida</t>
-  </si>
-  <si>
-    <t xml:space="preserve">14/10: pedido do PO para verificar a inserção de um agente LLM. No mesmo dia, o PO decidiu que o LLM conduz a conversa: a story foi fundida na US29. O ID fica, para a rastreabilidade.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total de story points</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Story points concluídos (Estado = Feito)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nota: a fatorização de matrizes (SVD, antiga US22) fica fora do plano da release. Épicos novos: E11 Orientação de curso (13/10) e E12 Candidatura (23/10). As stories das opcionais (Won't) ficam no fim, como fase 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plano de sprints — OptaBem</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Calculado a partir da folha «Product Backlog»: mudar o Sprint ou o Estado de uma story lá atualiza esta tabela.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Velocidade por sprint (SP) — real do Sprint 1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint Goal</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Stories</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP planeados</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP feitos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% feito</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Folga face à velocidade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nº stories</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Um aluno cria conta, entra e sai, e há um administrador com permissões próprias.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US01, US02, US03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uma pessoa indecisa conversa com o assistente (LLM), recebe 2 a 3 cursos do catálogo com explicação e escolhe um, ficando a decisão registada no percurso.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US29, US30, US31</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uma pessoa indecisa filtra, consulta e compara cursos de várias instituições, e pode apagar a sua conta e todos os seus dados (22/10 a 29/10; concluído a 23/10).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US05, US17</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quem escolheu um curso prepara a candidatura: vê as condições de acesso, a tendência e a procura de cada curso, calcula a sua nota e quanto precisa nos exames, descobre que exames lhe abrem mais portas, ordena as 6 opções, tem um plano B para a 2.ª fase e pode partilhar o plano; o catálogo passa a ter as licenciaturas da DGES (29/10 a 05/11; a confirmar com o docente).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US04, US33–US36, US40–US45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fora desta release (entrega a 05/11). As stories das opcionais passam a Won't (fase 2) a 23/10: o plano de candidatura substitui-as.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US37–US39, US06–US16, US18–US28 (US32 fundida na US29)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 07/10/2026 (decisão do Product Owner)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• O Sprint 1 tinha 24 SP planeados e a equipa concluiu 5 (registo e autenticação): o plano foi ajustado à velocidade real.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Story nova: US03 — Perfis de aluno e administrador (RF04, que não tinha story). Entra no Sprint 1 porque a importação do catálogo (US04) precisa de um administrador.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• As stories do catálogo, percurso e avaliações (US04 a US08) passam do Sprint 1 para o Sprint 2, com a pseudonimização (US09) para as avaliações serem anónimas desde o início.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• A explicação da recomendação passa para o Sprint 3; avaliação offline, períodos de avaliação, comentários e filtros para o Sprint 4.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Preferência de carga e comparação de estratégias passam para o Backlog; o SVD (antiga US22) fica fora do plano.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Escala das avaliações corrigida de 1–20 para 1–5 (igual ao resto do projeto).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• As stories foram renumeradas pela nova ordem (US01 a US28). A coluna «ID anterior» da folha «Product Backlog» mostra o número antigo.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 13/10/2026 (decisão dos Product Owners, com sugestões do docente)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Nova visão do produto: o utilizador pode ainda não ter curso; o OptaBem orienta a escolha do curso e depois a das opcionais (docs/geral/00-visao-do-produto.md).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Catálogo com várias instituições: MVP com 12 instituições e 30 licenciaturas (dados/catalogo-cursos-mvp.csv, fonte DGES).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Stories novas: US29 (questionário), US30 (sugestão de cursos com LLM) e US31 (escolher curso e linha do tempo). Épico novo E11.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• US04 e US05 passam a tratar instituições e cursos; US06 inclui a importação das UCs e passa para o Sprint 4.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• US08, US10 e US12 a US20 passam para o Backlog; as que eram Must passam a Should nesta release.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• A partir de 13/10 os IDs ficam fixos (stories novas recebem o número seguinte). A ordem de trabalho é a deste plano.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Atenção: o plano soma 13, 13 e 18 SP; a velocidade real do Sprint 1 foi 10 SP (ponto 10 da secção 5 dos requisitos).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Revisão de 14/10/2026 (decisões dos Product Owners)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• US03 revista: um só início de sessão para alunos e administradores (design patterns Strategy, Chain of Responsibility e Factory).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• US05 começada antes do Sprint 2: pesquisa de cursos reais na página de apresentação. Os SP contam no Sprint 2, quando a story estiver completa.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Story nova US32 (assistente LLM que conversa com o utilizador), no Backlog e por avaliar: decidir âmbito, custo e privacidade antes de estimar.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Redesenho visual do site (sem story própria): fica registado no PR #14 e no registo de uso de IA.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 14/10/2026 (decisão do PO na issue #15)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• As perguntas deixam de ser fixas: o LLM conduz a conversa. US29 reescrita (conversa, 5 SP) e US32 fundida nela; US30 passa a ser o fim da conversa (3 SP).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Spike técnico feito antes do Sprint 2 (PR #17): Gemini e Groq atrás de ClienteLLM, testes sem rede, conclusões em docs/geral/05-spike-llm.md. Não tem SP.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• O LLM passa para o Sprint 2. Velocidade ajustada à real (de 23 para 10 SP): Sprint 2 com 8 SP (2 de folga pela tecnologia nova), Sprints 3 e 4 com 10 SP.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• US05 passa para o Sprint 3. US04, US09 e US11 passam para o Backlog (Must → Should). A US07 guarda as avaliações com pseudo_id desde o início.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Consequência: nesta release não há recomendação de opcionais (US11). Se houver um Sprint 5, entram primeiro a US09 e a US11 (8 SP).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Por decidir antes do Sprint 2: idade mínima e plano do Gemini (os termos excluem menores de 18 e o plano gratuito com utilizadores no EEE).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint Planning do Sprint 2 (20/10/2026, decisão do PO)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• A US29 e a US30 (8 SP) foram feitas antes de o sprint começar (PR #19, #20 e #22 a #24). Para o sprint ter trabalho novo, entra a US31 (5 SP), antecipada do Sprint 3.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• O Sprint 2 fica com 13 SP planeados, acima da velocidade (10), mas só 5 SP são trabalho novo. O Sprint 3 fica com a US05 (5 SP) e 5 SP por planear: rever no fim do Sprint 2.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Ponto 14 decidido: o OptaBem é um protótipo usado pela equipa e na demonstração, com aviso de 18+ na conversa; fica escrito no relatório.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Servidor Ollama da faculdade testado e posto de parte: lento e não obedece ao pedido de sugestão (PR #25 e #26; 05-spike-llm.md, secção 7). Fica o Gemini.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint Review do Sprint 2 e Sprint Planning do Sprint 3 (22/10/2026, decisão dos PO)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Sprint Review: US29, US30 e US31 aceites, 13 de 13 SP. O percurso completo foi testado com o Gemini real, também noutro computador.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Até à entrega de 05/11, o centro do produto são os cursos. As opcionais saíram do site (PR #33) e as suas stories passam para segundo plano: US06 e US07 saem do Sprint 4 (Must → Should).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Sprints de uma semana: Sprint 3 de 22/10 a 29/10 e Sprint 4 de 29/10 a 05/11.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Sprint 3: US05 (5 SP) e US17 (3 SP, sobe do Backlog e passa a Must), com 2 SP de folga.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Sprint 4: uma story nova a decidir com o docente; a US04 entra se houver folga. O código fecha por volta de 03/11, para o relatório e a demonstração.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• A revisão de 22/10 (segurança do túnel, menu do aluno, textos) fica adiada por decisão do PO; o túnel é só para a equipa.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sprint Review do Sprint 3 (23/10/2026, decisão dos PO)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• US05 e US17 aceites, 7 de 7 SP. As duas stories foram testadas pelos PO (filtros, ficha, comparação e apagar a conta).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• O sprint fecha antes de 29/10 porque o objetivo foi cumprido. Entrou também, sem story, o menu fixo no topo (PR #40).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• No fecho, um teste da US17 que dependia da data em que corria foi corrigido (sem mudanças no código da aplicação).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Sprint 4 por planear: a story nova fica a decidir com o docente.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Replaneamento de 23/10/2026 (decisões do PO, com o protótipo do PR #44)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• O plano de candidatura ao Concurso Nacional de Acesso substitui as opcionais: épico novo E12 com a US33 (condições de acesso), US34 (notas), US35 (nota por curso), US36 (as 6 opções), US37 (assistente com as notas) e US38 (datas do concurso).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• As 22 stories das opcionais passam a Won't (fase 2) e ficam no fim do backlog, para a rastreabilidade.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• US04 reescrita: o catálogo vem da DGES por recolha, em vez de ser importado por CSV na gestão; passa a Must e entra no Sprint 4.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• US39 nova (gestão do catálogo), a partir da sugestão de um colega de editar a base de dados na área de gestão; fica no Backlog (Should).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Atenção: o Sprint 4 fica com 18 SP planeados, acima da velocidade (10). O código das US33 a US36 foi feito antes do sprint (protótipo), como a US29 e a US30 no Sprint 2. Se o docente achar demais, a US36 é a primeira a sair (é Should).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Sem story: o registo pede o nome, terminar sessão volta à página inicial e «As minhas decisões» sai do menu (PR #43 e #44).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Correção: o Sprint Planning de 22/10 dizia «US17 (3 SP)»; a US17 tem 2 SP (o total de 7 SP da Sprint Review está certo).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• A story do Sprint 4 tem de ser confirmada com o docente.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• (23/10, mais tarde) Stories novas US40 a US43, propostas pelo Claude e aceites pelo PO: quanto preciso no exame, tendência do último colocado, procura do curso e partilhar o plano. Feitas no PR #44.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Atenção: com elas, o Sprint 4 fica com 27 SP planeados para uma velocidade de 10. Quase todo o código já está feito (protótipo), mas a documentação de cada story (requisitos, use case, BPMN) não. Se o docente achar demais, saem primeiro a US43 (Could) e depois a US36, US40, US41 e US42 (Should).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Sem story: a gestão passa a ativar contas por confirmar, enquanto o site não envia emails reais (PR #43).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• (23/10, ao fim do dia) Stories novas US44 (que exames me abrem mais portas) e US45 (plano B: 2.ª fase), propostas pelo Claude e escolhidas pelo PO. Feitas no PR #44.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• O Sprint 4 fica com 32 SP planeados para uma velocidade de 10. Isto não é um planeamento realista em Scrum: o código foi feito antes do sprint, como protótipo. No Sprint Planning de 29/10, os PO e o docente decidem que stories entram; as restantes voltam ao Backlog com o código já feito.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Esclarecimento: o Sprint 4 ainda não começou (29/10 a 05/11). Um sprint fecha na Sprint Review, no fim do tempo marcado; aceitar um PR é o que faz uma story contar como Feita.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Resumo por prioridade (MoSCoW)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prioridade</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Significado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SP total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% do total de SP</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Obrigatório para o produto fazer sentido</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Importante, mas o produto funciona sem</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Desejável se houver folga</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fora desta release</t>
+    <t xml:space="preserve">Fundida na US29 a 14/10 (issue #15): a conversa com o assistente passou a ser a própria orientação.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total de story points arquivados</t>
   </si>
 </sst>
 </file>
@@ -1470,7 +1557,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1583,6 +1670,14 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1592,7 +1687,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="22">
+  <dxfs count="20">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1643,14 +1738,6 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFEDEDED"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
           <fgColor rgb="FFF8CBAD"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
@@ -1690,14 +1777,6 @@
     </dxf>
     <dxf>
       <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFEB9C"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
         </patternFill>
@@ -1713,14 +1792,14 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFF8CBAD"/>
+          <bgColor rgb="FFDDEBF7"/>
         </patternFill>
       </fill>
     </dxf>
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFDDEBF7"/>
+          <bgColor rgb="FFF8CBAD"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1954,7 +2033,7 @@
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>32</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2056,11 +2135,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="16294996"/>
-        <c:axId val="95851061"/>
+        <c:axId val="44034424"/>
+        <c:axId val="32648971"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="16294996"/>
+        <c:axId val="44034424"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2091,7 +2170,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="95851061"/>
+        <c:crossAx val="32648971"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2099,7 +2178,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="95851061"/>
+        <c:axId val="32648971"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2164,7 +2243,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="16294996"/>
+        <c:crossAx val="44034424"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2231,9 +2310,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2088000</xdr:colOff>
+      <xdr:colOff>2087280</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>84960</xdr:rowOff>
+      <xdr:rowOff>84240</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2242,7 +2321,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5753160" cy="2512800"/>
+        <a:ext cx="5752440" cy="2512080"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2253,6 +2332,10 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2783,16 +2866,16 @@
         <v>60</v>
       </c>
       <c r="C12" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="6" t="s">
+      <c r="E12" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="E12" s="6" t="s">
+      <c r="F12" s="6" t="s">
         <v>63</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>64</v>
       </c>
       <c r="G12" s="7" t="n">
         <v>2</v>
@@ -2808,10 +2891,10 @@
       </c>
       <c r="K12" s="8"/>
       <c r="L12" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="M12" s="5" t="s">
         <v>65</v>
-      </c>
-      <c r="M12" s="5" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2825,13 +2908,13 @@
         <v>53</v>
       </c>
       <c r="D13" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="E13" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="F13" s="6" t="s">
         <v>68</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>69</v>
       </c>
       <c r="G13" s="7" t="n">
         <v>5</v>
@@ -2840,14 +2923,14 @@
         <v>20</v>
       </c>
       <c r="I13" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="J13" s="7" t="s">
         <v>70</v>
-      </c>
-      <c r="J13" s="7" t="s">
-        <v>71</v>
       </c>
       <c r="K13" s="8"/>
       <c r="L13" s="8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="M13" s="5" t="s">
         <v>29</v>
@@ -2858,19 +2941,19 @@
         <v>10</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="E14" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="F14" s="6" t="s">
-        <v>77</v>
       </c>
       <c r="G14" s="7" t="n">
         <v>3</v>
@@ -2879,17 +2962,17 @@
         <v>20</v>
       </c>
       <c r="I14" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="J14" s="7" t="s">
         <v>70</v>
-      </c>
-      <c r="J14" s="7" t="s">
-        <v>71</v>
       </c>
       <c r="K14" s="8"/>
       <c r="L14" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="M14" s="5" t="s">
         <v>78</v>
-      </c>
-      <c r="M14" s="5" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2897,19 +2980,19 @@
         <v>11</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="C15" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D15" s="6" t="s">
+      <c r="E15" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="E15" s="6" t="s">
+      <c r="F15" s="6" t="s">
         <v>82</v>
-      </c>
-      <c r="F15" s="6" t="s">
-        <v>83</v>
       </c>
       <c r="G15" s="7" t="n">
         <v>2</v>
@@ -2918,17 +3001,17 @@
         <v>20</v>
       </c>
       <c r="I15" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="J15" s="7" t="s">
         <v>70</v>
-      </c>
-      <c r="J15" s="7" t="s">
-        <v>71</v>
       </c>
       <c r="K15" s="8"/>
       <c r="L15" s="8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="M15" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2936,19 +3019,19 @@
         <v>12</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D16" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="C16" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D16" s="6" t="s">
+      <c r="E16" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="E16" s="6" t="s">
+      <c r="F16" s="6" t="s">
         <v>87</v>
-      </c>
-      <c r="F16" s="6" t="s">
-        <v>88</v>
       </c>
       <c r="G16" s="7" t="n">
         <v>3</v>
@@ -2957,17 +3040,17 @@
         <v>20</v>
       </c>
       <c r="I16" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="J16" s="7" t="s">
         <v>70</v>
-      </c>
-      <c r="J16" s="7" t="s">
-        <v>71</v>
       </c>
       <c r="K16" s="8"/>
       <c r="L16" s="8" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="M16" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2975,38 +3058,38 @@
         <v>13</v>
       </c>
       <c r="B17" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="C17" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D17" s="6" t="s">
+      <c r="E17" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="E17" s="6" t="s">
+      <c r="F17" s="6" t="s">
         <v>92</v>
-      </c>
-      <c r="F17" s="6" t="s">
-        <v>93</v>
       </c>
       <c r="G17" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I17" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="J17" s="7" t="s">
         <v>70</v>
-      </c>
-      <c r="J17" s="7" t="s">
-        <v>71</v>
       </c>
       <c r="K17" s="8"/>
       <c r="L17" s="8" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M17" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3014,38 +3097,38 @@
         <v>14</v>
       </c>
       <c r="B18" s="5" t="s">
+        <v>95</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" s="6" t="s">
         <v>96</v>
       </c>
-      <c r="C18" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D18" s="6" t="s">
+      <c r="E18" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="E18" s="6" t="s">
+      <c r="F18" s="6" t="s">
         <v>98</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>99</v>
       </c>
       <c r="G18" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I18" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J18" s="7" t="s">
         <v>70</v>
-      </c>
-      <c r="J18" s="7" t="s">
-        <v>71</v>
       </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8" t="s">
         <v>100</v>
       </c>
       <c r="M18" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3056,7 +3139,7 @@
         <v>101</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D19" s="6" t="s">
         <v>102</v>
@@ -3071,20 +3154,20 @@
         <v>2</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I19" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J19" s="7" t="s">
         <v>70</v>
-      </c>
-      <c r="J19" s="7" t="s">
-        <v>71</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
         <v>100</v>
       </c>
       <c r="M19" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3095,7 +3178,7 @@
         <v>105</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D20" s="6" t="s">
         <v>106</v>
@@ -3110,20 +3193,20 @@
         <v>2</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I20" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J20" s="7" t="s">
         <v>70</v>
-      </c>
-      <c r="J20" s="7" t="s">
-        <v>71</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
         <v>100</v>
       </c>
       <c r="M20" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3134,7 +3217,7 @@
         <v>109</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D21" s="6" t="s">
         <v>110</v>
@@ -3149,20 +3232,20 @@
         <v>3</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="I21" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J21" s="7" t="s">
         <v>70</v>
-      </c>
-      <c r="J21" s="7" t="s">
-        <v>71</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="M21" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3170,38 +3253,38 @@
         <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="E22" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="C22" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D22" s="6" t="s">
+      <c r="F22" s="6" t="s">
         <v>116</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="F22" s="6" t="s">
-        <v>118</v>
       </c>
       <c r="G22" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>71</v>
+        <v>117</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
-        <v>100</v>
+        <v>118</v>
       </c>
       <c r="M22" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3212,7 +3295,7 @@
         <v>119</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>74</v>
+        <v>16</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>120</v>
@@ -3227,20 +3310,20 @@
         <v>2</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>113</v>
+        <v>93</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>71</v>
+        <v>117</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8" t="s">
-        <v>100</v>
+        <v>123</v>
       </c>
       <c r="M23" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3248,38 +3331,38 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>74</v>
+        <v>16</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="M24" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3287,38 +3370,38 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D25" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="E25" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="F25" s="6" t="s">
         <v>132</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="F25" s="6" t="s">
-        <v>134</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>5</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="M25" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3326,38 +3409,38 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
+        <v>134</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="E26" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="C26" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="D26" s="6" t="s">
+      <c r="F26" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="E26" s="6" t="s">
+      <c r="G26" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="H26" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="F26" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="G26" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H26" s="5" t="s">
-        <v>113</v>
-      </c>
       <c r="I26" s="7" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="M26" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3365,38 +3448,38 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="E27" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="F27" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="D27" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>144</v>
-      </c>
-      <c r="F27" s="6" t="s">
-        <v>145</v>
-      </c>
       <c r="G27" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>128</v>
+        <v>70</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
-        <v>147</v>
+        <v>100</v>
       </c>
       <c r="M27" s="5" t="s">
-        <v>52</v>
+        <v>78</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3404,934 +3487,143 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>142</v>
+        <v>73</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="G28" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>128</v>
+        <v>117</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="M28" s="5" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="n">
-        <v>25</v>
-      </c>
-      <c r="B29" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="F29" s="6" t="s">
-        <v>156</v>
-      </c>
-      <c r="G29" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="H29" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I29" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J29" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K29" s="8"/>
-      <c r="L29" s="8" t="s">
-        <v>157</v>
-      </c>
-      <c r="M29" s="5" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="n">
-        <v>26</v>
-      </c>
-      <c r="B30" s="5" t="s">
-        <v>158</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="F30" s="6" t="s">
-        <v>162</v>
-      </c>
-      <c r="G30" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H30" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I30" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J30" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K30" s="8"/>
-      <c r="L30" s="8" t="s">
-        <v>163</v>
-      </c>
-      <c r="M30" s="5" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="n">
-        <v>27</v>
-      </c>
-      <c r="B31" s="5" t="s">
-        <v>164</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>165</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>166</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>167</v>
-      </c>
-      <c r="G31" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H31" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I31" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J31" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K31" s="8"/>
-      <c r="L31" s="8" t="s">
-        <v>168</v>
-      </c>
-      <c r="M31" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F29" s="9" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="32" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>170</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>171</v>
-      </c>
-      <c r="F32" s="6" t="s">
-        <v>172</v>
-      </c>
-      <c r="G32" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="H32" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I32" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J32" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K32" s="8"/>
-      <c r="L32" s="8" t="s">
-        <v>173</v>
-      </c>
-      <c r="M32" s="5" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="n">
-        <v>29</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>159</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>176</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>177</v>
-      </c>
-      <c r="F33" s="6" t="s">
-        <v>178</v>
-      </c>
-      <c r="G33" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H33" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I33" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J33" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K33" s="8"/>
-      <c r="L33" s="8" t="s">
-        <v>173</v>
-      </c>
-      <c r="M33" s="5" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="n">
+      <c r="G29" s="9" t="n">
+        <f aca="false">SUM(G5:G28)</f>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F30" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="G30" s="9" t="n">
+        <f aca="false">SUMIF(J5:J28,"Feito",G5:G28)</f>
         <v>30</v>
       </c>
-      <c r="B34" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="C34" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>182</v>
-      </c>
-      <c r="F34" s="6" t="s">
-        <v>183</v>
-      </c>
-      <c r="G34" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H34" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I34" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J34" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K34" s="8"/>
-      <c r="L34" s="8" t="s">
-        <v>173</v>
-      </c>
-      <c r="M34" s="5" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="n">
-        <v>31</v>
-      </c>
-      <c r="B35" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="C35" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>188</v>
-      </c>
-      <c r="F35" s="6" t="s">
-        <v>189</v>
-      </c>
-      <c r="G35" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="H35" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I35" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J35" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K35" s="8"/>
-      <c r="L35" s="8" t="s">
-        <v>190</v>
-      </c>
-      <c r="M35" s="5" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="n">
-        <v>32</v>
-      </c>
-      <c r="B36" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="C36" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="D36" s="6" t="s">
-        <v>191</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>192</v>
-      </c>
-      <c r="F36" s="6" t="s">
-        <v>193</v>
-      </c>
-      <c r="G36" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="H36" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I36" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J36" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K36" s="8"/>
-      <c r="L36" s="8" t="s">
-        <v>194</v>
-      </c>
-      <c r="M36" s="5" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="n">
-        <v>33</v>
-      </c>
-      <c r="B37" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="C37" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>197</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>198</v>
-      </c>
-      <c r="F37" s="6" t="s">
-        <v>199</v>
-      </c>
-      <c r="G37" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H37" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I37" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J37" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K37" s="8"/>
-      <c r="L37" s="8" t="s">
-        <v>200</v>
-      </c>
-      <c r="M37" s="5" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="n">
-        <v>34</v>
-      </c>
-      <c r="B38" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="C38" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="D38" s="6" t="s">
-        <v>203</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>204</v>
-      </c>
-      <c r="F38" s="6" t="s">
-        <v>205</v>
-      </c>
-      <c r="G38" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H38" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I38" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J38" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K38" s="8"/>
-      <c r="L38" s="8" t="s">
-        <v>200</v>
-      </c>
-      <c r="M38" s="5" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="5" t="n">
-        <v>35</v>
-      </c>
-      <c r="B39" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="C39" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>207</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>208</v>
-      </c>
-      <c r="F39" s="6" t="s">
-        <v>209</v>
-      </c>
-      <c r="G39" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H39" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I39" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J39" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K39" s="8"/>
-      <c r="L39" s="8" t="s">
-        <v>210</v>
-      </c>
-      <c r="M39" s="5" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="n">
-        <v>36</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D40" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>213</v>
-      </c>
-      <c r="F40" s="6" t="s">
-        <v>214</v>
-      </c>
-      <c r="G40" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="H40" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I40" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J40" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K40" s="8"/>
-      <c r="L40" s="8" t="s">
-        <v>200</v>
-      </c>
-      <c r="M40" s="5" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5" t="n">
-        <v>37</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="C41" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D41" s="6" t="s">
-        <v>215</v>
-      </c>
-      <c r="E41" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="F41" s="6" t="s">
-        <v>217</v>
-      </c>
-      <c r="G41" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="H41" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I41" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J41" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K41" s="8"/>
-      <c r="L41" s="8" t="s">
-        <v>218</v>
-      </c>
-      <c r="M41" s="5" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="n">
-        <v>38</v>
-      </c>
-      <c r="B42" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="C42" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="D42" s="6" t="s">
-        <v>221</v>
-      </c>
-      <c r="E42" s="6" t="s">
-        <v>222</v>
-      </c>
-      <c r="F42" s="6" t="s">
-        <v>223</v>
-      </c>
-      <c r="G42" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H42" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I42" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J42" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K42" s="8"/>
-      <c r="L42" s="8" t="s">
-        <v>224</v>
-      </c>
-      <c r="M42" s="5" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="5" t="n">
-        <v>39</v>
-      </c>
-      <c r="B43" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D43" s="6" t="s">
-        <v>226</v>
-      </c>
-      <c r="E43" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="F43" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="G43" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H43" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I43" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J43" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K43" s="8"/>
-      <c r="L43" s="8" t="s">
-        <v>229</v>
-      </c>
-      <c r="M43" s="5" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="5" t="n">
-        <v>40</v>
-      </c>
-      <c r="B44" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="C44" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="D44" s="6" t="s">
-        <v>230</v>
-      </c>
-      <c r="E44" s="6" t="s">
-        <v>231</v>
-      </c>
-      <c r="F44" s="6" t="s">
-        <v>232</v>
-      </c>
-      <c r="G44" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H44" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I44" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J44" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K44" s="8"/>
-      <c r="L44" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="M44" s="5" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5" t="n">
-        <v>41</v>
-      </c>
-      <c r="B45" s="5" t="s">
-        <v>211</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="D45" s="6" t="s">
-        <v>234</v>
-      </c>
-      <c r="E45" s="6" t="s">
-        <v>235</v>
-      </c>
-      <c r="F45" s="6" t="s">
-        <v>236</v>
-      </c>
-      <c r="G45" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H45" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I45" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J45" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K45" s="8"/>
-      <c r="L45" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="M45" s="5" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="5" t="n">
-        <v>42</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>237</v>
-      </c>
-      <c r="C46" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="D46" s="6" t="s">
-        <v>238</v>
-      </c>
-      <c r="E46" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="F46" s="6" t="s">
-        <v>240</v>
-      </c>
-      <c r="G46" s="7" t="n">
-        <v>5</v>
-      </c>
-      <c r="H46" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I46" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J46" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K46" s="8"/>
-      <c r="L46" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="M46" s="5" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5" t="n">
-        <v>43</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>241</v>
-      </c>
-      <c r="C47" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="D47" s="6" t="s">
-        <v>242</v>
-      </c>
-      <c r="E47" s="6" t="s">
-        <v>243</v>
-      </c>
-      <c r="F47" s="6" t="s">
-        <v>244</v>
-      </c>
-      <c r="G47" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="H47" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I47" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J47" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K47" s="8"/>
-      <c r="L47" s="8" t="s">
-        <v>233</v>
-      </c>
-      <c r="M47" s="5" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="5" t="n">
-        <v>44</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>245</v>
-      </c>
-      <c r="C48" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="D48" s="6" t="s">
-        <v>246</v>
-      </c>
-      <c r="E48" s="6" t="s">
-        <v>247</v>
-      </c>
-      <c r="F48" s="6" t="s">
-        <v>248</v>
-      </c>
-      <c r="G48" s="7" t="n">
-        <v>3</v>
-      </c>
-      <c r="H48" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="I48" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J48" s="7" t="s">
-        <v>128</v>
-      </c>
-      <c r="K48" s="8"/>
-      <c r="L48" s="8" t="s">
-        <v>249</v>
-      </c>
-      <c r="M48" s="5" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="B49" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="C49" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="D49" s="6" t="s">
-        <v>251</v>
-      </c>
-      <c r="E49" s="6" t="s">
-        <v>252</v>
-      </c>
-      <c r="F49" s="6" t="s">
-        <v>253</v>
-      </c>
-      <c r="G49" s="7"/>
-      <c r="H49" s="5"/>
-      <c r="I49" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="J49" s="7" t="s">
-        <v>254</v>
-      </c>
-      <c r="K49" s="8"/>
-      <c r="L49" s="8" t="s">
-        <v>255</v>
-      </c>
-      <c r="M49" s="5" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F50" s="9" t="s">
-        <v>256</v>
-      </c>
-      <c r="G50" s="9" t="n">
-        <f aca="false">SUM(G5:G49)</f>
-        <v>162</v>
-      </c>
-    </row>
-    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F51" s="9" t="s">
-        <v>257</v>
-      </c>
-      <c r="G51" s="9" t="n">
-        <f aca="false">SUMIF(J5:J49,"Feito",G5:G49)</f>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F52" s="10" t="s">
-        <v>258</v>
-      </c>
-    </row>
+    </row>
+    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F31" s="10" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="35" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="36" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="37" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="38" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="39" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="40" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="41" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="42" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="43" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="44" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="45" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="46" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="47" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="48" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="49" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="50" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="52" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A4:M49"/>
-  <conditionalFormatting sqref="J5:J49">
-    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+  <autoFilter ref="A4:M28"/>
+  <conditionalFormatting sqref="J5:J28">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>"Feito"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12">
       <formula>"Em curso"</formula>
     </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+      <formula>"Protótipo"</formula>
+    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H49">
-    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+  <conditionalFormatting sqref="H5:H28">
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>"Must"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Should"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Could"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Won't"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I49">
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+  <conditionalFormatting sqref="I5:I28">
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Sprint 1"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Sprint 2"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>"Sprint 3"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Sprint 4"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="21">
+    <cfRule type="cellIs" priority="13" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"Backlog"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G49" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G28" type="list">
       <formula1>"1,2,3,5,8,13,21"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H49" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H28" type="list">
       <formula1>"Must,Should,Could,Won't"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I49" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I28" type="list">
       <formula1>"Sprint 1,Sprint 2,Sprint 3,Sprint 4,Backlog"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J49" type="list">
-      <formula1>"Por fazer,Em curso,Feito,Fundida"</formula1>
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J28" type="list">
+      <formula1>"Por fazer,Protótipo,Em curso,Feito"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -4352,7 +3644,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H94"/>
+  <dimension ref="A1:H103"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -4367,17 +3659,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>259</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>260</v>
+        <v>152</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>261</v>
+        <v>153</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>10</v>
@@ -4388,25 +3680,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>262</v>
+        <v>154</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>263</v>
+        <v>155</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>264</v>
+        <v>156</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>265</v>
+        <v>157</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>266</v>
+        <v>158</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>267</v>
+        <v>159</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>268</v>
+        <v>160</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4414,17 +3706,17 @@
         <v>21</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>269</v>
+        <v>161</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>270</v>
+        <v>162</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$49,$A6,'Product Backlog'!$G$5:$G$49)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$28,$A6,'Product Backlog'!$G$5:$G$28)</f>
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$49,'Product Backlog'!$I$5:$I$49,$A6,'Product Backlog'!$J$5:$J$49,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$28,'Product Backlog'!$I$5:$I$28,$A6,'Product Backlog'!$J$5:$J$28,"Feito")</f>
         <v>10</v>
       </c>
       <c r="F6" s="15" t="n">
@@ -4436,7 +3728,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$49,$A6)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$28,$A6)</f>
         <v>3</v>
       </c>
     </row>
@@ -4445,17 +3737,17 @@
         <v>40</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>271</v>
+        <v>163</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>272</v>
+        <v>164</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$49,$A7,'Product Backlog'!$G$5:$G$49)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$28,$A7,'Product Backlog'!$G$5:$G$28)</f>
         <v>13</v>
       </c>
       <c r="E7" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$49,'Product Backlog'!$I$5:$I$49,$A7,'Product Backlog'!$J$5:$J$49,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$28,'Product Backlog'!$I$5:$I$28,$A7,'Product Backlog'!$J$5:$J$28,"Feito")</f>
         <v>13</v>
       </c>
       <c r="F7" s="15" t="n">
@@ -4467,7 +3759,7 @@
         <v>-3</v>
       </c>
       <c r="H7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$49,$A7)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$28,$A7)</f>
         <v>3</v>
       </c>
     </row>
@@ -4476,17 +3768,17 @@
         <v>57</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>273</v>
+        <v>165</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>274</v>
+        <v>166</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$49,$A8,'Product Backlog'!$G$5:$G$49)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$28,$A8,'Product Backlog'!$G$5:$G$28)</f>
         <v>7</v>
       </c>
       <c r="E8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$49,'Product Backlog'!$I$5:$I$49,$A8,'Product Backlog'!$J$5:$J$49,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$28,'Product Backlog'!$I$5:$I$28,$A8,'Product Backlog'!$J$5:$J$28,"Feito")</f>
         <v>7</v>
       </c>
       <c r="F8" s="15" t="n">
@@ -4498,26 +3790,26 @@
         <v>3</v>
       </c>
       <c r="H8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$49,$A8)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$28,$A8)</f>
         <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>275</v>
+        <v>167</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>276</v>
+        <v>168</v>
       </c>
       <c r="D9" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$49,$A9,'Product Backlog'!$G$5:$G$49)</f>
-        <v>32</v>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$28,$A9,'Product Backlog'!$G$5:$G$28)</f>
+        <v>18</v>
       </c>
       <c r="E9" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$49,'Product Backlog'!$I$5:$I$49,$A9,'Product Backlog'!$J$5:$J$49,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$28,'Product Backlog'!$I$5:$I$28,$A9,'Product Backlog'!$J$5:$J$28,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F9" s="15" t="n">
@@ -4526,29 +3818,29 @@
       </c>
       <c r="G9" s="16" t="n">
         <f aca="false">$C$3-D9</f>
-        <v>-22</v>
+        <v>-8</v>
       </c>
       <c r="H9" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$49,$A9)</f>
-        <v>11</v>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$28,$A9)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>127</v>
+        <v>99</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>277</v>
+        <v>169</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>278</v>
+        <v>170</v>
       </c>
       <c r="D10" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$49,$A10,'Product Backlog'!$G$5:$G$49)</f>
-        <v>100</v>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$28,$A10,'Product Backlog'!$G$5:$G$28)</f>
+        <v>29</v>
       </c>
       <c r="E10" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$49,'Product Backlog'!$I$5:$I$49,$A10,'Product Backlog'!$J$5:$J$49,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$28,'Product Backlog'!$I$5:$I$28,$A10,'Product Backlog'!$J$5:$J$28,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F10" s="15" t="n">
@@ -4559,19 +3851,19 @@
         <v>34</v>
       </c>
       <c r="H10" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$49,$A10)</f>
-        <v>26</v>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$28,$A10)</f>
+        <v>11</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>279</v>
+        <v>171</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
       <c r="D11" s="21" t="n">
         <f aca="false">SUM(D6:D10)</f>
-        <v>162</v>
+        <v>77</v>
       </c>
       <c r="E11" s="21" t="n">
         <f aca="false">SUM(E6:E10)</f>
@@ -4579,312 +3871,352 @@
       </c>
       <c r="F11" s="22" t="n">
         <f aca="false">IF(D11=0,0,E11/D11)</f>
-        <v>0.185185185185185</v>
+        <v>0.38961038961039</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21" t="n">
         <f aca="false">SUM(H6:H10)</f>
-        <v>45</v>
+        <v>24</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>280</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>281</v>
+        <v>173</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>282</v>
+        <v>174</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>283</v>
+        <v>175</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>284</v>
+        <v>176</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>285</v>
+        <v>177</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>286</v>
+        <v>178</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>287</v>
+        <v>179</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>288</v>
+        <v>180</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
-        <v>289</v>
+        <v>181</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>290</v>
+        <v>182</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
-        <v>291</v>
+        <v>183</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>292</v>
+        <v>184</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="24" t="s">
-        <v>293</v>
+        <v>185</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="24" t="s">
-        <v>294</v>
+        <v>186</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="24" t="s">
-        <v>295</v>
+        <v>187</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="23" t="s">
-        <v>296</v>
+        <v>188</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="24" t="s">
-        <v>297</v>
+        <v>189</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="24" t="s">
-        <v>298</v>
+        <v>190</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="24" t="s">
-        <v>299</v>
+        <v>191</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="24" t="s">
-        <v>300</v>
+        <v>192</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="23" t="s">
-        <v>301</v>
+        <v>193</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="24" t="s">
-        <v>302</v>
+        <v>194</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="24" t="s">
-        <v>303</v>
+        <v>195</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="24" t="s">
-        <v>304</v>
+        <v>196</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="24" t="s">
-        <v>305</v>
+        <v>197</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="24" t="s">
-        <v>306</v>
+        <v>198</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="24" t="s">
-        <v>307</v>
+        <v>199</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="23" t="s">
-        <v>308</v>
+        <v>200</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="24" t="s">
-        <v>309</v>
+        <v>201</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="24" t="s">
-        <v>310</v>
+        <v>202</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="24" t="s">
-        <v>311</v>
+        <v>203</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="24" t="s">
-        <v>312</v>
+        <v>204</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="23" t="s">
-        <v>313</v>
+        <v>205</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="24" t="s">
-        <v>314</v>
+        <v>206</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="24" t="s">
-        <v>315</v>
+        <v>207</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="24" t="s">
-        <v>316</v>
+        <v>208</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="24" t="s">
-        <v>317</v>
+        <v>209</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="24" t="s">
-        <v>318</v>
+        <v>210</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="24" t="s">
-        <v>319</v>
+        <v>211</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="23" t="s">
-        <v>320</v>
+        <v>212</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="24" t="s">
-        <v>321</v>
+        <v>213</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="24" t="s">
-        <v>322</v>
+        <v>214</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="24" t="s">
-        <v>323</v>
+        <v>215</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="24" t="s">
-        <v>324</v>
+        <v>216</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="23" t="s">
-        <v>325</v>
+        <v>217</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="24" t="s">
-        <v>326</v>
+        <v>218</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="24" t="s">
-        <v>327</v>
+        <v>219</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="24" t="s">
-        <v>328</v>
+        <v>220</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="24" t="s">
-        <v>329</v>
+        <v>221</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="24" t="s">
-        <v>330</v>
+        <v>222</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="24" t="s">
-        <v>331</v>
+        <v>223</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="24" t="s">
-        <v>332</v>
+        <v>224</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="24" t="s">
-        <v>333</v>
+        <v>225</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="24" t="s">
-        <v>334</v>
+        <v>226</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="24" t="s">
-        <v>335</v>
+        <v>227</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="24" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="24" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="24" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="24" t="s">
-        <v>339</v>
+        <v>231</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A96" s="23" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A97" s="24" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A98" s="24" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A99" s="24" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A100" s="24" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A101" s="24" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A102" s="24" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A103" s="24" t="s">
+        <v>239</v>
       </c>
     </row>
   </sheetData>
@@ -4905,7 +4237,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
@@ -4917,24 +4249,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>340</v>
+        <v>240</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>341</v>
+        <v>241</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>342</v>
+        <v>242</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>268</v>
+        <v>160</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>343</v>
+        <v>243</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>344</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4942,92 +4274,97 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>345</v>
+        <v>245</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$49,A5)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$28,A5)</f>
         <v>12</v>
       </c>
       <c r="D5" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$49,A5,'Product Backlog'!$G$5:$G$49)</f>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$28,A5,'Product Backlog'!$G$5:$G$28)</f>
         <v>43</v>
       </c>
       <c r="E5" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D5/SUM($D$5:$D$8))</f>
-        <v>0.265432098765432</v>
+        <v>0.558441558441558</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>346</v>
+        <v>246</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$49,A6)</f>
-        <v>7</v>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$28,A6)</f>
+        <v>9</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$49,A6,'Product Backlog'!$G$5:$G$49)</f>
-        <v>22</v>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$28,A6,'Product Backlog'!$G$5:$G$28)</f>
+        <v>27</v>
       </c>
       <c r="E6" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D6/SUM($D$5:$D$8))</f>
-        <v>0.135802469135802</v>
+        <v>0.350649350649351</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>113</v>
+        <v>138</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>347</v>
+        <v>247</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$49,A7)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$28,A7)</f>
         <v>3</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$49,A7,'Product Backlog'!$G$5:$G$49)</f>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$28,A7,'Product Backlog'!$G$5:$G$28)</f>
         <v>7</v>
       </c>
       <c r="E7" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D7/SUM($D$5:$D$8))</f>
-        <v>0.0432098765432099</v>
+        <v>0.0909090909090909</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>146</v>
+        <v>248</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>348</v>
+        <v>249</v>
       </c>
       <c r="C8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$49,A8)</f>
-        <v>22</v>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$28,A8)</f>
+        <v>0</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$49,A8,'Product Backlog'!$G$5:$G$49)</f>
-        <v>90</v>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$28,A8,'Product Backlog'!$G$5:$G$28)</f>
+        <v>0</v>
       </c>
       <c r="E8" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D8/SUM($D$5:$D$8))</f>
-        <v>0.555555555555556</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>279</v>
+        <v>171</v>
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>
-        <v>44</v>
+        <v>24</v>
       </c>
       <c r="D9" s="27" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>162</v>
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="28" t="s">
+        <v>250</v>
       </c>
     </row>
   </sheetData>
@@ -5039,4 +4376,686 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:H28"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="44"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="29" t="s">
+        <v>252</v>
+      </c>
+      <c r="B2" s="29"/>
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+    </row>
+    <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>253</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>261</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>262</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>263</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="H6" s="6" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>267</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>268</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>270</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>284</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>289</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>290</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>301</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>302</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>303</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="s">
+        <v>297</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>305</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="E14" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>312</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>313</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>314</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>323</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>324</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>327</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>328</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>329</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>308</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>299</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="s">
+        <v>335</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>337</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="E20" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>342</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>315</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>300</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>346</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>348</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>321</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>350</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
+        <v>353</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>336</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>356</v>
+      </c>
+      <c r="E24" s="6" t="s">
+        <v>357</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="s">
+        <v>358</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>360</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>361</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>362</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>311</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>365</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>366</v>
+      </c>
+      <c r="E26" s="6" t="s">
+        <v>367</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>364</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="6" t="s">
+        <v>369</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>370</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>371</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>373</v>
+      </c>
+      <c r="F27" s="6"/>
+      <c r="G27" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="E28" s="9" t="s">
+        <v>375</v>
+      </c>
+      <c r="F28" s="9" t="n">
+        <f aca="false">SUM(F5:F27)</f>
+        <v>90</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:H27"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
US04 dividida: a recolha completa da DGES passa a ser a US48 (decisão do PO, 27/10)
A US04 fica com o catálogo recolhido da DGES (174 cursos, condições de
acesso, paginação, filtro para o LLM). Correr a recolha de todas as
licenciaturas exige o computador ligado uma noite inteira e passa para a
US48 (Backlog, 2 SP). Backlog, requisitos, visão e PROJETO.md atualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VGMz7jsnoKnqj32HjKSCN6
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -16,7 +16,7 @@
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Arquivo (opcionais)'!$A$4:$H$27</definedName>
     <definedName function="false" hidden="false" localSheetId="0" name="_xlnm.Print_Titles" vbProcedure="false">'Product Backlog'!$4:$4</definedName>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$28</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">'Product Backlog'!$A$4:$M$29</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="542" uniqueCount="376">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="382">
   <si>
     <t xml:space="preserve">Product Backlog — OptaBem (recomendador de cursos e plano de candidatura)</t>
   </si>
@@ -312,14 +312,14 @@
     <t xml:space="preserve">US10</t>
   </si>
   <si>
-    <t xml:space="preserve">Catálogo completo de licenciaturas (DGES)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como pessoa indecisa, quero procurar em todas as licenciaturas do concurso nacional, e não só numa amostra, para não deixar de fora um curso que me sirva.</t>
+    <t xml:space="preserve">Catálogo de licenciaturas recolhido da DGES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como pessoa indecisa, quero procurar num catálogo de licenciaturas recolhido da DGES, e não só numa amostra escrita à mão, para ver cursos de muitas instituições com dados oficiais.</t>
   </si>
   <si>
     <t xml:space="preserve">• Os cursos vêm das páginas públicas da DGES, por um script que corre no computador da equipa (dados/recolher_dges.py), devagar e retomável.
-• O catálogo tem as licenciaturas e mestrados integrados do concurso nacional, com vagas, nota do último colocado e condições de acesso.
+• O catálogo tem os cursos já recolhidos (174 no protótipo), com vagas, nota do último colocado e condições de acesso.
 • As descrições escritas pela equipa (catálogo do MVP) mantêm-se.
 • Lista de cursos com paginação (24 por página).
 • Acima de 150 cursos, o assistente (LLM) recebe só os cursos das áreas escolhidas.</t>
@@ -331,7 +331,7 @@
     <t xml:space="preserve">Protótipo</t>
   </si>
   <si>
-    <t xml:space="preserve">Protótipo no ramo feature/US04-catalogo-completo, incluído no PR #44: 174 cursos com condições de acesso. Falta a recolha completa e a documentação. Reescrita a 23/10 (antes: importar um CSV na gestão).</t>
+    <t xml:space="preserve">Protótipo no PR #44 (ramo feature/US04-catalogo-completo): 174 cursos com condições de acesso. 27/10 (decisão do PO): a recolha de todas as licenciaturas passa para a US48, porque exige o computador ligado uma noite inteira. Falta a documentação da story.</t>
   </si>
   <si>
     <t xml:space="preserve">US33</t>
@@ -535,6 +535,23 @@
     <t xml:space="preserve">27/10: story nova, para a parte do RF02 que não tinha story. Precisa de o site enviar emails reais (hoje não envia).</t>
   </si>
   <si>
+    <t xml:space="preserve">US48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recolha completa das licenciaturas (DGES)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como pessoa indecisa, quero que o catálogo tenha todas as licenciaturas e mestrados integrados do concurso nacional, para não deixar de fora um curso que me sirva.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• O script da US04 corre até ao fim sobre todas as instituições do concurso nacional.
+• O dados/README.md diz quantos cursos ficaram e quantos não têm condições de acesso ou nota do último colocado.
+• A aplicação e os testes continuam a funcionar com o catálogo completo (RNF03: páginas em menos de 2 s).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">27/10: separada da US04 (decisão do PO). O código já existe; falta correr a recolha, que exige o computador ligado uma noite inteira.</t>
+  </si>
+  <si>
     <t xml:space="preserve">US39</t>
   </si>
   <si>
@@ -667,7 +684,7 @@
     <t xml:space="preserve">Fora desta release, por ordem de prioridade. As US40 a US45 têm código pronto no PR #44 (protótipo). As opcionais estão na folha «Arquivo (opcionais)».</t>
   </si>
   <si>
-    <t xml:space="preserve">US40–US42, US44, US37, US46, US47, US39, US43, US45, US38</t>
+    <t xml:space="preserve">US40–US42, US44, US37, US46, US47, US48, US39, US43, US45, US38</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -869,6 +886,9 @@
   </si>
   <si>
     <t xml:space="preserve">• Stories novas no backlog: US46 (exportar os meus dados, a parte do RF17 que saiu da US17) e US47 (recuperar a palavra-passe, a parte do RF02 sem story).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• US04 dividida (decisão do PO): fica o catálogo recolhido da DGES com os 174 cursos já recolhidos; a recolha de todas as licenciaturas passa a ser a US48 (Backlog), porque exige o computador ligado uma noite inteira.</t>
   </si>
   <si>
     <t xml:space="preserve">• As notas de cada story passam a dizer só o estado atual; o histórico fica nesta folha.</t>
@@ -1687,7 +1707,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="21">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1800,6 +1820,13 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDDEBF7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2135,11 +2162,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="44034424"/>
-        <c:axId val="32648971"/>
+        <c:axId val="22608981"/>
+        <c:axId val="88979086"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="44034424"/>
+        <c:axId val="22608981"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2170,7 +2197,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="32648971"/>
+        <c:crossAx val="88979086"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2178,7 +2205,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="32648971"/>
+        <c:axId val="88979086"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2243,7 +2270,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44034424"/>
+        <c:crossAx val="22608981"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2310,9 +2337,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2087280</xdr:colOff>
+      <xdr:colOff>2087640</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>84240</xdr:rowOff>
+      <xdr:rowOff>84600</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2321,7 +2348,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5752440" cy="2512080"/>
+        <a:ext cx="5752800" cy="2512440"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3385,7 +3412,7 @@
         <v>132</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H25" s="5" t="s">
         <v>93</v>
@@ -3412,7 +3439,7 @@
         <v>134</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>73</v>
+        <v>53</v>
       </c>
       <c r="D26" s="6" t="s">
         <v>135</v>
@@ -3424,20 +3451,20 @@
         <v>137</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>138</v>
+        <v>93</v>
       </c>
       <c r="I26" s="7" t="s">
         <v>99</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>70</v>
+        <v>117</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
-        <v>100</v>
+        <v>138</v>
       </c>
       <c r="M26" s="5" t="s">
         <v>78</v>
@@ -3463,10 +3490,10 @@
         <v>142</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I27" s="7" t="s">
         <v>99</v>
@@ -3487,66 +3514,104 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>73</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G28" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="I28" s="7" t="s">
         <v>99</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>117</v>
+        <v>70</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8" t="s">
-        <v>147</v>
+        <v>100</v>
       </c>
       <c r="M28" s="5" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F29" s="9" t="s">
+    <row r="29" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="5" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="G29" s="9" t="n">
-        <f aca="false">SUM(G5:G28)</f>
-        <v>77</v>
+      <c r="C29" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="G29" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" s="5" t="s">
+        <v>143</v>
+      </c>
+      <c r="I29" s="7" t="s">
+        <v>99</v>
+      </c>
+      <c r="J29" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="K29" s="8"/>
+      <c r="L29" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="M29" s="5" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F30" s="9" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="G30" s="9" t="n">
-        <f aca="false">SUMIF(J5:J28,"Feito",G5:G28)</f>
+        <f aca="false">SUM(G5:G29)</f>
+        <v>79</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F31" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="G31" s="9" t="n">
+        <f aca="false">SUMIF(J5:J29,"Feito",G5:G29)</f>
         <v>30</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F31" s="10" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="F32" s="10" t="s">
+        <v>155</v>
+      </c>
+    </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="34" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="35" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="36" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="37" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3566,8 +3631,8 @@
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="52" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A4:M28"/>
-  <conditionalFormatting sqref="J5:J28">
+  <autoFilter ref="A4:M29"/>
+  <conditionalFormatting sqref="J5:J29">
     <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>"Feito"</formula>
     </cfRule>
@@ -3578,51 +3643,51 @@
       <formula>"Protótipo"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H5:H28">
+  <conditionalFormatting sqref="H5:H29">
     <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>"Must"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Should"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Could"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>"Won't"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:I28">
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+  <conditionalFormatting sqref="I5:I29">
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Sprint 1"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Sprint 2"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Sprint 3"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"Sprint 4"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="13" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="13" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
       <formula>"Backlog"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G28" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G5:G29" type="list">
       <formula1>"1,2,3,5,8,13,21"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H28" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="H5:H29" type="list">
       <formula1>"Must,Should,Could,Won't"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I28" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="I5:I29" type="list">
       <formula1>"Sprint 1,Sprint 2,Sprint 3,Sprint 4,Backlog"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J28" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="J5:J29" type="list">
       <formula1>"Por fazer,Protótipo,Em curso,Feito"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3644,7 +3709,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H103"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -3659,17 +3724,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>10</v>
@@ -3680,25 +3745,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3706,17 +3771,17 @@
         <v>21</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$28,$A6,'Product Backlog'!$G$5:$G$28)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$29,$A6,'Product Backlog'!$G$5:$G$29)</f>
         <v>10</v>
       </c>
       <c r="E6" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$28,'Product Backlog'!$I$5:$I$28,$A6,'Product Backlog'!$J$5:$J$28,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$29,'Product Backlog'!$I$5:$I$29,$A6,'Product Backlog'!$J$5:$J$29,"Feito")</f>
         <v>10</v>
       </c>
       <c r="F6" s="15" t="n">
@@ -3728,7 +3793,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$28,$A6)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$29,$A6)</f>
         <v>3</v>
       </c>
     </row>
@@ -3737,17 +3802,17 @@
         <v>40</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$28,$A7,'Product Backlog'!$G$5:$G$28)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$29,$A7,'Product Backlog'!$G$5:$G$29)</f>
         <v>13</v>
       </c>
       <c r="E7" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$28,'Product Backlog'!$I$5:$I$28,$A7,'Product Backlog'!$J$5:$J$28,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$29,'Product Backlog'!$I$5:$I$29,$A7,'Product Backlog'!$J$5:$J$29,"Feito")</f>
         <v>13</v>
       </c>
       <c r="F7" s="15" t="n">
@@ -3759,7 +3824,7 @@
         <v>-3</v>
       </c>
       <c r="H7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$28,$A7)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$29,$A7)</f>
         <v>3</v>
       </c>
     </row>
@@ -3768,17 +3833,17 @@
         <v>57</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$28,$A8,'Product Backlog'!$G$5:$G$28)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$29,$A8,'Product Backlog'!$G$5:$G$29)</f>
         <v>7</v>
       </c>
       <c r="E8" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$28,'Product Backlog'!$I$5:$I$28,$A8,'Product Backlog'!$J$5:$J$28,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$29,'Product Backlog'!$I$5:$I$29,$A8,'Product Backlog'!$J$5:$J$29,"Feito")</f>
         <v>7</v>
       </c>
       <c r="F8" s="15" t="n">
@@ -3790,7 +3855,7 @@
         <v>3</v>
       </c>
       <c r="H8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$28,$A8)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$29,$A8)</f>
         <v>2</v>
       </c>
     </row>
@@ -3799,17 +3864,17 @@
         <v>69</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D9" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$28,$A9,'Product Backlog'!$G$5:$G$28)</f>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$29,$A9,'Product Backlog'!$G$5:$G$29)</f>
         <v>18</v>
       </c>
       <c r="E9" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$28,'Product Backlog'!$I$5:$I$28,$A9,'Product Backlog'!$J$5:$J$28,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$29,'Product Backlog'!$I$5:$I$29,$A9,'Product Backlog'!$J$5:$J$29,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F9" s="15" t="n">
@@ -3821,7 +3886,7 @@
         <v>-8</v>
       </c>
       <c r="H9" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$28,$A9)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$29,$A9)</f>
         <v>5</v>
       </c>
     </row>
@@ -3830,17 +3895,17 @@
         <v>99</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="D10" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$28,$A10,'Product Backlog'!$G$5:$G$28)</f>
-        <v>29</v>
+        <f aca="false">SUMIF('Product Backlog'!$I$5:$I$29,$A10,'Product Backlog'!$G$5:$G$29)</f>
+        <v>31</v>
       </c>
       <c r="E10" s="5" t="n">
-        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$28,'Product Backlog'!$I$5:$I$28,$A10,'Product Backlog'!$J$5:$J$28,"Feito")</f>
+        <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$29,'Product Backlog'!$I$5:$I$29,$A10,'Product Backlog'!$J$5:$J$29,"Feito")</f>
         <v>0</v>
       </c>
       <c r="F10" s="15" t="n">
@@ -3851,19 +3916,19 @@
         <v>34</v>
       </c>
       <c r="H10" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$28,$A10)</f>
-        <v>11</v>
+        <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$29,$A10)</f>
+        <v>12</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
       <c r="D11" s="21" t="n">
         <f aca="false">SUM(D6:D10)</f>
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E11" s="21" t="n">
         <f aca="false">SUM(E6:E10)</f>
@@ -3871,352 +3936,357 @@
       </c>
       <c r="F11" s="22" t="n">
         <f aca="false">IF(D11=0,0,E11/D11)</f>
-        <v>0.38961038961039</v>
+        <v>0.379746835443038</v>
       </c>
       <c r="G11" s="21"/>
       <c r="H11" s="21" t="n">
         <f aca="false">SUM(H6:H10)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="24" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="24" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="24" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="23" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="24" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="24" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="24" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="24" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="23" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="24" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="24" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="24" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="24" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="24" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="24" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="23" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="24" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="24" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="24" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="24" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="23" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="24" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="24" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="24" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="24" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="24" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="24" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="23" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="24" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="24" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="24" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="24" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="23" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="24" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="24" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="24" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="24" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="24" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="24" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="24" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="24" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="24" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="24" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="24" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="24" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="24" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="24" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="23" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="24" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="24" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="24" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="24" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="24" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="24" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="24" t="s">
-        <v>239</v>
+        <v>244</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A104" s="24" t="s">
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -4249,24 +4319,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4274,19 +4344,19 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="C5" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$28,A5)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$29,A5)</f>
         <v>12</v>
       </c>
       <c r="D5" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$28,A5,'Product Backlog'!$G$5:$G$28)</f>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$29,A5,'Product Backlog'!$G$5:$G$29)</f>
         <v>43</v>
       </c>
       <c r="E5" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D5/SUM($D$5:$D$8))</f>
-        <v>0.558441558441558</v>
+        <v>0.544303797468354</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4294,54 +4364,54 @@
         <v>93</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="C6" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$28,A6)</f>
-        <v>9</v>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$29,A6)</f>
+        <v>10</v>
       </c>
       <c r="D6" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$28,A6,'Product Backlog'!$G$5:$G$28)</f>
-        <v>27</v>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$29,A6,'Product Backlog'!$G$5:$G$29)</f>
+        <v>29</v>
       </c>
       <c r="E6" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D6/SUM($D$5:$D$8))</f>
-        <v>0.350649350649351</v>
+        <v>0.367088607594937</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="C7" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$28,A7)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$29,A7)</f>
         <v>3</v>
       </c>
       <c r="D7" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$28,A7,'Product Backlog'!$G$5:$G$28)</f>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$29,A7,'Product Backlog'!$G$5:$G$29)</f>
         <v>7</v>
       </c>
       <c r="E7" s="15" t="n">
         <f aca="false">IF(SUM($D$5:$D$8)=0,0,D7/SUM($D$5:$D$8))</f>
-        <v>0.0909090909090909</v>
+        <v>0.0886075949367089</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="C8" s="5" t="n">
-        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$28,A8)</f>
+        <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$29,A8)</f>
         <v>0</v>
       </c>
       <c r="D8" s="5" t="n">
-        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$28,A8,'Product Backlog'!$G$5:$G$28)</f>
+        <f aca="false">SUMIF('Product Backlog'!$H$5:$H$29,A8,'Product Backlog'!$G$5:$G$29)</f>
         <v>0</v>
       </c>
       <c r="E8" s="15" t="n">
@@ -4351,20 +4421,20 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D9" s="27" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
     </row>
   </sheetData>
@@ -4386,24 +4456,24 @@
   <dimension ref="A1:H28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="44"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
@@ -4413,12 +4483,12 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>5</v>
@@ -4436,24 +4506,24 @@
         <v>14</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>5</v>
@@ -4462,111 +4532,111 @@
         <v>52</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>5</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>73</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4574,302 +4644,302 @@
         <v>65</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>5</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="F11" s="6" t="n">
         <v>8</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>295</v>
+        <v>301</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>296</v>
+        <v>302</v>
       </c>
       <c r="F12" s="6" t="n">
         <v>2</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>298</v>
+        <v>304</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>301</v>
+        <v>307</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>302</v>
+        <v>308</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>303</v>
+        <v>309</v>
       </c>
       <c r="F13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>304</v>
+        <v>310</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>297</v>
+        <v>303</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>305</v>
+        <v>311</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>306</v>
+        <v>312</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
       <c r="F14" s="6" t="n">
         <v>5</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
       <c r="F15" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>318</v>
+        <v>324</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>319</v>
+        <v>325</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
       <c r="F16" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>322</v>
+        <v>328</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>323</v>
+        <v>329</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>324</v>
+        <v>330</v>
       </c>
       <c r="F17" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>326</v>
+        <v>332</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>327</v>
+        <v>333</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>328</v>
+        <v>334</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="F18" s="6" t="n">
         <v>2</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="F19" s="6" t="n">
         <v>5</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>299</v>
+        <v>305</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>334</v>
+        <v>340</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>335</v>
+        <v>341</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>337</v>
+        <v>343</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>338</v>
+        <v>344</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>339</v>
+        <v>345</v>
       </c>
       <c r="F20" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>341</v>
+        <v>347</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>340</v>
+        <v>346</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>342</v>
+        <v>348</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>344</v>
+        <v>350</v>
       </c>
       <c r="F21" s="6" t="n">
         <v>3</v>
@@ -4878,166 +4948,166 @@
         <v>60</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>345</v>
+        <v>351</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>300</v>
+        <v>306</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>346</v>
+        <v>352</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>347</v>
+        <v>353</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>348</v>
+        <v>354</v>
       </c>
       <c r="F22" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>321</v>
+        <v>327</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>349</v>
+        <v>355</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>325</v>
+        <v>331</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>350</v>
+        <v>356</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>351</v>
+        <v>357</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="F23" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>336</v>
+        <v>342</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="F24" s="6" t="n">
         <v>5</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>359</v>
+        <v>365</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>358</v>
+        <v>364</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>360</v>
+        <v>366</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>361</v>
+        <v>367</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>362</v>
+        <v>368</v>
       </c>
       <c r="F25" s="6" t="n">
         <v>8</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>317</v>
+        <v>323</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>363</v>
+        <v>369</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>365</v>
+        <v>371</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>366</v>
+        <v>372</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>367</v>
+        <v>373</v>
       </c>
       <c r="F26" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>364</v>
+        <v>370</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>368</v>
+        <v>374</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>369</v>
+        <v>375</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>370</v>
+        <v>376</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="6" t="s">
         <v>78</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E28" s="9" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="F28" s="9" t="n">
         <f aca="false">SUM(F5:F27)</f>

</xml_diff>

<commit_message>
Documentação das stories do Sprint 4 (US04, US33 a US36) e testes em falta
- docs/US04 e docs/US33 a docs/US36: README, requisitos, use case, BPMN,
  prompt e diagramas (gerar.py), com a estrutura das stories anteriores.
- US35: a ficha do curso passa a mostrar o aviso de estimativa junto à nota
  (o critério de aceitação pedia-o; antes só o plano o tinha).
- Testes novos: leitura das condições de acesso nas páginas guardadas da DGES
  (US33), ficha sem sessão (US33), aviso de estimativa (US35), avisos de
  opções que não contam e de pré-requisitos (US36), curso escolhido como
  1.ª opção (US36). 430 testes a passar.
- Índices (docs/README.md, PROJETO.md), notas do backlog e registo de uso de IA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VGMz7jsnoKnqj32HjKSCN6
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -331,7 +331,7 @@
     <t xml:space="preserve">Protótipo</t>
   </si>
   <si>
-    <t xml:space="preserve">Protótipo no PR #44 (ramo feature/US04-catalogo-completo): 174 cursos com condições de acesso. 27/10 (decisão do PO): a recolha de todas as licenciaturas passa para a US48, porque exige o computador ligado uma noite inteira. Falta a documentação da story.</t>
+    <t xml:space="preserve">Protótipo no PR #44 (ramo feature/US04-catalogo-completo): 174 cursos com condições de acesso. 27/10 (decisão do PO): a recolha de todas as licenciaturas passa para a US48, porque exige o computador ligado uma noite inteira. Documentação em docs/US04/ (27/10).</t>
   </si>
   <si>
     <t xml:space="preserve">US33</t>
@@ -353,7 +353,7 @@
 • Funciona sem sessão iniciada.</t>
   </si>
   <si>
-    <t xml:space="preserve">Protótipo no PR #44, feito antes do sprint (23/10). Falta a documentação da story (requisitos, use case, BPMN).</t>
+    <t xml:space="preserve">Protótipo no PR #44, feito antes do sprint (23/10). Documentação em docs/US33/ (27/10).</t>
   </si>
   <si>
     <t xml:space="preserve">nova</t>
@@ -374,7 +374,7 @@
 • Matemática e Matemática A contam com o mesmo exame (a confirmar pela equipa na DGES).</t>
   </si>
   <si>
-    <t xml:space="preserve">Protótipo no PR #44, feito antes do sprint (23/10). Falta a documentação da story (requisitos, use case, BPMN). A equipa confirma na DGES se Matemática e Matemática A contam como o mesmo exame.</t>
+    <t xml:space="preserve">Protótipo no PR #44, feito antes do sprint (23/10). Documentação em docs/US34/ (27/10). A equipa confirma na DGES se Matemática e Matemática A contam como o mesmo exame.</t>
   </si>
   <si>
     <t xml:space="preserve">US35</t>
@@ -392,7 +392,7 @@
 • Aviso visível: estimativa para o contingente geral da 1.ª fase, não uma garantia.</t>
   </si>
   <si>
-    <t xml:space="preserve">Protótipo no PR #44, feito antes do sprint (23/10). Falta a documentação da story (requisitos, use case, BPMN). Contas em app/candidatura/calculos.py.</t>
+    <t xml:space="preserve">Protótipo no PR #44, feito antes do sprint (23/10). Documentação em docs/US35/ (27/10). Contas em app/candidatura/calculos.py.</t>
   </si>
   <si>
     <t xml:space="preserve">US36</t>
@@ -414,7 +414,7 @@
     <t xml:space="preserve">Should</t>
   </si>
   <si>
-    <t xml:space="preserve">Protótipo no PR #44, feito antes do sprint (23/10). Falta a documentação da story (requisitos, use case, BPMN). O OptaBem ajuda a preparar a candidatura, não a submete. Se o Sprint 4 for demais, é a primeira a sair.</t>
+    <t xml:space="preserve">Protótipo no PR #44, feito antes do sprint (23/10). Documentação em docs/US36/ (27/10). O OptaBem ajuda a preparar a candidatura, não a submete. Se o Sprint 4 for demais, é a primeira a sair.</t>
   </si>
   <si>
     <t xml:space="preserve">US40</t>
@@ -1690,7 +1690,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1707,7 +1707,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="21">
+  <dxfs count="20">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1820,13 +1820,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFF8CBAD"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFDDEBF7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2162,11 +2155,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="22608981"/>
-        <c:axId val="88979086"/>
+        <c:axId val="87705679"/>
+        <c:axId val="59618585"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="22608981"/>
+        <c:axId val="87705679"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2197,7 +2190,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="88979086"/>
+        <c:crossAx val="59618585"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2205,7 +2198,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="88979086"/>
+        <c:axId val="59618585"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2270,7 +2263,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="22608981"/>
+        <c:crossAx val="87705679"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2337,9 +2330,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2087640</xdr:colOff>
+      <xdr:colOff>2087280</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>84600</xdr:rowOff>
+      <xdr:rowOff>84240</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2348,7 +2341,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5752800" cy="2512440"/>
+        <a:ext cx="5752440" cy="2512080"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3647,30 +3640,30 @@
     <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>"Must"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Should"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Could"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Won't"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5:I29">
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
       <formula>"Sprint 1"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Sprint 2"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>"Sprint 3"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Sprint 4"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="13" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
+    <cfRule type="cellIs" priority="13" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"Backlog"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4244,47 +4237,47 @@
         <v>236</v>
       </c>
     </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="23" t="s">
         <v>237</v>
       </c>
     </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="24" t="s">
         <v>238</v>
       </c>
     </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="24" t="s">
         <v>239</v>
       </c>
     </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="24" t="s">
         <v>240</v>
       </c>
     </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="24" t="s">
         <v>241</v>
       </c>
     </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="24" t="s">
         <v>242</v>
       </c>
     </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="24" t="s">
         <v>243</v>
       </c>
     </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="24" t="s">
         <v>244</v>
       </c>
     </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="24" t="s">
         <v>245</v>
       </c>
@@ -4432,7 +4425,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
         <v>256</v>
       </c>
@@ -4456,17 +4449,17 @@
   <dimension ref="A1:H28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="44"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
         <v>257</v>
       </c>
@@ -4483,7 +4476,7 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
@@ -5105,7 +5098,7 @@
         <v>380</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="E28" s="9" t="s">
         <v>381</v>
       </c>

</xml_diff>

<commit_message>
US40 a US45 no Sprint 4 (decisão do PO, 27/10) e a sua documentação
- Backlog: US40 a US45 passam do Backlog para o Sprint 4 (32 SP), com a nota
  de que só se defende porque o código foi feito antes, como protótipo.
  Requisitos, visão e PROJETO.md alinhados.
- docs/US40 a docs/US45: README, requisitos, use case, BPMN, prompt e
  diagramas.
- Testes novos: «Precisa de X em Y» e tendência em cada opção do plano
  (US40, US41); aviso das vagas da 2.ª fase (US45).
- Texto do plano B vazio deixa de citar uma story.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VGMz7jsnoKnqj32HjKSCN6
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -84,7 +84,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="557" uniqueCount="391">
   <si>
     <t xml:space="preserve">Product Backlog — OptaBem (recomendador de cursos e plano de candidatura)</t>
   </si>
@@ -414,7 +414,7 @@
     <t xml:space="preserve">Should</t>
   </si>
   <si>
-    <t xml:space="preserve">Protótipo no PR #44, feito antes do sprint (23/10). Documentação em docs/US36/ (27/10). O OptaBem ajuda a preparar a candidatura, não a submete. Se o Sprint 4 for demais, é a primeira a sair.</t>
+    <t xml:space="preserve">Protótipo no PR #44, feito antes do sprint (23/10). Documentação em docs/US36/ (27/10). O OptaBem ajuda a preparar a candidatura, não a submete. Se o Sprint 4 for demais, saem primeiro as Could (US43 e US45).</t>
   </si>
   <si>
     <t xml:space="preserve">US40</t>
@@ -433,10 +433,7 @@
 • No plano, as opções a que falta uma prova mostram quanto precisa.</t>
   </si>
   <si>
-    <t xml:space="preserve">Backlog</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Código pronto no PR #44 (protótipo de 23/10, ideia proposta pelo Claude e aceite pelo PO). Fica no backlog porque o Sprint 4 já passa a velocidade; é aceite numa Sprint Review se houver folga.</t>
+    <t xml:space="preserve">Protótipo no PR #44 (23/10, ideia proposta pelo Claude e aceite pelo PO). 27/10: entra no Sprint 4 por decisão do PO. Documentação em docs/US40/ (27/10).</t>
   </si>
   <si>
     <t xml:space="preserve">US41</t>
@@ -453,6 +450,9 @@
 • A etiqueta aparece também em cada opção do plano.</t>
   </si>
   <si>
+    <t xml:space="preserve">Protótipo no PR #44 (23/10, ideia proposta pelo Claude e aceite pelo PO). 27/10: entra no Sprint 4 por decisão do PO. Documentação em docs/US41/ (27/10).</t>
+  </si>
+  <si>
     <t xml:space="preserve">US42</t>
   </si>
   <si>
@@ -464,6 +464,9 @@
   <si>
     <t xml:space="preserve">• Candidatos, candidatos em 1.ª opção, vagas e colocados da 1.ª fase de 2025 (DGES), na ficha do curso.
 • Etiqueta: «Sobraram vagas», «Muito procurado» (1,5 ou mais em 1.ª opção por vaga), «Procurado» (0,75 a 1,5) ou «Pouco escolhido em 1.ª opção».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protótipo no PR #44 (23/10, ideia proposta pelo Claude e aceite pelo PO). 27/10: entra no Sprint 4 por decisão do PO. Documentação em docs/US42/ (27/10).</t>
   </si>
   <si>
     <t xml:space="preserve">US44</t>
@@ -481,6 +484,47 @@
 • Matemática e Matemática A contam como o mesmo exame.</t>
   </si>
   <si>
+    <t xml:space="preserve">Protótipo no PR #44 (23/10, ideia proposta pelo Claude e aceite pelo PO). 27/10: entra no Sprint 4 por decisão do PO. Documentação em docs/US44/ (27/10).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partilhar o plano</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como candidato, quero partilhar o meu plano com quem me ajuda a decidir (pais, explicador), com uma ligação só de leitura, para pedir opinião sem dar a minha palavra-passe.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Ligação com um código aleatório; quem a tem vê o plano sem iniciar sessão.
+• Mostra o primeiro nome, as opções, a nota de candidatura e a situação; nunca o email, a média nem os exames.
+• «Deixar de partilhar» invalida a ligação de imediato.
+• A página não é indexada pelos motores de pesquisa.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Could</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protótipo no PR #44 (23/10, ideia proposta pelo Claude e aceite pelo PO). 27/10: entra no Sprint 4 por decisão do PO. Documentação em docs/US43/ (27/10).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Plano B: 2.ª fase</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Como candidato, quero ver cursos das áreas do meu plano que tiveram vagas na 2.ª fase e a que a minha nota chegava, para ter uma alternativa se não entrar na 1.ª fase.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Vagas, colocados e último colocado da 2.ª fase de 2025 (DGES).
+• Só cursos fora do plano, das mesmas áreas, onde a nota da pessoa chegava ao último colocado da 2.ª fase (ou, sem essa nota, onde sobraram vagas).
+• Aviso: as vagas da 2.ª fase são as que sobram da 1.ª e mudam todos os anos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Protótipo no PR #44 (23/10, ideia proposta pelo Claude e aceite pelo PO). 27/10: entra no Sprint 4 por decisão do PO. Documentação em docs/US45/ (27/10).</t>
+  </si>
+  <si>
     <t xml:space="preserve">US37</t>
   </si>
   <si>
@@ -493,6 +537,9 @@
     <t xml:space="preserve">• Só com autorização da pessoa, o LLM recebe as provas feitas e um intervalo de nota (nunca a média exata, RNF12).
 • Cursos a que falta uma prova não são sugeridos, ou vêm assinalados.
 • Os testes usam o LLM falso.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Backlog</t>
   </si>
   <si>
     <t xml:space="preserve">Por fazer</t>
@@ -570,38 +617,6 @@
     <t xml:space="preserve">Sugestão de um colega (editar a base de dados na gestão), reescrita com uma necessidade concreta: um editor genérico de tabelas daria aos administradores os dados dos alunos. Precisa do catálogo na base de dados.</t>
   </si>
   <si>
-    <t xml:space="preserve">US43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Partilhar o plano</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como candidato, quero partilhar o meu plano com quem me ajuda a decidir (pais, explicador), com uma ligação só de leitura, para pedir opinião sem dar a minha palavra-passe.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Ligação com um código aleatório; quem a tem vê o plano sem iniciar sessão.
-• Mostra o primeiro nome, as opções, a nota de candidatura e a situação; nunca o email, a média nem os exames.
-• «Deixar de partilhar» invalida a ligação de imediato.
-• A página não é indexada pelos motores de pesquisa.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Could</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Plano B: 2.ª fase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Como candidato, quero ver cursos das áreas do meu plano que tiveram vagas na 2.ª fase e a que a minha nota chegava, para ter uma alternativa se não entrar na 1.ª fase.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Vagas, colocados e último colocado da 2.ª fase de 2025 (DGES).
-• Só cursos fora do plano, das mesmas áreas, onde a nota da pessoa chegava ao último colocado da 2.ª fase (ou, sem essa nota, onde sobraram vagas).
-• Aviso: as vagas da 2.ª fase são as que sobram da 1.ª e mudam todos os anos.</t>
-  </si>
-  <si>
     <t xml:space="preserve">US38</t>
   </si>
   <si>
@@ -624,7 +639,7 @@
     <t xml:space="preserve">Story points concluídos (Estado = Feito)</t>
   </si>
   <si>
-    <t xml:space="preserve">Nota (27/10): as 22 stories das opcionais e a US32 (fundida na US29) estão na folha «Arquivo (opcionais)», com o motivo de cada uma. As US40 a US45 têm código no PR #44 mas ficam fora do Sprint 4, para o plano não passar ainda mais a velocidade.</t>
+    <t xml:space="preserve">Nota (27/10): as 22 stories das opcionais e a US32 (fundida na US29) estão na folha «Arquivo (opcionais)», com o motivo de cada uma. As US40 a US45 entraram no Sprint 4 a 27/10 (decisão do PO): o código estava feito; no sprint sobra documentação, testes e revisão.</t>
   </si>
   <si>
     <t xml:space="preserve">Plano de sprints — OptaBem</t>
@@ -675,16 +690,16 @@
     <t xml:space="preserve">US05, US17</t>
   </si>
   <si>
-    <t xml:space="preserve">Quem escolheu um curso prepara a candidatura: vê as condições de acesso de cada curso, indica as suas notas, vê a sua nota de candidatura em cada curso e ordena as 6 opções; o catálogo passa a ter as licenciaturas da DGES (29/10 a 05/11; a confirmar com o docente).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US04, US33–US36</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fora desta release, por ordem de prioridade. As US40 a US45 têm código pronto no PR #44 (protótipo). As opcionais estão na folha «Arquivo (opcionais)».</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US40–US42, US44, US37, US46, US47, US48, US39, US43, US45, US38</t>
+    <t xml:space="preserve">Quem escolheu um curso prepara a candidatura: vê as condições de acesso, a tendência e a procura de cada curso, indica as suas notas, vê a sua nota em cada curso e quanto precisa nos exames, ordena as 6 opções, descobre que exames lhe abrem mais portas, tem um plano B para a 2.ª fase e pode partilhar o plano; o catálogo passa a ter as licenciaturas da DGES (29/10 a 05/11; a confirmar com o docente).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US04, US33–US36, US40–US45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fora desta release, por ordem de prioridade. As opcionais estão na folha «Arquivo (opcionais)».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US37, US46, US47, US48, US39, US38</t>
   </si>
   <si>
     <t xml:space="preserve">Total</t>
@@ -895,6 +910,18 @@
   </si>
   <si>
     <t xml:space="preserve">• Atenção: mesmo assim, o Sprint 4 tem 18 SP para uma velocidade de 10. Só é defensável porque o código foi feito antes, como protótipo. A confirmar com o docente no Sprint Planning de 29/10.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sprint 4 alargado (27/10/2026, mais tarde; decisão do PO)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• As US40 a US45 voltam ao Sprint 4: são partes importantes do produto e o código já está feito (PR #44). O Sprint 4 passa de 18 para 32 SP.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Atenção: 32 SP para uma velocidade de 10 não é um planeamento realista de trabalho novo. Só se defende porque o código foi feito antes do sprint, como protótipo: no sprint sobra documentação, testes, revisão e aceitação. Fica escrito no relatório.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• A documentação das US04, US33 a US36 e US40 a US45 está em docs/USNN/ (PR #47), com testes novos para os critérios que não tinham teste.</t>
   </si>
   <si>
     <t xml:space="preserve">Resumo por prioridade (MoSCoW)</t>
@@ -1690,7 +1717,7 @@
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1707,7 +1734,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="20">
+  <dxfs count="21">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1820,6 +1847,13 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFF8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFDDEBF7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2053,7 +2087,7 @@
                   <c:v>7</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>18</c:v>
+                  <c:v>32</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2155,11 +2189,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="87705679"/>
-        <c:axId val="59618585"/>
+        <c:axId val="35237746"/>
+        <c:axId val="59396940"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="87705679"/>
+        <c:axId val="35237746"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2190,7 +2224,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="59618585"/>
+        <c:crossAx val="59396940"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2198,7 +2232,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="59618585"/>
+        <c:axId val="59396940"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2263,7 +2297,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87705679"/>
+        <c:crossAx val="35237746"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2330,9 +2364,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>2087280</xdr:colOff>
+      <xdr:colOff>2087640</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>84240</xdr:rowOff>
+      <xdr:rowOff>84600</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2341,7 +2375,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="775440" y="3992040"/>
-        <a:ext cx="5752440" cy="2512080"/>
+        <a:ext cx="5752800" cy="2512440"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -3138,14 +3172,14 @@
         <v>93</v>
       </c>
       <c r="I18" s="7" t="s">
-        <v>99</v>
+        <v>69</v>
       </c>
       <c r="J18" s="7" t="s">
         <v>70</v>
       </c>
       <c r="K18" s="8"/>
       <c r="L18" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="M18" s="5" t="s">
         <v>78</v>
@@ -3156,19 +3190,19 @@
         <v>15</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>73</v>
       </c>
       <c r="D19" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="E19" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="E19" s="6" t="s">
+      <c r="F19" s="6" t="s">
         <v>103</v>
-      </c>
-      <c r="F19" s="6" t="s">
-        <v>104</v>
       </c>
       <c r="G19" s="7" t="n">
         <v>2</v>
@@ -3177,14 +3211,14 @@
         <v>93</v>
       </c>
       <c r="I19" s="7" t="s">
-        <v>99</v>
+        <v>69</v>
       </c>
       <c r="J19" s="7" t="s">
         <v>70</v>
       </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="M19" s="5" t="s">
         <v>78</v>
@@ -3216,14 +3250,14 @@
         <v>93</v>
       </c>
       <c r="I20" s="7" t="s">
-        <v>99</v>
+        <v>69</v>
       </c>
       <c r="J20" s="7" t="s">
         <v>70</v>
       </c>
       <c r="K20" s="8"/>
       <c r="L20" s="8" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="M20" s="5" t="s">
         <v>78</v>
@@ -3234,19 +3268,19 @@
         <v>17</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>73</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G21" s="7" t="n">
         <v>3</v>
@@ -3255,14 +3289,14 @@
         <v>93</v>
       </c>
       <c r="I21" s="7" t="s">
-        <v>99</v>
+        <v>69</v>
       </c>
       <c r="J21" s="7" t="s">
         <v>70</v>
       </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8" t="s">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="M21" s="5" t="s">
         <v>78</v>
@@ -3273,35 +3307,35 @@
         <v>18</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="G22" s="7" t="n">
         <v>3</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>93</v>
+        <v>119</v>
       </c>
       <c r="I22" s="7" t="s">
-        <v>99</v>
+        <v>69</v>
       </c>
       <c r="J22" s="7" t="s">
-        <v>117</v>
+        <v>70</v>
       </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="M22" s="5" t="s">
         <v>78</v>
@@ -3312,35 +3346,35 @@
         <v>19</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>16</v>
+        <v>73</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F23" s="6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G23" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>93</v>
+        <v>119</v>
       </c>
       <c r="I23" s="7" t="s">
-        <v>99</v>
+        <v>69</v>
       </c>
       <c r="J23" s="7" t="s">
-        <v>117</v>
+        <v>70</v>
       </c>
       <c r="K23" s="8"/>
       <c r="L23" s="8" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="M23" s="5" t="s">
         <v>78</v>
@@ -3351,19 +3385,19 @@
         <v>20</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="F24" s="6" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G24" s="7" t="n">
         <v>3</v>
@@ -3372,14 +3406,14 @@
         <v>93</v>
       </c>
       <c r="I24" s="7" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
       <c r="J24" s="7" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="K24" s="8"/>
       <c r="L24" s="8" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="M24" s="5" t="s">
         <v>78</v>
@@ -3390,19 +3424,19 @@
         <v>21</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>53</v>
+        <v>16</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="F25" s="6" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="G25" s="7" t="n">
         <v>2</v>
@@ -3411,14 +3445,14 @@
         <v>93</v>
       </c>
       <c r="I25" s="7" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
       <c r="J25" s="7" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="K25" s="8"/>
       <c r="L25" s="8" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="M25" s="5" t="s">
         <v>78</v>
@@ -3429,35 +3463,35 @@
         <v>22</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>53</v>
+        <v>16</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="G26" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H26" s="5" t="s">
         <v>93</v>
       </c>
       <c r="I26" s="7" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
       <c r="J26" s="7" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="K26" s="8"/>
       <c r="L26" s="8" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="M26" s="5" t="s">
         <v>78</v>
@@ -3468,35 +3502,35 @@
         <v>23</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>73</v>
+        <v>53</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="G27" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>143</v>
+        <v>93</v>
       </c>
       <c r="I27" s="7" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
       <c r="J27" s="7" t="s">
-        <v>70</v>
+        <v>131</v>
       </c>
       <c r="K27" s="8"/>
       <c r="L27" s="8" t="s">
-        <v>100</v>
+        <v>147</v>
       </c>
       <c r="M27" s="5" t="s">
         <v>78</v>
@@ -3507,35 +3541,35 @@
         <v>24</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>73</v>
+        <v>53</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="F28" s="6" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="G28" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>143</v>
+        <v>93</v>
       </c>
       <c r="I28" s="7" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>70</v>
+        <v>131</v>
       </c>
       <c r="K28" s="8"/>
       <c r="L28" s="8" t="s">
-        <v>100</v>
+        <v>152</v>
       </c>
       <c r="M28" s="5" t="s">
         <v>78</v>
@@ -3546,35 +3580,35 @@
         <v>25</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>73</v>
       </c>
       <c r="D29" s="6" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="F29" s="6" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="G29" s="7" t="n">
         <v>2</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>143</v>
+        <v>119</v>
       </c>
       <c r="I29" s="7" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>117</v>
+        <v>131</v>
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="8" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="M29" s="5" t="s">
         <v>78</v>
@@ -3582,7 +3616,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F30" s="9" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="G30" s="9" t="n">
         <f aca="false">SUM(G5:G29)</f>
@@ -3591,7 +3625,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F31" s="9" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="G31" s="9" t="n">
         <f aca="false">SUMIF(J5:J29,"Feito",G5:G29)</f>
@@ -3600,7 +3634,7 @@
     </row>
     <row r="32" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F32" s="10" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -3640,30 +3674,30 @@
     <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>"Must"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="cellIs" priority="6" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Should"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="7" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Could"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
+    <cfRule type="cellIs" priority="8" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
       <formula>"Won't"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5:I29">
-    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13">
+    <cfRule type="cellIs" priority="9" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>"Sprint 1"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
+    <cfRule type="cellIs" priority="10" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="16">
       <formula>"Sprint 2"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="17">
+    <cfRule type="cellIs" priority="11" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
       <formula>"Sprint 3"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="18">
+    <cfRule type="cellIs" priority="12" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
       <formula>"Sprint 4"</formula>
     </cfRule>
-    <cfRule type="cellIs" priority="13" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="19">
+    <cfRule type="cellIs" priority="13" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="20">
       <formula>"Backlog"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3702,7 +3736,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H104"/>
+  <dimension ref="A1:H108"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
@@ -3717,17 +3751,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="12" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="C3" s="7" t="n">
         <v>10</v>
@@ -3738,25 +3772,25 @@
         <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3764,10 +3798,10 @@
         <v>21</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="C6" s="14" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="D6" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$29,$A6,'Product Backlog'!$G$5:$G$29)</f>
@@ -3795,10 +3829,10 @@
         <v>40</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="D7" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$29,$A7,'Product Backlog'!$G$5:$G$29)</f>
@@ -3826,10 +3860,10 @@
         <v>57</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="D8" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$29,$A8,'Product Backlog'!$G$5:$G$29)</f>
@@ -3857,14 +3891,14 @@
         <v>69</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="D9" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$29,$A9,'Product Backlog'!$G$5:$G$29)</f>
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="E9" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$29,'Product Backlog'!$I$5:$I$29,$A9,'Product Backlog'!$J$5:$J$29,"Feito")</f>
@@ -3876,26 +3910,26 @@
       </c>
       <c r="G9" s="16" t="n">
         <f aca="false">$C$3-D9</f>
-        <v>-8</v>
+        <v>-22</v>
       </c>
       <c r="H9" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$29,$A9)</f>
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>99</v>
+        <v>130</v>
       </c>
       <c r="B10" s="14" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">SUMIF('Product Backlog'!$I$5:$I$29,$A10,'Product Backlog'!$G$5:$G$29)</f>
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="E10" s="5" t="n">
         <f aca="false">SUMIFS('Product Backlog'!$G$5:$G$29,'Product Backlog'!$I$5:$I$29,$A10,'Product Backlog'!$J$5:$J$29,"Feito")</f>
@@ -3910,12 +3944,12 @@
       </c>
       <c r="H10" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$I$5:$I$29,$A10)</f>
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="20" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
@@ -3939,347 +3973,367 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="23" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="24" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="24" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="24" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="24" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="24" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="24" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="24" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="23" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="24" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="24" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="24" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="24" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="23" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="24" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="24" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="24" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="24" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="23" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="24" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="24" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="24" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="24" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="24" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="24" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="23" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="24" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="24" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="24" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="24" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="23" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="24" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="24" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="24" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="24" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="24" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="24" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="23" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="24" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="24" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="24" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="24" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="23" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="24" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="24" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="24" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="24" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="24" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="24" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="24" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="24" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="24" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="24" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="24" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="24" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="24" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="24" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="23" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="24" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="24" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="24" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="24" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="24" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="24" t="s">
-        <v>243</v>
-      </c>
-    </row>
-    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="24" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="24" t="s">
-        <v>245</v>
+        <v>250</v>
+      </c>
+    </row>
+    <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A105" s="23" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A106" s="24" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A107" s="24" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A108" s="24" t="s">
+        <v>254</v>
       </c>
     </row>
   </sheetData>
@@ -4312,24 +4366,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>246</v>
+        <v>255</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>248</v>
+        <v>257</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>249</v>
+        <v>258</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>250</v>
+        <v>259</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4337,7 +4391,7 @@
         <v>20</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>251</v>
+        <v>260</v>
       </c>
       <c r="C5" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$29,A5)</f>
@@ -4357,7 +4411,7 @@
         <v>93</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>252</v>
+        <v>261</v>
       </c>
       <c r="C6" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$29,A6)</f>
@@ -4374,10 +4428,10 @@
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>143</v>
+        <v>119</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>253</v>
+        <v>262</v>
       </c>
       <c r="C7" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$29,A7)</f>
@@ -4394,10 +4448,10 @@
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>254</v>
+        <v>263</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>255</v>
+        <v>264</v>
       </c>
       <c r="C8" s="5" t="n">
         <f aca="false">COUNTIF('Product Backlog'!$H$5:$H$29,A8)</f>
@@ -4414,7 +4468,7 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C9" s="27" t="n">
         <f aca="false">SUM(C5:C8)</f>
@@ -4425,9 +4479,9 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="102" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>256</v>
+        <v>265</v>
       </c>
     </row>
   </sheetData>
@@ -4449,24 +4503,24 @@
   <dimension ref="A1:H28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="44"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>257</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="29" t="s">
-        <v>258</v>
+        <v>267</v>
       </c>
       <c r="B2" s="29"/>
       <c r="C2" s="29"/>
@@ -4476,12 +4530,12 @@
       <c r="G2" s="29"/>
       <c r="H2" s="29"/>
     </row>
-    <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>259</v>
+        <v>268</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>5</v>
@@ -4499,24 +4553,24 @@
         <v>14</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>260</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="B5" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>262</v>
+        <v>271</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>263</v>
+        <v>272</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="F5" s="6" t="n">
         <v>5</v>
@@ -4525,111 +4579,111 @@
         <v>52</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>265</v>
+        <v>274</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>266</v>
+        <v>275</v>
       </c>
       <c r="B6" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>267</v>
+        <v>276</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>268</v>
+        <v>277</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>269</v>
+        <v>278</v>
       </c>
       <c r="F6" s="6" t="n">
         <v>5</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>261</v>
+        <v>270</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>270</v>
+        <v>279</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="B7" s="6" t="s">
         <v>73</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>272</v>
+        <v>281</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>273</v>
+        <v>282</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>274</v>
+        <v>283</v>
       </c>
       <c r="F7" s="6" t="n">
         <v>5</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>271</v>
+        <v>280</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>275</v>
+        <v>284</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>278</v>
+        <v>287</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>279</v>
+        <v>288</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>280</v>
+        <v>289</v>
       </c>
       <c r="F8" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>276</v>
+        <v>285</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>281</v>
+        <v>290</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="B9" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>283</v>
+        <v>292</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>284</v>
+        <v>293</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>285</v>
+        <v>294</v>
       </c>
       <c r="F9" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>266</v>
+        <v>275</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -4637,302 +4691,302 @@
         <v>65</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>287</v>
+        <v>296</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>288</v>
+        <v>297</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>289</v>
+        <v>298</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>290</v>
+        <v>299</v>
       </c>
       <c r="F10" s="6" t="n">
         <v>5</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>292</v>
+        <v>301</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>277</v>
+        <v>286</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="F11" s="6" t="n">
         <v>8</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>293</v>
+        <v>302</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>297</v>
+        <v>306</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>300</v>
+        <v>309</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>301</v>
+        <v>310</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>302</v>
+        <v>311</v>
       </c>
       <c r="F12" s="6" t="n">
         <v>2</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>304</v>
+        <v>313</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>305</v>
+        <v>314</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>306</v>
+        <v>315</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>307</v>
+        <v>316</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>308</v>
+        <v>317</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>309</v>
+        <v>318</v>
       </c>
       <c r="F13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>298</v>
+        <v>307</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>310</v>
+        <v>319</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>303</v>
+        <v>312</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>287</v>
+        <v>296</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>311</v>
+        <v>320</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>312</v>
+        <v>321</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>313</v>
+        <v>322</v>
       </c>
       <c r="F14" s="6" t="n">
         <v>5</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>314</v>
+        <v>323</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>315</v>
+        <v>324</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>317</v>
+        <v>326</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>318</v>
+        <v>327</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>319</v>
+        <v>328</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>320</v>
+        <v>329</v>
       </c>
       <c r="F15" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="B16" s="6" t="s">
         <v>36</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>324</v>
+        <v>333</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>325</v>
+        <v>334</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>326</v>
+        <v>335</v>
       </c>
       <c r="F16" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>282</v>
+        <v>291</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>322</v>
+        <v>331</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>327</v>
+        <v>336</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>317</v>
+        <v>326</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>328</v>
+        <v>337</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>329</v>
+        <v>338</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>330</v>
+        <v>339</v>
       </c>
       <c r="F17" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>331</v>
+        <v>340</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>332</v>
+        <v>341</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>333</v>
+        <v>342</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>334</v>
+        <v>343</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>335</v>
+        <v>344</v>
       </c>
       <c r="F18" s="6" t="n">
         <v>2</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>316</v>
+        <v>325</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>336</v>
+        <v>345</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>314</v>
+        <v>323</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>337</v>
+        <v>346</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>338</v>
+        <v>347</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>339</v>
+        <v>348</v>
       </c>
       <c r="F19" s="6" t="n">
         <v>5</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>305</v>
+        <v>314</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>340</v>
+        <v>349</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>341</v>
+        <v>350</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>343</v>
+        <v>352</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>344</v>
+        <v>353</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>345</v>
+        <v>354</v>
       </c>
       <c r="F20" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>346</v>
+        <v>355</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>347</v>
+        <v>356</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>346</v>
+        <v>355</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>348</v>
+        <v>357</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>349</v>
+        <v>358</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>350</v>
+        <v>359</v>
       </c>
       <c r="F21" s="6" t="n">
         <v>3</v>
@@ -4941,166 +4995,166 @@
         <v>60</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>351</v>
+        <v>360</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>306</v>
+        <v>315</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>352</v>
+        <v>361</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>353</v>
+        <v>362</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>354</v>
+        <v>363</v>
       </c>
       <c r="F22" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>327</v>
+        <v>336</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>355</v>
+        <v>364</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="6" t="s">
-        <v>331</v>
+        <v>340</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>317</v>
+        <v>326</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>356</v>
+        <v>365</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>357</v>
+        <v>366</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>358</v>
+        <v>367</v>
       </c>
       <c r="F23" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>359</v>
+        <v>368</v>
       </c>
       <c r="H23" s="6" t="s">
-        <v>360</v>
+        <v>369</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="6" t="s">
-        <v>359</v>
+        <v>368</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>342</v>
+        <v>351</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>361</v>
+        <v>370</v>
       </c>
       <c r="D24" s="6" t="s">
-        <v>362</v>
+        <v>371</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>363</v>
+        <v>372</v>
       </c>
       <c r="F24" s="6" t="n">
         <v>5</v>
       </c>
       <c r="G24" s="6" t="s">
-        <v>364</v>
+        <v>373</v>
       </c>
       <c r="H24" s="6" t="s">
-        <v>365</v>
+        <v>374</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>364</v>
+        <v>373</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>299</v>
+        <v>308</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>366</v>
+        <v>375</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>367</v>
+        <v>376</v>
       </c>
       <c r="E25" s="6" t="s">
-        <v>368</v>
+        <v>377</v>
       </c>
       <c r="F25" s="6" t="n">
         <v>8</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="H25" s="6" t="s">
-        <v>369</v>
+        <v>378</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="6" t="s">
-        <v>370</v>
+        <v>379</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>317</v>
+        <v>326</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>371</v>
+        <v>380</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>372</v>
+        <v>381</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>373</v>
+        <v>382</v>
       </c>
       <c r="F26" s="6" t="n">
         <v>3</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>370</v>
+        <v>379</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>374</v>
+        <v>383</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>375</v>
+        <v>384</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>376</v>
+        <v>385</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>377</v>
+        <v>386</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>378</v>
+        <v>387</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>379</v>
+        <v>388</v>
       </c>
       <c r="F27" s="6"/>
       <c r="G27" s="6" t="s">
         <v>78</v>
       </c>
       <c r="H27" s="6" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="E28" s="9" t="s">
-        <v>381</v>
+        <v>390</v>
       </c>
       <c r="F28" s="9" t="n">
         <f aca="false">SUM(F5:F27)</f>

</xml_diff>

<commit_message>
Definition of Done própria em cada story e preparação do fecho do Sprint 4
- Cada docs/USNN/README.md tem a sua Definition of Done: os critérios de
  aceitação dessa story, com os testes que os verificam (procurados no
  resultado dos 541 testes), e o mínimo da equipa. Regras (secção 11),
  modelo das issues e coluna N do backlog atualizados.
- docs/geral/07-cerimonias-scrum.md: o que está registado de cada
  cerimónia, retrospetivas por preencher e guião da Sprint Review.
- US48 no Sprint 4 como «Em curso» (por aceitar pelo PO).
- Comandos flask nos README em vez dos atalhos da pasta ferramentas,
  que não vai para o GitHub.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VGMz7ii8bx1E4vPrScuM4G
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Arquivo (opcionais)" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Product Backlog'!$A$4:$M$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Product Backlog'!$A$4:$N$29</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Product Backlog'!$4:$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Arquivo (opcionais)'!$A$4:$H$27</definedName>
   </definedNames>
@@ -724,7 +724,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
               </a:p>
             </txPr>
@@ -816,7 +816,7 @@
                   </a:defRPr>
                 </a:pPr>
                 <a:r>
-                  <a:t/>
+                  <a:t>None</a:t>
                 </a:r>
               </a:p>
             </txPr>
@@ -907,7 +907,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -985,7 +985,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -1017,7 +1017,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
         </a:p>
       </txPr>
@@ -1288,7 +1288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M32"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.66796875" defaultRowHeight="14.25" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="4" customWidth="1" style="30" min="1" max="1"/>
@@ -1302,6 +1302,7 @@
     <col width="14" customWidth="1" style="30" min="11" max="11"/>
     <col width="24" customWidth="1" style="30" min="12" max="12"/>
     <col width="10" customWidth="1" style="30" min="13" max="13"/>
+    <col width="46" customWidth="1" style="31" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="31">
@@ -1384,6 +1385,11 @@
           <t>ID anterior</t>
         </is>
       </c>
+      <c r="N4" s="34" t="inlineStr">
+        <is>
+          <t>Definition of Done (31/10)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="75" customHeight="1" s="31">
       <c r="A5" s="35" t="n">
@@ -1446,6 +1452,11 @@
           <t>US01</t>
         </is>
       </c>
+      <c r="N5" s="38" t="inlineStr">
+        <is>
+          <t>12 de 13 caixas marcadas (docs/US01/README.md). Falta: revisão do Simão.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="75" customHeight="1" s="31">
       <c r="A6" s="35" t="n">
@@ -1506,6 +1517,11 @@
       <c r="M6" s="35" t="inlineStr">
         <is>
           <t>US02</t>
+        </is>
+      </c>
+      <c r="N6" s="38" t="inlineStr">
+        <is>
+          <t>12 de 13 caixas marcadas (docs/US02/README.md). Falta: revisão do Simão.</t>
         </is>
       </c>
     </row>
@@ -1569,6 +1585,11 @@
       <c r="M7" s="35" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="N7" s="38" t="inlineStr">
+        <is>
+          <t>11 de 12 caixas marcadas (docs/US03/README.md). Falta: revisão do Simão.</t>
         </is>
       </c>
     </row>
@@ -1635,6 +1656,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="N8" s="38" t="inlineStr">
+        <is>
+          <t>14 de 14 caixas marcadas (docs/US29/README.md). Completa.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="75" customHeight="1" s="31">
       <c r="A9" s="35" t="n">
@@ -1698,6 +1724,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="N9" s="38" t="inlineStr">
+        <is>
+          <t>12 de 12 caixas marcadas (docs/US30/README.md). Completa.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="75" customHeight="1" s="31">
       <c r="A10" s="35" t="n">
@@ -1761,6 +1792,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="N10" s="38" t="inlineStr">
+        <is>
+          <t>11 de 12 caixas marcadas (docs/US31/README.md). Falta: revisão do Simão.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="75" customHeight="1" s="31">
       <c r="A11" s="35" t="n">
@@ -1823,6 +1859,11 @@
           <t>US04</t>
         </is>
       </c>
+      <c r="N11" s="38" t="inlineStr">
+        <is>
+          <t>11 de 11 caixas marcadas (docs/US05/README.md). Completa.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="75" customHeight="1" s="31">
       <c r="A12" s="35" t="n">
@@ -1882,6 +1923,11 @@
       <c r="M12" s="35" t="inlineStr">
         <is>
           <t>US10</t>
+        </is>
+      </c>
+      <c r="N12" s="38" t="inlineStr">
+        <is>
+          <t>10 de 10 caixas marcadas (docs/US17/README.md). Completa.</t>
         </is>
       </c>
     </row>
@@ -1947,6 +1993,11 @@
           <t>US03</t>
         </is>
       </c>
+      <c r="N13" s="38" t="inlineStr">
+        <is>
+          <t>10 de 12 caixas marcadas (docs/US04/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="75" customHeight="1" s="31">
       <c r="A14" s="35" t="n">
@@ -2010,6 +2061,11 @@
           <t>nova</t>
         </is>
       </c>
+      <c r="N14" s="38" t="inlineStr">
+        <is>
+          <t>10 de 12 caixas marcadas (docs/US33/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="75" customHeight="1" s="31">
       <c r="A15" s="35" t="n">
@@ -2072,6 +2128,11 @@
           <t>nova</t>
         </is>
       </c>
+      <c r="N15" s="38" t="inlineStr">
+        <is>
+          <t>10 de 12 caixas marcadas (docs/US34/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="75" customHeight="1" s="31">
       <c r="A16" s="35" t="n">
@@ -2132,6 +2193,11 @@
       <c r="M16" s="35" t="inlineStr">
         <is>
           <t>nova</t>
+        </is>
+      </c>
+      <c r="N16" s="38" t="inlineStr">
+        <is>
+          <t>10 de 12 caixas marcadas (docs/US35/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2198,6 +2264,11 @@
           <t>nova</t>
         </is>
       </c>
+      <c r="N17" s="38" t="inlineStr">
+        <is>
+          <t>13 de 15 caixas marcadas (docs/US36/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="75" customHeight="1" s="31">
       <c r="A18" s="35" t="n">
@@ -2261,6 +2332,11 @@
           <t>nova</t>
         </is>
       </c>
+      <c r="N18" s="38" t="inlineStr">
+        <is>
+          <t>10 de 12 caixas marcadas (docs/US40/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="75" customHeight="1" s="31">
       <c r="A19" s="35" t="n">
@@ -2322,6 +2398,11 @@
           <t>nova</t>
         </is>
       </c>
+      <c r="N19" s="38" t="inlineStr">
+        <is>
+          <t>8 de 10 caixas marcadas (docs/US41/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="75" customHeight="1" s="31">
       <c r="A20" s="35" t="n">
@@ -2380,6 +2461,11 @@
       <c r="M20" s="35" t="inlineStr">
         <is>
           <t>nova</t>
+        </is>
+      </c>
+      <c r="N20" s="38" t="inlineStr">
+        <is>
+          <t>7 de 9 caixas marcadas (docs/US42/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2444,6 +2530,11 @@
           <t>nova</t>
         </is>
       </c>
+      <c r="N21" s="38" t="inlineStr">
+        <is>
+          <t>9 de 11 caixas marcadas (docs/US44/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="75" customHeight="1" s="31">
       <c r="A22" s="35" t="n">
@@ -2506,6 +2597,11 @@
           <t>nova</t>
         </is>
       </c>
+      <c r="N22" s="38" t="inlineStr">
+        <is>
+          <t>10 de 12 caixas marcadas (docs/US43/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="75" customHeight="1" s="31">
       <c r="A23" s="35" t="n">
@@ -2567,6 +2663,11 @@
           <t>nova</t>
         </is>
       </c>
+      <c r="N23" s="38" t="inlineStr">
+        <is>
+          <t>8 de 10 caixas marcadas (docs/US45/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="75" customHeight="1" s="31">
       <c r="A24" s="35" t="n">
@@ -2628,6 +2729,11 @@
           <t>nova</t>
         </is>
       </c>
+      <c r="N24" s="38" t="inlineStr">
+        <is>
+          <t>8 de 10 caixas marcadas (docs/US37/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="75" customHeight="1" s="31">
       <c r="A25" s="35" t="n">
@@ -2681,12 +2787,17 @@
       <c r="K25" s="38" t="n"/>
       <c r="L25" s="38" t="inlineStr">
         <is>
-          <t>29/10: feita e aceite pelo PO (PR #50). Revisão do Simão pendente. Falta incluir a autorização da US37 na exportação, depois de as duas entrarem na main.</t>
+          <t>29/10: feita e aceite pelo PO (PR #50). Revisão do Simão pendente. 31/10: a exportação passou a dizer se a pessoa autorizou o assistente a usar as notas (US37).</t>
         </is>
       </c>
       <c r="M25" s="35" t="inlineStr">
         <is>
           <t>nova</t>
+        </is>
+      </c>
+      <c r="N25" s="38" t="inlineStr">
+        <is>
+          <t>9 de 11 caixas marcadas (docs/US46/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2742,12 +2853,17 @@
       <c r="K26" s="38" t="n"/>
       <c r="L26" s="38" t="inlineStr">
         <is>
-          <t>29/10: feita e aceite pelo PO (PR #51), com envio real de emails por SMTP. Revisão do Simão pendente.</t>
+          <t>29/10: feita e aceite pelo PO (PR #51), com envio real de emails por SMTP. Revisão do Simão pendente. 31/10: no máximo 3 emails de recuperação por conta e por hora (RF02.17).</t>
         </is>
       </c>
       <c r="M26" s="35" t="inlineStr">
         <is>
           <t>nova</t>
+        </is>
+      </c>
+      <c r="N26" s="38" t="inlineStr">
+        <is>
+          <t>10 de 12 caixas marcadas (docs/US47/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2812,6 +2928,11 @@
           <t>nova</t>
         </is>
       </c>
+      <c r="N27" s="38" t="inlineStr">
+        <is>
+          <t>9 de 11 caixas marcadas (docs/US39/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="75" customHeight="1" s="31">
       <c r="A28" s="35" t="n">
@@ -2872,6 +2993,11 @@
           <t>nova</t>
         </is>
       </c>
+      <c r="N28" s="38" t="inlineStr">
+        <is>
+          <t>7 de 9 caixas marcadas (docs/US38/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="75" customHeight="1" s="31">
       <c r="A29" s="35" t="n">
@@ -2914,23 +3040,28 @@
       </c>
       <c r="I29" s="37" t="inlineStr">
         <is>
-          <t>Backlog</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="J29" s="37" t="inlineStr">
         <is>
-          <t>Por fazer</t>
+          <t>Em curso</t>
         </is>
       </c>
       <c r="K29" s="38" t="n"/>
       <c r="L29" s="38" t="inlineStr">
         <is>
-          <t>27/10: separada da US04 (decisão do PO). O código já existe; falta correr a recolha, que exige o computador ligado uma noite inteira.</t>
+          <t>27/10: separada da US04 (decisão do PO). 29/10: recolha corrida pelo PO (1699 cursos, PR #58). 31/10: entra no Sprint 4; o PR #58 tinha ficado no ramo do #57 e só chegou à main no PR de fecho. Falta a aceitação do PO na Sprint Review e a revisão do Simão.</t>
         </is>
       </c>
       <c r="M29" s="35" t="inlineStr">
         <is>
           <t>nova</t>
+        </is>
+      </c>
+      <c r="N29" s="38" t="inlineStr">
+        <is>
+          <t>7 de 10 caixas marcadas (docs/US48/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11; aceitação do PO.</t>
         </is>
       </c>
     </row>
@@ -2984,7 +3115,7 @@
     <row r="51" ht="14.25" customHeight="1" s="31"/>
     <row r="52" ht="42.75" customHeight="1" s="31"/>
   </sheetData>
-  <autoFilter ref="A4:M29"/>
+  <autoFilter ref="A4:N29"/>
   <conditionalFormatting sqref="J5:J29">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="equal" aboveAverage="0" dxfId="11" text="" percent="0" bottom="0">
       <formula>"Feito"</formula>
@@ -3058,7 +3189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H117"/>
+  <dimension ref="A1:H123"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="30" min="1" max="1"/>
@@ -3095,7 +3226,6 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="23.25" customHeight="1" s="31">
       <c r="A5" s="34" t="inlineStr">
         <is>
@@ -3262,7 +3392,7 @@
       </c>
       <c r="C9" s="44" t="inlineStr">
         <is>
-          <t>US04, US33–US36, US40–US45, US37–US39, US46, US47</t>
+          <t>US04, US33–US36, US40–US45, US37–US39, US46–US48</t>
         </is>
       </c>
       <c r="D9" s="35">
@@ -3299,7 +3429,7 @@
       </c>
       <c r="C10" s="44" t="inlineStr">
         <is>
-          <t>US48</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D10" s="35">
@@ -3350,564 +3480,540 @@
         <v/>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
-    <row r="23"/>
-    <row r="24"/>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27"/>
-    <row r="28"/>
     <row r="29" ht="15" customHeight="1" s="31">
-      <c r="A29" s="53" t="inlineStr">
+      <c r="A29" s="55" t="inlineStr">
         <is>
           <t>Replaneamento de 07/10/2026 (decisão do Product Owner)</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1" s="31">
-      <c r="A30" s="54" t="inlineStr">
+      <c r="A30" s="56" t="inlineStr">
         <is>
           <t>• O Sprint 1 tinha 24 SP planeados e a equipa concluiu 5 (registo e autenticação): o plano foi ajustado à velocidade real.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1" s="31">
-      <c r="A31" s="54" t="inlineStr">
+      <c r="A31" s="56" t="inlineStr">
         <is>
           <t>• Story nova: US03 — Perfis de aluno e administrador (RF04, que não tinha story). Entra no Sprint 1 porque a importação do catálogo (US04) precisa de um administrador.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1" s="31">
-      <c r="A32" s="54" t="inlineStr">
+      <c r="A32" s="56" t="inlineStr">
         <is>
           <t>• As stories do catálogo, percurso e avaliações (US04 a US08) passam do Sprint 1 para o Sprint 2, com a pseudonimização (US09) para as avaliações serem anónimas desde o início.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1" s="31">
-      <c r="A33" s="54" t="inlineStr">
+      <c r="A33" s="56" t="inlineStr">
         <is>
           <t>• A explicação da recomendação passa para o Sprint 3; avaliação offline, períodos de avaliação, comentários e filtros para o Sprint 4.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1" s="31">
-      <c r="A34" s="54" t="inlineStr">
+      <c r="A34" s="56" t="inlineStr">
         <is>
           <t>• Preferência de carga e comparação de estratégias passam para o Backlog; o SVD (antiga US22) fica fora do plano.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="31">
-      <c r="A35" s="54" t="inlineStr">
+      <c r="A35" s="56" t="inlineStr">
         <is>
           <t>• Escala das avaliações corrigida de 1–20 para 1–5 (igual ao resto do projeto).</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1" s="31">
-      <c r="A36" s="54" t="inlineStr">
+      <c r="A36" s="56" t="inlineStr">
         <is>
           <t>• As stories foram renumeradas pela nova ordem (US01 a US28). A coluna «ID anterior» da folha «Product Backlog» mostra o número antigo.</t>
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38" ht="15" customHeight="1" s="31">
-      <c r="A38" s="53" t="inlineStr">
+      <c r="A38" s="55" t="inlineStr">
         <is>
           <t>Replaneamento de 13/10/2026 (decisão dos Product Owners, com sugestões do docente)</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1" s="31">
-      <c r="A39" s="54" t="inlineStr">
+      <c r="A39" s="56" t="inlineStr">
         <is>
           <t>• Nova visão do produto: o utilizador pode ainda não ter curso; o OptaBem orienta a escolha do curso e depois a das opcionais (docs/geral/00-visao-do-produto.md).</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1" s="31">
-      <c r="A40" s="54" t="inlineStr">
+      <c r="A40" s="56" t="inlineStr">
         <is>
           <t>• Catálogo com várias instituições: MVP com 12 instituições e 30 licenciaturas (dados/catalogo-cursos-mvp.csv, fonte DGES).</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1" s="31">
-      <c r="A41" s="54" t="inlineStr">
+      <c r="A41" s="56" t="inlineStr">
         <is>
           <t>• Stories novas: US29 (questionário), US30 (sugestão de cursos com LLM) e US31 (escolher curso e linha do tempo). Épico novo E11.</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1" s="31">
-      <c r="A42" s="54" t="inlineStr">
+      <c r="A42" s="56" t="inlineStr">
         <is>
           <t>• US04 e US05 passam a tratar instituições e cursos; US06 inclui a importação das UCs e passa para o Sprint 4.</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1" s="31">
-      <c r="A43" s="54" t="inlineStr">
+      <c r="A43" s="56" t="inlineStr">
         <is>
           <t>• US08, US10 e US12 a US20 passam para o Backlog; as que eram Must passam a Should nesta release.</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1" s="31">
-      <c r="A44" s="54" t="inlineStr">
+      <c r="A44" s="56" t="inlineStr">
         <is>
           <t>• A partir de 13/10 os IDs ficam fixos (stories novas recebem o número seguinte). A ordem de trabalho é a deste plano.</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1" s="31">
-      <c r="A45" s="54" t="inlineStr">
+      <c r="A45" s="56" t="inlineStr">
         <is>
           <t>• Atenção: o plano soma 13, 13 e 18 SP; a velocidade real do Sprint 1 foi 10 SP (ponto 10 da secção 5 dos requisitos).</t>
         </is>
       </c>
     </row>
-    <row r="46"/>
     <row r="47" ht="15" customHeight="1" s="31">
-      <c r="A47" s="53" t="inlineStr">
+      <c r="A47" s="55" t="inlineStr">
         <is>
           <t>Revisão de 14/10/2026 (decisões dos Product Owners)</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15" customHeight="1" s="31">
-      <c r="A48" s="54" t="inlineStr">
+      <c r="A48" s="56" t="inlineStr">
         <is>
           <t>• US03 revista: um só início de sessão para alunos e administradores (design patterns Strategy, Chain of Responsibility e Factory).</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1" s="31">
-      <c r="A49" s="54" t="inlineStr">
+      <c r="A49" s="56" t="inlineStr">
         <is>
           <t>• US05 começada antes do Sprint 2: pesquisa de cursos reais na página de apresentação. Os SP contam no Sprint 2, quando a story estiver completa.</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1" s="31">
-      <c r="A50" s="54" t="inlineStr">
+      <c r="A50" s="56" t="inlineStr">
         <is>
           <t>• Story nova US32 (assistente LLM que conversa com o utilizador), no Backlog e por avaliar: decidir âmbito, custo e privacidade antes de estimar.</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1" s="31">
-      <c r="A51" s="54" t="inlineStr">
+      <c r="A51" s="56" t="inlineStr">
         <is>
           <t>• Redesenho visual do site (sem story própria): fica registado no PR #14 e no registo de uso de IA.</t>
         </is>
       </c>
     </row>
-    <row r="52"/>
     <row r="53" ht="15" customHeight="1" s="31">
-      <c r="A53" s="53" t="inlineStr">
+      <c r="A53" s="55" t="inlineStr">
         <is>
           <t>Replaneamento de 14/10/2026 (decisão do PO na issue #15)</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1" s="31">
-      <c r="A54" s="54" t="inlineStr">
+      <c r="A54" s="56" t="inlineStr">
         <is>
           <t>• As perguntas deixam de ser fixas: o LLM conduz a conversa. US29 reescrita (conversa, 5 SP) e US32 fundida nela; US30 passa a ser o fim da conversa (3 SP).</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1" s="31">
-      <c r="A55" s="54" t="inlineStr">
+      <c r="A55" s="56" t="inlineStr">
         <is>
           <t>• Spike técnico feito antes do Sprint 2 (PR #17): Gemini e Groq atrás de ClienteLLM, testes sem rede, conclusões em docs/geral/05-spike-llm.md. Não tem SP.</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1" s="31">
-      <c r="A56" s="54" t="inlineStr">
+      <c r="A56" s="56" t="inlineStr">
         <is>
           <t>• O LLM passa para o Sprint 2. Velocidade ajustada à real (de 23 para 10 SP): Sprint 2 com 8 SP (2 de folga pela tecnologia nova), Sprints 3 e 4 com 10 SP.</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1" s="31">
-      <c r="A57" s="54" t="inlineStr">
+      <c r="A57" s="56" t="inlineStr">
         <is>
           <t>• US05 passa para o Sprint 3. US04, US09 e US11 passam para o Backlog (Must → Should). A US07 guarda as avaliações com pseudo_id desde o início.</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1" s="31">
-      <c r="A58" s="54" t="inlineStr">
+      <c r="A58" s="56" t="inlineStr">
         <is>
           <t>• Consequência: nesta release não há recomendação de opcionais (US11). Se houver um Sprint 5, entram primeiro a US09 e a US11 (8 SP).</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1" s="31">
-      <c r="A59" s="54" t="inlineStr">
+      <c r="A59" s="56" t="inlineStr">
         <is>
           <t>• Por decidir antes do Sprint 2: idade mínima e plano do Gemini (os termos excluem menores de 18 e o plano gratuito com utilizadores no EEE).</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1" s="31">
-      <c r="A60" s="53" t="inlineStr">
+      <c r="A60" s="55" t="inlineStr">
         <is>
           <t>Sprint Planning do Sprint 2 (20/10/2026, decisão do PO)</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1" s="31">
-      <c r="A61" s="54" t="inlineStr">
+      <c r="A61" s="56" t="inlineStr">
         <is>
           <t>• A US29 e a US30 (8 SP) foram feitas antes de o sprint começar (PR #19, #20 e #22 a #24). Para o sprint ter trabalho novo, entra a US31 (5 SP), antecipada do Sprint 3.</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1" s="31">
-      <c r="A62" s="54" t="inlineStr">
+      <c r="A62" s="56" t="inlineStr">
         <is>
           <t>• O Sprint 2 fica com 13 SP planeados, acima da velocidade (10), mas só 5 SP são trabalho novo. O Sprint 3 fica com a US05 (5 SP) e 5 SP por planear: rever no fim do Sprint 2.</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1" s="31">
-      <c r="A63" s="54" t="inlineStr">
+      <c r="A63" s="56" t="inlineStr">
         <is>
           <t>• Ponto 14 decidido: o OptaBem é um protótipo usado pela equipa e na demonstração, com aviso de 18+ na conversa; fica escrito no relatório.</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1" s="31">
-      <c r="A64" s="54" t="inlineStr">
+      <c r="A64" s="56" t="inlineStr">
         <is>
           <t>• Servidor Ollama da faculdade testado e posto de parte: lento e não obedece ao pedido de sugestão (PR #25 e #26; 05-spike-llm.md, secção 7). Fica o Gemini.</t>
         </is>
       </c>
     </row>
-    <row r="65"/>
     <row r="66" ht="15" customHeight="1" s="31">
-      <c r="A66" s="53" t="inlineStr">
+      <c r="A66" s="55" t="inlineStr">
         <is>
           <t>Sprint Review do Sprint 2 e Sprint Planning do Sprint 3 (22/10/2026, decisão dos PO)</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1" s="31">
-      <c r="A67" s="54" t="inlineStr">
+      <c r="A67" s="56" t="inlineStr">
         <is>
           <t>• Sprint Review: US29, US30 e US31 aceites, 13 de 13 SP. O percurso completo foi testado com o Gemini real, também noutro computador.</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1" s="31">
-      <c r="A68" s="54" t="inlineStr">
+      <c r="A68" s="56" t="inlineStr">
         <is>
           <t>• Até à entrega de 05/11, o centro do produto são os cursos. As opcionais saíram do site (PR #33) e as suas stories passam para segundo plano: US06 e US07 saem do Sprint 4 (Must → Should).</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1" s="31">
-      <c r="A69" s="54" t="inlineStr">
+      <c r="A69" s="56" t="inlineStr">
         <is>
           <t>• Sprints de uma semana: Sprint 3 de 22/10 a 29/10 e Sprint 4 de 29/10 a 05/11.</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1" s="31">
-      <c r="A70" s="54" t="inlineStr">
+      <c r="A70" s="56" t="inlineStr">
         <is>
           <t>• Sprint 3: US05 (5 SP) e US17 (3 SP, sobe do Backlog e passa a Must), com 2 SP de folga.</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1" s="31">
-      <c r="A71" s="54" t="inlineStr">
+      <c r="A71" s="56" t="inlineStr">
         <is>
           <t>• Sprint 4: uma story nova a decidir com o docente; a US04 entra se houver folga. O código fecha por volta de 03/11, para o relatório e a demonstração.</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1" s="31">
-      <c r="A72" s="54" t="inlineStr">
+      <c r="A72" s="56" t="inlineStr">
         <is>
           <t>• A revisão de 22/10 (segurança do túnel, menu do aluno, textos) fica adiada por decisão do PO; o túnel é só para a equipa.</t>
         </is>
       </c>
     </row>
-    <row r="73"/>
     <row r="74" ht="15" customHeight="1" s="31">
-      <c r="A74" s="53" t="inlineStr">
+      <c r="A74" s="55" t="inlineStr">
         <is>
           <t>Sprint Review do Sprint 3 (23/10/2026, decisão dos PO)</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1" s="31">
-      <c r="A75" s="54" t="inlineStr">
+      <c r="A75" s="56" t="inlineStr">
         <is>
           <t>• US05 e US17 aceites, 7 de 7 SP. As duas stories foram testadas pelos PO (filtros, ficha, comparação e apagar a conta).</t>
         </is>
       </c>
     </row>
     <row r="76" ht="15" customHeight="1" s="31">
-      <c r="A76" s="54" t="inlineStr">
+      <c r="A76" s="56" t="inlineStr">
         <is>
           <t>• O sprint fecha antes de 29/10 porque o objetivo foi cumprido. Entrou também, sem story, o menu fixo no topo (PR #40).</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1" s="31">
-      <c r="A77" s="54" t="inlineStr">
+      <c r="A77" s="56" t="inlineStr">
         <is>
           <t>• No fecho, um teste da US17 que dependia da data em que corria foi corrigido (sem mudanças no código da aplicação).</t>
         </is>
       </c>
     </row>
     <row r="78" ht="15" customHeight="1" s="31">
-      <c r="A78" s="54" t="inlineStr">
+      <c r="A78" s="56" t="inlineStr">
         <is>
           <t>• Sprint 4 por planear: a story nova fica a decidir com o docente.</t>
         </is>
       </c>
     </row>
-    <row r="79"/>
     <row r="80" ht="15" customHeight="1" s="31">
-      <c r="A80" s="53" t="inlineStr">
+      <c r="A80" s="55" t="inlineStr">
         <is>
           <t>Replaneamento de 23/10/2026 (decisões do PO, com o protótipo do PR #44)</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1" s="31">
-      <c r="A81" s="54" t="inlineStr">
+      <c r="A81" s="56" t="inlineStr">
         <is>
           <t>• O plano de candidatura ao Concurso Nacional de Acesso substitui as opcionais: épico novo E12 com a US33 (condições de acesso), US34 (notas), US35 (nota por curso), US36 (as 6 opções), US37 (assistente com as notas) e US38 (datas do concurso).</t>
         </is>
       </c>
     </row>
     <row r="82" ht="15" customHeight="1" s="31">
-      <c r="A82" s="54" t="inlineStr">
+      <c r="A82" s="56" t="inlineStr">
         <is>
           <t>• As 22 stories das opcionais passam a Won't (fase 2) e ficam no fim do backlog, para a rastreabilidade.</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1" s="31">
-      <c r="A83" s="54" t="inlineStr">
+      <c r="A83" s="56" t="inlineStr">
         <is>
           <t>• US04 reescrita: o catálogo vem da DGES por recolha, em vez de ser importado por CSV na gestão; passa a Must e entra no Sprint 4.</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1" s="31">
-      <c r="A84" s="54" t="inlineStr">
+      <c r="A84" s="56" t="inlineStr">
         <is>
           <t>• US39 nova (gestão do catálogo), a partir da sugestão de um colega de editar a base de dados na área de gestão; fica no Backlog (Should).</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1" s="31">
-      <c r="A85" s="54" t="inlineStr">
+      <c r="A85" s="56" t="inlineStr">
         <is>
           <t>• Atenção: o Sprint 4 fica com 18 SP planeados, acima da velocidade (10). O código das US33 a US36 foi feito antes do sprint (protótipo), como a US29 e a US30 no Sprint 2. Se o docente achar demais, a US36 é a primeira a sair (é Should).</t>
         </is>
       </c>
     </row>
     <row r="86" ht="15" customHeight="1" s="31">
-      <c r="A86" s="54" t="inlineStr">
+      <c r="A86" s="56" t="inlineStr">
         <is>
           <t>• Sem story: o registo pede o nome, terminar sessão volta à página inicial e «As minhas decisões» sai do menu (PR #43 e #44).</t>
         </is>
       </c>
     </row>
     <row r="87" ht="15" customHeight="1" s="31">
-      <c r="A87" s="54" t="inlineStr">
+      <c r="A87" s="56" t="inlineStr">
         <is>
           <t>• Correção: o Sprint Planning de 22/10 dizia «US17 (3 SP)»; a US17 tem 2 SP (o total de 7 SP da Sprint Review está certo).</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1" s="31">
-      <c r="A88" s="54" t="inlineStr">
+      <c r="A88" s="56" t="inlineStr">
         <is>
           <t>• A story do Sprint 4 tem de ser confirmada com o docente.</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1" s="31">
-      <c r="A89" s="54" t="inlineStr">
+      <c r="A89" s="56" t="inlineStr">
         <is>
           <t>• (23/10, mais tarde) Stories novas US40 a US43, propostas pelo Claude e aceites pelo PO: quanto preciso no exame, tendência do último colocado, procura do curso e partilhar o plano. Feitas no PR #44.</t>
         </is>
       </c>
     </row>
     <row r="90" ht="15" customHeight="1" s="31">
-      <c r="A90" s="54" t="inlineStr">
+      <c r="A90" s="56" t="inlineStr">
         <is>
           <t>• Atenção: com elas, o Sprint 4 fica com 27 SP planeados para uma velocidade de 10. Quase todo o código já está feito (protótipo), mas a documentação de cada story (requisitos, use case, BPMN) não. Se o docente achar demais, saem primeiro a US43 (Could) e depois a US36, US40, US41 e US42 (Should).</t>
         </is>
       </c>
     </row>
     <row r="91" ht="15" customHeight="1" s="31">
-      <c r="A91" s="54" t="inlineStr">
+      <c r="A91" s="56" t="inlineStr">
         <is>
           <t>• Sem story: a gestão passa a ativar contas por confirmar, enquanto o site não envia emails reais (PR #43).</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1" s="31">
-      <c r="A92" s="54" t="inlineStr">
+      <c r="A92" s="56" t="inlineStr">
         <is>
           <t>• (23/10, ao fim do dia) Stories novas US44 (que exames me abrem mais portas) e US45 (plano B: 2.ª fase), propostas pelo Claude e escolhidas pelo PO. Feitas no PR #44.</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1" s="31">
-      <c r="A93" s="54" t="inlineStr">
+      <c r="A93" s="56" t="inlineStr">
         <is>
           <t>• O Sprint 4 fica com 32 SP planeados para uma velocidade de 10. Isto não é um planeamento realista em Scrum: o código foi feito antes do sprint, como protótipo. No Sprint Planning de 29/10, os PO e o docente decidem que stories entram; as restantes voltam ao Backlog com o código já feito.</t>
         </is>
       </c>
     </row>
     <row r="94" ht="15" customHeight="1" s="31">
-      <c r="A94" s="54" t="inlineStr">
+      <c r="A94" s="56" t="inlineStr">
         <is>
           <t>• Esclarecimento: o Sprint 4 ainda não começou (29/10 a 05/11). Um sprint fecha na Sprint Review, no fim do tempo marcado; aceitar um PR é o que faz uma story contar como Feita.</t>
         </is>
       </c>
     </row>
-    <row r="95"/>
     <row r="96" ht="15" customHeight="1" s="31">
-      <c r="A96" s="53" t="inlineStr">
+      <c r="A96" s="55" t="inlineStr">
         <is>
           <t>Reestruturação de 27/10/2026 (autorizada pelo docente; decisão do PO)</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1" s="31">
-      <c r="A97" s="54" t="inlineStr">
+      <c r="A97" s="56" t="inlineStr">
         <is>
           <t>• O docente autorizou mudar o backlog a fundo, para corresponder a um recomendador de cursos e não de opcionais.</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1" s="31">
-      <c r="A98" s="54" t="inlineStr">
+      <c r="A98" s="56" t="inlineStr">
         <is>
           <t>• As 22 stories das opcionais (US06 a US16 e US18 a US28) e a US32 (fundida na US29) saem do Product Backlog para a folha «Arquivo (opcionais)», com o motivo de cada uma. Os IDs não são reutilizados.</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1" s="31">
-      <c r="A99" s="54" t="inlineStr">
+      <c r="A99" s="56" t="inlineStr">
         <is>
           <t>• Épicos reorganizados: E1 Conta e privacidade, E2 Catálogo de cursos, E3 Orientação com o assistente, E4 Plano de candidatura. Os épicos antigos ficam no arquivo.</t>
         </is>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1" s="31">
-      <c r="A100" s="54" t="inlineStr">
+      <c r="A100" s="56" t="inlineStr">
         <is>
           <t>• Sprint 4 reduzido ao essencial: US04 e US33 a US36 (18 SP). As US40 a US45 (14 SP) voltam ao backlog com o código pronto, no estado novo «Protótipo».</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1" s="31">
-      <c r="A101" s="54" t="inlineStr">
+      <c r="A101" s="56" t="inlineStr">
         <is>
           <t>• Stories novas no backlog: US46 (exportar os meus dados, a parte do RF17 que saiu da US17) e US47 (recuperar a palavra-passe, a parte do RF02 sem story).</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1" s="31">
-      <c r="A102" s="54" t="inlineStr">
+      <c r="A102" s="56" t="inlineStr">
         <is>
           <t>• US04 dividida (decisão do PO): fica o catálogo recolhido da DGES com os 174 cursos já recolhidos; a recolha de todas as licenciaturas passa a ser a US48 (Backlog), porque exige o computador ligado uma noite inteira.</t>
         </is>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1" s="31">
-      <c r="A103" s="54" t="inlineStr">
+      <c r="A103" s="56" t="inlineStr">
         <is>
           <t>• As notas de cada story passam a dizer só o estado atual; o histórico fica nesta folha.</t>
         </is>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1" s="31">
-      <c r="A104" s="54" t="inlineStr">
+      <c r="A104" s="56" t="inlineStr">
         <is>
           <t>• Atenção: mesmo assim, o Sprint 4 tem 18 SP para uma velocidade de 10. Só é defensável porque o código foi feito antes, como protótipo. A confirmar com o docente no Sprint Planning de 29/10.</t>
         </is>
       </c>
     </row>
     <row r="105" ht="15" customHeight="1" s="31">
-      <c r="A105" s="53" t="inlineStr">
+      <c r="A105" s="55" t="inlineStr">
         <is>
           <t>Sprint 4 alargado (27/10/2026, mais tarde; decisão do PO)</t>
         </is>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1" s="31">
-      <c r="A106" s="54" t="inlineStr">
+      <c r="A106" s="56" t="inlineStr">
         <is>
           <t>• As US40 a US45 voltam ao Sprint 4: são partes importantes do produto e o código já está feito (PR #44). O Sprint 4 passa de 18 para 32 SP.</t>
         </is>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1" s="31">
-      <c r="A107" s="54" t="inlineStr">
+      <c r="A107" s="56" t="inlineStr">
         <is>
           <t>• Atenção: 32 SP para uma velocidade de 10 não é um planeamento realista de trabalho novo. Só se defende porque o código foi feito antes do sprint, como protótipo: no sprint sobra documentação, testes, revisão e aceitação. Fica escrito no relatório.</t>
         </is>
       </c>
     </row>
     <row r="108" ht="15" customHeight="1" s="31">
-      <c r="A108" s="54" t="inlineStr">
+      <c r="A108" s="56" t="inlineStr">
         <is>
           <t>• A documentação das US04, US33 a US36 e US40 a US45 está em docs/USNN/ (PR #47), com testes novos para os critérios que não tinham teste.</t>
         </is>
       </c>
     </row>
     <row r="109" ht="15" customHeight="1" s="31">
-      <c r="A109" s="53" t="inlineStr">
+      <c r="A109" s="55" t="inlineStr">
         <is>
           <t>Aceitação das stories do Sprint 4 (27/10/2026, decisão do PO)</t>
         </is>
       </c>
     </row>
     <row r="110" ht="15" customHeight="1" s="31">
-      <c r="A110" s="54" t="inlineStr">
+      <c r="A110" s="56" t="inlineStr">
         <is>
           <t>• O PO aceitou as 11 stories do Sprint 4 (US04, US33 a US36, US40 a US45): o código foi feito a 23/10, antes do sprint, e a documentação e os testes em falta a 27/10. Passam a Feito: 32 de 32 SP.</t>
         </is>
       </c>
     </row>
     <row r="111" ht="15" customHeight="1" s="31">
-      <c r="A111" s="54" t="inlineStr">
+      <c r="A111" s="56" t="inlineStr">
         <is>
           <t>• Antes de aceitar, o Claude verificou as 11 stories com o catálogo real e encontrou dois erros, corrigidos no mesmo dia: os cursos do ensino privado entravam no plano do concurso nacional (US36, US35, US44, US45), e as Matemáticas só ligavam a prova 16 à 19 (US34, US35, US44; correspondência da DGES: a Matemática A dá as provas 16, 17 e 19, a Matemática B a 16 e a 17, o MACS a 17).</t>
         </is>
       </c>
     </row>
     <row r="112" ht="15" customHeight="1" s="31">
-      <c r="A112" s="54" t="inlineStr">
+      <c r="A112" s="56" t="inlineStr">
         <is>
           <t>• Fica registado que a aceitação aconteceu antes da data de início marcada para o Sprint 4 (29/10) e com a revisão do Simão (PR #48) ainda pendente.</t>
         </is>
@@ -3945,6 +4051,41 @@
       <c r="A117" s="56" t="inlineStr">
         <is>
           <t>• Sem story: envio real de emails por SMTP (configurado no .env), textos antigos das opcionais (PR #55) e o visual calmo, com menos texto à vista e a letra do sistema (PR #56).</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="55" t="inlineStr">
+        <is>
+          <t>Preparação do fecho do Sprint 4 (31/10/2026; feita pelo Claude a pedido do PO)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="56" t="inlineStr">
+        <is>
+          <t>• A US48 entra no Sprint 4 como «Em curso»: o código e os dados estão na main, mas falta o PO aceitá-la na Sprint Review. Se for aceite, o Sprint 4 fica com 49 SP feitos, para uma velocidade de 10.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="56" t="inlineStr">
+        <is>
+          <t>• Cada story tem agora a sua Definition of Done no README da pasta docs/USNN/: os critérios de aceitação dessa story (com os testes que os verificam) e o mínimo da equipa. A coluna N da folha «Product Backlog» resume o que falta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="56" t="inlineStr">
+        <is>
+          <t>• O que falta em quase todas: a revisão do Simão (nenhum PR tem revisão formal no GitHub) e mostrar as stories do Sprint 4 na Sprint Review de 05/11.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="56" t="inlineStr">
+        <is>
+          <t>• Sem story: limite de 3 emails de recuperação por conta e por hora (US47), autorização da US37 na exportação dos dados (US46), ícone do separador com as cores do visual calmo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fecho: revisão no GitHub dispensada pelos Product Owners e US48 aceite
Decisão dos PO a 31/10: o Simão acompanhou todo o trabalho, por isso a
revisão do código no GitHub é dispensada e fica escrita na Definition of
Done de cada story. A US48 é aceite (Sprint 4 com 49 SP). Falta só a
caixa «Funciona na demonstração», a marcar na Sprint Review de 05/11.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VGMz7ii8bx1E4vPrScuM4G
</commit_message>
<xml_diff>
--- a/docs/geral/product-backlog.xlsx
+++ b/docs/geral/product-backlog.xlsx
@@ -1454,7 +1454,7 @@
       </c>
       <c r="N5" s="38" t="inlineStr">
         <is>
-          <t>12 de 13 caixas marcadas (docs/US01/README.md). Falta: revisão do Simão.</t>
+          <t>13 de 13 caixas marcadas (docs/US01/README.md). Completa.</t>
         </is>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="N6" s="38" t="inlineStr">
         <is>
-          <t>12 de 13 caixas marcadas (docs/US02/README.md). Falta: revisão do Simão.</t>
+          <t>13 de 13 caixas marcadas (docs/US02/README.md). Completa.</t>
         </is>
       </c>
     </row>
@@ -1589,7 +1589,7 @@
       </c>
       <c r="N7" s="38" t="inlineStr">
         <is>
-          <t>11 de 12 caixas marcadas (docs/US03/README.md). Falta: revisão do Simão.</t>
+          <t>12 de 12 caixas marcadas (docs/US03/README.md). Completa.</t>
         </is>
       </c>
     </row>
@@ -1794,7 +1794,7 @@
       </c>
       <c r="N10" s="38" t="inlineStr">
         <is>
-          <t>11 de 12 caixas marcadas (docs/US31/README.md). Falta: revisão do Simão.</t>
+          <t>12 de 12 caixas marcadas (docs/US31/README.md). Completa.</t>
         </is>
       </c>
     </row>
@@ -1995,7 +1995,7 @@
       </c>
       <c r="N13" s="38" t="inlineStr">
         <is>
-          <t>10 de 12 caixas marcadas (docs/US04/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>11 de 12 caixas marcadas (docs/US04/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2063,7 +2063,7 @@
       </c>
       <c r="N14" s="38" t="inlineStr">
         <is>
-          <t>10 de 12 caixas marcadas (docs/US33/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>11 de 12 caixas marcadas (docs/US33/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2130,7 @@
       </c>
       <c r="N15" s="38" t="inlineStr">
         <is>
-          <t>10 de 12 caixas marcadas (docs/US34/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>11 de 12 caixas marcadas (docs/US34/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="N16" s="38" t="inlineStr">
         <is>
-          <t>10 de 12 caixas marcadas (docs/US35/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>11 de 12 caixas marcadas (docs/US35/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2266,7 +2266,7 @@
       </c>
       <c r="N17" s="38" t="inlineStr">
         <is>
-          <t>13 de 15 caixas marcadas (docs/US36/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>14 de 15 caixas marcadas (docs/US36/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2334,7 +2334,7 @@
       </c>
       <c r="N18" s="38" t="inlineStr">
         <is>
-          <t>10 de 12 caixas marcadas (docs/US40/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>11 de 12 caixas marcadas (docs/US40/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2400,7 +2400,7 @@
       </c>
       <c r="N19" s="38" t="inlineStr">
         <is>
-          <t>8 de 10 caixas marcadas (docs/US41/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>9 de 10 caixas marcadas (docs/US41/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="N20" s="38" t="inlineStr">
         <is>
-          <t>7 de 9 caixas marcadas (docs/US42/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>8 de 9 caixas marcadas (docs/US42/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2532,7 +2532,7 @@
       </c>
       <c r="N21" s="38" t="inlineStr">
         <is>
-          <t>9 de 11 caixas marcadas (docs/US44/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>10 de 11 caixas marcadas (docs/US44/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2599,7 +2599,7 @@
       </c>
       <c r="N22" s="38" t="inlineStr">
         <is>
-          <t>10 de 12 caixas marcadas (docs/US43/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>11 de 12 caixas marcadas (docs/US43/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2665,7 +2665,7 @@
       </c>
       <c r="N23" s="38" t="inlineStr">
         <is>
-          <t>8 de 10 caixas marcadas (docs/US45/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>9 de 10 caixas marcadas (docs/US45/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2721,7 +2721,7 @@
       <c r="K24" s="38" t="n"/>
       <c r="L24" s="38" t="inlineStr">
         <is>
-          <t>29/10: feita e aceite pelo PO (PR #54). Só com autorização, o LLM recebe os exames e um intervalo da média. Revisão do Simão pendente. A conversa continua só para maiores de 18 (ponto 14 dos requisitos).</t>
+          <t>29/10: feita e aceite pelo PO (PR #54). Só com autorização, o LLM recebe os exames e um intervalo da média. Revisão no GitHub dispensada pelos PO a 31/10. A conversa continua só para maiores de 18 (ponto 14 dos requisitos).</t>
         </is>
       </c>
       <c r="M24" s="35" t="inlineStr">
@@ -2731,7 +2731,7 @@
       </c>
       <c r="N24" s="38" t="inlineStr">
         <is>
-          <t>8 de 10 caixas marcadas (docs/US37/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>9 de 10 caixas marcadas (docs/US37/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2787,7 +2787,7 @@
       <c r="K25" s="38" t="n"/>
       <c r="L25" s="38" t="inlineStr">
         <is>
-          <t>29/10: feita e aceite pelo PO (PR #50). Revisão do Simão pendente. 31/10: a exportação passou a dizer se a pessoa autorizou o assistente a usar as notas (US37).</t>
+          <t>29/10: feita e aceite pelo PO (PR #50). Revisão no GitHub dispensada pelos PO a 31/10. 31/10: a exportação passou a dizer se a pessoa autorizou o assistente a usar as notas (US37).</t>
         </is>
       </c>
       <c r="M25" s="35" t="inlineStr">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="N25" s="38" t="inlineStr">
         <is>
-          <t>9 de 11 caixas marcadas (docs/US46/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>10 de 11 caixas marcadas (docs/US46/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2853,7 @@
       <c r="K26" s="38" t="n"/>
       <c r="L26" s="38" t="inlineStr">
         <is>
-          <t>29/10: feita e aceite pelo PO (PR #51), com envio real de emails por SMTP. Revisão do Simão pendente. 31/10: no máximo 3 emails de recuperação por conta e por hora (RF02.17).</t>
+          <t>29/10: feita e aceite pelo PO (PR #51), com envio real de emails por SMTP. Revisão no GitHub dispensada pelos PO a 31/10. 31/10: no máximo 3 emails de recuperação por conta e por hora (RF02.17).</t>
         </is>
       </c>
       <c r="M26" s="35" t="inlineStr">
@@ -2863,7 +2863,7 @@
       </c>
       <c r="N26" s="38" t="inlineStr">
         <is>
-          <t>10 de 12 caixas marcadas (docs/US47/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>11 de 12 caixas marcadas (docs/US47/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
       <c r="K27" s="38" t="n"/>
       <c r="L27" s="38" t="inlineStr">
         <is>
-          <t>29/10: feita e aceite pelo PO (PR #53). Sem acesso aos dados dos alunos. Revisão do Simão pendente. Medir o desempenho com o catálogo completo (US48).</t>
+          <t>29/10: feita e aceite pelo PO (PR #53). Sem acesso aos dados dos alunos. Revisão no GitHub dispensada pelos PO a 31/10. Medir o desempenho com o catálogo completo (US48).</t>
         </is>
       </c>
       <c r="M27" s="35" t="inlineStr">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="N27" s="38" t="inlineStr">
         <is>
-          <t>9 de 11 caixas marcadas (docs/US39/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>10 de 11 caixas marcadas (docs/US39/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -2985,7 +2985,7 @@
       <c r="K28" s="38" t="n"/>
       <c r="L28" s="38" t="inlineStr">
         <is>
-          <t>29/10: feita e aceite pelo PO (PR #52), com as datas de 2026. Revisão do Simão pendente. Acrescentar as datas de 2027 quando forem publicadas.</t>
+          <t>29/10: feita e aceite pelo PO (PR #52), com as datas de 2026. Revisão no GitHub dispensada pelos PO a 31/10. Acrescentar as datas de 2027 quando forem publicadas.</t>
         </is>
       </c>
       <c r="M28" s="35" t="inlineStr">
@@ -2995,7 +2995,7 @@
       </c>
       <c r="N28" s="38" t="inlineStr">
         <is>
-          <t>7 de 9 caixas marcadas (docs/US38/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11.</t>
+          <t>8 de 9 caixas marcadas (docs/US38/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -3045,13 +3045,13 @@
       </c>
       <c r="J29" s="37" t="inlineStr">
         <is>
-          <t>Em curso</t>
+          <t>Feito</t>
         </is>
       </c>
       <c r="K29" s="38" t="n"/>
       <c r="L29" s="38" t="inlineStr">
         <is>
-          <t>27/10: separada da US04 (decisão do PO). 29/10: recolha corrida pelo PO (1699 cursos, PR #58). 31/10: entra no Sprint 4; o PR #58 tinha ficado no ramo do #57 e só chegou à main no PR de fecho. Falta a aceitação do PO na Sprint Review e a revisão do Simão.</t>
+          <t>27/10: separada da US04 (decisão do PO). 29/10: recolha corrida pelo PO (1699 cursos, PR #58). 31/10: entra no Sprint 4 e é aceite pelo PO; o PR #58 tinha ficado no ramo do #57 e chegou à main no PR #61.</t>
         </is>
       </c>
       <c r="M29" s="35" t="inlineStr">
@@ -3061,7 +3061,7 @@
       </c>
       <c r="N29" s="38" t="inlineStr">
         <is>
-          <t>7 de 10 caixas marcadas (docs/US48/README.md). Falta: revisão do Simão; mostrar na Sprint Review de 05/11; aceitação do PO.</t>
+          <t>9 de 10 caixas marcadas (docs/US48/README.md). Falta: mostrar na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -3189,7 +3189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H123"/>
+  <dimension ref="A1:H129"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="11" customWidth="1" style="30" min="1" max="1"/>
@@ -4054,6 +4054,7 @@
         </is>
       </c>
     </row>
+    <row r="118"/>
     <row r="119">
       <c r="A119" s="55" t="inlineStr">
         <is>
@@ -4064,7 +4065,7 @@
     <row r="120">
       <c r="A120" s="56" t="inlineStr">
         <is>
-          <t>• A US48 entra no Sprint 4 como «Em curso»: o código e os dados estão na main, mas falta o PO aceitá-la na Sprint Review. Se for aceite, o Sprint 4 fica com 49 SP feitos, para uma velocidade de 10.</t>
+          <t>• A US48 entra no Sprint 4 e é aceite pelo PO a 31/10: o Sprint 4 fica com 49 SP feitos, para uma velocidade de 10.</t>
         </is>
       </c>
     </row>
@@ -4078,7 +4079,7 @@
     <row r="122">
       <c r="A122" s="56" t="inlineStr">
         <is>
-          <t>• O que falta em quase todas: a revisão do Simão (nenhum PR tem revisão formal no GitHub) e mostrar as stories do Sprint 4 na Sprint Review de 05/11.</t>
+          <t>• Os Product Owners dispensaram a revisão do código no GitHub (o Simão acompanhou todo o trabalho). Falta só mostrar as stories do Sprint 4 na Sprint Review de 05/11.</t>
         </is>
       </c>
     </row>
@@ -4089,6 +4090,12 @@
         </is>
       </c>
     </row>
+    <row r="124"/>
+    <row r="125"/>
+    <row r="126"/>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
   </sheetData>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.4" right="0.4" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>